<commit_message>
Přidána nová závada ID 742
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E742"/>
+  <dimension ref="A1:E743"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17596,6 +17596,27 @@
       </c>
       <c r="E742" t="inlineStr"/>
     </row>
+    <row r="743">
+      <c r="A743" t="n">
+        <v>742</v>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Smazána závada ID 731
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E743"/>
+  <dimension ref="A1:E742"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17383,53 +17383,49 @@
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
           <t>844 028</t>
         </is>
       </c>
-      <c r="C732" t="inlineStr"/>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>28.01.2026</t>
+        </is>
+      </c>
       <c r="D732" t="inlineStr">
         <is>
-          <t>neukazuje hladinu oleje na A</t>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
         </is>
       </c>
       <c r="E732" t="inlineStr">
         <is>
-          <t>po vytáhnutí a zacvaknutí konektoru OK</t>
+          <t>opraven a vyrobena provizorní krytka</t>
         </is>
       </c>
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C733" t="inlineStr">
-        <is>
-          <t>28.01.2026</t>
-        </is>
-      </c>
+          <t>844 029</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr"/>
       <c r="D733" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E733" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr"/>
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
@@ -17439,14 +17435,14 @@
       <c r="C734" t="inlineStr"/>
       <c r="D734" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E734" t="inlineStr"/>
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
@@ -17456,14 +17452,14 @@
       <c r="C735" t="inlineStr"/>
       <c r="D735" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E735" t="inlineStr"/>
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
@@ -17473,14 +17469,14 @@
       <c r="C736" t="inlineStr"/>
       <c r="D736" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E736" t="inlineStr"/>
     </row>
     <row r="737">
       <c r="A737" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
@@ -17490,35 +17486,35 @@
       <c r="C737" t="inlineStr"/>
       <c r="D737" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E737" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
     </row>
     <row r="738">
       <c r="A738" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C738" t="inlineStr"/>
       <c r="D738" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E738" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr"/>
     </row>
     <row r="739">
       <c r="A739" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B739" t="inlineStr">
         <is>
@@ -17528,56 +17524,60 @@
       <c r="C739" t="inlineStr"/>
       <c r="D739" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E739" t="inlineStr"/>
     </row>
     <row r="740">
       <c r="A740" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>954 212</t>
-        </is>
-      </c>
-      <c r="C740" t="inlineStr"/>
+          <t>954 214</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>29.1:2026</t>
+        </is>
+      </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E740" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
     </row>
     <row r="741">
       <c r="A741" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
         <is>
-          <t>29.1:2026</t>
+          <t>19.08.2026</t>
         </is>
       </c>
       <c r="D741" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E741" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr"/>
     </row>
     <row r="742">
       <c r="A742" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B742" t="inlineStr">
         <is>
@@ -17591,31 +17591,10 @@
       </c>
       <c r="D742" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E742" t="inlineStr"/>
-    </row>
-    <row r="743">
-      <c r="A743" t="n">
-        <v>742</v>
-      </c>
-      <c r="B743" t="inlineStr">
-        <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C743" t="inlineStr">
-        <is>
-          <t>19.08.2026</t>
-        </is>
-      </c>
-      <c r="D743" t="inlineStr">
-        <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E743" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Smazána závada ID 685
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E742"/>
+  <dimension ref="A1:E741"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16529,105 +16529,105 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>029 227</t>
+          <t>714 226</t>
         </is>
       </c>
       <c r="C686" t="inlineStr"/>
-      <c r="D686" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
+      <c r="D686" t="inlineStr"/>
       <c r="E686" t="inlineStr"/>
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>714 226</t>
+          <t>742 263</t>
         </is>
       </c>
       <c r="C687" t="inlineStr"/>
-      <c r="D687" t="inlineStr"/>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="E687" t="inlineStr"/>
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>742 263</t>
+          <t>814  188</t>
         </is>
       </c>
       <c r="C688" t="inlineStr"/>
       <c r="D688" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>výměna obrazovky Lokel na 914</t>
         </is>
       </c>
       <c r="E688" t="inlineStr"/>
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>814  188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E689" t="inlineStr"/>
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="E690" t="inlineStr"/>
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E691" t="inlineStr"/>
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
@@ -16637,35 +16637,35 @@
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E692" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E693" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr"/>
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
@@ -16675,48 +16675,52 @@
       <c r="C694" t="inlineStr"/>
       <c r="D694" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E694" t="inlineStr"/>
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C695" t="inlineStr"/>
       <c r="D695" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E695" t="inlineStr"/>
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C696" t="inlineStr"/>
       <c r="D696" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E696" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
@@ -16726,39 +16730,35 @@
       <c r="C697" t="inlineStr"/>
       <c r="D697" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E697" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>814 118</t>
+          <t>842 011</t>
         </is>
       </c>
       <c r="C698" t="inlineStr"/>
       <c r="D698" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E698" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr"/>
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
@@ -16768,14 +16768,14 @@
       <c r="C699" t="inlineStr"/>
       <c r="D699" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E699" t="inlineStr"/>
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
@@ -16785,14 +16785,14 @@
       <c r="C700" t="inlineStr"/>
       <c r="D700" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E700" t="inlineStr"/>
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
@@ -16802,14 +16802,18 @@
       <c r="C701" t="inlineStr"/>
       <c r="D701" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E701" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
@@ -16819,18 +16823,18 @@
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E702" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
@@ -16840,56 +16844,52 @@
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E703" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr"/>
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>842 011</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E704" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E705" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr"/>
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
@@ -16899,31 +16899,31 @@
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
         </is>
       </c>
       <c r="E706" t="inlineStr"/>
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E707" t="inlineStr"/>
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
@@ -16933,35 +16933,35 @@
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E708" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C709" t="inlineStr"/>
       <c r="D709" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E709" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr"/>
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
@@ -16971,14 +16971,14 @@
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E710" t="inlineStr"/>
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
@@ -16988,31 +16988,31 @@
       <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E711" t="inlineStr"/>
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C712" t="inlineStr"/>
       <c r="D712" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E712" t="inlineStr"/>
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
@@ -17022,14 +17022,18 @@
       <c r="C713" t="inlineStr"/>
       <c r="D713" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="E713" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
@@ -17039,18 +17043,14 @@
       <c r="C714" t="inlineStr"/>
       <c r="D714" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E714" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr"/>
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
@@ -17060,14 +17060,18 @@
       <c r="C715" t="inlineStr"/>
       <c r="D715" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E715" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
@@ -17077,18 +17081,14 @@
       <c r="C716" t="inlineStr"/>
       <c r="D716" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E716" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr"/>
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
@@ -17098,14 +17098,14 @@
       <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E717" t="inlineStr"/>
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
@@ -17115,35 +17115,43 @@
       <c r="C718" t="inlineStr"/>
       <c r="D718" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E718" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
           <t>844 020</t>
         </is>
       </c>
-      <c r="C719" t="inlineStr"/>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>19.1.202ž</t>
+        </is>
+      </c>
       <c r="D719" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E719" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
@@ -17152,48 +17160,40 @@
       </c>
       <c r="C720" t="inlineStr">
         <is>
-          <t>19.1.202ž</t>
+          <t>2.2:2026</t>
         </is>
       </c>
       <c r="D720" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E720" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>844 020</t>
-        </is>
-      </c>
-      <c r="C721" t="inlineStr">
-        <is>
-          <t>2.2:2026</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr"/>
       <c r="D721" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E721" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr"/>
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
@@ -17203,14 +17203,18 @@
       <c r="C722" t="inlineStr"/>
       <c r="D722" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E722" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
@@ -17220,18 +17224,18 @@
       <c r="C723" t="inlineStr"/>
       <c r="D723" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E723" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
@@ -17241,35 +17245,31 @@
       <c r="C724" t="inlineStr"/>
       <c r="D724" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E724" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr"/>
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C725" t="inlineStr"/>
       <c r="D725" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E725" t="inlineStr"/>
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
@@ -17279,14 +17279,14 @@
       <c r="C726" t="inlineStr"/>
       <c r="D726" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E726" t="inlineStr"/>
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
@@ -17296,35 +17296,39 @@
       <c r="C727" t="inlineStr"/>
       <c r="D727" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E727" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C728" t="inlineStr"/>
       <c r="D728" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E728" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
@@ -17334,81 +17338,77 @@
       <c r="C729" t="inlineStr"/>
       <c r="D729" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E729" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C730" t="inlineStr"/>
       <c r="D730" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E730" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr"/>
     </row>
     <row r="731">
       <c r="A731" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>844 026</t>
-        </is>
-      </c>
-      <c r="C731" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>28.01.2026</t>
+        </is>
+      </c>
       <c r="D731" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E731" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C732" t="inlineStr">
-        <is>
-          <t>28.01.2026</t>
-        </is>
-      </c>
+          <t>844 029</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr"/>
       <c r="D732" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E732" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr"/>
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
@@ -17418,14 +17418,14 @@
       <c r="C733" t="inlineStr"/>
       <c r="D733" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E733" t="inlineStr"/>
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
@@ -17435,14 +17435,14 @@
       <c r="C734" t="inlineStr"/>
       <c r="D734" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E734" t="inlineStr"/>
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
@@ -17452,14 +17452,14 @@
       <c r="C735" t="inlineStr"/>
       <c r="D735" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E735" t="inlineStr"/>
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
@@ -17469,35 +17469,35 @@
       <c r="C736" t="inlineStr"/>
       <c r="D736" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E736" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
     </row>
     <row r="737">
       <c r="A737" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C737" t="inlineStr"/>
       <c r="D737" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E737" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr"/>
     </row>
     <row r="738">
       <c r="A738" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
@@ -17507,56 +17507,60 @@
       <c r="C738" t="inlineStr"/>
       <c r="D738" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E738" t="inlineStr"/>
     </row>
     <row r="739">
       <c r="A739" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>954 212</t>
-        </is>
-      </c>
-      <c r="C739" t="inlineStr"/>
+          <t>954 214</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>29.1:2026</t>
+        </is>
+      </c>
       <c r="D739" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E739" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
     </row>
     <row r="740">
       <c r="A740" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C740" t="inlineStr">
         <is>
-          <t>29.1:2026</t>
+          <t>19.08.2026</t>
         </is>
       </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E740" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr"/>
     </row>
     <row r="741">
       <c r="A741" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B741" t="inlineStr">
         <is>
@@ -17570,31 +17574,10 @@
       </c>
       <c r="D741" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E741" t="inlineStr"/>
-    </row>
-    <row r="742">
-      <c r="A742" t="n">
-        <v>742</v>
-      </c>
-      <c r="B742" t="inlineStr">
-        <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C742" t="inlineStr">
-        <is>
-          <t>19.08.2026</t>
-        </is>
-      </c>
-      <c r="D742" t="inlineStr">
-        <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E742" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidána nová závada ID 743
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E741"/>
+  <dimension ref="A1:E742"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17133,11 +17133,7 @@
           <t>844 020</t>
         </is>
       </c>
-      <c r="C719" t="inlineStr">
-        <is>
-          <t>19.1.202ž</t>
-        </is>
-      </c>
+      <c r="C719" t="inlineStr"/>
       <c r="D719" t="inlineStr">
         <is>
           <t>nejdou přeředit směry na žádné straně</t>
@@ -17158,11 +17154,7 @@
           <t>844 020</t>
         </is>
       </c>
-      <c r="C720" t="inlineStr">
-        <is>
-          <t>2.2:2026</t>
-        </is>
-      </c>
+      <c r="C720" t="inlineStr"/>
       <c r="D720" t="inlineStr">
         <is>
           <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
@@ -17521,11 +17513,7 @@
           <t>954 214</t>
         </is>
       </c>
-      <c r="C739" t="inlineStr">
-        <is>
-          <t>29.1:2026</t>
-        </is>
-      </c>
+      <c r="C739" t="inlineStr"/>
       <c r="D739" t="inlineStr">
         <is>
           <t>přijea na poruchu protismyku</t>
@@ -17578,6 +17566,31 @@
         </is>
       </c>
       <c r="E741" t="inlineStr"/>
+    </row>
+    <row r="742">
+      <c r="A742" t="n">
+        <v>743</v>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>814190</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidána nová závada ID 744
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E742"/>
+  <dimension ref="A1:E743"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,7 +475,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-11-02</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2025-08-11</t>
+          <t>2025-11-08</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2025-11-10</t>
+          <t>2025-10-11</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2025-11-10</t>
+          <t>2025-10-11</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2025-08-10</t>
+          <t>2025-10-08</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2025-08-10</t>
+          <t>2025-10-08</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2025-07-10</t>
+          <t>2025-10-07</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2025-07-10</t>
+          <t>2025-10-07</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2025-05-10</t>
+          <t>2025-10-05</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2025-03-10</t>
+          <t>2025-10-03</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2025-03-10</t>
+          <t>2025-10-03</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2025-07-09</t>
+          <t>2025-09-07</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2025-07-09</t>
+          <t>2025-09-07</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>2025-09-05</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2025-04-09</t>
+          <t>2025-09-04</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2025-01-09</t>
+          <t>2025-09-01</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2025-08-12</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2025-01-08</t>
+          <t>2025-08-01</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2025-01-08</t>
+          <t>2025-08-01</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2025-08-07</t>
+          <t>2025-07-08</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2025-11-06</t>
+          <t>2025-06-11</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-05-12</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-05-12</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-05-12</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-05-12</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2025-09-05</t>
+          <t>2025-05-09</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2025-06-04</t>
+          <t>2025-04-06</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2025-06-04</t>
+          <t>2025-04-06</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2025-06-04</t>
+          <t>2025-04-06</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2025-02-04</t>
+          <t>2025-04-02</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-02-12</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-02-12</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2025-03-02</t>
+          <t>2025-02-03</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -3640,7 +3640,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2025-03-02</t>
+          <t>2025-02-03</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2025-03-02</t>
+          <t>2025-02-03</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-01-12</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2024-03-12</t>
+          <t>2024-12-03</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2024-03-12</t>
+          <t>2024-12-03</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -3988,7 +3988,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2024-11-10</t>
+          <t>2024-10-11</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -4013,7 +4013,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2024-11-10</t>
+          <t>2024-10-11</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2024-08-10</t>
+          <t>2024-10-08</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -4088,7 +4088,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2024-02-10</t>
+          <t>2024-10-02</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2024-12-09</t>
+          <t>2024-09-12</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -4252,7 +4252,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2024-02-09</t>
+          <t>2024-09-02</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -4622,7 +4622,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2024-11-08</t>
+          <t>2024-08-11</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2024-11-08</t>
+          <t>2024-08-11</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2024-11-08</t>
+          <t>2024-08-11</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2024-10-08</t>
+          <t>2024-08-10</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2024-10-08</t>
+          <t>2024-08-10</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -4739,7 +4739,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2024-07-08</t>
+          <t>2024-08-07</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>2024-07-08</t>
+          <t>2024-08-07</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -4789,7 +4789,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>2024-07-08</t>
+          <t>2024-08-07</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>2024-05-08</t>
+          <t>2024-08-05</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -4835,7 +4835,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>2024-05-08</t>
+          <t>2024-08-05</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -4856,7 +4856,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>2024-02-08</t>
+          <t>2024-08-02</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -4877,7 +4877,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>2024-02-08</t>
+          <t>2024-08-02</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -4898,7 +4898,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>2024-01-08</t>
+          <t>2024-08-01</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>2024-12-07</t>
+          <t>2024-07-12</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>2024-10-07</t>
+          <t>2024-07-10</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>2024-10-07</t>
+          <t>2024-07-10</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -5388,7 +5388,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>2024-10-07</t>
+          <t>2024-07-10</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -5409,7 +5409,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>2024-09-07</t>
+          <t>2024-07-09</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>2024-09-07</t>
+          <t>2024-07-09</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -5451,7 +5451,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>2024-08-07</t>
+          <t>2024-07-08</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -5476,7 +5476,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>2024-06-07</t>
+          <t>2024-07-06</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -5497,7 +5497,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>2024-02-07</t>
+          <t>2024-07-02</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>2024-02-07</t>
+          <t>2024-07-02</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>2024-02-07</t>
+          <t>2024-07-02</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>2024-02-07</t>
+          <t>2024-07-02</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -5813,7 +5813,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2024-04-06</t>
+          <t>2024-06-04</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -5838,7 +5838,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2024-01-06</t>
+          <t>2024-06-01</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2024-08-05</t>
+          <t>2024-05-08</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -6112,7 +6112,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>2024-12-04</t>
+          <t>2024-04-12</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>2024-11-04</t>
+          <t>2024-04-11</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -6154,7 +6154,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>2024-09-04</t>
+          <t>2024-04-09</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2024-08-04</t>
+          <t>2024-04-08</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -6196,7 +6196,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>2024-08-04</t>
+          <t>2024-04-08</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -6217,7 +6217,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>2024-07-04</t>
+          <t>2024-04-07</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -6238,7 +6238,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>2024-07-04</t>
+          <t>2024-04-07</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -6259,7 +6259,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>2024-05-04</t>
+          <t>2024-04-05</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>2024-05-04</t>
+          <t>2024-04-05</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>2024-03-04</t>
+          <t>2024-04-03</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2024-03-04</t>
+          <t>2024-04-03</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -6385,7 +6385,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2024-03-04</t>
+          <t>2024-04-03</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -6410,7 +6410,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2024-01-04</t>
+          <t>2024-04-01</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -6952,7 +6952,7 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>2024-12-03</t>
+          <t>2024-03-12</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
@@ -6973,7 +6973,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>2024-12-03</t>
+          <t>2024-03-12</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
@@ -6994,7 +6994,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>2024-12-03</t>
+          <t>2024-03-12</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
@@ -7015,7 +7015,7 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>2024-10-03</t>
+          <t>2024-03-10</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
@@ -7036,7 +7036,7 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>2024-10-03</t>
+          <t>2024-03-10</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
@@ -7057,7 +7057,7 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>2024-10-03</t>
+          <t>2024-03-10</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
@@ -7330,7 +7330,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>2023-08-12</t>
+          <t>2023-12-08</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>2023-07-11</t>
+          <t>2023-11-07</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
@@ -7607,7 +7607,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>2023-12-10</t>
+          <t>2023-10-12</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>2023-08-10</t>
+          <t>2023-10-08</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
@@ -7653,7 +7653,7 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>2023-08-10</t>
+          <t>2023-10-08</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>2023-08-10</t>
+          <t>2023-10-08</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
@@ -7703,7 +7703,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>2023-07-10</t>
+          <t>2023-10-07</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
@@ -7728,7 +7728,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>2023-05-10</t>
+          <t>2023-10-05</t>
         </is>
       </c>
       <c r="D352" t="inlineStr">
@@ -7753,7 +7753,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>2023-04-10</t>
+          <t>2023-10-04</t>
         </is>
       </c>
       <c r="D353" t="inlineStr"/>
@@ -7774,7 +7774,7 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>2023-04-10</t>
+          <t>2023-10-04</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
@@ -7795,7 +7795,7 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>2023-04-10</t>
+          <t>2023-10-04</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
@@ -7820,7 +7820,7 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>2023-02-10</t>
+          <t>2023-10-02</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
@@ -7845,7 +7845,7 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>2023-02-10</t>
+          <t>2023-10-02</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
@@ -7870,7 +7870,7 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>2023-02-10</t>
+          <t>2023-10-02</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>2023-02-10</t>
+          <t>2023-10-02</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
@@ -7916,7 +7916,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>2023-02-10</t>
+          <t>2023-10-02</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
@@ -8665,7 +8665,7 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>2023-12-09</t>
+          <t>2023-09-12</t>
         </is>
       </c>
       <c r="D397" t="inlineStr">
@@ -8690,7 +8690,7 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>2023-12-09</t>
+          <t>2023-09-12</t>
         </is>
       </c>
       <c r="D398" t="inlineStr">
@@ -8715,7 +8715,7 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>2023-12-09</t>
+          <t>2023-09-12</t>
         </is>
       </c>
       <c r="D399" t="inlineStr">
@@ -8736,7 +8736,7 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>2023-12-09</t>
+          <t>2023-09-12</t>
         </is>
       </c>
       <c r="D400" t="inlineStr">
@@ -8803,7 +8803,7 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>2023-06-09</t>
+          <t>2023-09-06</t>
         </is>
       </c>
       <c r="D403" t="inlineStr">
@@ -9649,7 +9649,7 @@
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>2023-12-08</t>
+          <t>2023-08-12</t>
         </is>
       </c>
       <c r="D445" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>2023-12-08</t>
+          <t>2023-08-12</t>
         </is>
       </c>
       <c r="D446" t="inlineStr"/>
@@ -9695,7 +9695,7 @@
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>2023-12-08</t>
+          <t>2023-08-12</t>
         </is>
       </c>
       <c r="D447" t="inlineStr"/>
@@ -9716,7 +9716,7 @@
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>2023-12-08</t>
+          <t>2023-08-12</t>
         </is>
       </c>
       <c r="D448" t="inlineStr">
@@ -9737,7 +9737,7 @@
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>2023-09-08</t>
+          <t>2023-08-09</t>
         </is>
       </c>
       <c r="D449" t="inlineStr">
@@ -9758,7 +9758,7 @@
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>2023-09-08</t>
+          <t>2023-08-09</t>
         </is>
       </c>
       <c r="D450" t="inlineStr">
@@ -9783,7 +9783,7 @@
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>2023-07-08</t>
+          <t>2023-08-07</t>
         </is>
       </c>
       <c r="D451" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>2023-06-08</t>
+          <t>2023-08-06</t>
         </is>
       </c>
       <c r="D452" t="inlineStr">
@@ -9833,7 +9833,7 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>2023-06-08</t>
+          <t>2023-08-06</t>
         </is>
       </c>
       <c r="D453" t="inlineStr">
@@ -9858,7 +9858,7 @@
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>2023-06-08</t>
+          <t>2023-08-06</t>
         </is>
       </c>
       <c r="D454" t="inlineStr">
@@ -9883,7 +9883,7 @@
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>2023-06-08</t>
+          <t>2023-08-06</t>
         </is>
       </c>
       <c r="D455" t="inlineStr">
@@ -9908,7 +9908,7 @@
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>2023-06-08</t>
+          <t>2023-08-06</t>
         </is>
       </c>
       <c r="D456" t="inlineStr">
@@ -9933,7 +9933,7 @@
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>2023-04-08</t>
+          <t>2023-08-04</t>
         </is>
       </c>
       <c r="D457" t="inlineStr">
@@ -9958,7 +9958,7 @@
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>2023-04-08</t>
+          <t>2023-08-04</t>
         </is>
       </c>
       <c r="D458" t="inlineStr">
@@ -9983,7 +9983,7 @@
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>2023-03-08</t>
+          <t>2023-08-03</t>
         </is>
       </c>
       <c r="D459" t="inlineStr">
@@ -10008,7 +10008,7 @@
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>2023-03-08</t>
+          <t>2023-08-03</t>
         </is>
       </c>
       <c r="D460" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>2023-03-08</t>
+          <t>2023-08-03</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>2023-02-08</t>
+          <t>2023-08-02</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>2023-02-08</t>
+          <t>2023-08-02</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
@@ -10104,7 +10104,7 @@
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>2023-02-08</t>
+          <t>2023-08-02</t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
@@ -10129,7 +10129,7 @@
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>2023-02-08</t>
+          <t>2023-08-02</t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>2023-01-08</t>
+          <t>2023-08-01</t>
         </is>
       </c>
       <c r="D466" t="inlineStr">
@@ -10179,7 +10179,7 @@
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>2023-01-08</t>
+          <t>2023-08-01</t>
         </is>
       </c>
       <c r="D467" t="inlineStr">
@@ -10204,7 +10204,7 @@
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>2023-01-08</t>
+          <t>2023-08-01</t>
         </is>
       </c>
       <c r="D468" t="inlineStr">
@@ -11169,7 +11169,7 @@
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>2023-12-07</t>
+          <t>2023-07-12</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
@@ -11194,7 +11194,7 @@
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>2023-12-07</t>
+          <t>2023-07-12</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
@@ -11219,7 +11219,7 @@
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>2023-12-07</t>
+          <t>2023-07-12</t>
         </is>
       </c>
       <c r="D519" t="inlineStr"/>
@@ -11240,7 +11240,7 @@
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>2023-11-07</t>
+          <t>2023-07-11</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
@@ -11265,7 +11265,7 @@
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>2023-11-07</t>
+          <t>2023-07-11</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
@@ -11290,7 +11290,7 @@
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>2023-11-07</t>
+          <t>2023-07-11</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
@@ -11311,7 +11311,7 @@
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>2023-11-07</t>
+          <t>2023-07-11</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
@@ -11336,7 +11336,7 @@
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>2023-10-07</t>
+          <t>2023-07-10</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
@@ -11357,7 +11357,7 @@
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>2023-10-07</t>
+          <t>2023-07-10</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
@@ -11382,7 +11382,7 @@
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>2023-10-07</t>
+          <t>2023-07-10</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>2023-09-07</t>
+          <t>2023-07-09</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
@@ -11428,7 +11428,7 @@
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>2023-09-07</t>
+          <t>2023-07-09</t>
         </is>
       </c>
       <c r="D528" t="inlineStr"/>
@@ -11449,7 +11449,7 @@
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>2023-09-07</t>
+          <t>2023-07-09</t>
         </is>
       </c>
       <c r="D529" t="inlineStr"/>
@@ -11470,7 +11470,7 @@
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>2023-08-07</t>
+          <t>2023-07-08</t>
         </is>
       </c>
       <c r="D530" t="inlineStr">
@@ -11495,7 +11495,7 @@
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>2023-08-07</t>
+          <t>2023-07-08</t>
         </is>
       </c>
       <c r="D531" t="inlineStr"/>
@@ -11516,7 +11516,7 @@
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>2023-08-07</t>
+          <t>2023-07-08</t>
         </is>
       </c>
       <c r="D532" t="inlineStr">
@@ -11566,7 +11566,7 @@
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>2023-06-07</t>
+          <t>2023-07-06</t>
         </is>
       </c>
       <c r="D534" t="inlineStr"/>
@@ -11587,7 +11587,7 @@
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>2023-06-07</t>
+          <t>2023-07-06</t>
         </is>
       </c>
       <c r="D535" t="inlineStr">
@@ -11612,7 +11612,7 @@
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>2023-06-07</t>
+          <t>2023-07-06</t>
         </is>
       </c>
       <c r="D536" t="inlineStr">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>2023-06-07</t>
+          <t>2023-07-06</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>2023-05-07</t>
+          <t>2023-07-05</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
@@ -11683,7 +11683,7 @@
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>2023-05-07</t>
+          <t>2023-07-05</t>
         </is>
       </c>
       <c r="D539" t="inlineStr"/>
@@ -11704,7 +11704,7 @@
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>2023-05-07</t>
+          <t>2023-07-05</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
@@ -11729,7 +11729,7 @@
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>2023-05-07</t>
+          <t>2023-07-05</t>
         </is>
       </c>
       <c r="D541" t="inlineStr">
@@ -11754,7 +11754,7 @@
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>2023-04-07</t>
+          <t>2023-07-04</t>
         </is>
       </c>
       <c r="D542" t="inlineStr">
@@ -11779,7 +11779,7 @@
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>2023-04-07</t>
+          <t>2023-07-04</t>
         </is>
       </c>
       <c r="D543" t="inlineStr">
@@ -11800,7 +11800,7 @@
       </c>
       <c r="C544" t="inlineStr">
         <is>
-          <t>2023-04-07</t>
+          <t>2023-07-04</t>
         </is>
       </c>
       <c r="D544" t="inlineStr"/>
@@ -11821,7 +11821,7 @@
       </c>
       <c r="C545" t="inlineStr">
         <is>
-          <t>2023-04-07</t>
+          <t>2023-07-04</t>
         </is>
       </c>
       <c r="D545" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="C546" t="inlineStr">
         <is>
-          <t>2023-03-07</t>
+          <t>2023-07-03</t>
         </is>
       </c>
       <c r="D546" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="C547" t="inlineStr">
         <is>
-          <t>2023-03-07</t>
+          <t>2023-07-03</t>
         </is>
       </c>
       <c r="D547" t="inlineStr">
@@ -11896,7 +11896,7 @@
       </c>
       <c r="C548" t="inlineStr">
         <is>
-          <t>2023-02-07</t>
+          <t>2023-07-02</t>
         </is>
       </c>
       <c r="D548" t="inlineStr">
@@ -11921,7 +11921,7 @@
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>2023-01-07</t>
+          <t>2023-07-01</t>
         </is>
       </c>
       <c r="D549" t="inlineStr">
@@ -11942,7 +11942,7 @@
       </c>
       <c r="C550" t="inlineStr">
         <is>
-          <t>2023-01-07</t>
+          <t>2023-07-01</t>
         </is>
       </c>
       <c r="D550" t="inlineStr">
@@ -11967,7 +11967,7 @@
       </c>
       <c r="C551" t="inlineStr">
         <is>
-          <t>2023-01-07</t>
+          <t>2023-07-01</t>
         </is>
       </c>
       <c r="D551" t="inlineStr">
@@ -11992,7 +11992,7 @@
       </c>
       <c r="C552" t="inlineStr">
         <is>
-          <t>2023-01-07</t>
+          <t>2023-07-01</t>
         </is>
       </c>
       <c r="D552" t="inlineStr">
@@ -12017,7 +12017,7 @@
       </c>
       <c r="C553" t="inlineStr">
         <is>
-          <t>2023-01-07</t>
+          <t>2023-07-01</t>
         </is>
       </c>
       <c r="D553" t="inlineStr">
@@ -12042,7 +12042,7 @@
       </c>
       <c r="C554" t="inlineStr">
         <is>
-          <t>2023-01-07</t>
+          <t>2023-07-01</t>
         </is>
       </c>
       <c r="D554" t="inlineStr">
@@ -13249,7 +13249,7 @@
       </c>
       <c r="C613" t="inlineStr">
         <is>
-          <t>2023-12-06</t>
+          <t>2023-06-12</t>
         </is>
       </c>
       <c r="D613" t="inlineStr">
@@ -13270,7 +13270,7 @@
       </c>
       <c r="C614" t="inlineStr">
         <is>
-          <t>2023-12-06</t>
+          <t>2023-06-12</t>
         </is>
       </c>
       <c r="D614" t="inlineStr">
@@ -13291,7 +13291,7 @@
       </c>
       <c r="C615" t="inlineStr">
         <is>
-          <t>2023-12-06</t>
+          <t>2023-06-12</t>
         </is>
       </c>
       <c r="D615" t="inlineStr">
@@ -13312,7 +13312,7 @@
       </c>
       <c r="C616" t="inlineStr">
         <is>
-          <t>2023-11-06</t>
+          <t>2023-06-11</t>
         </is>
       </c>
       <c r="D616" t="inlineStr">
@@ -13337,7 +13337,7 @@
       </c>
       <c r="C617" t="inlineStr">
         <is>
-          <t>2023-11-06</t>
+          <t>2023-06-11</t>
         </is>
       </c>
       <c r="D617" t="inlineStr">
@@ -13362,7 +13362,7 @@
       </c>
       <c r="C618" t="inlineStr">
         <is>
-          <t>2023-11-06</t>
+          <t>2023-06-11</t>
         </is>
       </c>
       <c r="D618" t="inlineStr">
@@ -13383,7 +13383,7 @@
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>2023-10-06</t>
+          <t>2023-06-10</t>
         </is>
       </c>
       <c r="D619" t="inlineStr">
@@ -13408,7 +13408,7 @@
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>2023-10-06</t>
+          <t>2023-06-10</t>
         </is>
       </c>
       <c r="D620" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="C621" t="inlineStr">
         <is>
-          <t>2023-10-06</t>
+          <t>2023-06-10</t>
         </is>
       </c>
       <c r="D621" t="inlineStr">
@@ -13454,7 +13454,7 @@
       </c>
       <c r="C622" t="inlineStr">
         <is>
-          <t>2023-09-06</t>
+          <t>2023-06-09</t>
         </is>
       </c>
       <c r="D622" t="inlineStr">
@@ -13479,7 +13479,7 @@
       </c>
       <c r="C623" t="inlineStr">
         <is>
-          <t>2023-09-06</t>
+          <t>2023-06-09</t>
         </is>
       </c>
       <c r="D623" t="inlineStr">
@@ -13504,7 +13504,7 @@
       </c>
       <c r="C624" t="inlineStr">
         <is>
-          <t>2023-09-06</t>
+          <t>2023-06-09</t>
         </is>
       </c>
       <c r="D624" t="inlineStr">
@@ -13529,7 +13529,7 @@
       </c>
       <c r="C625" t="inlineStr">
         <is>
-          <t>2023-08-06</t>
+          <t>2023-06-08</t>
         </is>
       </c>
       <c r="D625" t="inlineStr">
@@ -13554,7 +13554,7 @@
       </c>
       <c r="C626" t="inlineStr">
         <is>
-          <t>2023-08-06</t>
+          <t>2023-06-08</t>
         </is>
       </c>
       <c r="D626" t="inlineStr">
@@ -13579,7 +13579,7 @@
       </c>
       <c r="C627" t="inlineStr">
         <is>
-          <t>2023-08-06</t>
+          <t>2023-06-08</t>
         </is>
       </c>
       <c r="D627" t="inlineStr">
@@ -13604,7 +13604,7 @@
       </c>
       <c r="C628" t="inlineStr">
         <is>
-          <t>2023-08-06</t>
+          <t>2023-06-08</t>
         </is>
       </c>
       <c r="D628" t="inlineStr">
@@ -13629,7 +13629,7 @@
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>2023-07-06</t>
+          <t>2023-06-07</t>
         </is>
       </c>
       <c r="D629" t="inlineStr">
@@ -13654,7 +13654,7 @@
       </c>
       <c r="C630" t="inlineStr">
         <is>
-          <t>2023-07-06</t>
+          <t>2023-06-07</t>
         </is>
       </c>
       <c r="D630" t="inlineStr">
@@ -13675,7 +13675,7 @@
       </c>
       <c r="C631" t="inlineStr">
         <is>
-          <t>2023-07-06</t>
+          <t>2023-06-07</t>
         </is>
       </c>
       <c r="D631" t="inlineStr">
@@ -13721,7 +13721,7 @@
       </c>
       <c r="C633" t="inlineStr">
         <is>
-          <t>2023-05-06</t>
+          <t>2023-06-05</t>
         </is>
       </c>
       <c r="D633" t="inlineStr">
@@ -13894,7 +13894,7 @@
       </c>
       <c r="C642" t="inlineStr">
         <is>
-          <t>2023-12-04</t>
+          <t>2023-04-12</t>
         </is>
       </c>
       <c r="D642" t="inlineStr">
@@ -14046,7 +14046,7 @@
       </c>
       <c r="C650" t="inlineStr">
         <is>
-          <t>2023-09-02</t>
+          <t>2023-02-09</t>
         </is>
       </c>
       <c r="D650" t="inlineStr">
@@ -14067,7 +14067,7 @@
       </c>
       <c r="C651" t="inlineStr">
         <is>
-          <t>2023-03-02</t>
+          <t>2023-02-03</t>
         </is>
       </c>
       <c r="D651" t="inlineStr">
@@ -14147,7 +14147,7 @@
       </c>
       <c r="C655" t="inlineStr">
         <is>
-          <t>2023-10-01</t>
+          <t>2023-01-10</t>
         </is>
       </c>
       <c r="D655" t="inlineStr">
@@ -14240,7 +14240,7 @@
       </c>
       <c r="C660" t="inlineStr">
         <is>
-          <t>2022-06-12</t>
+          <t>2022-12-06</t>
         </is>
       </c>
       <c r="D660" t="inlineStr">
@@ -14265,7 +14265,7 @@
       </c>
       <c r="C661" t="inlineStr">
         <is>
-          <t>2022-06-12</t>
+          <t>2022-12-06</t>
         </is>
       </c>
       <c r="D661" t="inlineStr">
@@ -14286,7 +14286,7 @@
       </c>
       <c r="C662" t="inlineStr">
         <is>
-          <t>2022-03-12</t>
+          <t>2022-12-03</t>
         </is>
       </c>
       <c r="D662" t="inlineStr">
@@ -14353,7 +14353,7 @@
       </c>
       <c r="C665" t="inlineStr">
         <is>
-          <t>2022-06-11</t>
+          <t>2022-11-06</t>
         </is>
       </c>
       <c r="D665" t="inlineStr">
@@ -14374,7 +14374,7 @@
       </c>
       <c r="C666" t="inlineStr">
         <is>
-          <t>2022-06-11</t>
+          <t>2022-11-06</t>
         </is>
       </c>
       <c r="D666" t="inlineStr">
@@ -14395,7 +14395,7 @@
       </c>
       <c r="C667" t="inlineStr">
         <is>
-          <t>2022-06-11</t>
+          <t>2022-11-06</t>
         </is>
       </c>
       <c r="D667" t="inlineStr">
@@ -14420,7 +14420,7 @@
       </c>
       <c r="C668" t="inlineStr">
         <is>
-          <t>2022-05-11</t>
+          <t>2022-11-05</t>
         </is>
       </c>
       <c r="D668" t="inlineStr">
@@ -14445,7 +14445,7 @@
       </c>
       <c r="C669" t="inlineStr">
         <is>
-          <t>2022-05-11</t>
+          <t>2022-11-05</t>
         </is>
       </c>
       <c r="D669" t="inlineStr">
@@ -14525,7 +14525,7 @@
       </c>
       <c r="C673" t="inlineStr">
         <is>
-          <t>2022-07-09</t>
+          <t>2022-09-07</t>
         </is>
       </c>
       <c r="D673" t="inlineStr">
@@ -14550,7 +14550,7 @@
       </c>
       <c r="C674" t="inlineStr">
         <is>
-          <t>2022-03-09</t>
+          <t>2022-09-03</t>
         </is>
       </c>
       <c r="D674" t="inlineStr">
@@ -14659,7 +14659,7 @@
       </c>
       <c r="C679" t="inlineStr">
         <is>
-          <t>2021-08-10</t>
+          <t>2021-10-08</t>
         </is>
       </c>
       <c r="D679" t="inlineStr">
@@ -14705,7 +14705,7 @@
       </c>
       <c r="C681" t="inlineStr">
         <is>
-          <t>2021-06-09</t>
+          <t>2021-09-06</t>
         </is>
       </c>
       <c r="D681" t="inlineStr">
@@ -15825,6 +15825,31 @@
       <c r="E742" t="inlineStr">
         <is>
           <t>asdasd</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="n">
+        <v>744</v>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>814 190</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>testik</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>test</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Úprava závady ID 744
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -454,7 +454,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2021-01-01</t>
+          <t>01.01.2021</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -475,7 +475,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>04.06.2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>04.05.2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>04.05.2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>04.04.2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>03.10.2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>03.10.2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>03.08.2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>02.11.2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>02.03.2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>02.02.2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>02.01.2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>01.09.2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>01.07.2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>01.05.2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2025-11-11</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2025-11-08</t>
+          <t>11.08.2025</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2025-10-11</t>
+          <t>10.11.2025</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2025-10-11</t>
+          <t>10.11.2025</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2025-10-10</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2025-10-08</t>
+          <t>10.08.2025</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2025-10-08</t>
+          <t>10.08.2025</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2025-10-07</t>
+          <t>10.07.2025</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2025-10-07</t>
+          <t>10.07.2025</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2025-10-05</t>
+          <t>10.05.2025</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2025-10-03</t>
+          <t>10.03.2025</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2025-10-03</t>
+          <t>10.03.2025</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2025-09-07</t>
+          <t>09.07.2025</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2025-09-07</t>
+          <t>09.07.2025</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2025-09-05</t>
+          <t>09.05.2025</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2025-09-04</t>
+          <t>09.04.2025</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2025-09-01</t>
+          <t>09.01.2025</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2025-08-12</t>
+          <t>08.12.2025</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2025-08-01</t>
+          <t>08.01.2025</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2025-08-01</t>
+          <t>08.01.2025</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2025-07-08</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2025-06-11</t>
+          <t>06.11.2025</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2025-06-06</t>
+          <t>06.06.2025</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2025-06-06</t>
+          <t>06.06.2025</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2025-05-12</t>
+          <t>05.12.2025</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2025-05-12</t>
+          <t>05.12.2025</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2025-05-12</t>
+          <t>05.12.2025</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2025-05-12</t>
+          <t>05.12.2025</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>05.09.2025</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2025-04-06</t>
+          <t>04.06.2025</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2025-04-06</t>
+          <t>04.06.2025</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2025-04-06</t>
+          <t>04.06.2025</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2025-04-02</t>
+          <t>04.02.2025</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2025-02-12</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2025-02-12</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2025-02-03</t>
+          <t>02.03.2025</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -3640,7 +3640,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2025-02-03</t>
+          <t>02.03.2025</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2025-02-03</t>
+          <t>02.03.2025</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2025-01-12</t>
+          <t>01.12.2025</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2024-12-03</t>
+          <t>12.03.2024</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2024-12-03</t>
+          <t>12.03.2024</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -3900,7 +3900,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2024-11-11</t>
+          <t>11.11.2024</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -3988,7 +3988,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2024-10-11</t>
+          <t>10.11.2024</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -4013,7 +4013,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2024-10-11</t>
+          <t>10.11.2024</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2024-10-10</t>
+          <t>10.10.2024</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2024-10-08</t>
+          <t>10.08.2024</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -4088,7 +4088,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2024-10-02</t>
+          <t>10.02.2024</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2024-09-12</t>
+          <t>09.12.2024</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -4252,7 +4252,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2024-09-02</t>
+          <t>09.02.2024</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -4622,7 +4622,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2024-08-11</t>
+          <t>08.11.2024</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2024-08-11</t>
+          <t>08.11.2024</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2024-08-11</t>
+          <t>08.11.2024</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2024-08-10</t>
+          <t>08.10.2024</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2024-08-10</t>
+          <t>08.10.2024</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -4739,7 +4739,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2024-08-07</t>
+          <t>08.07.2024</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>2024-08-07</t>
+          <t>08.07.2024</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -4789,7 +4789,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>2024-08-07</t>
+          <t>08.07.2024</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>2024-08-05</t>
+          <t>08.05.2024</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -4835,7 +4835,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>2024-08-05</t>
+          <t>08.05.2024</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -4856,7 +4856,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
+          <t>08.02.2024</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -4877,7 +4877,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
+          <t>08.02.2024</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -4898,7 +4898,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>2024-08-01</t>
+          <t>08.01.2024</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>2024-07-12</t>
+          <t>07.12.2024</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>2024-07-10</t>
+          <t>07.10.2024</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>2024-07-10</t>
+          <t>07.10.2024</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -5388,7 +5388,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>2024-07-10</t>
+          <t>07.10.2024</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -5409,7 +5409,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>2024-07-09</t>
+          <t>07.09.2024</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>2024-07-09</t>
+          <t>07.09.2024</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -5451,7 +5451,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>2024-07-08</t>
+          <t>07.08.2024</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -5476,7 +5476,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>2024-07-06</t>
+          <t>07.06.2024</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -5497,7 +5497,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>2024-07-02</t>
+          <t>07.02.2024</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>2024-07-02</t>
+          <t>07.02.2024</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>2024-07-02</t>
+          <t>07.02.2024</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>2024-07-02</t>
+          <t>07.02.2024</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -5813,7 +5813,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2024-06-04</t>
+          <t>06.04.2024</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -5838,7 +5838,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2024-06-01</t>
+          <t>06.01.2024</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2024-05-08</t>
+          <t>05.08.2024</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -6112,7 +6112,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>2024-04-12</t>
+          <t>04.12.2024</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>2024-04-11</t>
+          <t>04.11.2024</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -6154,7 +6154,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>2024-04-09</t>
+          <t>04.09.2024</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2024-04-08</t>
+          <t>04.08.2024</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -6196,7 +6196,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>2024-04-08</t>
+          <t>04.08.2024</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -6217,7 +6217,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>2024-04-07</t>
+          <t>04.07.2024</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -6238,7 +6238,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>2024-04-07</t>
+          <t>04.07.2024</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -6259,7 +6259,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>2024-04-05</t>
+          <t>04.05.2024</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>2024-04-05</t>
+          <t>04.05.2024</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -6301,7 +6301,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>2024-04-04</t>
+          <t>04.04.2024</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -6322,7 +6322,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>2024-04-04</t>
+          <t>04.04.2024</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>2024-04-03</t>
+          <t>04.03.2024</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2024-04-03</t>
+          <t>04.03.2024</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -6385,7 +6385,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2024-04-03</t>
+          <t>04.03.2024</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -6410,7 +6410,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2024-04-01</t>
+          <t>04.01.2024</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -6952,7 +6952,7 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>2024-03-12</t>
+          <t>03.12.2024</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
@@ -6973,7 +6973,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>2024-03-12</t>
+          <t>03.12.2024</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
@@ -6994,7 +6994,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>2024-03-12</t>
+          <t>03.12.2024</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
@@ -7015,7 +7015,7 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>2024-03-10</t>
+          <t>03.10.2024</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
@@ -7036,7 +7036,7 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>2024-03-10</t>
+          <t>03.10.2024</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
@@ -7057,7 +7057,7 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>2024-03-10</t>
+          <t>03.10.2024</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>2024-03-03</t>
+          <t>03.03.2024</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
@@ -7330,7 +7330,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>2023-12-08</t>
+          <t>12.08.2023</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>2023-11-07</t>
+          <t>11.07.2023</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
@@ -7607,7 +7607,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>2023-10-12</t>
+          <t>10.12.2023</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>2023-10-08</t>
+          <t>10.08.2023</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
@@ -7653,7 +7653,7 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>2023-10-08</t>
+          <t>10.08.2023</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>2023-10-08</t>
+          <t>10.08.2023</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
@@ -7703,7 +7703,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>2023-10-07</t>
+          <t>10.07.2023</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
@@ -7728,7 +7728,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>2023-10-05</t>
+          <t>10.05.2023</t>
         </is>
       </c>
       <c r="D352" t="inlineStr">
@@ -7753,7 +7753,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>2023-10-04</t>
+          <t>10.04.2023</t>
         </is>
       </c>
       <c r="D353" t="inlineStr"/>
@@ -7774,7 +7774,7 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>2023-10-04</t>
+          <t>10.04.2023</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
@@ -7795,7 +7795,7 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>2023-10-04</t>
+          <t>10.04.2023</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
@@ -7820,7 +7820,7 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>2023-10-02</t>
+          <t>10.02.2023</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
@@ -7845,7 +7845,7 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>2023-10-02</t>
+          <t>10.02.2023</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
@@ -7870,7 +7870,7 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>2023-10-02</t>
+          <t>10.02.2023</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>2023-10-02</t>
+          <t>10.02.2023</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
@@ -7916,7 +7916,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>2023-10-02</t>
+          <t>10.02.2023</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
@@ -8665,7 +8665,7 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>2023-09-12</t>
+          <t>09.12.2023</t>
         </is>
       </c>
       <c r="D397" t="inlineStr">
@@ -8690,7 +8690,7 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>2023-09-12</t>
+          <t>09.12.2023</t>
         </is>
       </c>
       <c r="D398" t="inlineStr">
@@ -8715,7 +8715,7 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>2023-09-12</t>
+          <t>09.12.2023</t>
         </is>
       </c>
       <c r="D399" t="inlineStr">
@@ -8736,7 +8736,7 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>2023-09-12</t>
+          <t>09.12.2023</t>
         </is>
       </c>
       <c r="D400" t="inlineStr">
@@ -8757,7 +8757,7 @@
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>2023-09-09</t>
+          <t>09.09.2023</t>
         </is>
       </c>
       <c r="D401" t="inlineStr">
@@ -8778,7 +8778,7 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>2023-09-09</t>
+          <t>09.09.2023</t>
         </is>
       </c>
       <c r="D402" t="inlineStr">
@@ -8803,7 +8803,7 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>2023-09-06</t>
+          <t>09.06.2023</t>
         </is>
       </c>
       <c r="D403" t="inlineStr">
@@ -9649,7 +9649,7 @@
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>2023-08-12</t>
+          <t>08.12.2023</t>
         </is>
       </c>
       <c r="D445" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>2023-08-12</t>
+          <t>08.12.2023</t>
         </is>
       </c>
       <c r="D446" t="inlineStr"/>
@@ -9695,7 +9695,7 @@
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>2023-08-12</t>
+          <t>08.12.2023</t>
         </is>
       </c>
       <c r="D447" t="inlineStr"/>
@@ -9716,7 +9716,7 @@
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>2023-08-12</t>
+          <t>08.12.2023</t>
         </is>
       </c>
       <c r="D448" t="inlineStr">
@@ -9737,7 +9737,7 @@
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>2023-08-09</t>
+          <t>08.09.2023</t>
         </is>
       </c>
       <c r="D449" t="inlineStr">
@@ -9758,7 +9758,7 @@
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>2023-08-09</t>
+          <t>08.09.2023</t>
         </is>
       </c>
       <c r="D450" t="inlineStr">
@@ -9783,7 +9783,7 @@
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>2023-08-07</t>
+          <t>08.07.2023</t>
         </is>
       </c>
       <c r="D451" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>2023-08-06</t>
+          <t>08.06.2023</t>
         </is>
       </c>
       <c r="D452" t="inlineStr">
@@ -9833,7 +9833,7 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>2023-08-06</t>
+          <t>08.06.2023</t>
         </is>
       </c>
       <c r="D453" t="inlineStr">
@@ -9858,7 +9858,7 @@
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>2023-08-06</t>
+          <t>08.06.2023</t>
         </is>
       </c>
       <c r="D454" t="inlineStr">
@@ -9883,7 +9883,7 @@
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>2023-08-06</t>
+          <t>08.06.2023</t>
         </is>
       </c>
       <c r="D455" t="inlineStr">
@@ -9908,7 +9908,7 @@
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>2023-08-06</t>
+          <t>08.06.2023</t>
         </is>
       </c>
       <c r="D456" t="inlineStr">
@@ -9933,7 +9933,7 @@
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>2023-08-04</t>
+          <t>08.04.2023</t>
         </is>
       </c>
       <c r="D457" t="inlineStr">
@@ -9958,7 +9958,7 @@
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>2023-08-04</t>
+          <t>08.04.2023</t>
         </is>
       </c>
       <c r="D458" t="inlineStr">
@@ -9983,7 +9983,7 @@
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>2023-08-03</t>
+          <t>08.03.2023</t>
         </is>
       </c>
       <c r="D459" t="inlineStr">
@@ -10008,7 +10008,7 @@
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>2023-08-03</t>
+          <t>08.03.2023</t>
         </is>
       </c>
       <c r="D460" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>2023-08-03</t>
+          <t>08.03.2023</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>2023-08-02</t>
+          <t>08.02.2023</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>2023-08-02</t>
+          <t>08.02.2023</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
@@ -10104,7 +10104,7 @@
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>2023-08-02</t>
+          <t>08.02.2023</t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
@@ -10129,7 +10129,7 @@
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>2023-08-02</t>
+          <t>08.02.2023</t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>2023-08-01</t>
+          <t>08.01.2023</t>
         </is>
       </c>
       <c r="D466" t="inlineStr">
@@ -10179,7 +10179,7 @@
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>2023-08-01</t>
+          <t>08.01.2023</t>
         </is>
       </c>
       <c r="D467" t="inlineStr">
@@ -10204,7 +10204,7 @@
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>2023-08-01</t>
+          <t>08.01.2023</t>
         </is>
       </c>
       <c r="D468" t="inlineStr">
@@ -11169,7 +11169,7 @@
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>2023-07-12</t>
+          <t>07.12.2023</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
@@ -11194,7 +11194,7 @@
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>2023-07-12</t>
+          <t>07.12.2023</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
@@ -11219,7 +11219,7 @@
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>2023-07-12</t>
+          <t>07.12.2023</t>
         </is>
       </c>
       <c r="D519" t="inlineStr"/>
@@ -11240,7 +11240,7 @@
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>2023-07-11</t>
+          <t>07.11.2023</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
@@ -11265,7 +11265,7 @@
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>2023-07-11</t>
+          <t>07.11.2023</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
@@ -11290,7 +11290,7 @@
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>2023-07-11</t>
+          <t>07.11.2023</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
@@ -11311,7 +11311,7 @@
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>2023-07-11</t>
+          <t>07.11.2023</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
@@ -11336,7 +11336,7 @@
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>2023-07-10</t>
+          <t>07.10.2023</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
@@ -11357,7 +11357,7 @@
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>2023-07-10</t>
+          <t>07.10.2023</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
@@ -11382,7 +11382,7 @@
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>2023-07-10</t>
+          <t>07.10.2023</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>2023-07-09</t>
+          <t>07.09.2023</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
@@ -11428,7 +11428,7 @@
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>2023-07-09</t>
+          <t>07.09.2023</t>
         </is>
       </c>
       <c r="D528" t="inlineStr"/>
@@ -11449,7 +11449,7 @@
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>2023-07-09</t>
+          <t>07.09.2023</t>
         </is>
       </c>
       <c r="D529" t="inlineStr"/>
@@ -11470,7 +11470,7 @@
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>2023-07-08</t>
+          <t>07.08.2023</t>
         </is>
       </c>
       <c r="D530" t="inlineStr">
@@ -11495,7 +11495,7 @@
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>2023-07-08</t>
+          <t>07.08.2023</t>
         </is>
       </c>
       <c r="D531" t="inlineStr"/>
@@ -11516,7 +11516,7 @@
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>2023-07-08</t>
+          <t>07.08.2023</t>
         </is>
       </c>
       <c r="D532" t="inlineStr">
@@ -11541,7 +11541,7 @@
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>2023-07-07</t>
+          <t>07.07.2023</t>
         </is>
       </c>
       <c r="D533" t="inlineStr">
@@ -11566,7 +11566,7 @@
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>2023-07-06</t>
+          <t>07.06.2023</t>
         </is>
       </c>
       <c r="D534" t="inlineStr"/>
@@ -11587,7 +11587,7 @@
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>2023-07-06</t>
+          <t>07.06.2023</t>
         </is>
       </c>
       <c r="D535" t="inlineStr">
@@ -11612,7 +11612,7 @@
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>2023-07-06</t>
+          <t>07.06.2023</t>
         </is>
       </c>
       <c r="D536" t="inlineStr">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>2023-07-06</t>
+          <t>07.06.2023</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>2023-07-05</t>
+          <t>07.05.2023</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
@@ -11683,7 +11683,7 @@
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>2023-07-05</t>
+          <t>07.05.2023</t>
         </is>
       </c>
       <c r="D539" t="inlineStr"/>
@@ -11704,7 +11704,7 @@
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>2023-07-05</t>
+          <t>07.05.2023</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
@@ -11729,7 +11729,7 @@
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>2023-07-05</t>
+          <t>07.05.2023</t>
         </is>
       </c>
       <c r="D541" t="inlineStr">
@@ -11754,7 +11754,7 @@
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>2023-07-04</t>
+          <t>07.04.2023</t>
         </is>
       </c>
       <c r="D542" t="inlineStr">
@@ -11779,7 +11779,7 @@
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>2023-07-04</t>
+          <t>07.04.2023</t>
         </is>
       </c>
       <c r="D543" t="inlineStr">
@@ -11800,7 +11800,7 @@
       </c>
       <c r="C544" t="inlineStr">
         <is>
-          <t>2023-07-04</t>
+          <t>07.04.2023</t>
         </is>
       </c>
       <c r="D544" t="inlineStr"/>
@@ -11821,7 +11821,7 @@
       </c>
       <c r="C545" t="inlineStr">
         <is>
-          <t>2023-07-04</t>
+          <t>07.04.2023</t>
         </is>
       </c>
       <c r="D545" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="C546" t="inlineStr">
         <is>
-          <t>2023-07-03</t>
+          <t>07.03.2023</t>
         </is>
       </c>
       <c r="D546" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="C547" t="inlineStr">
         <is>
-          <t>2023-07-03</t>
+          <t>07.03.2023</t>
         </is>
       </c>
       <c r="D547" t="inlineStr">
@@ -11896,7 +11896,7 @@
       </c>
       <c r="C548" t="inlineStr">
         <is>
-          <t>2023-07-02</t>
+          <t>07.02.2023</t>
         </is>
       </c>
       <c r="D548" t="inlineStr">
@@ -11921,7 +11921,7 @@
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>2023-07-01</t>
+          <t>07.01.2023</t>
         </is>
       </c>
       <c r="D549" t="inlineStr">
@@ -11942,7 +11942,7 @@
       </c>
       <c r="C550" t="inlineStr">
         <is>
-          <t>2023-07-01</t>
+          <t>07.01.2023</t>
         </is>
       </c>
       <c r="D550" t="inlineStr">
@@ -11967,7 +11967,7 @@
       </c>
       <c r="C551" t="inlineStr">
         <is>
-          <t>2023-07-01</t>
+          <t>07.01.2023</t>
         </is>
       </c>
       <c r="D551" t="inlineStr">
@@ -11992,7 +11992,7 @@
       </c>
       <c r="C552" t="inlineStr">
         <is>
-          <t>2023-07-01</t>
+          <t>07.01.2023</t>
         </is>
       </c>
       <c r="D552" t="inlineStr">
@@ -12017,7 +12017,7 @@
       </c>
       <c r="C553" t="inlineStr">
         <is>
-          <t>2023-07-01</t>
+          <t>07.01.2023</t>
         </is>
       </c>
       <c r="D553" t="inlineStr">
@@ -12042,7 +12042,7 @@
       </c>
       <c r="C554" t="inlineStr">
         <is>
-          <t>2023-07-01</t>
+          <t>07.01.2023</t>
         </is>
       </c>
       <c r="D554" t="inlineStr">
@@ -13249,7 +13249,7 @@
       </c>
       <c r="C613" t="inlineStr">
         <is>
-          <t>2023-06-12</t>
+          <t>06.12.2023</t>
         </is>
       </c>
       <c r="D613" t="inlineStr">
@@ -13270,7 +13270,7 @@
       </c>
       <c r="C614" t="inlineStr">
         <is>
-          <t>2023-06-12</t>
+          <t>06.12.2023</t>
         </is>
       </c>
       <c r="D614" t="inlineStr">
@@ -13291,7 +13291,7 @@
       </c>
       <c r="C615" t="inlineStr">
         <is>
-          <t>2023-06-12</t>
+          <t>06.12.2023</t>
         </is>
       </c>
       <c r="D615" t="inlineStr">
@@ -13312,7 +13312,7 @@
       </c>
       <c r="C616" t="inlineStr">
         <is>
-          <t>2023-06-11</t>
+          <t>06.11.2023</t>
         </is>
       </c>
       <c r="D616" t="inlineStr">
@@ -13337,7 +13337,7 @@
       </c>
       <c r="C617" t="inlineStr">
         <is>
-          <t>2023-06-11</t>
+          <t>06.11.2023</t>
         </is>
       </c>
       <c r="D617" t="inlineStr">
@@ -13362,7 +13362,7 @@
       </c>
       <c r="C618" t="inlineStr">
         <is>
-          <t>2023-06-11</t>
+          <t>06.11.2023</t>
         </is>
       </c>
       <c r="D618" t="inlineStr">
@@ -13383,7 +13383,7 @@
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>2023-06-10</t>
+          <t>06.10.2023</t>
         </is>
       </c>
       <c r="D619" t="inlineStr">
@@ -13408,7 +13408,7 @@
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>2023-06-10</t>
+          <t>06.10.2023</t>
         </is>
       </c>
       <c r="D620" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="C621" t="inlineStr">
         <is>
-          <t>2023-06-10</t>
+          <t>06.10.2023</t>
         </is>
       </c>
       <c r="D621" t="inlineStr">
@@ -13454,7 +13454,7 @@
       </c>
       <c r="C622" t="inlineStr">
         <is>
-          <t>2023-06-09</t>
+          <t>06.09.2023</t>
         </is>
       </c>
       <c r="D622" t="inlineStr">
@@ -13479,7 +13479,7 @@
       </c>
       <c r="C623" t="inlineStr">
         <is>
-          <t>2023-06-09</t>
+          <t>06.09.2023</t>
         </is>
       </c>
       <c r="D623" t="inlineStr">
@@ -13504,7 +13504,7 @@
       </c>
       <c r="C624" t="inlineStr">
         <is>
-          <t>2023-06-09</t>
+          <t>06.09.2023</t>
         </is>
       </c>
       <c r="D624" t="inlineStr">
@@ -13529,7 +13529,7 @@
       </c>
       <c r="C625" t="inlineStr">
         <is>
-          <t>2023-06-08</t>
+          <t>06.08.2023</t>
         </is>
       </c>
       <c r="D625" t="inlineStr">
@@ -13554,7 +13554,7 @@
       </c>
       <c r="C626" t="inlineStr">
         <is>
-          <t>2023-06-08</t>
+          <t>06.08.2023</t>
         </is>
       </c>
       <c r="D626" t="inlineStr">
@@ -13579,7 +13579,7 @@
       </c>
       <c r="C627" t="inlineStr">
         <is>
-          <t>2023-06-08</t>
+          <t>06.08.2023</t>
         </is>
       </c>
       <c r="D627" t="inlineStr">
@@ -13604,7 +13604,7 @@
       </c>
       <c r="C628" t="inlineStr">
         <is>
-          <t>2023-06-08</t>
+          <t>06.08.2023</t>
         </is>
       </c>
       <c r="D628" t="inlineStr">
@@ -13629,7 +13629,7 @@
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>2023-06-07</t>
+          <t>06.07.2023</t>
         </is>
       </c>
       <c r="D629" t="inlineStr">
@@ -13654,7 +13654,7 @@
       </c>
       <c r="C630" t="inlineStr">
         <is>
-          <t>2023-06-07</t>
+          <t>06.07.2023</t>
         </is>
       </c>
       <c r="D630" t="inlineStr">
@@ -13675,7 +13675,7 @@
       </c>
       <c r="C631" t="inlineStr">
         <is>
-          <t>2023-06-07</t>
+          <t>06.07.2023</t>
         </is>
       </c>
       <c r="D631" t="inlineStr">
@@ -13700,7 +13700,7 @@
       </c>
       <c r="C632" t="inlineStr">
         <is>
-          <t>2023-06-06</t>
+          <t>06.06.2023</t>
         </is>
       </c>
       <c r="D632" t="inlineStr">
@@ -13721,7 +13721,7 @@
       </c>
       <c r="C633" t="inlineStr">
         <is>
-          <t>2023-06-05</t>
+          <t>06.05.2023</t>
         </is>
       </c>
       <c r="D633" t="inlineStr">
@@ -13894,7 +13894,7 @@
       </c>
       <c r="C642" t="inlineStr">
         <is>
-          <t>2023-04-12</t>
+          <t>04.12.2023</t>
         </is>
       </c>
       <c r="D642" t="inlineStr">
@@ -13966,7 +13966,7 @@
       </c>
       <c r="C646" t="inlineStr">
         <is>
-          <t>2023-03-03</t>
+          <t>03.03.2023</t>
         </is>
       </c>
       <c r="D646" t="inlineStr">
@@ -13987,7 +13987,7 @@
       </c>
       <c r="C647" t="inlineStr">
         <is>
-          <t>2023-03-03</t>
+          <t>03.03.2023</t>
         </is>
       </c>
       <c r="D647" t="inlineStr">
@@ -14046,7 +14046,7 @@
       </c>
       <c r="C650" t="inlineStr">
         <is>
-          <t>2023-02-09</t>
+          <t>02.09.2023</t>
         </is>
       </c>
       <c r="D650" t="inlineStr">
@@ -14067,7 +14067,7 @@
       </c>
       <c r="C651" t="inlineStr">
         <is>
-          <t>2023-02-03</t>
+          <t>02.03.2023</t>
         </is>
       </c>
       <c r="D651" t="inlineStr">
@@ -14147,7 +14147,7 @@
       </c>
       <c r="C655" t="inlineStr">
         <is>
-          <t>2023-01-10</t>
+          <t>01.10.2023</t>
         </is>
       </c>
       <c r="D655" t="inlineStr">
@@ -14240,7 +14240,7 @@
       </c>
       <c r="C660" t="inlineStr">
         <is>
-          <t>2022-12-06</t>
+          <t>12.06.2022</t>
         </is>
       </c>
       <c r="D660" t="inlineStr">
@@ -14265,7 +14265,7 @@
       </c>
       <c r="C661" t="inlineStr">
         <is>
-          <t>2022-12-06</t>
+          <t>12.06.2022</t>
         </is>
       </c>
       <c r="D661" t="inlineStr">
@@ -14286,7 +14286,7 @@
       </c>
       <c r="C662" t="inlineStr">
         <is>
-          <t>2022-12-03</t>
+          <t>12.03.2022</t>
         </is>
       </c>
       <c r="D662" t="inlineStr">
@@ -14353,7 +14353,7 @@
       </c>
       <c r="C665" t="inlineStr">
         <is>
-          <t>2022-11-06</t>
+          <t>11.06.2022</t>
         </is>
       </c>
       <c r="D665" t="inlineStr">
@@ -14374,7 +14374,7 @@
       </c>
       <c r="C666" t="inlineStr">
         <is>
-          <t>2022-11-06</t>
+          <t>11.06.2022</t>
         </is>
       </c>
       <c r="D666" t="inlineStr">
@@ -14395,7 +14395,7 @@
       </c>
       <c r="C667" t="inlineStr">
         <is>
-          <t>2022-11-06</t>
+          <t>11.06.2022</t>
         </is>
       </c>
       <c r="D667" t="inlineStr">
@@ -14420,7 +14420,7 @@
       </c>
       <c r="C668" t="inlineStr">
         <is>
-          <t>2022-11-05</t>
+          <t>11.05.2022</t>
         </is>
       </c>
       <c r="D668" t="inlineStr">
@@ -14445,7 +14445,7 @@
       </c>
       <c r="C669" t="inlineStr">
         <is>
-          <t>2022-11-05</t>
+          <t>11.05.2022</t>
         </is>
       </c>
       <c r="D669" t="inlineStr">
@@ -14525,7 +14525,7 @@
       </c>
       <c r="C673" t="inlineStr">
         <is>
-          <t>2022-09-07</t>
+          <t>09.07.2022</t>
         </is>
       </c>
       <c r="D673" t="inlineStr">
@@ -14550,7 +14550,7 @@
       </c>
       <c r="C674" t="inlineStr">
         <is>
-          <t>2022-09-03</t>
+          <t>09.03.2022</t>
         </is>
       </c>
       <c r="D674" t="inlineStr">
@@ -14659,7 +14659,7 @@
       </c>
       <c r="C679" t="inlineStr">
         <is>
-          <t>2021-10-08</t>
+          <t>10.08.2021</t>
         </is>
       </c>
       <c r="D679" t="inlineStr">
@@ -14705,7 +14705,7 @@
       </c>
       <c r="C681" t="inlineStr">
         <is>
-          <t>2021-09-06</t>
+          <t>09.06.2021</t>
         </is>
       </c>
       <c r="D681" t="inlineStr">
@@ -15839,7 +15839,7 @@
       </c>
       <c r="C743" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>19.08.2026</t>
         </is>
       </c>
       <c r="D743" t="inlineStr">

</xml_diff>

<commit_message>
Smazána závada ID 744
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E743"/>
+  <dimension ref="A1:E742"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15828,31 +15828,6 @@
         </is>
       </c>
     </row>
-    <row r="743">
-      <c r="A743" t="n">
-        <v>744</v>
-      </c>
-      <c r="B743" t="inlineStr">
-        <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C743" t="inlineStr">
-        <is>
-          <t>19.08.2026</t>
-        </is>
-      </c>
-      <c r="D743" t="inlineStr">
-        <is>
-          <t>testik</t>
-        </is>
-      </c>
-      <c r="E743" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 745 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F743"/>
+  <dimension ref="A1:F744"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19564,6 +19564,36 @@
         </is>
       </c>
     </row>
+    <row r="744">
+      <c r="A744" t="n">
+        <v>745</v>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>814 143</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>Nešly přeřadit směry</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>Výměna čidla pro odblokování směru</t>
+        </is>
+      </c>
+      <c r="F744" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 746 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F744"/>
+  <dimension ref="A1:F745"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19594,6 +19594,36 @@
         </is>
       </c>
     </row>
+    <row r="745">
+      <c r="A745" t="n">
+        <v>746</v>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>03.07.2026</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>výměna A2.6</t>
+        </is>
+      </c>
+      <c r="F745" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Úprava závady ID 744 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -19554,10 +19554,14 @@
       </c>
       <c r="D743" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6 dneska výměna A2.7</t>
-        </is>
-      </c>
-      <c r="E743" t="inlineStr"/>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>Výměna A2.7</t>
+        </is>
+      </c>
       <c r="F743" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>

</xml_diff>

<commit_message>
Hromadná úprava z tabulky (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -6761,7 +6761,11 @@
           <t>netlačí tlak ADBlue na 5 baru - výměna filtru a vyčistění sítka OK</t>
         </is>
       </c>
-      <c r="E243" t="inlineStr"/>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Zkouška</t>
+        </is>
+      </c>
       <c r="F243" t="inlineStr">
         <is>
           <t>Neuvedeno</t>

</xml_diff>

<commit_message>
Přidána nová závada ID 747 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F745"/>
+  <dimension ref="A1:F746"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19628,6 +19628,32 @@
         </is>
       </c>
     </row>
+    <row r="746">
+      <c r="A746" t="n">
+        <v>747</v>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>29.07.2026</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr"/>
+      <c r="F746" t="inlineStr">
+        <is>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 748 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F746"/>
+  <dimension ref="A1:F747"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19654,6 +19654,32 @@
         </is>
       </c>
     </row>
+    <row r="747">
+      <c r="A747" t="n">
+        <v>748</v>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>01.08.2026</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr"/>
+      <c r="F747" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 749 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F747"/>
+  <dimension ref="A1:F748"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19680,6 +19680,32 @@
         </is>
       </c>
     </row>
+    <row r="748">
+      <c r="A748" t="n">
+        <v>749</v>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>08.08.2026</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>Zavaz motoru B</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr"/>
+      <c r="F748" t="inlineStr">
+        <is>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 750 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F748"/>
+  <dimension ref="A1:F749"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19706,6 +19706,32 @@
         </is>
       </c>
     </row>
+    <row r="749">
+      <c r="A749" t="n">
+        <v>750</v>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>18.08.2026</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr"/>
+      <c r="F749" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 751 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F749"/>
+  <dimension ref="A1:F750"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19732,6 +19732,36 @@
         </is>
       </c>
     </row>
+    <row r="750">
+      <c r="A750" t="n">
+        <v>751</v>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>954 218</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>17.08.2026</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
+      <c r="F750" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 752 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F750"/>
+  <dimension ref="A1:F751"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19762,6 +19762,32 @@
         </is>
       </c>
     </row>
+    <row r="751">
+      <c r="A751" t="n">
+        <v>752</v>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>842 036</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>17.08.2026</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>MSV výměna BIS02</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr"/>
+      <c r="F751" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 753 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F751"/>
+  <dimension ref="A1:F752"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19788,6 +19788,32 @@
         </is>
       </c>
     </row>
+    <row r="752">
+      <c r="A752" t="n">
+        <v>753</v>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>17.08.2026</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>Výměna BIS02</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr"/>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Smazána závada ID 681 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F752"/>
+  <dimension ref="A1:F751"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18294,11 +18294,11 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>842 011</t>
+          <t>842 015</t>
         </is>
       </c>
       <c r="C682" t="inlineStr"/>
@@ -18312,15 +18312,19 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>029 221</t>
         </is>
       </c>
       <c r="C683" t="inlineStr"/>
-      <c r="D683" t="inlineStr"/>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="E683" t="inlineStr"/>
       <c r="F683" t="inlineStr">
         <is>
@@ -18330,11 +18334,11 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>029 221</t>
+          <t>029 222</t>
         </is>
       </c>
       <c r="C684" t="inlineStr"/>
@@ -18352,19 +18356,15 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>029 222</t>
+          <t>714 226</t>
         </is>
       </c>
       <c r="C685" t="inlineStr"/>
-      <c r="D685" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
+      <c r="D685" t="inlineStr"/>
       <c r="E685" t="inlineStr"/>
       <c r="F685" t="inlineStr">
         <is>
@@ -18374,15 +18374,19 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>714 226</t>
+          <t>742 263</t>
         </is>
       </c>
       <c r="C686" t="inlineStr"/>
-      <c r="D686" t="inlineStr"/>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="E686" t="inlineStr"/>
       <c r="F686" t="inlineStr">
         <is>
@@ -18392,17 +18396,17 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>742 263</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C687" t="inlineStr"/>
       <c r="D687" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>výměna obrazovky Lokel na 914</t>
         </is>
       </c>
       <c r="E687" t="inlineStr"/>
@@ -18414,17 +18418,17 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C688" t="inlineStr"/>
       <c r="D688" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E688" t="inlineStr"/>
@@ -18436,17 +18440,17 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="E689" t="inlineStr"/>
@@ -18458,17 +18462,17 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E690" t="inlineStr"/>
@@ -18480,7 +18484,7 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
@@ -18490,10 +18494,14 @@
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E691" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F691" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -18502,24 +18510,20 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E692" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr"/>
       <c r="F692" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -18528,7 +18532,7 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
@@ -18538,7 +18542,7 @@
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E693" t="inlineStr"/>
@@ -18550,17 +18554,17 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C694" t="inlineStr"/>
       <c r="D694" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E694" t="inlineStr"/>
@@ -18572,20 +18576,24 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C695" t="inlineStr"/>
       <c r="D695" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E695" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F695" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -18594,7 +18602,7 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
@@ -18604,12 +18612,12 @@
       <c r="C696" t="inlineStr"/>
       <c r="D696" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E696" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F696" t="inlineStr">
@@ -18620,24 +18628,24 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C697" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D697" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E697" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr"/>
       <c r="F697" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -18646,7 +18654,7 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
@@ -18655,12 +18663,12 @@
       </c>
       <c r="C698" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D698" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E698" t="inlineStr"/>
@@ -18672,7 +18680,7 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
@@ -18686,7 +18694,7 @@
       </c>
       <c r="D699" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E699" t="inlineStr"/>
@@ -18698,7 +18706,7 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
@@ -18712,10 +18720,14 @@
       </c>
       <c r="D700" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E700" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F700" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -18724,7 +18736,7 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
@@ -18738,12 +18750,12 @@
       </c>
       <c r="D701" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E701" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F701" t="inlineStr">
@@ -18754,7 +18766,7 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
@@ -18768,14 +18780,10 @@
       </c>
       <c r="D702" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E702" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr"/>
       <c r="F702" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -18784,24 +18792,24 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C703" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E703" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F703" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -18810,24 +18818,20 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E704" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr"/>
       <c r="F704" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -18836,7 +18840,7 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
@@ -18846,7 +18850,7 @@
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
         </is>
       </c>
       <c r="E705" t="inlineStr"/>
@@ -18858,17 +18862,17 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E706" t="inlineStr"/>
@@ -18880,7 +18884,7 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
@@ -18890,10 +18894,14 @@
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E707" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F707" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -18902,24 +18910,20 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E708" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr"/>
       <c r="F708" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -18928,7 +18932,7 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
@@ -18938,7 +18942,7 @@
       <c r="C709" t="inlineStr"/>
       <c r="D709" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E709" t="inlineStr"/>
@@ -18950,7 +18954,7 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
@@ -18960,7 +18964,7 @@
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E710" t="inlineStr"/>
@@ -18972,17 +18976,17 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E711" t="inlineStr"/>
@@ -18994,7 +18998,7 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
@@ -19004,10 +19008,14 @@
       <c r="C712" t="inlineStr"/>
       <c r="D712" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="E712" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F712" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19016,7 +19024,7 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
@@ -19026,14 +19034,10 @@
       <c r="C713" t="inlineStr"/>
       <c r="D713" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E713" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr"/>
       <c r="F713" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19042,7 +19046,7 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
@@ -19052,10 +19056,14 @@
       <c r="C714" t="inlineStr"/>
       <c r="D714" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E714" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F714" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19064,7 +19072,7 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
@@ -19074,14 +19082,10 @@
       <c r="C715" t="inlineStr"/>
       <c r="D715" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E715" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr"/>
       <c r="F715" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19090,7 +19094,7 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
@@ -19100,7 +19104,7 @@
       <c r="C716" t="inlineStr"/>
       <c r="D716" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E716" t="inlineStr"/>
@@ -19112,7 +19116,7 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
@@ -19122,10 +19126,14 @@
       <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E717" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F717" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19134,7 +19142,7 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
@@ -19144,12 +19152,12 @@
       <c r="C718" t="inlineStr"/>
       <c r="D718" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E718" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F718" t="inlineStr">
@@ -19160,7 +19168,7 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
@@ -19170,12 +19178,12 @@
       <c r="C719" t="inlineStr"/>
       <c r="D719" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E719" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F719" t="inlineStr">
@@ -19186,24 +19194,20 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C720" t="inlineStr"/>
       <c r="D720" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E720" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr"/>
       <c r="F720" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19212,7 +19216,7 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
@@ -19222,10 +19226,14 @@
       <c r="C721" t="inlineStr"/>
       <c r="D721" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E721" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F721" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19234,7 +19242,7 @@
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
@@ -19244,12 +19252,12 @@
       <c r="C722" t="inlineStr"/>
       <c r="D722" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E722" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F722" t="inlineStr">
@@ -19260,7 +19268,7 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
@@ -19270,14 +19278,10 @@
       <c r="C723" t="inlineStr"/>
       <c r="D723" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E723" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr"/>
       <c r="F723" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19286,17 +19290,17 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C724" t="inlineStr"/>
       <c r="D724" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E724" t="inlineStr"/>
@@ -19308,7 +19312,7 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
@@ -19318,7 +19322,7 @@
       <c r="C725" t="inlineStr"/>
       <c r="D725" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E725" t="inlineStr"/>
@@ -19330,7 +19334,7 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
@@ -19340,10 +19344,14 @@
       <c r="C726" t="inlineStr"/>
       <c r="D726" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E726" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F726" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19352,22 +19360,22 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C727" t="inlineStr"/>
       <c r="D727" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E727" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F727" t="inlineStr">
@@ -19378,7 +19386,7 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
@@ -19388,12 +19396,12 @@
       <c r="C728" t="inlineStr"/>
       <c r="D728" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E728" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F728" t="inlineStr">
@@ -19404,24 +19412,20 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C729" t="inlineStr"/>
       <c r="D729" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E729" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr"/>
       <c r="F729" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19430,20 +19434,24 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C730" t="inlineStr"/>
       <c r="D730" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E730" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F730" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19452,24 +19460,20 @@
     </row>
     <row r="731">
       <c r="A731" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C731" t="inlineStr"/>
       <c r="D731" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E731" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr"/>
       <c r="F731" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19478,7 +19482,7 @@
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
@@ -19488,7 +19492,7 @@
       <c r="C732" t="inlineStr"/>
       <c r="D732" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E732" t="inlineStr"/>
@@ -19500,7 +19504,7 @@
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
@@ -19510,7 +19514,7 @@
       <c r="C733" t="inlineStr"/>
       <c r="D733" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E733" t="inlineStr"/>
@@ -19522,7 +19526,7 @@
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
@@ -19532,7 +19536,7 @@
       <c r="C734" t="inlineStr"/>
       <c r="D734" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E734" t="inlineStr"/>
@@ -19544,7 +19548,7 @@
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
@@ -19554,10 +19558,14 @@
       <c r="C735" t="inlineStr"/>
       <c r="D735" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E735" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F735" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19566,24 +19574,20 @@
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C736" t="inlineStr"/>
       <c r="D736" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E736" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr"/>
       <c r="F736" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19592,7 +19596,7 @@
     </row>
     <row r="737">
       <c r="A737" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
@@ -19602,7 +19606,7 @@
       <c r="C737" t="inlineStr"/>
       <c r="D737" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E737" t="inlineStr"/>
@@ -19614,20 +19618,24 @@
     </row>
     <row r="738">
       <c r="A738" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C738" t="inlineStr"/>
       <c r="D738" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E738" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F738" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19636,24 +19644,20 @@
     </row>
     <row r="739">
       <c r="A739" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C739" t="inlineStr"/>
       <c r="D739" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E739" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr"/>
       <c r="F739" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19662,7 +19666,7 @@
     </row>
     <row r="740">
       <c r="A740" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B740" t="inlineStr">
         <is>
@@ -19672,7 +19676,7 @@
       <c r="C740" t="inlineStr"/>
       <c r="D740" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E740" t="inlineStr"/>
@@ -19684,20 +19688,24 @@
     </row>
     <row r="741">
       <c r="A741" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C741" t="inlineStr"/>
       <c r="D741" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E741" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F741" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19706,37 +19714,41 @@
     </row>
     <row r="742">
       <c r="A742" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C742" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D742" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E742" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F742" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
     </row>
     <row r="743">
       <c r="A743" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C743" t="inlineStr">
@@ -19746,12 +19758,12 @@
       </c>
       <c r="D743" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E743" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F743" t="inlineStr">
@@ -19762,26 +19774,26 @@
     </row>
     <row r="744">
       <c r="A744" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C744" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D744" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E744" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F744" t="inlineStr">
@@ -19792,132 +19804,132 @@
     </row>
     <row r="745">
       <c r="A745" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B745" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C745" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D745" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E745" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr"/>
       <c r="F745" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
     </row>
     <row r="746">
       <c r="A746" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C746" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D746" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E746" t="inlineStr"/>
       <c r="F746" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
     </row>
     <row r="747">
       <c r="A747" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C747" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D747" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E747" t="inlineStr"/>
       <c r="F747" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
     </row>
     <row r="748">
       <c r="A748" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C748" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D748" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E748" t="inlineStr"/>
       <c r="F748" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
     </row>
     <row r="749">
       <c r="A749" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B749" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C749" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D749" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E749" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F749" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -19926,11 +19938,11 @@
     </row>
     <row r="750">
       <c r="A750" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B750" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C750" t="inlineStr">
@@ -19940,12 +19952,12 @@
       </c>
       <c r="D750" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E750" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F750" t="inlineStr">
@@ -19956,11 +19968,11 @@
     </row>
     <row r="751">
       <c r="A751" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B751" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C751" t="inlineStr">
@@ -19970,7 +19982,7 @@
       </c>
       <c r="D751" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E751" t="inlineStr">
@@ -19979,36 +19991,6 @@
         </is>
       </c>
       <c r="F751" t="inlineStr">
-        <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-    </row>
-    <row r="752">
-      <c r="A752" t="n">
-        <v>753</v>
-      </c>
-      <c r="B752" t="inlineStr">
-        <is>
-          <t>842 025</t>
-        </is>
-      </c>
-      <c r="C752" t="inlineStr">
-        <is>
-          <t>17.08.2026</t>
-        </is>
-      </c>
-      <c r="D752" t="inlineStr">
-        <is>
-          <t>Výměna BIS02</t>
-        </is>
-      </c>
-      <c r="E752" t="inlineStr">
-        <is>
-          <t>MSV</t>
-        </is>
-      </c>
-      <c r="F752" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
         </is>

</xml_diff>

<commit_message>
Přidána nová závada ID 754 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F750"/>
+  <dimension ref="A1:F751"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19994,6 +19994,36 @@
         </is>
       </c>
     </row>
+    <row r="751">
+      <c r="A751" t="n">
+        <v>754</v>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>844 029</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>22.08.2026</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>závaz</t>
+        </is>
+      </c>
+      <c r="F751" t="inlineStr">
+        <is>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 755 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F751"/>
+  <dimension ref="A1:F752"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20024,6 +20024,32 @@
         </is>
       </c>
     </row>
+    <row r="752">
+      <c r="A752" t="n">
+        <v>755</v>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>814 188</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>21.08.2026</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr"/>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>IS - Infosystém</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Smazána závada ID 756 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G753"/>
+  <dimension ref="A1:G752"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23810,37 +23810,6 @@
         </is>
       </c>
     </row>
-    <row r="753">
-      <c r="A753" t="n">
-        <v>756</v>
-      </c>
-      <c r="B753" t="inlineStr">
-        <is>
-          <t>844 029</t>
-        </is>
-      </c>
-      <c r="C753" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
-      <c r="D753" t="inlineStr">
-        <is>
-          <t>Zkouška nahrání fotky</t>
-        </is>
-      </c>
-      <c r="E753" t="inlineStr"/>
-      <c r="F753" t="inlineStr">
-        <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G753" t="inlineStr">
-        <is>
-          <t>Bez fotky</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 756 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G752"/>
+  <dimension ref="A1:G753"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23810,6 +23810,37 @@
         </is>
       </c>
     </row>
+    <row r="753">
+      <c r="A753" t="n">
+        <v>756</v>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>844 029</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>22.08.2026</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>zkouska fotky</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr"/>
+      <c r="F753" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>Bez fotky</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 757 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G753"/>
+  <dimension ref="A1:G754"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23841,6 +23841,37 @@
         </is>
       </c>
     </row>
+    <row r="754">
+      <c r="A754" t="n">
+        <v>757</v>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>844 029</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>22.08.2026</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>zkouska fotky</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr"/>
+      <c r="F754" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G754" t="inlineStr">
+        <is>
+          <t>Bez fotky</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 758 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G754"/>
+  <dimension ref="A1:G755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23872,6 +23872,37 @@
         </is>
       </c>
     </row>
+    <row r="755">
+      <c r="A755" t="n">
+        <v>758</v>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>844 029</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>22.08.2026</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>zkouska fotky</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr"/>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/0yNQXdNM/72da06f000a6.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Smazána závada ID 757 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G754"/>
+  <dimension ref="A1:G753"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23812,7 +23812,7 @@
     </row>
     <row r="753">
       <c r="A753" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B753" t="inlineStr">
         <is>
@@ -23836,37 +23836,6 @@
         </is>
       </c>
       <c r="G753" t="inlineStr">
-        <is>
-          <t>Bez fotky</t>
-        </is>
-      </c>
-    </row>
-    <row r="754">
-      <c r="A754" t="n">
-        <v>758</v>
-      </c>
-      <c r="B754" t="inlineStr">
-        <is>
-          <t>844 029</t>
-        </is>
-      </c>
-      <c r="C754" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
-      <c r="D754" t="inlineStr">
-        <is>
-          <t>zkouska fotky</t>
-        </is>
-      </c>
-      <c r="E754" t="inlineStr"/>
-      <c r="F754" t="inlineStr">
-        <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G754" t="inlineStr">
         <is>
           <t>https://i.ibb.co/0yNQXdNM/72da06f000a6.jpg</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 758 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G753"/>
+  <dimension ref="A1:G752"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23810,37 +23810,6 @@
         </is>
       </c>
     </row>
-    <row r="753">
-      <c r="A753" t="n">
-        <v>758</v>
-      </c>
-      <c r="B753" t="inlineStr">
-        <is>
-          <t>844 029</t>
-        </is>
-      </c>
-      <c r="C753" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
-      <c r="D753" t="inlineStr">
-        <is>
-          <t>zkouska fotky</t>
-        </is>
-      </c>
-      <c r="E753" t="inlineStr"/>
-      <c r="F753" t="inlineStr">
-        <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G753" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/0yNQXdNM/72da06f000a6.jpg</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Úprava závady ID 756 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -23829,7 +23829,11 @@
           <t>adsasdads</t>
         </is>
       </c>
-      <c r="E753" t="inlineStr"/>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F753" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -23837,7 +23841,7 @@
       </c>
       <c r="G753" t="inlineStr">
         <is>
-          <t>https://i.ibb.co/0yNQXdNM/72da06f000a6.jpg</t>
+          <t>https://i.ibb.co/N6fv63hs/f5dae1b76bf9.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Úprava závady ID 758 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -23881,23 +23881,27 @@
           <t>844 015</t>
         </is>
       </c>
-      <c r="C755" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
+      <c r="C755" t="inlineStr"/>
       <c r="D755" t="inlineStr">
         <is>
-          <t>Vývaz motoru B</t>
-        </is>
-      </c>
-      <c r="E755" t="inlineStr"/>
+          <t>Vývaz motoru "B"</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F755" t="inlineStr">
         <is>
           <t>Spalovací motor / Pohon</t>
         </is>
       </c>
-      <c r="G755" t="inlineStr"/>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidána nová závada ID 759 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G755"/>
+  <dimension ref="A1:G756"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23887,21 +23887,44 @@
           <t>Vývaz motoru "B"</t>
         </is>
       </c>
-      <c r="E755" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E755" t="inlineStr"/>
       <c r="F755" t="inlineStr">
         <is>
           <t>Spalovací motor / Pohon</t>
         </is>
       </c>
-      <c r="G755" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G755" t="inlineStr"/>
+    </row>
+    <row r="756">
+      <c r="A756" t="n">
+        <v>759</v>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>814 120</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>22.08.2026</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr">
+        <is>
+          <t>Vadná černá karta v bobku</t>
+        </is>
+      </c>
+      <c r="F756" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G756" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Smazána závada ID 604 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G755"/>
+  <dimension ref="A1:G754"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19198,22 +19198,22 @@
     </row>
     <row r="603">
       <c r="A603" t="n">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="B603" t="inlineStr">
         <is>
-          <t>810 015</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C603" t="inlineStr"/>
       <c r="D603" t="inlineStr">
         <is>
-          <t>AVJ propádávájí mince</t>
+          <t>nelze odbrzdit, tlak ve válcích zůstáva 0,3 bar závada jen z 914</t>
         </is>
       </c>
       <c r="E603" t="inlineStr">
         <is>
-          <t>výměna mincovníku</t>
+          <t>zk. Jízda OK</t>
         </is>
       </c>
       <c r="F603" t="inlineStr">
@@ -19229,22 +19229,22 @@
     </row>
     <row r="604">
       <c r="A604" t="n">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B604" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C604" t="inlineStr"/>
       <c r="D604" t="inlineStr">
         <is>
-          <t>nelze odbrzdit, tlak ve válcích zůstáva 0,3 bar závada jen z 914</t>
+          <t>2.SM samovolně zvyšuje otáčky, seřízení GAC</t>
         </is>
       </c>
       <c r="E604" t="inlineStr">
         <is>
-          <t>zk. Jízda OK</t>
+          <t>přístě vyměnit GAC musela jet ven</t>
         </is>
       </c>
       <c r="F604" t="inlineStr">
@@ -19260,22 +19260,22 @@
     </row>
     <row r="605">
       <c r="A605" t="n">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C605" t="inlineStr"/>
       <c r="D605" t="inlineStr">
         <is>
-          <t>2.SM samovolně zvyšuje otáčky, seřízení GAC</t>
+          <t>nehlási IS na stan. A</t>
         </is>
       </c>
       <c r="E605" t="inlineStr">
         <is>
-          <t>přístě vyměnit GAC musela jet ven</t>
+          <t>ztlumen potenciometr</t>
         </is>
       </c>
       <c r="F605" t="inlineStr">
@@ -19291,7 +19291,7 @@
     </row>
     <row r="606">
       <c r="A606" t="n">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B606" t="inlineStr">
         <is>
@@ -19301,12 +19301,12 @@
       <c r="C606" t="inlineStr"/>
       <c r="D606" t="inlineStr">
         <is>
-          <t>nehlási IS na stan. A</t>
+          <t>lednice nechladí</t>
         </is>
       </c>
       <c r="E606" t="inlineStr">
         <is>
-          <t>ztlumen potenciometr</t>
+          <t>odzkoušeno OK</t>
         </is>
       </c>
       <c r="F606" t="inlineStr">
@@ -19322,7 +19322,7 @@
     </row>
     <row r="607">
       <c r="A607" t="n">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B607" t="inlineStr">
         <is>
@@ -19332,12 +19332,12 @@
       <c r="C607" t="inlineStr"/>
       <c r="D607" t="inlineStr">
         <is>
-          <t>lednice nechladí</t>
+          <t>údajně rázy převodovky</t>
         </is>
       </c>
       <c r="E607" t="inlineStr">
         <is>
-          <t>odzkoušeno OK</t>
+          <t>řesí p. Šípek vyčítal jsi obě HMP</t>
         </is>
       </c>
       <c r="F607" t="inlineStr">
@@ -19353,22 +19353,22 @@
     </row>
     <row r="608">
       <c r="A608" t="n">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B608" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C608" t="inlineStr"/>
       <c r="D608" t="inlineStr">
         <is>
-          <t>údajně rázy převodovky</t>
+          <t>lok. Nejde nastartovat</t>
         </is>
       </c>
       <c r="E608" t="inlineStr">
         <is>
-          <t>řesí p. Šípek vyčítal jsi obě HMP</t>
+          <t>naftová netěsnost</t>
         </is>
       </c>
       <c r="F608" t="inlineStr">
@@ -19384,22 +19384,22 @@
     </row>
     <row r="609">
       <c r="A609" t="n">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C609" t="inlineStr"/>
       <c r="D609" t="inlineStr">
         <is>
-          <t>lok. Nejde nastartovat</t>
+          <t>izolačni stav odztraněny zkraty na vodiči 80 a 50</t>
         </is>
       </c>
       <c r="E609" t="inlineStr">
         <is>
-          <t>naftová netěsnost</t>
+          <t>startéry vyfoukany,ale nakonec výměna M2(volný pomocný vodič) seřízení GAC 2. SM , zkušební jízda se zdá v pořádku</t>
         </is>
       </c>
       <c r="F609" t="inlineStr">
@@ -19415,24 +19415,24 @@
     </row>
     <row r="610">
       <c r="A610" t="n">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B610" t="inlineStr">
         <is>
-          <t>842 035</t>
-        </is>
-      </c>
-      <c r="C610" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>06.12.2023</t>
+        </is>
+      </c>
       <c r="D610" t="inlineStr">
         <is>
-          <t>izolačni stav odztraněny zkraty na vodiči 80 a 50</t>
-        </is>
-      </c>
-      <c r="E610" t="inlineStr">
-        <is>
-          <t>startéry vyfoukany,ale nakonec výměna M2(volný pomocný vodič) seřízení GAC 2. SM , zkušební jízda se zdá v pořádku</t>
-        </is>
-      </c>
+          <t>Výměna obrazovky na 914 (občas zamrzá)</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr"/>
       <c r="F610" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19446,11 +19446,11 @@
     </row>
     <row r="611">
       <c r="A611" t="n">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B611" t="inlineStr">
         <is>
-          <t>814 003</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C611" t="inlineStr">
@@ -19460,7 +19460,7 @@
       </c>
       <c r="D611" t="inlineStr">
         <is>
-          <t>Výměna obrazovky na 914 (občas zamrzá)</t>
+          <t>údajně se rozpadá IS přezkoušeno (kontrola konektoru)</t>
         </is>
       </c>
       <c r="E611" t="inlineStr"/>
@@ -19477,11 +19477,11 @@
     </row>
     <row r="612">
       <c r="A612" t="n">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B612" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 072</t>
         </is>
       </c>
       <c r="C612" t="inlineStr">
@@ -19491,7 +19491,7 @@
       </c>
       <c r="D612" t="inlineStr">
         <is>
-          <t>údajně se rozpadá IS přezkoušeno (kontrola konektoru)</t>
+          <t>tozpadáva se IS, oprava dispeleje na 914 byl volný</t>
         </is>
       </c>
       <c r="E612" t="inlineStr"/>
@@ -19508,24 +19508,28 @@
     </row>
     <row r="613">
       <c r="A613" t="n">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>814 072</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C613" t="inlineStr">
         <is>
-          <t>06.12.2023</t>
+          <t>06.11.2023</t>
         </is>
       </c>
       <c r="D613" t="inlineStr">
         <is>
-          <t>tozpadáva se IS, oprava dispeleje na 914 byl volný</t>
-        </is>
-      </c>
-      <c r="E613" t="inlineStr"/>
+          <t>tabule vnitřní , venkovní nekomunikují</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>výměna konektoru C na 914</t>
+        </is>
+      </c>
       <c r="F613" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19539,11 +19543,11 @@
     </row>
     <row r="614">
       <c r="A614" t="n">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B614" t="inlineStr">
         <is>
-          <t>814 118</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C614" t="inlineStr">
@@ -19553,12 +19557,12 @@
       </c>
       <c r="D614" t="inlineStr">
         <is>
-          <t>tabule vnitřní , venkovní nekomunikují</t>
+          <t>korekce vody 2</t>
         </is>
       </c>
       <c r="E614" t="inlineStr">
         <is>
-          <t>výměna konektoru C na 914</t>
+          <t>izolačni stav špatný  stáhlé zemni relé</t>
         </is>
       </c>
       <c r="F614" t="inlineStr">
@@ -19574,11 +19578,11 @@
     </row>
     <row r="615">
       <c r="A615" t="n">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C615" t="inlineStr">
@@ -19588,14 +19592,10 @@
       </c>
       <c r="D615" t="inlineStr">
         <is>
-          <t>korekce vody 2</t>
-        </is>
-      </c>
-      <c r="E615" t="inlineStr">
-        <is>
-          <t>izolačni stav špatný  stáhlé zemni relé</t>
-        </is>
-      </c>
+          <t>výměna ARR na B stan. Nefunkční</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr"/>
       <c r="F615" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19609,24 +19609,28 @@
     </row>
     <row r="616">
       <c r="A616" t="n">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B616" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>810 329</t>
         </is>
       </c>
       <c r="C616" t="inlineStr">
         <is>
-          <t>06.11.2023</t>
+          <t>06.10.2023</t>
         </is>
       </c>
       <c r="D616" t="inlineStr">
         <is>
-          <t>výměna ARR na B stan. Nefunkční</t>
-        </is>
-      </c>
-      <c r="E616" t="inlineStr"/>
+          <t>nejde rychloměr</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>výměna</t>
+        </is>
+      </c>
       <c r="F616" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19640,11 +19644,11 @@
     </row>
     <row r="617">
       <c r="A617" t="n">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>810 329</t>
+          <t>842 011</t>
         </is>
       </c>
       <c r="C617" t="inlineStr">
@@ -19654,14 +19658,10 @@
       </c>
       <c r="D617" t="inlineStr">
         <is>
-          <t>nejde rychloměr</t>
-        </is>
-      </c>
-      <c r="E617" t="inlineStr">
-        <is>
-          <t>výměna</t>
-        </is>
-      </c>
+          <t>udajně zateklo do pultu na 2st.(kontrola)</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr"/>
       <c r="F617" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19675,11 +19675,11 @@
     </row>
     <row r="618">
       <c r="A618" t="n">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B618" t="inlineStr">
         <is>
-          <t>842 011</t>
+          <t>842 021</t>
         </is>
       </c>
       <c r="C618" t="inlineStr">
@@ -19689,10 +19689,14 @@
       </c>
       <c r="D618" t="inlineStr">
         <is>
-          <t>udajně zateklo do pultu na 2st.(kontrola)</t>
-        </is>
-      </c>
-      <c r="E618" t="inlineStr"/>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>vadné čidlo vody v míse</t>
+        </is>
+      </c>
       <c r="F618" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19706,26 +19710,26 @@
     </row>
     <row r="619">
       <c r="A619" t="n">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>842 021</t>
+          <t>810 015</t>
         </is>
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>06.10.2023</t>
+          <t>06.09.2023</t>
         </is>
       </c>
       <c r="D619" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>nejde AVJF</t>
         </is>
       </c>
       <c r="E619" t="inlineStr">
         <is>
-          <t>vadné čidlo vody v míse</t>
+          <t>byla vypadlá vratná pojistka,baterka měla 11V.Výměna baterie.Odzkoušení OK</t>
         </is>
       </c>
       <c r="F619" t="inlineStr">
@@ -19741,11 +19745,11 @@
     </row>
     <row r="620">
       <c r="A620" t="n">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>810 015</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C620" t="inlineStr">
@@ -19755,12 +19759,12 @@
       </c>
       <c r="D620" t="inlineStr">
         <is>
-          <t>nejde AVJF</t>
+          <t>Nejdou dvěře WC</t>
         </is>
       </c>
       <c r="E620" t="inlineStr">
         <is>
-          <t>byla vypadlá vratná pojistka,baterka měla 11V.Výměna baterie.Odzkoušení OK</t>
+          <t>upadlý drát na přepínači funkce WC (zapnuto,bez dveří, vypnuto). Seřízení zámykání dveří. Frýdek</t>
         </is>
       </c>
       <c r="F620" t="inlineStr">
@@ -19776,11 +19780,11 @@
     </row>
     <row r="621">
       <c r="A621" t="n">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C621" t="inlineStr">
@@ -19790,12 +19794,12 @@
       </c>
       <c r="D621" t="inlineStr">
         <is>
-          <t>Nejdou dvěře WC</t>
+          <t>údajně nejdou někdy schody u levých dveří strany A</t>
         </is>
       </c>
       <c r="E621" t="inlineStr">
         <is>
-          <t>upadlý drát na přepínači funkce WC (zapnuto,bez dveří, vypnuto). Seřízení zámykání dveří. Frýdek</t>
+          <t>vyčištění od kamínků,odzkoušení-OK</t>
         </is>
       </c>
       <c r="F621" t="inlineStr">
@@ -19811,26 +19815,26 @@
     </row>
     <row r="622">
       <c r="A622" t="n">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C622" t="inlineStr">
         <is>
-          <t>06.09.2023</t>
+          <t>06.08.2023</t>
         </is>
       </c>
       <c r="D622" t="inlineStr">
         <is>
-          <t>údajně nejdou někdy schody u levých dveří strany A</t>
+          <t>zapůjčena z HB</t>
         </is>
       </c>
       <c r="E622" t="inlineStr">
         <is>
-          <t>vyčištění od kamínků,odzkoušení-OK</t>
+          <t>nahrány data IS ( funguje preš radiostanici)</t>
         </is>
       </c>
       <c r="F622" t="inlineStr">
@@ -19846,11 +19850,11 @@
     </row>
     <row r="623">
       <c r="A623" t="n">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B623" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C623" t="inlineStr">
@@ -19860,12 +19864,12 @@
       </c>
       <c r="D623" t="inlineStr">
         <is>
-          <t>zapůjčena z HB</t>
+          <t>Opět problémy se startováním</t>
         </is>
       </c>
       <c r="E623" t="inlineStr">
         <is>
-          <t>nahrány data IS ( funguje preš radiostanici)</t>
+          <t>(asi už vadný capos kondy)říkali veselani jak tu byli</t>
         </is>
       </c>
       <c r="F623" t="inlineStr">
@@ -19881,7 +19885,7 @@
     </row>
     <row r="624">
       <c r="A624" t="n">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B624" t="inlineStr">
         <is>
@@ -19895,12 +19899,12 @@
       </c>
       <c r="D624" t="inlineStr">
         <is>
-          <t>Opět problémy se startováním</t>
+          <t>oprava hlasitosti na stanovišti A</t>
         </is>
       </c>
       <c r="E624" t="inlineStr">
         <is>
-          <t>(asi už vadný capos kondy)říkali veselani jak tu byli</t>
+          <t>přechod na kontaktech u reproduktoru v pultě</t>
         </is>
       </c>
       <c r="F624" t="inlineStr">
@@ -19916,11 +19920,11 @@
     </row>
     <row r="625">
       <c r="A625" t="n">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B625" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C625" t="inlineStr">
@@ -19930,12 +19934,12 @@
       </c>
       <c r="D625" t="inlineStr">
         <is>
-          <t>oprava hlasitosti na stanovišti A</t>
+          <t>výměna ARR na B</t>
         </is>
       </c>
       <c r="E625" t="inlineStr">
         <is>
-          <t>přechod na kontaktech u reproduktoru v pultě</t>
+          <t>vadná linka CAN</t>
         </is>
       </c>
       <c r="F625" t="inlineStr">
@@ -19951,26 +19955,26 @@
     </row>
     <row r="626">
       <c r="A626" t="n">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>842 015</t>
         </is>
       </c>
       <c r="C626" t="inlineStr">
         <is>
-          <t>06.08.2023</t>
+          <t>06.07.2023</t>
         </is>
       </c>
       <c r="D626" t="inlineStr">
         <is>
-          <t>výměna ARR na B</t>
+          <t>někdy nejde brzda PB</t>
         </is>
       </c>
       <c r="E626" t="inlineStr">
         <is>
-          <t>vadná linka CAN</t>
+          <t>výměna karty DS a OUT z 842 025</t>
         </is>
       </c>
       <c r="F626" t="inlineStr">
@@ -19986,11 +19990,11 @@
     </row>
     <row r="627">
       <c r="A627" t="n">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C627" t="inlineStr">
@@ -20000,14 +20004,10 @@
       </c>
       <c r="D627" t="inlineStr">
         <is>
-          <t>někdy nejde brzda PB</t>
-        </is>
-      </c>
-      <c r="E627" t="inlineStr">
-        <is>
-          <t>výměna karty DS a OUT z 842 025</t>
-        </is>
-      </c>
+          <t>dosazeny karty z 842 015 (DS a OUT)</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr"/>
       <c r="F627" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20021,11 +20021,11 @@
     </row>
     <row r="628">
       <c r="A628" t="n">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C628" t="inlineStr">
@@ -20035,10 +20035,14 @@
       </c>
       <c r="D628" t="inlineStr">
         <is>
-          <t>dosazeny karty z 842 015 (DS a OUT)</t>
-        </is>
-      </c>
-      <c r="E628" t="inlineStr"/>
+          <t>dosazen asi 5 dobíječ na B funkční</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>ve skladu nefunkční jenom (má řešit asi Mlíčko)</t>
+        </is>
+      </c>
       <c r="F628" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20052,28 +20056,24 @@
     </row>
     <row r="629">
       <c r="A629" t="n">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 076</t>
         </is>
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>06.07.2023</t>
+          <t>06.06.2023</t>
         </is>
       </c>
       <c r="D629" t="inlineStr">
         <is>
-          <t>dosazen asi 5 dobíječ na B funkční</t>
-        </is>
-      </c>
-      <c r="E629" t="inlineStr">
-        <is>
-          <t>ve skladu nefunkční jenom (má řešit asi Mlíčko)</t>
-        </is>
-      </c>
+          <t>NEHODA V HOLEŠOVĚ</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr"/>
       <c r="F629" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20087,21 +20087,21 @@
     </row>
     <row r="630">
       <c r="A630" t="n">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>814 076</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C630" t="inlineStr">
         <is>
-          <t>06.06.2023</t>
+          <t>06.05.2023</t>
         </is>
       </c>
       <c r="D630" t="inlineStr">
         <is>
-          <t>NEHODA V HOLEŠOVĚ</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E630" t="inlineStr"/>
@@ -20118,21 +20118,17 @@
     </row>
     <row r="631">
       <c r="A631" t="n">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C631" t="inlineStr">
-        <is>
-          <t>06.05.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr"/>
       <c r="D631" t="inlineStr">
         <is>
-          <t>MM</t>
+          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
         </is>
       </c>
       <c r="E631" t="inlineStr"/>
@@ -20149,7 +20145,7 @@
     </row>
     <row r="632">
       <c r="A632" t="n">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="B632" t="inlineStr">
         <is>
@@ -20159,7 +20155,7 @@
       <c r="C632" t="inlineStr"/>
       <c r="D632" t="inlineStr">
         <is>
-          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
+          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
         </is>
       </c>
       <c r="E632" t="inlineStr"/>
@@ -20176,7 +20172,7 @@
     </row>
     <row r="633">
       <c r="A633" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B633" t="inlineStr">
         <is>
@@ -20186,7 +20182,7 @@
       <c r="C633" t="inlineStr"/>
       <c r="D633" t="inlineStr">
         <is>
-          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
+          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
         </is>
       </c>
       <c r="E633" t="inlineStr"/>
@@ -20203,20 +20199,24 @@
     </row>
     <row r="634">
       <c r="A634" t="n">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C634" t="inlineStr"/>
       <c r="D634" t="inlineStr">
         <is>
-          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
-        </is>
-      </c>
-      <c r="E634" t="inlineStr"/>
+          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>vyměnili dobíječ stacionární (Veselí)</t>
+        </is>
+      </c>
       <c r="F634" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20230,22 +20230,22 @@
     </row>
     <row r="635">
       <c r="A635" t="n">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C635" t="inlineStr"/>
       <c r="D635" t="inlineStr">
         <is>
-          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
         </is>
       </c>
       <c r="E635" t="inlineStr">
         <is>
-          <t>vyměnili dobíječ stacionární (Veselí)</t>
+          <t>jela ven</t>
         </is>
       </c>
       <c r="F635" t="inlineStr">
@@ -20261,24 +20261,20 @@
     </row>
     <row r="636">
       <c r="A636" t="n">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C636" t="inlineStr"/>
       <c r="D636" t="inlineStr">
         <is>
-          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
-        </is>
-      </c>
-      <c r="E636" t="inlineStr">
-        <is>
-          <t>jela ven</t>
-        </is>
-      </c>
+          <t>seřízení kamer přes program v notasu(obraz)</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr"/>
       <c r="F636" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20292,20 +20288,24 @@
     </row>
     <row r="637">
       <c r="A637" t="n">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C637" t="inlineStr"/>
       <c r="D637" t="inlineStr">
         <is>
-          <t>seřízení kamer přes program v notasu(obraz)</t>
-        </is>
-      </c>
-      <c r="E637" t="inlineStr"/>
+          <t>po startu někdy nenabíjí "B"</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+        </is>
+      </c>
       <c r="F637" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20319,22 +20319,22 @@
     </row>
     <row r="638">
       <c r="A638" t="n">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C638" t="inlineStr"/>
       <c r="D638" t="inlineStr">
         <is>
-          <t>po startu někdy nenabíjí "B"</t>
+          <t>2. motor korekce vody  vystup</t>
         </is>
       </c>
       <c r="E638" t="inlineStr">
         <is>
-          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
         </is>
       </c>
       <c r="F638" t="inlineStr">
@@ -20350,24 +20350,24 @@
     </row>
     <row r="639">
       <c r="A639" t="n">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>842 035</t>
-        </is>
-      </c>
-      <c r="C639" t="inlineStr"/>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>04.12.2023</t>
+        </is>
+      </c>
       <c r="D639" t="inlineStr">
         <is>
-          <t>2. motor korekce vody  vystup</t>
-        </is>
-      </c>
-      <c r="E639" t="inlineStr">
-        <is>
-          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
-        </is>
-      </c>
+          <t>Výměna motoru A</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr"/>
       <c r="F639" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20381,21 +20381,17 @@
     </row>
     <row r="640">
       <c r="A640" t="n">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C640" t="inlineStr">
-        <is>
-          <t>04.12.2023</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr"/>
       <c r="D640" t="inlineStr">
         <is>
-          <t>Výměna motoru A</t>
+          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
         </is>
       </c>
       <c r="E640" t="inlineStr"/>
@@ -20412,17 +20408,17 @@
     </row>
     <row r="641">
       <c r="A641" t="n">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C641" t="inlineStr"/>
       <c r="D641" t="inlineStr">
         <is>
-          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
+          <t>dosazena nahadni Mirelka + NO z 844 013</t>
         </is>
       </c>
       <c r="E641" t="inlineStr"/>
@@ -20439,17 +20435,17 @@
     </row>
     <row r="642">
       <c r="A642" t="n">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 062</t>
         </is>
       </c>
       <c r="C642" t="inlineStr"/>
       <c r="D642" t="inlineStr">
         <is>
-          <t>dosazena nahadni Mirelka + NO z 844 013</t>
+          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
         </is>
       </c>
       <c r="E642" t="inlineStr"/>
@@ -20466,17 +20462,21 @@
     </row>
     <row r="643">
       <c r="A643" t="n">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>814 062</t>
-        </is>
-      </c>
-      <c r="C643" t="inlineStr"/>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>03.03.2023</t>
+        </is>
+      </c>
       <c r="D643" t="inlineStr">
         <is>
-          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E643" t="inlineStr"/>
@@ -20493,11 +20493,11 @@
     </row>
     <row r="644">
       <c r="A644" t="n">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C644" t="inlineStr">
@@ -20507,7 +20507,7 @@
       </c>
       <c r="D644" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
+          <t>Dosazení ŘJ kamer</t>
         </is>
       </c>
       <c r="E644" t="inlineStr"/>
@@ -20524,24 +20524,24 @@
     </row>
     <row r="645">
       <c r="A645" t="n">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>844 013</t>
-        </is>
-      </c>
-      <c r="C645" t="inlineStr">
-        <is>
-          <t>03.03.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr"/>
       <c r="D645" t="inlineStr">
         <is>
-          <t>Dosazení ŘJ kamer</t>
-        </is>
-      </c>
-      <c r="E645" t="inlineStr"/>
+          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>hlášeno p. Škodovi</t>
+        </is>
+      </c>
       <c r="F645" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20555,24 +20555,20 @@
     </row>
     <row r="646">
       <c r="A646" t="n">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C646" t="inlineStr"/>
       <c r="D646" t="inlineStr">
         <is>
-          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
-        </is>
-      </c>
-      <c r="E646" t="inlineStr">
-        <is>
-          <t>hlášeno p. Škodovi</t>
-        </is>
-      </c>
+          <t>ŘJ kamer dosazena z 013</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr"/>
       <c r="F646" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20586,17 +20582,21 @@
     </row>
     <row r="647">
       <c r="A647" t="n">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B647" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C647" t="inlineStr"/>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>02.09.2023</t>
+        </is>
+      </c>
       <c r="D647" t="inlineStr">
         <is>
-          <t>ŘJ kamer dosazena z 013</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E647" t="inlineStr"/>
@@ -20613,21 +20613,21 @@
     </row>
     <row r="648">
       <c r="A648" t="n">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 072</t>
         </is>
       </c>
       <c r="C648" t="inlineStr">
         <is>
-          <t>02.09.2023</t>
+          <t>02.03.2023</t>
         </is>
       </c>
       <c r="D648" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E648" t="inlineStr"/>
@@ -20644,24 +20644,24 @@
     </row>
     <row r="649">
       <c r="A649" t="n">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>814 072</t>
-        </is>
-      </c>
-      <c r="C649" t="inlineStr">
-        <is>
-          <t>02.03.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr"/>
       <c r="D649" t="inlineStr">
         <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E649" t="inlineStr"/>
+          <t>dosazen opraveny MIREL</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+        </is>
+      </c>
       <c r="F649" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20675,22 +20675,22 @@
     </row>
     <row r="650">
       <c r="A650" t="n">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C650" t="inlineStr"/>
       <c r="D650" t="inlineStr">
         <is>
-          <t>dosazen opraveny MIREL</t>
+          <t>Odpojen trojcestný ventil na A i B</t>
         </is>
       </c>
       <c r="E650" t="inlineStr">
         <is>
-          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+          <t>Zapojeny zpět 24.2.2023</t>
         </is>
       </c>
       <c r="F650" t="inlineStr">
@@ -20706,24 +20706,20 @@
     </row>
     <row r="651">
       <c r="A651" t="n">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C651" t="inlineStr"/>
       <c r="D651" t="inlineStr">
         <is>
-          <t>Odpojen trojcestný ventil na A i B</t>
-        </is>
-      </c>
-      <c r="E651" t="inlineStr">
-        <is>
-          <t>Zapojeny zpět 24.2.2023</t>
-        </is>
-      </c>
+          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr"/>
       <c r="F651" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20737,17 +20733,21 @@
     </row>
     <row r="652">
       <c r="A652" t="n">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B652" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C652" t="inlineStr"/>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>01.10.2023</t>
+        </is>
+      </c>
       <c r="D652" t="inlineStr">
         <is>
-          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E652" t="inlineStr"/>
@@ -20764,21 +20764,17 @@
     </row>
     <row r="653">
       <c r="A653" t="n">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C653" t="inlineStr">
-        <is>
-          <t>01.10.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr"/>
       <c r="D653" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
         </is>
       </c>
       <c r="E653" t="inlineStr"/>
@@ -20795,17 +20791,17 @@
     </row>
     <row r="654">
       <c r="A654" t="n">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C654" t="inlineStr"/>
       <c r="D654" t="inlineStr">
         <is>
-          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
+          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
         </is>
       </c>
       <c r="E654" t="inlineStr"/>
@@ -20822,7 +20818,7 @@
     </row>
     <row r="655">
       <c r="A655" t="n">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B655" t="inlineStr">
         <is>
@@ -20832,7 +20828,7 @@
       <c r="C655" t="inlineStr"/>
       <c r="D655" t="inlineStr">
         <is>
-          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
+          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
         </is>
       </c>
       <c r="E655" t="inlineStr"/>
@@ -20849,20 +20845,24 @@
     </row>
     <row r="656">
       <c r="A656" t="n">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C656" t="inlineStr"/>
       <c r="D656" t="inlineStr">
         <is>
-          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
-        </is>
-      </c>
-      <c r="E656" t="inlineStr"/>
+          <t>Přišel opravený Mirel ve skladu</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>dosazen na 29.12.2022</t>
+        </is>
+      </c>
       <c r="F656" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20876,22 +20876,26 @@
     </row>
     <row r="657">
       <c r="A657" t="n">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C657" t="inlineStr"/>
+          <t>844 014</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>12.06.2022</t>
+        </is>
+      </c>
       <c r="D657" t="inlineStr">
         <is>
-          <t>Přišel opravený Mirel ve skladu</t>
+          <t>rychloměr do opravy hazí !!</t>
         </is>
       </c>
       <c r="E657" t="inlineStr">
         <is>
-          <t>dosazen na 29.12.2022</t>
+          <t>zapujcen z 844 028 z veselí</t>
         </is>
       </c>
       <c r="F657" t="inlineStr">
@@ -20907,11 +20911,11 @@
     </row>
     <row r="658">
       <c r="A658" t="n">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C658" t="inlineStr">
@@ -20921,14 +20925,10 @@
       </c>
       <c r="D658" t="inlineStr">
         <is>
-          <t>rychloměr do opravy hazí !!</t>
-        </is>
-      </c>
-      <c r="E658" t="inlineStr">
-        <is>
-          <t>zapujcen z 844 028 z veselí</t>
-        </is>
-      </c>
+          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr"/>
       <c r="F658" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20942,24 +20942,28 @@
     </row>
     <row r="659">
       <c r="A659" t="n">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B659" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C659" t="inlineStr">
         <is>
-          <t>12.06.2022</t>
+          <t>12.03.2022</t>
         </is>
       </c>
       <c r="D659" t="inlineStr">
         <is>
-          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
-        </is>
-      </c>
-      <c r="E659" t="inlineStr"/>
+          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>bude řešit Škoda</t>
+        </is>
+      </c>
       <c r="F659" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20973,26 +20977,22 @@
     </row>
     <row r="660">
       <c r="A660" t="n">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B660" t="inlineStr">
         <is>
           <t>844 003</t>
         </is>
       </c>
-      <c r="C660" t="inlineStr">
-        <is>
-          <t>12.03.2022</t>
-        </is>
-      </c>
+      <c r="C660" t="inlineStr"/>
       <c r="D660" t="inlineStr">
         <is>
-          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+          <t>na A strane asi vadna expanzní nadrz topení ?</t>
         </is>
       </c>
       <c r="E660" t="inlineStr">
         <is>
-          <t>bude řešit Škoda</t>
+          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
         </is>
       </c>
       <c r="F660" t="inlineStr">
@@ -21008,22 +21008,22 @@
     </row>
     <row r="661">
       <c r="A661" t="n">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B661" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C661" t="inlineStr"/>
       <c r="D661" t="inlineStr">
         <is>
-          <t>na A strane asi vadna expanzní nadrz topení ?</t>
+          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
         </is>
       </c>
       <c r="E661" t="inlineStr">
         <is>
-          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
+          <t>nová obrazovka hazela vykricnik porad</t>
         </is>
       </c>
       <c r="F661" t="inlineStr">
@@ -21039,24 +21039,24 @@
     </row>
     <row r="662">
       <c r="A662" t="n">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B662" t="inlineStr">
         <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C662" t="inlineStr"/>
+          <t>842 010</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>11.06.2022</t>
+        </is>
+      </c>
       <c r="D662" t="inlineStr">
         <is>
-          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
-        </is>
-      </c>
-      <c r="E662" t="inlineStr">
-        <is>
-          <t>nová obrazovka hazela vykricnik porad</t>
-        </is>
-      </c>
+          <t>Přehození karty TBA v DPV na 842 036</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr"/>
       <c r="F662" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21070,11 +21070,11 @@
     </row>
     <row r="663">
       <c r="A663" t="n">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>842 010</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C663" t="inlineStr">
@@ -21084,7 +21084,7 @@
       </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 036</t>
+          <t>Přehození karty TBA v DPV na 842 010</t>
         </is>
       </c>
       <c r="E663" t="inlineStr"/>
@@ -21101,11 +21101,11 @@
     </row>
     <row r="664">
       <c r="A664" t="n">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C664" t="inlineStr">
@@ -21115,10 +21115,14 @@
       </c>
       <c r="D664" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 010</t>
-        </is>
-      </c>
-      <c r="E664" t="inlineStr"/>
+          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>mirel byl špatný po opravě</t>
+        </is>
+      </c>
       <c r="F664" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21132,26 +21136,26 @@
     </row>
     <row r="665">
       <c r="A665" t="n">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C665" t="inlineStr">
         <is>
-          <t>11.06.2022</t>
+          <t>11.05.2022</t>
         </is>
       </c>
       <c r="D665" t="inlineStr">
         <is>
-          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
         </is>
       </c>
       <c r="E665" t="inlineStr">
         <is>
-          <t>mirel byl špatný po opravě</t>
+          <t>25.11. opraveno</t>
         </is>
       </c>
       <c r="F665" t="inlineStr">
@@ -21167,11 +21171,11 @@
     </row>
     <row r="666">
       <c r="A666" t="n">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C666" t="inlineStr">
@@ -21181,14 +21185,10 @@
       </c>
       <c r="D666" t="inlineStr">
         <is>
-          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
-        </is>
-      </c>
-      <c r="E666" t="inlineStr">
-        <is>
-          <t>25.11. opraveno</t>
-        </is>
-      </c>
+          <t>VESELÍ R3 (odjela)</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr"/>
       <c r="F666" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21202,24 +21202,24 @@
     </row>
     <row r="667">
       <c r="A667" t="n">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>844 020</t>
-        </is>
-      </c>
-      <c r="C667" t="inlineStr">
-        <is>
-          <t>11.05.2022</t>
-        </is>
-      </c>
+          <t>814 190</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr"/>
       <c r="D667" t="inlineStr">
         <is>
-          <t>VESELÍ R3 (odjela)</t>
-        </is>
-      </c>
-      <c r="E667" t="inlineStr"/>
+          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>hlášeno p.Škodovi</t>
+        </is>
+      </c>
       <c r="F667" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21233,22 +21233,22 @@
     </row>
     <row r="668">
       <c r="A668" t="n">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B668" t="inlineStr">
         <is>
-          <t>814 190</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C668" t="inlineStr"/>
       <c r="D668" t="inlineStr">
         <is>
-          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
         </is>
       </c>
       <c r="E668" t="inlineStr">
         <is>
-          <t>hlášeno p.Škodovi</t>
+          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
         </is>
       </c>
       <c r="F668" t="inlineStr">
@@ -21264,24 +21264,20 @@
     </row>
     <row r="669">
       <c r="A669" t="n">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C669" t="inlineStr"/>
       <c r="D669" t="inlineStr">
         <is>
-          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
-        </is>
-      </c>
-      <c r="E669" t="inlineStr">
-        <is>
-          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
-        </is>
-      </c>
+          <t>dosazen předzesilovač linky</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr"/>
       <c r="F669" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21295,20 +21291,28 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
           <t>814 073</t>
         </is>
       </c>
-      <c r="C670" t="inlineStr"/>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>09.07.2022</t>
+        </is>
+      </c>
       <c r="D670" t="inlineStr">
         <is>
-          <t>dosazen předzesilovač linky</t>
-        </is>
-      </c>
-      <c r="E670" t="inlineStr"/>
+          <t>chybějící díl</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>předzasilovač linky - objednán nový</t>
+        </is>
+      </c>
       <c r="F670" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21322,26 +21326,26 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 003</t>
         </is>
       </c>
       <c r="C671" t="inlineStr">
         <is>
-          <t>09.07.2022</t>
+          <t>09.03.2022</t>
         </is>
       </c>
       <c r="D671" t="inlineStr">
         <is>
-          <t>chybějící díl</t>
+          <t>dosazen díl</t>
         </is>
       </c>
       <c r="E671" t="inlineStr">
         <is>
-          <t>předzasilovač linky - objednán nový</t>
+          <t>dosazen předzasilovač linky A23</t>
         </is>
       </c>
       <c r="F671" t="inlineStr">
@@ -21357,26 +21361,22 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C672" t="inlineStr">
-        <is>
-          <t>09.03.2022</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr"/>
       <c r="D672" t="inlineStr">
         <is>
-          <t>dosazen díl</t>
+          <t>oprava dveří na B pravé po směru jízdy</t>
         </is>
       </c>
       <c r="E672" t="inlineStr">
         <is>
-          <t>dosazen předzasilovač linky A23</t>
+          <t>vadný motorek</t>
         </is>
       </c>
       <c r="F672" t="inlineStr">
@@ -21392,22 +21392,22 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C673" t="inlineStr"/>
       <c r="D673" t="inlineStr">
         <is>
-          <t>oprava dveří na B pravé po směru jízdy</t>
+          <t>vadné čidlo množství písku M5</t>
         </is>
       </c>
       <c r="E673" t="inlineStr">
         <is>
-          <t>vadný motorek</t>
+          <t>2. osa pravo po smeru jizdy z B</t>
         </is>
       </c>
       <c r="F673" t="inlineStr">
@@ -21423,22 +21423,22 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C674" t="inlineStr"/>
       <c r="D674" t="inlineStr">
         <is>
-          <t>vadné čidlo množství písku M5</t>
+          <t>rychloměr dán do skladu na opravu</t>
         </is>
       </c>
       <c r="E674" t="inlineStr">
         <is>
-          <t>2. osa pravo po smeru jizdy z B</t>
+          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
         </is>
       </c>
       <c r="F674" t="inlineStr">
@@ -21454,22 +21454,22 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C675" t="inlineStr"/>
       <c r="D675" t="inlineStr">
         <is>
-          <t>rychloměr dán do skladu na opravu</t>
+          <t>rychloměr nekomunikuje</t>
         </is>
       </c>
       <c r="E675" t="inlineStr">
         <is>
-          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
+          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
         </is>
       </c>
       <c r="F675" t="inlineStr">
@@ -21485,22 +21485,26 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
-          <t>844 022</t>
-        </is>
-      </c>
-      <c r="C676" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>10.08.2021</t>
+        </is>
+      </c>
       <c r="D676" t="inlineStr">
         <is>
-          <t>rychloměr nekomunikuje</t>
+          <t>dosazeny díly</t>
         </is>
       </c>
       <c r="E676" t="inlineStr">
         <is>
-          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
+          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
         </is>
       </c>
       <c r="F676" t="inlineStr">
@@ -21516,18 +21520,14 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C677" t="inlineStr">
-        <is>
-          <t>10.08.2021</t>
-        </is>
-      </c>
+      <c r="C677" t="inlineStr"/>
       <c r="D677" t="inlineStr">
         <is>
           <t>dosazeny díly</t>
@@ -21535,7 +21535,7 @@
       </c>
       <c r="E677" t="inlineStr">
         <is>
-          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
+          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
         </is>
       </c>
       <c r="F677" t="inlineStr">
@@ -21551,22 +21551,26 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C678" t="inlineStr"/>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>09.06.2021</t>
+        </is>
+      </c>
       <c r="D678" t="inlineStr">
         <is>
-          <t>dosazeny díly</t>
+          <t>Chybějící díly z důvodu použití na jinou lok.</t>
         </is>
       </c>
       <c r="E678" t="inlineStr">
         <is>
-          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
+          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
         </is>
       </c>
       <c r="F678" t="inlineStr">
@@ -21582,28 +21586,16 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C679" t="inlineStr">
-        <is>
-          <t>09.06.2021</t>
-        </is>
-      </c>
-      <c r="D679" t="inlineStr">
-        <is>
-          <t>Chybějící díly z důvodu použití na jinou lok.</t>
-        </is>
-      </c>
-      <c r="E679" t="inlineStr">
-        <is>
-          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
-        </is>
-      </c>
+          <t>842 015</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr"/>
+      <c r="D679" t="inlineStr"/>
+      <c r="E679" t="inlineStr"/>
       <c r="F679" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21617,15 +21609,19 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>029 221</t>
         </is>
       </c>
       <c r="C680" t="inlineStr"/>
-      <c r="D680" t="inlineStr"/>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="E680" t="inlineStr"/>
       <c r="F680" t="inlineStr">
         <is>
@@ -21640,11 +21636,11 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
-          <t>029 221</t>
+          <t>029 222</t>
         </is>
       </c>
       <c r="C681" t="inlineStr"/>
@@ -21667,19 +21663,15 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>029 222</t>
+          <t>714 226</t>
         </is>
       </c>
       <c r="C682" t="inlineStr"/>
-      <c r="D682" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
+      <c r="D682" t="inlineStr"/>
       <c r="E682" t="inlineStr"/>
       <c r="F682" t="inlineStr">
         <is>
@@ -21694,15 +21686,19 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>714 226</t>
+          <t>742 263</t>
         </is>
       </c>
       <c r="C683" t="inlineStr"/>
-      <c r="D683" t="inlineStr"/>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="E683" t="inlineStr"/>
       <c r="F683" t="inlineStr">
         <is>
@@ -21717,17 +21713,17 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>742 263</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C684" t="inlineStr"/>
       <c r="D684" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>výměna obrazovky Lokel na 914</t>
         </is>
       </c>
       <c r="E684" t="inlineStr"/>
@@ -21744,17 +21740,17 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C685" t="inlineStr"/>
       <c r="D685" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E685" t="inlineStr"/>
@@ -21771,17 +21767,17 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C686" t="inlineStr"/>
       <c r="D686" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="E686" t="inlineStr"/>
@@ -21798,17 +21794,17 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C687" t="inlineStr"/>
       <c r="D687" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E687" t="inlineStr"/>
@@ -21825,7 +21821,7 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
@@ -21835,10 +21831,14 @@
       <c r="C688" t="inlineStr"/>
       <c r="D688" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E688" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F688" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21852,24 +21852,20 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E689" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr"/>
       <c r="F689" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21883,7 +21879,7 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
@@ -21893,7 +21889,7 @@
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E690" t="inlineStr"/>
@@ -21910,17 +21906,17 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E691" t="inlineStr"/>
@@ -21937,20 +21933,24 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E692" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F692" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21964,7 +21964,7 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
@@ -21974,12 +21974,12 @@
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E693" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F693" t="inlineStr">
@@ -21995,24 +21995,24 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C694" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D694" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E694" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr"/>
       <c r="F694" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22026,7 +22026,7 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
@@ -22035,12 +22035,12 @@
       </c>
       <c r="C695" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D695" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E695" t="inlineStr"/>
@@ -22057,7 +22057,7 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
@@ -22071,7 +22071,7 @@
       </c>
       <c r="D696" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E696" t="inlineStr"/>
@@ -22088,7 +22088,7 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
@@ -22102,10 +22102,14 @@
       </c>
       <c r="D697" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E697" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F697" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22119,7 +22123,7 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
@@ -22133,12 +22137,12 @@
       </c>
       <c r="D698" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E698" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F698" t="inlineStr">
@@ -22154,7 +22158,7 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
@@ -22168,14 +22172,10 @@
       </c>
       <c r="D699" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E699" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr"/>
       <c r="F699" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22189,24 +22189,24 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C700" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr"/>
       <c r="D700" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E700" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F700" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22220,24 +22220,20 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C701" t="inlineStr"/>
       <c r="D701" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E701" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr"/>
       <c r="F701" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22251,7 +22247,7 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
@@ -22261,7 +22257,7 @@
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
         </is>
       </c>
       <c r="E702" t="inlineStr"/>
@@ -22278,17 +22274,17 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E703" t="inlineStr"/>
@@ -22305,7 +22301,7 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
@@ -22315,10 +22311,14 @@
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E704" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F704" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22332,24 +22332,20 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E705" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr"/>
       <c r="F705" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22363,7 +22359,7 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
@@ -22373,7 +22369,7 @@
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E706" t="inlineStr"/>
@@ -22390,7 +22386,7 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
@@ -22400,7 +22396,7 @@
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E707" t="inlineStr"/>
@@ -22417,17 +22413,17 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E708" t="inlineStr"/>
@@ -22444,7 +22440,7 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
@@ -22454,10 +22450,14 @@
       <c r="C709" t="inlineStr"/>
       <c r="D709" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="E709" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F709" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22471,7 +22471,7 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
@@ -22481,14 +22481,10 @@
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E710" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr"/>
       <c r="F710" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22502,7 +22498,7 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
@@ -22512,10 +22508,14 @@
       <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E711" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F711" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22529,7 +22529,7 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
@@ -22539,14 +22539,10 @@
       <c r="C712" t="inlineStr"/>
       <c r="D712" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E712" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr"/>
       <c r="F712" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22560,7 +22556,7 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
@@ -22570,7 +22566,7 @@
       <c r="C713" t="inlineStr"/>
       <c r="D713" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E713" t="inlineStr"/>
@@ -22587,7 +22583,7 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
@@ -22597,10 +22593,14 @@
       <c r="C714" t="inlineStr"/>
       <c r="D714" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E714" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F714" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22614,7 +22614,7 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
@@ -22624,12 +22624,12 @@
       <c r="C715" t="inlineStr"/>
       <c r="D715" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E715" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F715" t="inlineStr">
@@ -22645,7 +22645,7 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
@@ -22655,12 +22655,12 @@
       <c r="C716" t="inlineStr"/>
       <c r="D716" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E716" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F716" t="inlineStr">
@@ -22676,24 +22676,20 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E717" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr"/>
       <c r="F717" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22707,7 +22703,7 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
@@ -22717,10 +22713,14 @@
       <c r="C718" t="inlineStr"/>
       <c r="D718" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E718" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F718" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22734,7 +22734,7 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
@@ -22744,12 +22744,12 @@
       <c r="C719" t="inlineStr"/>
       <c r="D719" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E719" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F719" t="inlineStr">
@@ -22765,7 +22765,7 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
@@ -22775,14 +22775,10 @@
       <c r="C720" t="inlineStr"/>
       <c r="D720" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E720" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr"/>
       <c r="F720" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22796,17 +22792,17 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C721" t="inlineStr"/>
       <c r="D721" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E721" t="inlineStr"/>
@@ -22823,7 +22819,7 @@
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
@@ -22833,7 +22829,7 @@
       <c r="C722" t="inlineStr"/>
       <c r="D722" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E722" t="inlineStr"/>
@@ -22850,7 +22846,7 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
@@ -22860,10 +22856,14 @@
       <c r="C723" t="inlineStr"/>
       <c r="D723" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E723" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F723" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22877,22 +22877,22 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C724" t="inlineStr"/>
       <c r="D724" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E724" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F724" t="inlineStr">
@@ -22908,7 +22908,7 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
@@ -22918,12 +22918,12 @@
       <c r="C725" t="inlineStr"/>
       <c r="D725" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E725" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F725" t="inlineStr">
@@ -22939,24 +22939,20 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C726" t="inlineStr"/>
       <c r="D726" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E726" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr"/>
       <c r="F726" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22970,20 +22966,24 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C727" t="inlineStr"/>
       <c r="D727" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E727" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F727" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22997,24 +22997,20 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C728" t="inlineStr"/>
       <c r="D728" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E728" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr"/>
       <c r="F728" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23028,7 +23024,7 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
@@ -23038,7 +23034,7 @@
       <c r="C729" t="inlineStr"/>
       <c r="D729" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E729" t="inlineStr"/>
@@ -23055,7 +23051,7 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
@@ -23065,7 +23061,7 @@
       <c r="C730" t="inlineStr"/>
       <c r="D730" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E730" t="inlineStr"/>
@@ -23082,7 +23078,7 @@
     </row>
     <row r="731">
       <c r="A731" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
@@ -23092,7 +23088,7 @@
       <c r="C731" t="inlineStr"/>
       <c r="D731" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E731" t="inlineStr"/>
@@ -23109,7 +23105,7 @@
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
@@ -23119,10 +23115,14 @@
       <c r="C732" t="inlineStr"/>
       <c r="D732" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E732" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F732" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23136,24 +23136,20 @@
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C733" t="inlineStr"/>
       <c r="D733" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E733" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr"/>
       <c r="F733" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23167,7 +23163,7 @@
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
@@ -23177,7 +23173,7 @@
       <c r="C734" t="inlineStr"/>
       <c r="D734" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E734" t="inlineStr"/>
@@ -23194,20 +23190,24 @@
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C735" t="inlineStr"/>
       <c r="D735" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E735" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F735" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23221,24 +23221,20 @@
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C736" t="inlineStr"/>
       <c r="D736" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E736" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr"/>
       <c r="F736" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23252,7 +23248,7 @@
     </row>
     <row r="737">
       <c r="A737" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
@@ -23262,7 +23258,7 @@
       <c r="C737" t="inlineStr"/>
       <c r="D737" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E737" t="inlineStr"/>
@@ -23279,20 +23275,24 @@
     </row>
     <row r="738">
       <c r="A738" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C738" t="inlineStr"/>
       <c r="D738" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E738" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F738" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23306,27 +23306,31 @@
     </row>
     <row r="739">
       <c r="A739" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C739" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D739" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E739" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F739" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G739" t="inlineStr">
@@ -23337,11 +23341,11 @@
     </row>
     <row r="740">
       <c r="A740" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C740" t="inlineStr">
@@ -23351,12 +23355,12 @@
       </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E740" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F740" t="inlineStr">
@@ -23372,26 +23376,26 @@
     </row>
     <row r="741">
       <c r="A741" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D741" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E741" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F741" t="inlineStr">
@@ -23407,31 +23411,27 @@
     </row>
     <row r="742">
       <c r="A742" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C742" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D742" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E742" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr"/>
       <c r="F742" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G742" t="inlineStr">
@@ -23442,27 +23442,27 @@
     </row>
     <row r="743">
       <c r="A743" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C743" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D743" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E743" t="inlineStr"/>
       <c r="F743" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G743" t="inlineStr">
@@ -23473,27 +23473,27 @@
     </row>
     <row r="744">
       <c r="A744" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C744" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D744" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E744" t="inlineStr"/>
       <c r="F744" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G744" t="inlineStr">
@@ -23504,27 +23504,27 @@
     </row>
     <row r="745">
       <c r="A745" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B745" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C745" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D745" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E745" t="inlineStr"/>
       <c r="F745" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G745" t="inlineStr">
@@ -23535,24 +23535,28 @@
     </row>
     <row r="746">
       <c r="A746" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C746" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D746" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E746" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F746" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -23566,11 +23570,11 @@
     </row>
     <row r="747">
       <c r="A747" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C747" t="inlineStr">
@@ -23580,12 +23584,12 @@
       </c>
       <c r="D747" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E747" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F747" t="inlineStr">
@@ -23601,11 +23605,11 @@
     </row>
     <row r="748">
       <c r="A748" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C748" t="inlineStr">
@@ -23615,7 +23619,7 @@
       </c>
       <c r="D748" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E748" t="inlineStr">
@@ -23636,31 +23640,31 @@
     </row>
     <row r="749">
       <c r="A749" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B749" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C749" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D749" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E749" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F749" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G749" t="inlineStr">
@@ -23671,31 +23675,27 @@
     </row>
     <row r="750">
       <c r="A750" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B750" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C750" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D750" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E750" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr"/>
       <c r="F750" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G750" t="inlineStr">
@@ -23706,57 +23706,53 @@
     </row>
     <row r="751">
       <c r="A751" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B751" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C751" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D751" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E751" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F751" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
-        </is>
-      </c>
-      <c r="G751" t="inlineStr">
-        <is>
-          <t>Bez fotky</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G751" t="inlineStr"/>
     </row>
     <row r="752">
       <c r="A752" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B752" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C752" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr"/>
       <c r="D752" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E752" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F752" t="inlineStr">
@@ -23768,92 +23764,65 @@
     </row>
     <row r="753">
       <c r="A753" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B753" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C753" t="inlineStr"/>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D753" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
-        </is>
-      </c>
-      <c r="E753" t="inlineStr">
-        <is>
-          <t>Prohozní s 844 028 - A2.6</t>
-        </is>
-      </c>
+          <t>Vývaz motoru "B"</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr"/>
       <c r="F753" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G753" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="754">
       <c r="A754" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B754" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C754" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D754" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
-        </is>
-      </c>
-      <c r="E754" t="inlineStr"/>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>Vadná černá karta v bobku</t>
+        </is>
+      </c>
       <c r="F754" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G754" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="755">
-      <c r="A755" t="n">
-        <v>759</v>
-      </c>
-      <c r="B755" t="inlineStr">
-        <is>
-          <t>814 120</t>
-        </is>
-      </c>
-      <c r="C755" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
-      <c r="D755" t="inlineStr">
-        <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
-        </is>
-      </c>
-      <c r="E755" t="inlineStr">
-        <is>
-          <t>Vadná černá karta v bobku</t>
-        </is>
-      </c>
-      <c r="F755" t="inlineStr">
-        <is>
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G755" t="inlineStr"/>
+      <c r="G754" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Smazána závada ID 621 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G754"/>
+  <dimension ref="A1:G753"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19710,11 +19710,11 @@
     </row>
     <row r="619">
       <c r="A619" t="n">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>810 015</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C619" t="inlineStr">
@@ -19724,12 +19724,12 @@
       </c>
       <c r="D619" t="inlineStr">
         <is>
-          <t>nejde AVJF</t>
+          <t>Nejdou dvěře WC</t>
         </is>
       </c>
       <c r="E619" t="inlineStr">
         <is>
-          <t>byla vypadlá vratná pojistka,baterka měla 11V.Výměna baterie.Odzkoušení OK</t>
+          <t>upadlý drát na přepínači funkce WC (zapnuto,bez dveří, vypnuto). Seřízení zámykání dveří. Frýdek</t>
         </is>
       </c>
       <c r="F619" t="inlineStr">
@@ -19745,11 +19745,11 @@
     </row>
     <row r="620">
       <c r="A620" t="n">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C620" t="inlineStr">
@@ -19759,12 +19759,12 @@
       </c>
       <c r="D620" t="inlineStr">
         <is>
-          <t>Nejdou dvěře WC</t>
+          <t>údajně nejdou někdy schody u levých dveří strany A</t>
         </is>
       </c>
       <c r="E620" t="inlineStr">
         <is>
-          <t>upadlý drát na přepínači funkce WC (zapnuto,bez dveří, vypnuto). Seřízení zámykání dveří. Frýdek</t>
+          <t>vyčištění od kamínků,odzkoušení-OK</t>
         </is>
       </c>
       <c r="F620" t="inlineStr">
@@ -19780,26 +19780,26 @@
     </row>
     <row r="621">
       <c r="A621" t="n">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C621" t="inlineStr">
         <is>
-          <t>06.09.2023</t>
+          <t>06.08.2023</t>
         </is>
       </c>
       <c r="D621" t="inlineStr">
         <is>
-          <t>údajně nejdou někdy schody u levých dveří strany A</t>
+          <t>zapůjčena z HB</t>
         </is>
       </c>
       <c r="E621" t="inlineStr">
         <is>
-          <t>vyčištění od kamínků,odzkoušení-OK</t>
+          <t>nahrány data IS ( funguje preš radiostanici)</t>
         </is>
       </c>
       <c r="F621" t="inlineStr">
@@ -19815,11 +19815,11 @@
     </row>
     <row r="622">
       <c r="A622" t="n">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C622" t="inlineStr">
@@ -19829,12 +19829,12 @@
       </c>
       <c r="D622" t="inlineStr">
         <is>
-          <t>zapůjčena z HB</t>
+          <t>Opět problémy se startováním</t>
         </is>
       </c>
       <c r="E622" t="inlineStr">
         <is>
-          <t>nahrány data IS ( funguje preš radiostanici)</t>
+          <t>(asi už vadný capos kondy)říkali veselani jak tu byli</t>
         </is>
       </c>
       <c r="F622" t="inlineStr">
@@ -19850,7 +19850,7 @@
     </row>
     <row r="623">
       <c r="A623" t="n">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B623" t="inlineStr">
         <is>
@@ -19864,12 +19864,12 @@
       </c>
       <c r="D623" t="inlineStr">
         <is>
-          <t>Opět problémy se startováním</t>
+          <t>oprava hlasitosti na stanovišti A</t>
         </is>
       </c>
       <c r="E623" t="inlineStr">
         <is>
-          <t>(asi už vadný capos kondy)říkali veselani jak tu byli</t>
+          <t>přechod na kontaktech u reproduktoru v pultě</t>
         </is>
       </c>
       <c r="F623" t="inlineStr">
@@ -19885,11 +19885,11 @@
     </row>
     <row r="624">
       <c r="A624" t="n">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C624" t="inlineStr">
@@ -19899,12 +19899,12 @@
       </c>
       <c r="D624" t="inlineStr">
         <is>
-          <t>oprava hlasitosti na stanovišti A</t>
+          <t>výměna ARR na B</t>
         </is>
       </c>
       <c r="E624" t="inlineStr">
         <is>
-          <t>přechod na kontaktech u reproduktoru v pultě</t>
+          <t>vadná linka CAN</t>
         </is>
       </c>
       <c r="F624" t="inlineStr">
@@ -19920,26 +19920,26 @@
     </row>
     <row r="625">
       <c r="A625" t="n">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B625" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>842 015</t>
         </is>
       </c>
       <c r="C625" t="inlineStr">
         <is>
-          <t>06.08.2023</t>
+          <t>06.07.2023</t>
         </is>
       </c>
       <c r="D625" t="inlineStr">
         <is>
-          <t>výměna ARR na B</t>
+          <t>někdy nejde brzda PB</t>
         </is>
       </c>
       <c r="E625" t="inlineStr">
         <is>
-          <t>vadná linka CAN</t>
+          <t>výměna karty DS a OUT z 842 025</t>
         </is>
       </c>
       <c r="F625" t="inlineStr">
@@ -19955,11 +19955,11 @@
     </row>
     <row r="626">
       <c r="A626" t="n">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C626" t="inlineStr">
@@ -19969,14 +19969,10 @@
       </c>
       <c r="D626" t="inlineStr">
         <is>
-          <t>někdy nejde brzda PB</t>
-        </is>
-      </c>
-      <c r="E626" t="inlineStr">
-        <is>
-          <t>výměna karty DS a OUT z 842 025</t>
-        </is>
-      </c>
+          <t>dosazeny karty z 842 015 (DS a OUT)</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr"/>
       <c r="F626" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19990,11 +19986,11 @@
     </row>
     <row r="627">
       <c r="A627" t="n">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C627" t="inlineStr">
@@ -20004,10 +20000,14 @@
       </c>
       <c r="D627" t="inlineStr">
         <is>
-          <t>dosazeny karty z 842 015 (DS a OUT)</t>
-        </is>
-      </c>
-      <c r="E627" t="inlineStr"/>
+          <t>dosazen asi 5 dobíječ na B funkční</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>ve skladu nefunkční jenom (má řešit asi Mlíčko)</t>
+        </is>
+      </c>
       <c r="F627" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20021,28 +20021,24 @@
     </row>
     <row r="628">
       <c r="A628" t="n">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 076</t>
         </is>
       </c>
       <c r="C628" t="inlineStr">
         <is>
-          <t>06.07.2023</t>
+          <t>06.06.2023</t>
         </is>
       </c>
       <c r="D628" t="inlineStr">
         <is>
-          <t>dosazen asi 5 dobíječ na B funkční</t>
-        </is>
-      </c>
-      <c r="E628" t="inlineStr">
-        <is>
-          <t>ve skladu nefunkční jenom (má řešit asi Mlíčko)</t>
-        </is>
-      </c>
+          <t>NEHODA V HOLEŠOVĚ</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr"/>
       <c r="F628" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20056,21 +20052,21 @@
     </row>
     <row r="629">
       <c r="A629" t="n">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>814 076</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>06.06.2023</t>
+          <t>06.05.2023</t>
         </is>
       </c>
       <c r="D629" t="inlineStr">
         <is>
-          <t>NEHODA V HOLEŠOVĚ</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E629" t="inlineStr"/>
@@ -20087,21 +20083,17 @@
     </row>
     <row r="630">
       <c r="A630" t="n">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C630" t="inlineStr">
-        <is>
-          <t>06.05.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr"/>
       <c r="D630" t="inlineStr">
         <is>
-          <t>MM</t>
+          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
         </is>
       </c>
       <c r="E630" t="inlineStr"/>
@@ -20118,7 +20110,7 @@
     </row>
     <row r="631">
       <c r="A631" t="n">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="B631" t="inlineStr">
         <is>
@@ -20128,7 +20120,7 @@
       <c r="C631" t="inlineStr"/>
       <c r="D631" t="inlineStr">
         <is>
-          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
+          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
         </is>
       </c>
       <c r="E631" t="inlineStr"/>
@@ -20145,7 +20137,7 @@
     </row>
     <row r="632">
       <c r="A632" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B632" t="inlineStr">
         <is>
@@ -20155,7 +20147,7 @@
       <c r="C632" t="inlineStr"/>
       <c r="D632" t="inlineStr">
         <is>
-          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
+          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
         </is>
       </c>
       <c r="E632" t="inlineStr"/>
@@ -20172,20 +20164,24 @@
     </row>
     <row r="633">
       <c r="A633" t="n">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C633" t="inlineStr"/>
       <c r="D633" t="inlineStr">
         <is>
-          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
-        </is>
-      </c>
-      <c r="E633" t="inlineStr"/>
+          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>vyměnili dobíječ stacionární (Veselí)</t>
+        </is>
+      </c>
       <c r="F633" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20199,22 +20195,22 @@
     </row>
     <row r="634">
       <c r="A634" t="n">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C634" t="inlineStr"/>
       <c r="D634" t="inlineStr">
         <is>
-          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
         </is>
       </c>
       <c r="E634" t="inlineStr">
         <is>
-          <t>vyměnili dobíječ stacionární (Veselí)</t>
+          <t>jela ven</t>
         </is>
       </c>
       <c r="F634" t="inlineStr">
@@ -20230,24 +20226,20 @@
     </row>
     <row r="635">
       <c r="A635" t="n">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C635" t="inlineStr"/>
       <c r="D635" t="inlineStr">
         <is>
-          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
-        </is>
-      </c>
-      <c r="E635" t="inlineStr">
-        <is>
-          <t>jela ven</t>
-        </is>
-      </c>
+          <t>seřízení kamer přes program v notasu(obraz)</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr"/>
       <c r="F635" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20261,20 +20253,24 @@
     </row>
     <row r="636">
       <c r="A636" t="n">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C636" t="inlineStr"/>
       <c r="D636" t="inlineStr">
         <is>
-          <t>seřízení kamer přes program v notasu(obraz)</t>
-        </is>
-      </c>
-      <c r="E636" t="inlineStr"/>
+          <t>po startu někdy nenabíjí "B"</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+        </is>
+      </c>
       <c r="F636" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20288,22 +20284,22 @@
     </row>
     <row r="637">
       <c r="A637" t="n">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C637" t="inlineStr"/>
       <c r="D637" t="inlineStr">
         <is>
-          <t>po startu někdy nenabíjí "B"</t>
+          <t>2. motor korekce vody  vystup</t>
         </is>
       </c>
       <c r="E637" t="inlineStr">
         <is>
-          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
         </is>
       </c>
       <c r="F637" t="inlineStr">
@@ -20319,24 +20315,24 @@
     </row>
     <row r="638">
       <c r="A638" t="n">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>842 035</t>
-        </is>
-      </c>
-      <c r="C638" t="inlineStr"/>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>04.12.2023</t>
+        </is>
+      </c>
       <c r="D638" t="inlineStr">
         <is>
-          <t>2. motor korekce vody  vystup</t>
-        </is>
-      </c>
-      <c r="E638" t="inlineStr">
-        <is>
-          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
-        </is>
-      </c>
+          <t>Výměna motoru A</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr"/>
       <c r="F638" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20350,21 +20346,17 @@
     </row>
     <row r="639">
       <c r="A639" t="n">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C639" t="inlineStr">
-        <is>
-          <t>04.12.2023</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr"/>
       <c r="D639" t="inlineStr">
         <is>
-          <t>Výměna motoru A</t>
+          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
         </is>
       </c>
       <c r="E639" t="inlineStr"/>
@@ -20381,17 +20373,17 @@
     </row>
     <row r="640">
       <c r="A640" t="n">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C640" t="inlineStr"/>
       <c r="D640" t="inlineStr">
         <is>
-          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
+          <t>dosazena nahadni Mirelka + NO z 844 013</t>
         </is>
       </c>
       <c r="E640" t="inlineStr"/>
@@ -20408,17 +20400,17 @@
     </row>
     <row r="641">
       <c r="A641" t="n">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 062</t>
         </is>
       </c>
       <c r="C641" t="inlineStr"/>
       <c r="D641" t="inlineStr">
         <is>
-          <t>dosazena nahadni Mirelka + NO z 844 013</t>
+          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
         </is>
       </c>
       <c r="E641" t="inlineStr"/>
@@ -20435,17 +20427,21 @@
     </row>
     <row r="642">
       <c r="A642" t="n">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>814 062</t>
-        </is>
-      </c>
-      <c r="C642" t="inlineStr"/>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>03.03.2023</t>
+        </is>
+      </c>
       <c r="D642" t="inlineStr">
         <is>
-          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E642" t="inlineStr"/>
@@ -20462,11 +20458,11 @@
     </row>
     <row r="643">
       <c r="A643" t="n">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C643" t="inlineStr">
@@ -20476,7 +20472,7 @@
       </c>
       <c r="D643" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
+          <t>Dosazení ŘJ kamer</t>
         </is>
       </c>
       <c r="E643" t="inlineStr"/>
@@ -20493,24 +20489,24 @@
     </row>
     <row r="644">
       <c r="A644" t="n">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>844 013</t>
-        </is>
-      </c>
-      <c r="C644" t="inlineStr">
-        <is>
-          <t>03.03.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr"/>
       <c r="D644" t="inlineStr">
         <is>
-          <t>Dosazení ŘJ kamer</t>
-        </is>
-      </c>
-      <c r="E644" t="inlineStr"/>
+          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>hlášeno p. Škodovi</t>
+        </is>
+      </c>
       <c r="F644" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20524,24 +20520,20 @@
     </row>
     <row r="645">
       <c r="A645" t="n">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C645" t="inlineStr"/>
       <c r="D645" t="inlineStr">
         <is>
-          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
-        </is>
-      </c>
-      <c r="E645" t="inlineStr">
-        <is>
-          <t>hlášeno p. Škodovi</t>
-        </is>
-      </c>
+          <t>ŘJ kamer dosazena z 013</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr"/>
       <c r="F645" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20555,17 +20547,21 @@
     </row>
     <row r="646">
       <c r="A646" t="n">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B646" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C646" t="inlineStr"/>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>02.09.2023</t>
+        </is>
+      </c>
       <c r="D646" t="inlineStr">
         <is>
-          <t>ŘJ kamer dosazena z 013</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E646" t="inlineStr"/>
@@ -20582,21 +20578,21 @@
     </row>
     <row r="647">
       <c r="A647" t="n">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 072</t>
         </is>
       </c>
       <c r="C647" t="inlineStr">
         <is>
-          <t>02.09.2023</t>
+          <t>02.03.2023</t>
         </is>
       </c>
       <c r="D647" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E647" t="inlineStr"/>
@@ -20613,24 +20609,24 @@
     </row>
     <row r="648">
       <c r="A648" t="n">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>814 072</t>
-        </is>
-      </c>
-      <c r="C648" t="inlineStr">
-        <is>
-          <t>02.03.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr"/>
       <c r="D648" t="inlineStr">
         <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E648" t="inlineStr"/>
+          <t>dosazen opraveny MIREL</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+        </is>
+      </c>
       <c r="F648" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20644,22 +20640,22 @@
     </row>
     <row r="649">
       <c r="A649" t="n">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C649" t="inlineStr"/>
       <c r="D649" t="inlineStr">
         <is>
-          <t>dosazen opraveny MIREL</t>
+          <t>Odpojen trojcestný ventil na A i B</t>
         </is>
       </c>
       <c r="E649" t="inlineStr">
         <is>
-          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+          <t>Zapojeny zpět 24.2.2023</t>
         </is>
       </c>
       <c r="F649" t="inlineStr">
@@ -20675,24 +20671,20 @@
     </row>
     <row r="650">
       <c r="A650" t="n">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C650" t="inlineStr"/>
       <c r="D650" t="inlineStr">
         <is>
-          <t>Odpojen trojcestný ventil na A i B</t>
-        </is>
-      </c>
-      <c r="E650" t="inlineStr">
-        <is>
-          <t>Zapojeny zpět 24.2.2023</t>
-        </is>
-      </c>
+          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr"/>
       <c r="F650" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20706,17 +20698,21 @@
     </row>
     <row r="651">
       <c r="A651" t="n">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B651" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C651" t="inlineStr"/>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>01.10.2023</t>
+        </is>
+      </c>
       <c r="D651" t="inlineStr">
         <is>
-          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E651" t="inlineStr"/>
@@ -20733,21 +20729,17 @@
     </row>
     <row r="652">
       <c r="A652" t="n">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C652" t="inlineStr">
-        <is>
-          <t>01.10.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr"/>
       <c r="D652" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
         </is>
       </c>
       <c r="E652" t="inlineStr"/>
@@ -20764,17 +20756,17 @@
     </row>
     <row r="653">
       <c r="A653" t="n">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C653" t="inlineStr"/>
       <c r="D653" t="inlineStr">
         <is>
-          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
+          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
         </is>
       </c>
       <c r="E653" t="inlineStr"/>
@@ -20791,7 +20783,7 @@
     </row>
     <row r="654">
       <c r="A654" t="n">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B654" t="inlineStr">
         <is>
@@ -20801,7 +20793,7 @@
       <c r="C654" t="inlineStr"/>
       <c r="D654" t="inlineStr">
         <is>
-          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
+          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
         </is>
       </c>
       <c r="E654" t="inlineStr"/>
@@ -20818,20 +20810,24 @@
     </row>
     <row r="655">
       <c r="A655" t="n">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C655" t="inlineStr"/>
       <c r="D655" t="inlineStr">
         <is>
-          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
-        </is>
-      </c>
-      <c r="E655" t="inlineStr"/>
+          <t>Přišel opravený Mirel ve skladu</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>dosazen na 29.12.2022</t>
+        </is>
+      </c>
       <c r="F655" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20845,22 +20841,26 @@
     </row>
     <row r="656">
       <c r="A656" t="n">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C656" t="inlineStr"/>
+          <t>844 014</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>12.06.2022</t>
+        </is>
+      </c>
       <c r="D656" t="inlineStr">
         <is>
-          <t>Přišel opravený Mirel ve skladu</t>
+          <t>rychloměr do opravy hazí !!</t>
         </is>
       </c>
       <c r="E656" t="inlineStr">
         <is>
-          <t>dosazen na 29.12.2022</t>
+          <t>zapujcen z 844 028 z veselí</t>
         </is>
       </c>
       <c r="F656" t="inlineStr">
@@ -20876,11 +20876,11 @@
     </row>
     <row r="657">
       <c r="A657" t="n">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C657" t="inlineStr">
@@ -20890,14 +20890,10 @@
       </c>
       <c r="D657" t="inlineStr">
         <is>
-          <t>rychloměr do opravy hazí !!</t>
-        </is>
-      </c>
-      <c r="E657" t="inlineStr">
-        <is>
-          <t>zapujcen z 844 028 z veselí</t>
-        </is>
-      </c>
+          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr"/>
       <c r="F657" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20911,24 +20907,28 @@
     </row>
     <row r="658">
       <c r="A658" t="n">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C658" t="inlineStr">
         <is>
-          <t>12.06.2022</t>
+          <t>12.03.2022</t>
         </is>
       </c>
       <c r="D658" t="inlineStr">
         <is>
-          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
-        </is>
-      </c>
-      <c r="E658" t="inlineStr"/>
+          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>bude řešit Škoda</t>
+        </is>
+      </c>
       <c r="F658" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20942,26 +20942,22 @@
     </row>
     <row r="659">
       <c r="A659" t="n">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B659" t="inlineStr">
         <is>
           <t>844 003</t>
         </is>
       </c>
-      <c r="C659" t="inlineStr">
-        <is>
-          <t>12.03.2022</t>
-        </is>
-      </c>
+      <c r="C659" t="inlineStr"/>
       <c r="D659" t="inlineStr">
         <is>
-          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+          <t>na A strane asi vadna expanzní nadrz topení ?</t>
         </is>
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>bude řešit Škoda</t>
+          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
         </is>
       </c>
       <c r="F659" t="inlineStr">
@@ -20977,22 +20973,22 @@
     </row>
     <row r="660">
       <c r="A660" t="n">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B660" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C660" t="inlineStr"/>
       <c r="D660" t="inlineStr">
         <is>
-          <t>na A strane asi vadna expanzní nadrz topení ?</t>
+          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
         </is>
       </c>
       <c r="E660" t="inlineStr">
         <is>
-          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
+          <t>nová obrazovka hazela vykricnik porad</t>
         </is>
       </c>
       <c r="F660" t="inlineStr">
@@ -21008,24 +21004,24 @@
     </row>
     <row r="661">
       <c r="A661" t="n">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B661" t="inlineStr">
         <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C661" t="inlineStr"/>
+          <t>842 010</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>11.06.2022</t>
+        </is>
+      </c>
       <c r="D661" t="inlineStr">
         <is>
-          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
-        </is>
-      </c>
-      <c r="E661" t="inlineStr">
-        <is>
-          <t>nová obrazovka hazela vykricnik porad</t>
-        </is>
-      </c>
+          <t>Přehození karty TBA v DPV na 842 036</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr"/>
       <c r="F661" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21039,11 +21035,11 @@
     </row>
     <row r="662">
       <c r="A662" t="n">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B662" t="inlineStr">
         <is>
-          <t>842 010</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C662" t="inlineStr">
@@ -21053,7 +21049,7 @@
       </c>
       <c r="D662" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 036</t>
+          <t>Přehození karty TBA v DPV na 842 010</t>
         </is>
       </c>
       <c r="E662" t="inlineStr"/>
@@ -21070,11 +21066,11 @@
     </row>
     <row r="663">
       <c r="A663" t="n">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C663" t="inlineStr">
@@ -21084,10 +21080,14 @@
       </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 010</t>
-        </is>
-      </c>
-      <c r="E663" t="inlineStr"/>
+          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>mirel byl špatný po opravě</t>
+        </is>
+      </c>
       <c r="F663" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21101,26 +21101,26 @@
     </row>
     <row r="664">
       <c r="A664" t="n">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C664" t="inlineStr">
         <is>
-          <t>11.06.2022</t>
+          <t>11.05.2022</t>
         </is>
       </c>
       <c r="D664" t="inlineStr">
         <is>
-          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
         </is>
       </c>
       <c r="E664" t="inlineStr">
         <is>
-          <t>mirel byl špatný po opravě</t>
+          <t>25.11. opraveno</t>
         </is>
       </c>
       <c r="F664" t="inlineStr">
@@ -21136,11 +21136,11 @@
     </row>
     <row r="665">
       <c r="A665" t="n">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C665" t="inlineStr">
@@ -21150,14 +21150,10 @@
       </c>
       <c r="D665" t="inlineStr">
         <is>
-          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
-        </is>
-      </c>
-      <c r="E665" t="inlineStr">
-        <is>
-          <t>25.11. opraveno</t>
-        </is>
-      </c>
+          <t>VESELÍ R3 (odjela)</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr"/>
       <c r="F665" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21171,24 +21167,24 @@
     </row>
     <row r="666">
       <c r="A666" t="n">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>844 020</t>
-        </is>
-      </c>
-      <c r="C666" t="inlineStr">
-        <is>
-          <t>11.05.2022</t>
-        </is>
-      </c>
+          <t>814 190</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr"/>
       <c r="D666" t="inlineStr">
         <is>
-          <t>VESELÍ R3 (odjela)</t>
-        </is>
-      </c>
-      <c r="E666" t="inlineStr"/>
+          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>hlášeno p.Škodovi</t>
+        </is>
+      </c>
       <c r="F666" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21202,22 +21198,22 @@
     </row>
     <row r="667">
       <c r="A667" t="n">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>814 190</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C667" t="inlineStr"/>
       <c r="D667" t="inlineStr">
         <is>
-          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
         </is>
       </c>
       <c r="E667" t="inlineStr">
         <is>
-          <t>hlášeno p.Škodovi</t>
+          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
         </is>
       </c>
       <c r="F667" t="inlineStr">
@@ -21233,24 +21229,20 @@
     </row>
     <row r="668">
       <c r="A668" t="n">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B668" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C668" t="inlineStr"/>
       <c r="D668" t="inlineStr">
         <is>
-          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
-        </is>
-      </c>
-      <c r="E668" t="inlineStr">
-        <is>
-          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
-        </is>
-      </c>
+          <t>dosazen předzesilovač linky</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr"/>
       <c r="F668" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21264,20 +21256,28 @@
     </row>
     <row r="669">
       <c r="A669" t="n">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B669" t="inlineStr">
         <is>
           <t>814 073</t>
         </is>
       </c>
-      <c r="C669" t="inlineStr"/>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>09.07.2022</t>
+        </is>
+      </c>
       <c r="D669" t="inlineStr">
         <is>
-          <t>dosazen předzesilovač linky</t>
-        </is>
-      </c>
-      <c r="E669" t="inlineStr"/>
+          <t>chybějící díl</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>předzasilovač linky - objednán nový</t>
+        </is>
+      </c>
       <c r="F669" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21291,26 +21291,26 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 003</t>
         </is>
       </c>
       <c r="C670" t="inlineStr">
         <is>
-          <t>09.07.2022</t>
+          <t>09.03.2022</t>
         </is>
       </c>
       <c r="D670" t="inlineStr">
         <is>
-          <t>chybějící díl</t>
+          <t>dosazen díl</t>
         </is>
       </c>
       <c r="E670" t="inlineStr">
         <is>
-          <t>předzasilovač linky - objednán nový</t>
+          <t>dosazen předzasilovač linky A23</t>
         </is>
       </c>
       <c r="F670" t="inlineStr">
@@ -21326,26 +21326,22 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C671" t="inlineStr">
-        <is>
-          <t>09.03.2022</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr"/>
       <c r="D671" t="inlineStr">
         <is>
-          <t>dosazen díl</t>
+          <t>oprava dveří na B pravé po směru jízdy</t>
         </is>
       </c>
       <c r="E671" t="inlineStr">
         <is>
-          <t>dosazen předzasilovač linky A23</t>
+          <t>vadný motorek</t>
         </is>
       </c>
       <c r="F671" t="inlineStr">
@@ -21361,22 +21357,22 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C672" t="inlineStr"/>
       <c r="D672" t="inlineStr">
         <is>
-          <t>oprava dveří na B pravé po směru jízdy</t>
+          <t>vadné čidlo množství písku M5</t>
         </is>
       </c>
       <c r="E672" t="inlineStr">
         <is>
-          <t>vadný motorek</t>
+          <t>2. osa pravo po smeru jizdy z B</t>
         </is>
       </c>
       <c r="F672" t="inlineStr">
@@ -21392,22 +21388,22 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C673" t="inlineStr"/>
       <c r="D673" t="inlineStr">
         <is>
-          <t>vadné čidlo množství písku M5</t>
+          <t>rychloměr dán do skladu na opravu</t>
         </is>
       </c>
       <c r="E673" t="inlineStr">
         <is>
-          <t>2. osa pravo po smeru jizdy z B</t>
+          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
         </is>
       </c>
       <c r="F673" t="inlineStr">
@@ -21423,22 +21419,22 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C674" t="inlineStr"/>
       <c r="D674" t="inlineStr">
         <is>
-          <t>rychloměr dán do skladu na opravu</t>
+          <t>rychloměr nekomunikuje</t>
         </is>
       </c>
       <c r="E674" t="inlineStr">
         <is>
-          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
+          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
         </is>
       </c>
       <c r="F674" t="inlineStr">
@@ -21454,22 +21450,26 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
-          <t>844 022</t>
-        </is>
-      </c>
-      <c r="C675" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>10.08.2021</t>
+        </is>
+      </c>
       <c r="D675" t="inlineStr">
         <is>
-          <t>rychloměr nekomunikuje</t>
+          <t>dosazeny díly</t>
         </is>
       </c>
       <c r="E675" t="inlineStr">
         <is>
-          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
+          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
         </is>
       </c>
       <c r="F675" t="inlineStr">
@@ -21485,18 +21485,14 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C676" t="inlineStr">
-        <is>
-          <t>10.08.2021</t>
-        </is>
-      </c>
+      <c r="C676" t="inlineStr"/>
       <c r="D676" t="inlineStr">
         <is>
           <t>dosazeny díly</t>
@@ -21504,7 +21500,7 @@
       </c>
       <c r="E676" t="inlineStr">
         <is>
-          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
+          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
         </is>
       </c>
       <c r="F676" t="inlineStr">
@@ -21520,22 +21516,26 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C677" t="inlineStr"/>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>09.06.2021</t>
+        </is>
+      </c>
       <c r="D677" t="inlineStr">
         <is>
-          <t>dosazeny díly</t>
+          <t>Chybějící díly z důvodu použití na jinou lok.</t>
         </is>
       </c>
       <c r="E677" t="inlineStr">
         <is>
-          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
+          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
         </is>
       </c>
       <c r="F677" t="inlineStr">
@@ -21551,28 +21551,16 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C678" t="inlineStr">
-        <is>
-          <t>09.06.2021</t>
-        </is>
-      </c>
-      <c r="D678" t="inlineStr">
-        <is>
-          <t>Chybějící díly z důvodu použití na jinou lok.</t>
-        </is>
-      </c>
-      <c r="E678" t="inlineStr">
-        <is>
-          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
-        </is>
-      </c>
+          <t>842 015</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr"/>
+      <c r="D678" t="inlineStr"/>
+      <c r="E678" t="inlineStr"/>
       <c r="F678" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21586,15 +21574,19 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>029 221</t>
         </is>
       </c>
       <c r="C679" t="inlineStr"/>
-      <c r="D679" t="inlineStr"/>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="E679" t="inlineStr"/>
       <c r="F679" t="inlineStr">
         <is>
@@ -21609,11 +21601,11 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>029 221</t>
+          <t>029 222</t>
         </is>
       </c>
       <c r="C680" t="inlineStr"/>
@@ -21636,19 +21628,15 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
-          <t>029 222</t>
+          <t>714 226</t>
         </is>
       </c>
       <c r="C681" t="inlineStr"/>
-      <c r="D681" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
+      <c r="D681" t="inlineStr"/>
       <c r="E681" t="inlineStr"/>
       <c r="F681" t="inlineStr">
         <is>
@@ -21663,15 +21651,19 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>714 226</t>
+          <t>742 263</t>
         </is>
       </c>
       <c r="C682" t="inlineStr"/>
-      <c r="D682" t="inlineStr"/>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="E682" t="inlineStr"/>
       <c r="F682" t="inlineStr">
         <is>
@@ -21686,17 +21678,17 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>742 263</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C683" t="inlineStr"/>
       <c r="D683" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>výměna obrazovky Lokel na 914</t>
         </is>
       </c>
       <c r="E683" t="inlineStr"/>
@@ -21713,17 +21705,17 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C684" t="inlineStr"/>
       <c r="D684" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E684" t="inlineStr"/>
@@ -21740,17 +21732,17 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C685" t="inlineStr"/>
       <c r="D685" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="E685" t="inlineStr"/>
@@ -21767,17 +21759,17 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C686" t="inlineStr"/>
       <c r="D686" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E686" t="inlineStr"/>
@@ -21794,7 +21786,7 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
@@ -21804,10 +21796,14 @@
       <c r="C687" t="inlineStr"/>
       <c r="D687" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E687" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F687" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21821,24 +21817,20 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C688" t="inlineStr"/>
       <c r="D688" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E688" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr"/>
       <c r="F688" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21852,7 +21844,7 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
@@ -21862,7 +21854,7 @@
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E689" t="inlineStr"/>
@@ -21879,17 +21871,17 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E690" t="inlineStr"/>
@@ -21906,20 +21898,24 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E691" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F691" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21933,7 +21929,7 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
@@ -21943,12 +21939,12 @@
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E692" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F692" t="inlineStr">
@@ -21964,24 +21960,24 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C693" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D693" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E693" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr"/>
       <c r="F693" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21995,7 +21991,7 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
@@ -22004,12 +22000,12 @@
       </c>
       <c r="C694" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D694" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E694" t="inlineStr"/>
@@ -22026,7 +22022,7 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
@@ -22040,7 +22036,7 @@
       </c>
       <c r="D695" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E695" t="inlineStr"/>
@@ -22057,7 +22053,7 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
@@ -22071,10 +22067,14 @@
       </c>
       <c r="D696" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E696" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F696" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22088,7 +22088,7 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
@@ -22102,12 +22102,12 @@
       </c>
       <c r="D697" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E697" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F697" t="inlineStr">
@@ -22123,7 +22123,7 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
@@ -22137,14 +22137,10 @@
       </c>
       <c r="D698" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E698" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr"/>
       <c r="F698" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22158,24 +22154,24 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C699" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr"/>
       <c r="D699" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E699" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F699" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22189,24 +22185,20 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C700" t="inlineStr"/>
       <c r="D700" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E700" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr"/>
       <c r="F700" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22220,7 +22212,7 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
@@ -22230,7 +22222,7 @@
       <c r="C701" t="inlineStr"/>
       <c r="D701" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
         </is>
       </c>
       <c r="E701" t="inlineStr"/>
@@ -22247,17 +22239,17 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E702" t="inlineStr"/>
@@ -22274,7 +22266,7 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
@@ -22284,10 +22276,14 @@
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E703" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F703" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22301,24 +22297,20 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E704" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr"/>
       <c r="F704" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22332,7 +22324,7 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
@@ -22342,7 +22334,7 @@
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E705" t="inlineStr"/>
@@ -22359,7 +22351,7 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
@@ -22369,7 +22361,7 @@
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E706" t="inlineStr"/>
@@ -22386,17 +22378,17 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E707" t="inlineStr"/>
@@ -22413,7 +22405,7 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
@@ -22423,10 +22415,14 @@
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="E708" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F708" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22440,7 +22436,7 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
@@ -22450,14 +22446,10 @@
       <c r="C709" t="inlineStr"/>
       <c r="D709" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E709" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr"/>
       <c r="F709" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22471,7 +22463,7 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
@@ -22481,10 +22473,14 @@
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E710" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F710" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22498,7 +22494,7 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
@@ -22508,14 +22504,10 @@
       <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E711" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr"/>
       <c r="F711" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22529,7 +22521,7 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
@@ -22539,7 +22531,7 @@
       <c r="C712" t="inlineStr"/>
       <c r="D712" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E712" t="inlineStr"/>
@@ -22556,7 +22548,7 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
@@ -22566,10 +22558,14 @@
       <c r="C713" t="inlineStr"/>
       <c r="D713" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E713" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F713" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22583,7 +22579,7 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
@@ -22593,12 +22589,12 @@
       <c r="C714" t="inlineStr"/>
       <c r="D714" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E714" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F714" t="inlineStr">
@@ -22614,7 +22610,7 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
@@ -22624,12 +22620,12 @@
       <c r="C715" t="inlineStr"/>
       <c r="D715" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E715" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F715" t="inlineStr">
@@ -22645,24 +22641,20 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C716" t="inlineStr"/>
       <c r="D716" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E716" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr"/>
       <c r="F716" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22676,7 +22668,7 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
@@ -22686,10 +22678,14 @@
       <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E717" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F717" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22703,7 +22699,7 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
@@ -22713,12 +22709,12 @@
       <c r="C718" t="inlineStr"/>
       <c r="D718" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E718" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F718" t="inlineStr">
@@ -22734,7 +22730,7 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
@@ -22744,14 +22740,10 @@
       <c r="C719" t="inlineStr"/>
       <c r="D719" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E719" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr"/>
       <c r="F719" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22765,17 +22757,17 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C720" t="inlineStr"/>
       <c r="D720" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E720" t="inlineStr"/>
@@ -22792,7 +22784,7 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
@@ -22802,7 +22794,7 @@
       <c r="C721" t="inlineStr"/>
       <c r="D721" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E721" t="inlineStr"/>
@@ -22819,7 +22811,7 @@
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
@@ -22829,10 +22821,14 @@
       <c r="C722" t="inlineStr"/>
       <c r="D722" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E722" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F722" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22846,22 +22842,22 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C723" t="inlineStr"/>
       <c r="D723" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E723" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F723" t="inlineStr">
@@ -22877,7 +22873,7 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
@@ -22887,12 +22883,12 @@
       <c r="C724" t="inlineStr"/>
       <c r="D724" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E724" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F724" t="inlineStr">
@@ -22908,24 +22904,20 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C725" t="inlineStr"/>
       <c r="D725" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E725" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr"/>
       <c r="F725" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22939,20 +22931,24 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C726" t="inlineStr"/>
       <c r="D726" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E726" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F726" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22966,24 +22962,20 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C727" t="inlineStr"/>
       <c r="D727" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E727" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr"/>
       <c r="F727" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22997,7 +22989,7 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
@@ -23007,7 +22999,7 @@
       <c r="C728" t="inlineStr"/>
       <c r="D728" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E728" t="inlineStr"/>
@@ -23024,7 +23016,7 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
@@ -23034,7 +23026,7 @@
       <c r="C729" t="inlineStr"/>
       <c r="D729" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E729" t="inlineStr"/>
@@ -23051,7 +23043,7 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
@@ -23061,7 +23053,7 @@
       <c r="C730" t="inlineStr"/>
       <c r="D730" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E730" t="inlineStr"/>
@@ -23078,7 +23070,7 @@
     </row>
     <row r="731">
       <c r="A731" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
@@ -23088,10 +23080,14 @@
       <c r="C731" t="inlineStr"/>
       <c r="D731" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E731" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F731" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23105,24 +23101,20 @@
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C732" t="inlineStr"/>
       <c r="D732" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E732" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr"/>
       <c r="F732" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23136,7 +23128,7 @@
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
@@ -23146,7 +23138,7 @@
       <c r="C733" t="inlineStr"/>
       <c r="D733" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E733" t="inlineStr"/>
@@ -23163,20 +23155,24 @@
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C734" t="inlineStr"/>
       <c r="D734" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E734" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F734" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23190,24 +23186,20 @@
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C735" t="inlineStr"/>
       <c r="D735" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E735" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr"/>
       <c r="F735" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23221,7 +23213,7 @@
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
@@ -23231,7 +23223,7 @@
       <c r="C736" t="inlineStr"/>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E736" t="inlineStr"/>
@@ -23248,20 +23240,24 @@
     </row>
     <row r="737">
       <c r="A737" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C737" t="inlineStr"/>
       <c r="D737" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E737" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F737" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23275,27 +23271,31 @@
     </row>
     <row r="738">
       <c r="A738" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C738" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D738" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E738" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F738" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G738" t="inlineStr">
@@ -23306,11 +23306,11 @@
     </row>
     <row r="739">
       <c r="A739" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C739" t="inlineStr">
@@ -23320,12 +23320,12 @@
       </c>
       <c r="D739" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E739" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F739" t="inlineStr">
@@ -23341,26 +23341,26 @@
     </row>
     <row r="740">
       <c r="A740" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C740" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E740" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F740" t="inlineStr">
@@ -23376,31 +23376,27 @@
     </row>
     <row r="741">
       <c r="A741" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D741" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E741" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr"/>
       <c r="F741" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G741" t="inlineStr">
@@ -23411,27 +23407,27 @@
     </row>
     <row r="742">
       <c r="A742" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C742" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D742" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E742" t="inlineStr"/>
       <c r="F742" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G742" t="inlineStr">
@@ -23442,27 +23438,27 @@
     </row>
     <row r="743">
       <c r="A743" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C743" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D743" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E743" t="inlineStr"/>
       <c r="F743" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G743" t="inlineStr">
@@ -23473,27 +23469,27 @@
     </row>
     <row r="744">
       <c r="A744" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C744" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D744" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E744" t="inlineStr"/>
       <c r="F744" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G744" t="inlineStr">
@@ -23504,24 +23500,28 @@
     </row>
     <row r="745">
       <c r="A745" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B745" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C745" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D745" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E745" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F745" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -23535,11 +23535,11 @@
     </row>
     <row r="746">
       <c r="A746" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C746" t="inlineStr">
@@ -23549,12 +23549,12 @@
       </c>
       <c r="D746" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E746" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F746" t="inlineStr">
@@ -23570,11 +23570,11 @@
     </row>
     <row r="747">
       <c r="A747" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C747" t="inlineStr">
@@ -23584,7 +23584,7 @@
       </c>
       <c r="D747" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E747" t="inlineStr">
@@ -23605,31 +23605,31 @@
     </row>
     <row r="748">
       <c r="A748" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C748" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D748" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E748" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F748" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G748" t="inlineStr">
@@ -23640,31 +23640,27 @@
     </row>
     <row r="749">
       <c r="A749" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B749" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C749" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D749" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E749" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr"/>
       <c r="F749" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G749" t="inlineStr">
@@ -23675,57 +23671,53 @@
     </row>
     <row r="750">
       <c r="A750" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B750" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C750" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D750" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E750" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F750" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
-        </is>
-      </c>
-      <c r="G750" t="inlineStr">
-        <is>
-          <t>Bez fotky</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G750" t="inlineStr"/>
     </row>
     <row r="751">
       <c r="A751" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B751" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C751" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr"/>
       <c r="D751" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E751" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F751" t="inlineStr">
@@ -23737,92 +23729,65 @@
     </row>
     <row r="752">
       <c r="A752" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B752" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C752" t="inlineStr"/>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D752" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
-        </is>
-      </c>
-      <c r="E752" t="inlineStr">
-        <is>
-          <t>Prohozní s 844 028 - A2.6</t>
-        </is>
-      </c>
+          <t>Vývaz motoru "B"</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr"/>
       <c r="F752" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G752" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G752" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="753">
       <c r="A753" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B753" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C753" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D753" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
-        </is>
-      </c>
-      <c r="E753" t="inlineStr"/>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>Vadná černá karta v bobku</t>
+        </is>
+      </c>
       <c r="F753" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G753" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="754">
-      <c r="A754" t="n">
-        <v>759</v>
-      </c>
-      <c r="B754" t="inlineStr">
-        <is>
-          <t>814 120</t>
-        </is>
-      </c>
-      <c r="C754" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
-      <c r="D754" t="inlineStr">
-        <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
-        </is>
-      </c>
-      <c r="E754" t="inlineStr">
-        <is>
-          <t>Vadná černá karta v bobku</t>
-        </is>
-      </c>
-      <c r="F754" t="inlineStr">
-        <is>
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G754" t="inlineStr"/>
+      <c r="G753" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Přidána nová závada ID 760 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G753"/>
+  <dimension ref="A1:G754"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23789,6 +23789,37 @@
       </c>
       <c r="G753" t="inlineStr"/>
     </row>
+    <row r="754">
+      <c r="A754" t="n">
+        <v>760</v>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>Opět závada motoru A CAN předtím výměna A2.6 a A2.7 nyní nasimulováno</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>Výměna A2.5</t>
+        </is>
+      </c>
+      <c r="F754" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G754" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 761 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G754"/>
+  <dimension ref="A1:G755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23820,6 +23820,37 @@
       </c>
       <c r="G754" t="inlineStr"/>
     </row>
+    <row r="755">
+      <c r="A755" t="n">
+        <v>761</v>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>závada viz video</t>
+        </is>
+      </c>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G755" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 762 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G755"/>
+  <dimension ref="A1:G756"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23851,6 +23851,41 @@
       </c>
       <c r="G755" t="inlineStr"/>
     </row>
+    <row r="756">
+      <c r="A756" t="n">
+        <v>762</v>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr">
+        <is>
+          <t>závada viz video</t>
+        </is>
+      </c>
+      <c r="F756" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G756" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Smazána závada ID 760 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G756"/>
+  <dimension ref="A1:G755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23791,7 +23791,7 @@
     </row>
     <row r="754">
       <c r="A754" t="n">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="B754" t="inlineStr">
         <is>
@@ -23805,12 +23805,12 @@
       </c>
       <c r="D754" t="inlineStr">
         <is>
-          <t>Opět závada motoru A CAN předtím výměna A2.6 a A2.7 nyní nasimulováno</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E754" t="inlineStr">
         <is>
-          <t>Výměna A2.5</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F754" t="inlineStr">
@@ -23822,7 +23822,7 @@
     </row>
     <row r="755">
       <c r="A755" t="n">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="B755" t="inlineStr">
         <is>
@@ -23849,38 +23849,7 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G755" t="inlineStr"/>
-    </row>
-    <row r="756">
-      <c r="A756" t="n">
-        <v>762</v>
-      </c>
-      <c r="B756" t="inlineStr">
-        <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C756" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D756" t="inlineStr">
-        <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
-        </is>
-      </c>
-      <c r="E756" t="inlineStr">
-        <is>
-          <t>závada viz video</t>
-        </is>
-      </c>
-      <c r="F756" t="inlineStr">
-        <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G756" t="inlineStr">
+      <c r="G755" t="inlineStr">
         <is>
           <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 761 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G755"/>
+  <dimension ref="A1:G754"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23791,7 +23791,7 @@
     </row>
     <row r="754">
       <c r="A754" t="n">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="B754" t="inlineStr">
         <is>
@@ -23818,38 +23818,7 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G754" t="inlineStr"/>
-    </row>
-    <row r="755">
-      <c r="A755" t="n">
-        <v>762</v>
-      </c>
-      <c r="B755" t="inlineStr">
-        <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C755" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D755" t="inlineStr">
-        <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
-        </is>
-      </c>
-      <c r="E755" t="inlineStr">
-        <is>
-          <t>závada viz video</t>
-        </is>
-      </c>
-      <c r="F755" t="inlineStr">
-        <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G755" t="inlineStr">
+      <c r="G754" t="inlineStr">
         <is>
           <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
         </is>

</xml_diff>

<commit_message>
Přidána nová závada ID 763 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G754"/>
+  <dimension ref="A1:G755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23824,6 +23824,37 @@
         </is>
       </c>
     </row>
+    <row r="755">
+      <c r="A755" t="n">
+        <v>763</v>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>844 111</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>Proste test</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr"/>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_0986.mov</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Smazána závada ID 763 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G755"/>
+  <dimension ref="A1:G754"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23824,37 +23824,6 @@
         </is>
       </c>
     </row>
-    <row r="755">
-      <c r="A755" t="n">
-        <v>763</v>
-      </c>
-      <c r="B755" t="inlineStr">
-        <is>
-          <t>844 111</t>
-        </is>
-      </c>
-      <c r="C755" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D755" t="inlineStr">
-        <is>
-          <t>Proste test</t>
-        </is>
-      </c>
-      <c r="E755" t="inlineStr"/>
-      <c r="F755" t="inlineStr">
-        <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G755" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_0986.mov</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 763 (autor: Dan)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G754"/>
+  <dimension ref="A1:G755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23824,6 +23824,41 @@
         </is>
       </c>
     </row>
+    <row r="755">
+      <c r="A755" t="n">
+        <v>763</v>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>844 014</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
+        </is>
+      </c>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Smazána závada ID 764 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I756"/>
+  <dimension ref="A1:I755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25381,43 +25381,6 @@
       <c r="H755" t="inlineStr"/>
       <c r="I755" t="inlineStr"/>
     </row>
-    <row r="756">
-      <c r="A756" t="n">
-        <v>764</v>
-      </c>
-      <c r="B756" t="inlineStr">
-        <is>
-          <t>844 111</t>
-        </is>
-      </c>
-      <c r="C756" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D756" t="inlineStr">
-        <is>
-          <t>test textu</t>
-        </is>
-      </c>
-      <c r="E756" t="inlineStr"/>
-      <c r="F756" t="inlineStr">
-        <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G756" t="inlineStr"/>
-      <c r="H756" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-      <c r="I756" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hromadná úprava z tabulky (Radek) (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -3659,7 +3659,11 @@
           <t>844 003</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>25.08.2025</t>
+        </is>
+      </c>
       <c r="D93" t="inlineStr">
         <is>
           <t>chyba CAN1 SH3 po restartu DDC 732-TG na SH3 věe v pořádku</t>
@@ -3997,7 +4001,11 @@
           <t>844 003</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr"/>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>28.07.2025</t>
+        </is>
+      </c>
       <c r="D103" t="inlineStr">
         <is>
           <t>při rozjezdu  a jizde nad 30km dochází k zabrždění podvozku (hnaného) prostřední</t>
@@ -4773,7 +4781,11 @@
           <t>844 003</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr"/>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>29.04.2025</t>
+        </is>
+      </c>
       <c r="D127" t="inlineStr">
         <is>
           <t>vývaz motoru A vadný</t>

</xml_diff>

<commit_message>
Smazána závada ID 705 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I755"/>
+  <dimension ref="A1:I754"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23619,7 +23619,7 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
@@ -23629,7 +23629,7 @@
       <c r="C700" t="inlineStr"/>
       <c r="D700" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
         </is>
       </c>
       <c r="E700" t="inlineStr"/>
@@ -23648,17 +23648,17 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C701" t="inlineStr"/>
       <c r="D701" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E701" t="inlineStr"/>
@@ -23677,7 +23677,7 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
@@ -23687,10 +23687,14 @@
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E702" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F702" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23706,24 +23710,20 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E703" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr"/>
       <c r="F703" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23739,7 +23739,7 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
@@ -23749,7 +23749,7 @@
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E704" t="inlineStr"/>
@@ -23768,7 +23768,7 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
@@ -23778,7 +23778,7 @@
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E705" t="inlineStr"/>
@@ -23797,17 +23797,17 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E706" t="inlineStr"/>
@@ -23826,7 +23826,7 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
@@ -23836,10 +23836,14 @@
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="E707" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F707" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23855,7 +23859,7 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
@@ -23865,14 +23869,10 @@
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E708" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr"/>
       <c r="F708" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23888,7 +23888,7 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
@@ -23898,10 +23898,14 @@
       <c r="C709" t="inlineStr"/>
       <c r="D709" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E709" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F709" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23917,7 +23921,7 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
@@ -23927,14 +23931,10 @@
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E710" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr"/>
       <c r="F710" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23950,7 +23950,7 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
@@ -23960,7 +23960,7 @@
       <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E711" t="inlineStr"/>
@@ -23979,7 +23979,7 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
@@ -23989,10 +23989,14 @@
       <c r="C712" t="inlineStr"/>
       <c r="D712" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E712" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F712" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24008,7 +24012,7 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
@@ -24018,12 +24022,12 @@
       <c r="C713" t="inlineStr"/>
       <c r="D713" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E713" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F713" t="inlineStr">
@@ -24041,7 +24045,7 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
@@ -24051,12 +24055,12 @@
       <c r="C714" t="inlineStr"/>
       <c r="D714" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E714" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F714" t="inlineStr">
@@ -24074,24 +24078,20 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C715" t="inlineStr"/>
       <c r="D715" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E715" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr"/>
       <c r="F715" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24107,7 +24107,7 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
@@ -24117,10 +24117,14 @@
       <c r="C716" t="inlineStr"/>
       <c r="D716" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E716" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F716" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24136,7 +24140,7 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
@@ -24146,12 +24150,12 @@
       <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E717" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F717" t="inlineStr">
@@ -24169,7 +24173,7 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
@@ -24179,14 +24183,10 @@
       <c r="C718" t="inlineStr"/>
       <c r="D718" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E718" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr"/>
       <c r="F718" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24202,17 +24202,17 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C719" t="inlineStr"/>
       <c r="D719" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E719" t="inlineStr"/>
@@ -24231,7 +24231,7 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
@@ -24241,7 +24241,7 @@
       <c r="C720" t="inlineStr"/>
       <c r="D720" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E720" t="inlineStr"/>
@@ -24260,7 +24260,7 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
@@ -24270,10 +24270,14 @@
       <c r="C721" t="inlineStr"/>
       <c r="D721" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E721" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F721" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24289,22 +24293,22 @@
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C722" t="inlineStr"/>
       <c r="D722" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E722" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F722" t="inlineStr">
@@ -24322,7 +24326,7 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
@@ -24332,12 +24336,12 @@
       <c r="C723" t="inlineStr"/>
       <c r="D723" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E723" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F723" t="inlineStr">
@@ -24355,24 +24359,20 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C724" t="inlineStr"/>
       <c r="D724" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E724" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr"/>
       <c r="F724" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24388,23 +24388,27 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C725" t="inlineStr"/>
       <c r="D725" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E725" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F725" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G725" t="inlineStr"/>
@@ -24417,27 +24421,23 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C726" t="inlineStr"/>
       <c r="D726" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E726" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr"/>
       <c r="F726" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G726" t="inlineStr"/>
@@ -24450,7 +24450,7 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
@@ -24460,7 +24460,7 @@
       <c r="C727" t="inlineStr"/>
       <c r="D727" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E727" t="inlineStr"/>
@@ -24479,7 +24479,7 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
@@ -24489,7 +24489,7 @@
       <c r="C728" t="inlineStr"/>
       <c r="D728" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E728" t="inlineStr"/>
@@ -24508,7 +24508,7 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
@@ -24518,7 +24518,7 @@
       <c r="C729" t="inlineStr"/>
       <c r="D729" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E729" t="inlineStr"/>
@@ -24537,7 +24537,7 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
@@ -24547,10 +24547,14 @@
       <c r="C730" t="inlineStr"/>
       <c r="D730" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E730" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F730" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24566,24 +24570,20 @@
     </row>
     <row r="731">
       <c r="A731" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C731" t="inlineStr"/>
       <c r="D731" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E731" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr"/>
       <c r="F731" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24599,7 +24599,7 @@
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
@@ -24609,7 +24609,7 @@
       <c r="C732" t="inlineStr"/>
       <c r="D732" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E732" t="inlineStr"/>
@@ -24628,20 +24628,24 @@
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C733" t="inlineStr"/>
       <c r="D733" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E733" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F733" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24657,27 +24661,23 @@
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C734" t="inlineStr"/>
       <c r="D734" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E734" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr"/>
       <c r="F734" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G734" t="inlineStr"/>
@@ -24690,7 +24690,7 @@
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
@@ -24700,7 +24700,7 @@
       <c r="C735" t="inlineStr"/>
       <c r="D735" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E735" t="inlineStr"/>
@@ -24719,23 +24719,27 @@
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C736" t="inlineStr"/>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E736" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F736" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G736" t="inlineStr"/>
@@ -24748,27 +24752,31 @@
     </row>
     <row r="737">
       <c r="A737" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C737" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D737" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E737" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F737" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G737" t="inlineStr"/>
@@ -24781,11 +24789,11 @@
     </row>
     <row r="738">
       <c r="A738" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C738" t="inlineStr">
@@ -24795,12 +24803,12 @@
       </c>
       <c r="D738" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E738" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F738" t="inlineStr">
@@ -24818,26 +24826,26 @@
     </row>
     <row r="739">
       <c r="A739" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C739" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D739" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E739" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F739" t="inlineStr">
@@ -24855,31 +24863,27 @@
     </row>
     <row r="740">
       <c r="A740" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C740" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E740" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr"/>
       <c r="F740" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G740" t="inlineStr"/>
@@ -24892,27 +24896,27 @@
     </row>
     <row r="741">
       <c r="A741" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D741" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E741" t="inlineStr"/>
       <c r="F741" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G741" t="inlineStr"/>
@@ -24925,27 +24929,27 @@
     </row>
     <row r="742">
       <c r="A742" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C742" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D742" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E742" t="inlineStr"/>
       <c r="F742" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G742" t="inlineStr"/>
@@ -24958,27 +24962,27 @@
     </row>
     <row r="743">
       <c r="A743" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C743" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D743" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E743" t="inlineStr"/>
       <c r="F743" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G743" t="inlineStr"/>
@@ -24991,24 +24995,28 @@
     </row>
     <row r="744">
       <c r="A744" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C744" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D744" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E744" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F744" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -25024,11 +25032,11 @@
     </row>
     <row r="745">
       <c r="A745" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B745" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C745" t="inlineStr">
@@ -25038,12 +25046,12 @@
       </c>
       <c r="D745" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E745" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F745" t="inlineStr">
@@ -25061,11 +25069,11 @@
     </row>
     <row r="746">
       <c r="A746" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C746" t="inlineStr">
@@ -25075,7 +25083,7 @@
       </c>
       <c r="D746" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E746" t="inlineStr">
@@ -25098,31 +25106,31 @@
     </row>
     <row r="747">
       <c r="A747" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C747" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D747" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E747" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F747" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G747" t="inlineStr"/>
@@ -25135,31 +25143,27 @@
     </row>
     <row r="748">
       <c r="A748" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C748" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D748" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E748" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr"/>
       <c r="F748" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G748" t="inlineStr"/>
@@ -25172,27 +25176,31 @@
     </row>
     <row r="749">
       <c r="A749" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B749" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C749" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D749" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E749" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F749" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G749" t="inlineStr"/>
@@ -25205,26 +25213,22 @@
     </row>
     <row r="750">
       <c r="A750" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B750" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C750" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr"/>
       <c r="D750" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E750" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F750" t="inlineStr">
@@ -25242,30 +25246,38 @@
     </row>
     <row r="751">
       <c r="A751" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B751" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C751" t="inlineStr"/>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D751" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E751" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F751" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G751" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G751" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H751" t="inlineStr"/>
       <c r="I751" t="inlineStr">
         <is>
@@ -25275,38 +25287,34 @@
     </row>
     <row r="752">
       <c r="A752" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B752" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C752" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D752" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E752" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F752" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G752" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G752" t="inlineStr"/>
       <c r="H752" t="inlineStr"/>
       <c r="I752" t="inlineStr">
         <is>
@@ -25316,26 +25324,26 @@
     </row>
     <row r="753">
       <c r="A753" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B753" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C753" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D753" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E753" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F753" t="inlineStr">
@@ -25343,7 +25351,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G753" t="inlineStr"/>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H753" t="inlineStr"/>
       <c r="I753" t="inlineStr">
         <is>
@@ -25353,11 +25365,11 @@
     </row>
     <row r="754">
       <c r="A754" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B754" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C754" t="inlineStr">
@@ -25367,67 +25379,26 @@
       </c>
       <c r="D754" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E754" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F754" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G754" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H754" t="inlineStr"/>
       <c r="I754" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="755">
-      <c r="A755" t="n">
-        <v>763</v>
-      </c>
-      <c r="B755" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C755" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D755" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E755" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F755" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G755" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H755" t="inlineStr"/>
-      <c r="I755" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 683 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I744"/>
+  <dimension ref="A1:I743"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22676,11 +22676,11 @@
     </row>
     <row r="669">
       <c r="A669" t="n">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>029 221</t>
+          <t>029 222</t>
         </is>
       </c>
       <c r="C669" t="inlineStr"/>
@@ -22705,19 +22705,15 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>029 222</t>
+          <t>714 226</t>
         </is>
       </c>
       <c r="C670" t="inlineStr"/>
-      <c r="D670" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
+      <c r="D670" t="inlineStr"/>
       <c r="E670" t="inlineStr"/>
       <c r="F670" t="inlineStr">
         <is>
@@ -22734,15 +22730,19 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>714 226</t>
+          <t>742 263</t>
         </is>
       </c>
       <c r="C671" t="inlineStr"/>
-      <c r="D671" t="inlineStr"/>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="E671" t="inlineStr"/>
       <c r="F671" t="inlineStr">
         <is>
@@ -22759,17 +22759,17 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>742 263</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C672" t="inlineStr"/>
       <c r="D672" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>výměna obrazovky Lokel na 914</t>
         </is>
       </c>
       <c r="E672" t="inlineStr"/>
@@ -22788,17 +22788,17 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C673" t="inlineStr"/>
       <c r="D673" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E673" t="inlineStr"/>
@@ -22817,17 +22817,17 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C674" t="inlineStr"/>
       <c r="D674" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="E674" t="inlineStr"/>
@@ -22846,17 +22846,17 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C675" t="inlineStr"/>
       <c r="D675" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E675" t="inlineStr"/>
@@ -22875,7 +22875,7 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
@@ -22885,10 +22885,14 @@
       <c r="C676" t="inlineStr"/>
       <c r="D676" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E676" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F676" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22904,24 +22908,20 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C677" t="inlineStr"/>
       <c r="D677" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E677" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr"/>
       <c r="F677" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22937,7 +22937,7 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
@@ -22947,7 +22947,7 @@
       <c r="C678" t="inlineStr"/>
       <c r="D678" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E678" t="inlineStr"/>
@@ -22966,17 +22966,17 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C679" t="inlineStr"/>
       <c r="D679" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E679" t="inlineStr"/>
@@ -22995,20 +22995,24 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C680" t="inlineStr"/>
       <c r="D680" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E680" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F680" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23024,7 +23028,7 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
@@ -23034,12 +23038,12 @@
       <c r="C681" t="inlineStr"/>
       <c r="D681" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E681" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F681" t="inlineStr">
@@ -23057,24 +23061,24 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C682" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D682" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E682" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr"/>
       <c r="F682" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23090,7 +23094,7 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
@@ -23099,12 +23103,12 @@
       </c>
       <c r="C683" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D683" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E683" t="inlineStr"/>
@@ -23123,7 +23127,7 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
@@ -23137,7 +23141,7 @@
       </c>
       <c r="D684" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E684" t="inlineStr"/>
@@ -23156,7 +23160,7 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
@@ -23170,10 +23174,14 @@
       </c>
       <c r="D685" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E685" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F685" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23189,7 +23197,7 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
@@ -23203,12 +23211,12 @@
       </c>
       <c r="D686" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E686" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F686" t="inlineStr">
@@ -23226,7 +23234,7 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
@@ -23240,14 +23248,10 @@
       </c>
       <c r="D687" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E687" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr"/>
       <c r="F687" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23263,24 +23267,24 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C688" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr"/>
       <c r="D688" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E688" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F688" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23296,24 +23300,20 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E689" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr"/>
       <c r="F689" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23329,17 +23329,17 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E690" t="inlineStr"/>
@@ -23358,7 +23358,7 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
@@ -23368,10 +23368,14 @@
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E691" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F691" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23387,24 +23391,20 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E692" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr"/>
       <c r="F692" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23420,7 +23420,7 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
@@ -23430,7 +23430,7 @@
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E693" t="inlineStr"/>
@@ -23449,7 +23449,7 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
@@ -23459,7 +23459,7 @@
       <c r="C694" t="inlineStr"/>
       <c r="D694" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E694" t="inlineStr"/>
@@ -23478,17 +23478,17 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C695" t="inlineStr"/>
       <c r="D695" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E695" t="inlineStr"/>
@@ -23507,7 +23507,7 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
@@ -23517,10 +23517,14 @@
       <c r="C696" t="inlineStr"/>
       <c r="D696" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="E696" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F696" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23536,7 +23540,7 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
@@ -23546,14 +23550,10 @@
       <c r="C697" t="inlineStr"/>
       <c r="D697" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E697" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr"/>
       <c r="F697" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23569,7 +23569,7 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
@@ -23579,10 +23579,14 @@
       <c r="C698" t="inlineStr"/>
       <c r="D698" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E698" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F698" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23598,7 +23602,7 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
@@ -23608,14 +23612,10 @@
       <c r="C699" t="inlineStr"/>
       <c r="D699" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E699" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr"/>
       <c r="F699" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23631,7 +23631,7 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
@@ -23641,7 +23641,7 @@
       <c r="C700" t="inlineStr"/>
       <c r="D700" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E700" t="inlineStr"/>
@@ -23660,7 +23660,7 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
@@ -23670,10 +23670,14 @@
       <c r="C701" t="inlineStr"/>
       <c r="D701" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E701" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F701" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23689,7 +23693,7 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
@@ -23699,12 +23703,12 @@
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E702" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F702" t="inlineStr">
@@ -23722,7 +23726,7 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
@@ -23732,12 +23736,12 @@
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E703" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F703" t="inlineStr">
@@ -23755,24 +23759,20 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E704" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr"/>
       <c r="F704" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23788,7 +23788,7 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
@@ -23798,10 +23798,14 @@
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E705" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F705" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23817,7 +23821,7 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
@@ -23827,12 +23831,12 @@
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E706" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F706" t="inlineStr">
@@ -23850,7 +23854,7 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
@@ -23860,14 +23864,10 @@
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E707" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr"/>
       <c r="F707" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23883,17 +23883,17 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E708" t="inlineStr"/>
@@ -23912,7 +23912,7 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
@@ -23922,7 +23922,7 @@
       <c r="C709" t="inlineStr"/>
       <c r="D709" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E709" t="inlineStr"/>
@@ -23941,7 +23941,7 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
@@ -23951,10 +23951,14 @@
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E710" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F710" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23970,22 +23974,22 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E711" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F711" t="inlineStr">
@@ -24003,7 +24007,7 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
@@ -24013,12 +24017,12 @@
       <c r="C712" t="inlineStr"/>
       <c r="D712" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E712" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F712" t="inlineStr">
@@ -24036,24 +24040,20 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C713" t="inlineStr"/>
       <c r="D713" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E713" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr"/>
       <c r="F713" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24069,23 +24069,27 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C714" t="inlineStr"/>
       <c r="D714" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E714" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F714" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G714" t="inlineStr"/>
@@ -24098,27 +24102,23 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C715" t="inlineStr"/>
       <c r="D715" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E715" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr"/>
       <c r="F715" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G715" t="inlineStr"/>
@@ -24131,7 +24131,7 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
@@ -24141,7 +24141,7 @@
       <c r="C716" t="inlineStr"/>
       <c r="D716" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E716" t="inlineStr"/>
@@ -24160,7 +24160,7 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
@@ -24170,7 +24170,7 @@
       <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E717" t="inlineStr"/>
@@ -24189,7 +24189,7 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
@@ -24199,7 +24199,7 @@
       <c r="C718" t="inlineStr"/>
       <c r="D718" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E718" t="inlineStr"/>
@@ -24218,7 +24218,7 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
@@ -24228,10 +24228,14 @@
       <c r="C719" t="inlineStr"/>
       <c r="D719" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E719" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F719" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24247,24 +24251,20 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C720" t="inlineStr"/>
       <c r="D720" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E720" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr"/>
       <c r="F720" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24280,7 +24280,7 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
@@ -24290,7 +24290,7 @@
       <c r="C721" t="inlineStr"/>
       <c r="D721" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E721" t="inlineStr"/>
@@ -24309,20 +24309,24 @@
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C722" t="inlineStr"/>
       <c r="D722" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E722" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F722" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24338,27 +24342,23 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C723" t="inlineStr"/>
       <c r="D723" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E723" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr"/>
       <c r="F723" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G723" t="inlineStr"/>
@@ -24371,7 +24371,7 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
@@ -24381,7 +24381,7 @@
       <c r="C724" t="inlineStr"/>
       <c r="D724" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E724" t="inlineStr"/>
@@ -24400,23 +24400,27 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C725" t="inlineStr"/>
       <c r="D725" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E725" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F725" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G725" t="inlineStr"/>
@@ -24429,27 +24433,31 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C726" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D726" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E726" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F726" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G726" t="inlineStr"/>
@@ -24462,11 +24470,11 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C727" t="inlineStr">
@@ -24476,12 +24484,12 @@
       </c>
       <c r="D727" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E727" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F727" t="inlineStr">
@@ -24499,26 +24507,26 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D728" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E728" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F728" t="inlineStr">
@@ -24536,31 +24544,27 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C729" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D729" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E729" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr"/>
       <c r="F729" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G729" t="inlineStr"/>
@@ -24573,27 +24577,27 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D730" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E730" t="inlineStr"/>
       <c r="F730" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G730" t="inlineStr"/>
@@ -24606,27 +24610,27 @@
     </row>
     <row r="731">
       <c r="A731" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C731" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D731" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E731" t="inlineStr"/>
       <c r="F731" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G731" t="inlineStr"/>
@@ -24639,27 +24643,27 @@
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C732" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D732" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E732" t="inlineStr"/>
       <c r="F732" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G732" t="inlineStr"/>
@@ -24672,24 +24676,28 @@
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C733" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D733" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E733" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F733" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -24705,11 +24713,11 @@
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C734" t="inlineStr">
@@ -24719,12 +24727,12 @@
       </c>
       <c r="D734" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E734" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F734" t="inlineStr">
@@ -24742,11 +24750,11 @@
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C735" t="inlineStr">
@@ -24756,7 +24764,7 @@
       </c>
       <c r="D735" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E735" t="inlineStr">
@@ -24779,31 +24787,31 @@
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C736" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E736" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F736" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G736" t="inlineStr"/>
@@ -24816,31 +24824,27 @@
     </row>
     <row r="737">
       <c r="A737" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C737" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D737" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E737" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr"/>
       <c r="F737" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G737" t="inlineStr"/>
@@ -24853,27 +24857,31 @@
     </row>
     <row r="738">
       <c r="A738" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C738" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D738" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E738" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F738" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G738" t="inlineStr"/>
@@ -24886,26 +24894,22 @@
     </row>
     <row r="739">
       <c r="A739" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C739" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr"/>
       <c r="D739" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E739" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F739" t="inlineStr">
@@ -24923,30 +24927,38 @@
     </row>
     <row r="740">
       <c r="A740" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B740" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C740" t="inlineStr"/>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E740" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F740" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G740" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G740" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H740" t="inlineStr"/>
       <c r="I740" t="inlineStr">
         <is>
@@ -24956,38 +24968,34 @@
     </row>
     <row r="741">
       <c r="A741" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D741" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E741" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F741" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G741" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G741" t="inlineStr"/>
       <c r="H741" t="inlineStr"/>
       <c r="I741" t="inlineStr">
         <is>
@@ -24997,26 +25005,26 @@
     </row>
     <row r="742">
       <c r="A742" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C742" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D742" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E742" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F742" t="inlineStr">
@@ -25024,7 +25032,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G742" t="inlineStr"/>
+      <c r="G742" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H742" t="inlineStr"/>
       <c r="I742" t="inlineStr">
         <is>
@@ -25034,11 +25046,11 @@
     </row>
     <row r="743">
       <c r="A743" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C743" t="inlineStr">
@@ -25048,67 +25060,26 @@
       </c>
       <c r="D743" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E743" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F743" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G743" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H743" t="inlineStr"/>
       <c r="I743" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="744">
-      <c r="A744" t="n">
-        <v>763</v>
-      </c>
-      <c r="B744" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C744" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D744" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E744" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F744" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G744" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H744" t="inlineStr"/>
-      <c r="I744" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 684 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I743"/>
+  <dimension ref="A1:I742"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22676,19 +22676,15 @@
     </row>
     <row r="669">
       <c r="A669" t="n">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>029 222</t>
+          <t>714 226</t>
         </is>
       </c>
       <c r="C669" t="inlineStr"/>
-      <c r="D669" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
+      <c r="D669" t="inlineStr"/>
       <c r="E669" t="inlineStr"/>
       <c r="F669" t="inlineStr">
         <is>
@@ -22705,15 +22701,19 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>714 226</t>
+          <t>742 263</t>
         </is>
       </c>
       <c r="C670" t="inlineStr"/>
-      <c r="D670" t="inlineStr"/>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="E670" t="inlineStr"/>
       <c r="F670" t="inlineStr">
         <is>
@@ -22730,17 +22730,17 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>742 263</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C671" t="inlineStr"/>
       <c r="D671" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>výměna obrazovky Lokel na 914</t>
         </is>
       </c>
       <c r="E671" t="inlineStr"/>
@@ -22759,17 +22759,17 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C672" t="inlineStr"/>
       <c r="D672" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E672" t="inlineStr"/>
@@ -22788,17 +22788,17 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C673" t="inlineStr"/>
       <c r="D673" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="E673" t="inlineStr"/>
@@ -22817,17 +22817,17 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C674" t="inlineStr"/>
       <c r="D674" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E674" t="inlineStr"/>
@@ -22846,7 +22846,7 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
@@ -22856,10 +22856,14 @@
       <c r="C675" t="inlineStr"/>
       <c r="D675" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E675" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F675" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22875,24 +22879,20 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C676" t="inlineStr"/>
       <c r="D676" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E676" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr"/>
       <c r="F676" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22908,7 +22908,7 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
@@ -22918,7 +22918,7 @@
       <c r="C677" t="inlineStr"/>
       <c r="D677" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E677" t="inlineStr"/>
@@ -22937,17 +22937,17 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C678" t="inlineStr"/>
       <c r="D678" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E678" t="inlineStr"/>
@@ -22966,20 +22966,24 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C679" t="inlineStr"/>
       <c r="D679" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E679" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F679" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22995,7 +22999,7 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
@@ -23005,12 +23009,12 @@
       <c r="C680" t="inlineStr"/>
       <c r="D680" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E680" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F680" t="inlineStr">
@@ -23028,24 +23032,24 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C681" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D681" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E681" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr"/>
       <c r="F681" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23061,7 +23065,7 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
@@ -23070,12 +23074,12 @@
       </c>
       <c r="C682" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D682" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E682" t="inlineStr"/>
@@ -23094,7 +23098,7 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
@@ -23108,7 +23112,7 @@
       </c>
       <c r="D683" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E683" t="inlineStr"/>
@@ -23127,7 +23131,7 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
@@ -23141,10 +23145,14 @@
       </c>
       <c r="D684" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E684" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F684" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23160,7 +23168,7 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
@@ -23174,12 +23182,12 @@
       </c>
       <c r="D685" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E685" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F685" t="inlineStr">
@@ -23197,7 +23205,7 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
@@ -23211,14 +23219,10 @@
       </c>
       <c r="D686" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E686" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr"/>
       <c r="F686" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23234,24 +23238,24 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C687" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr"/>
       <c r="D687" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E687" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F687" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23267,24 +23271,20 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C688" t="inlineStr"/>
       <c r="D688" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E688" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr"/>
       <c r="F688" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23300,17 +23300,17 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E689" t="inlineStr"/>
@@ -23329,7 +23329,7 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
@@ -23339,10 +23339,14 @@
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E690" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F690" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23358,24 +23362,20 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E691" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr"/>
       <c r="F691" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23391,7 +23391,7 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
@@ -23401,7 +23401,7 @@
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E692" t="inlineStr"/>
@@ -23420,7 +23420,7 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
@@ -23430,7 +23430,7 @@
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E693" t="inlineStr"/>
@@ -23449,17 +23449,17 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C694" t="inlineStr"/>
       <c r="D694" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E694" t="inlineStr"/>
@@ -23478,7 +23478,7 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
@@ -23488,10 +23488,14 @@
       <c r="C695" t="inlineStr"/>
       <c r="D695" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="E695" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F695" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23507,7 +23511,7 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
@@ -23517,14 +23521,10 @@
       <c r="C696" t="inlineStr"/>
       <c r="D696" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E696" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr"/>
       <c r="F696" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23540,7 +23540,7 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
@@ -23550,10 +23550,14 @@
       <c r="C697" t="inlineStr"/>
       <c r="D697" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E697" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F697" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23569,7 +23573,7 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
@@ -23579,14 +23583,10 @@
       <c r="C698" t="inlineStr"/>
       <c r="D698" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E698" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr"/>
       <c r="F698" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23602,7 +23602,7 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
@@ -23612,7 +23612,7 @@
       <c r="C699" t="inlineStr"/>
       <c r="D699" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E699" t="inlineStr"/>
@@ -23631,7 +23631,7 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
@@ -23641,10 +23641,14 @@
       <c r="C700" t="inlineStr"/>
       <c r="D700" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E700" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F700" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23660,7 +23664,7 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
@@ -23670,12 +23674,12 @@
       <c r="C701" t="inlineStr"/>
       <c r="D701" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E701" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F701" t="inlineStr">
@@ -23693,7 +23697,7 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
@@ -23703,12 +23707,12 @@
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E702" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F702" t="inlineStr">
@@ -23726,24 +23730,20 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E703" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr"/>
       <c r="F703" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23759,7 +23759,7 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
@@ -23769,10 +23769,14 @@
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E704" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F704" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23788,7 +23792,7 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
@@ -23798,12 +23802,12 @@
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E705" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F705" t="inlineStr">
@@ -23821,7 +23825,7 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
@@ -23831,14 +23835,10 @@
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E706" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr"/>
       <c r="F706" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23854,17 +23854,17 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E707" t="inlineStr"/>
@@ -23883,7 +23883,7 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
@@ -23893,7 +23893,7 @@
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E708" t="inlineStr"/>
@@ -23912,7 +23912,7 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
@@ -23922,10 +23922,14 @@
       <c r="C709" t="inlineStr"/>
       <c r="D709" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E709" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F709" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23941,22 +23945,22 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E710" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F710" t="inlineStr">
@@ -23974,7 +23978,7 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
@@ -23984,12 +23988,12 @@
       <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E711" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F711" t="inlineStr">
@@ -24007,24 +24011,20 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C712" t="inlineStr"/>
       <c r="D712" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E712" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr"/>
       <c r="F712" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24040,23 +24040,27 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C713" t="inlineStr"/>
       <c r="D713" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E713" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F713" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G713" t="inlineStr"/>
@@ -24069,27 +24073,23 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C714" t="inlineStr"/>
       <c r="D714" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E714" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr"/>
       <c r="F714" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G714" t="inlineStr"/>
@@ -24102,7 +24102,7 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
@@ -24112,7 +24112,7 @@
       <c r="C715" t="inlineStr"/>
       <c r="D715" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E715" t="inlineStr"/>
@@ -24131,7 +24131,7 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
@@ -24141,7 +24141,7 @@
       <c r="C716" t="inlineStr"/>
       <c r="D716" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E716" t="inlineStr"/>
@@ -24160,7 +24160,7 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
@@ -24170,7 +24170,7 @@
       <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E717" t="inlineStr"/>
@@ -24189,7 +24189,7 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
@@ -24199,10 +24199,14 @@
       <c r="C718" t="inlineStr"/>
       <c r="D718" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E718" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F718" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24218,24 +24222,20 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C719" t="inlineStr"/>
       <c r="D719" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E719" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr"/>
       <c r="F719" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24251,7 +24251,7 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
@@ -24261,7 +24261,7 @@
       <c r="C720" t="inlineStr"/>
       <c r="D720" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E720" t="inlineStr"/>
@@ -24280,20 +24280,24 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C721" t="inlineStr"/>
       <c r="D721" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E721" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F721" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24309,27 +24313,23 @@
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C722" t="inlineStr"/>
       <c r="D722" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E722" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr"/>
       <c r="F722" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G722" t="inlineStr"/>
@@ -24342,7 +24342,7 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
@@ -24352,7 +24352,7 @@
       <c r="C723" t="inlineStr"/>
       <c r="D723" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E723" t="inlineStr"/>
@@ -24371,23 +24371,27 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C724" t="inlineStr"/>
       <c r="D724" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E724" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F724" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G724" t="inlineStr"/>
@@ -24400,27 +24404,31 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C725" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D725" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E725" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F725" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G725" t="inlineStr"/>
@@ -24433,11 +24441,11 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
@@ -24447,12 +24455,12 @@
       </c>
       <c r="D726" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E726" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F726" t="inlineStr">
@@ -24470,26 +24478,26 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C727" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D727" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E727" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F727" t="inlineStr">
@@ -24507,31 +24515,27 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D728" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E728" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr"/>
       <c r="F728" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G728" t="inlineStr"/>
@@ -24544,27 +24548,27 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C729" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D729" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E729" t="inlineStr"/>
       <c r="F729" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G729" t="inlineStr"/>
@@ -24577,27 +24581,27 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D730" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E730" t="inlineStr"/>
       <c r="F730" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G730" t="inlineStr"/>
@@ -24610,27 +24614,27 @@
     </row>
     <row r="731">
       <c r="A731" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C731" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D731" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E731" t="inlineStr"/>
       <c r="F731" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G731" t="inlineStr"/>
@@ -24643,24 +24647,28 @@
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C732" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D732" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E732" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F732" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -24676,11 +24684,11 @@
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C733" t="inlineStr">
@@ -24690,12 +24698,12 @@
       </c>
       <c r="D733" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E733" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F733" t="inlineStr">
@@ -24713,11 +24721,11 @@
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C734" t="inlineStr">
@@ -24727,7 +24735,7 @@
       </c>
       <c r="D734" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E734" t="inlineStr">
@@ -24750,31 +24758,31 @@
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C735" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D735" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E735" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F735" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G735" t="inlineStr"/>
@@ -24787,31 +24795,27 @@
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C736" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E736" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr"/>
       <c r="F736" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G736" t="inlineStr"/>
@@ -24824,27 +24828,31 @@
     </row>
     <row r="737">
       <c r="A737" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C737" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D737" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E737" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F737" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G737" t="inlineStr"/>
@@ -24857,26 +24865,22 @@
     </row>
     <row r="738">
       <c r="A738" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C738" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr"/>
       <c r="D738" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E738" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F738" t="inlineStr">
@@ -24894,30 +24898,38 @@
     </row>
     <row r="739">
       <c r="A739" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B739" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C739" t="inlineStr"/>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D739" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E739" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F739" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G739" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G739" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H739" t="inlineStr"/>
       <c r="I739" t="inlineStr">
         <is>
@@ -24927,38 +24939,34 @@
     </row>
     <row r="740">
       <c r="A740" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C740" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E740" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F740" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G740" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G740" t="inlineStr"/>
       <c r="H740" t="inlineStr"/>
       <c r="I740" t="inlineStr">
         <is>
@@ -24968,26 +24976,26 @@
     </row>
     <row r="741">
       <c r="A741" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D741" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E741" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F741" t="inlineStr">
@@ -24995,7 +25003,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G741" t="inlineStr"/>
+      <c r="G741" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H741" t="inlineStr"/>
       <c r="I741" t="inlineStr">
         <is>
@@ -25005,11 +25017,11 @@
     </row>
     <row r="742">
       <c r="A742" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C742" t="inlineStr">
@@ -25019,67 +25031,26 @@
       </c>
       <c r="D742" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E742" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F742" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G742" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H742" t="inlineStr"/>
       <c r="I742" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="743">
-      <c r="A743" t="n">
-        <v>763</v>
-      </c>
-      <c r="B743" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C743" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D743" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E743" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F743" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G743" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H743" t="inlineStr"/>
-      <c r="I743" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 687 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I742"/>
+  <dimension ref="A1:I741"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22701,17 +22701,17 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>742 263</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C670" t="inlineStr"/>
       <c r="D670" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>výměna obrazovky Lokel na 914</t>
         </is>
       </c>
       <c r="E670" t="inlineStr"/>
@@ -22730,17 +22730,17 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C671" t="inlineStr"/>
       <c r="D671" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E671" t="inlineStr"/>
@@ -22759,17 +22759,17 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C672" t="inlineStr"/>
       <c r="D672" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="E672" t="inlineStr"/>
@@ -22788,17 +22788,17 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C673" t="inlineStr"/>
       <c r="D673" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E673" t="inlineStr"/>
@@ -22817,7 +22817,7 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
@@ -22827,10 +22827,14 @@
       <c r="C674" t="inlineStr"/>
       <c r="D674" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E674" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F674" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22846,24 +22850,20 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C675" t="inlineStr"/>
       <c r="D675" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E675" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr"/>
       <c r="F675" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22879,7 +22879,7 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
@@ -22889,7 +22889,7 @@
       <c r="C676" t="inlineStr"/>
       <c r="D676" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E676" t="inlineStr"/>
@@ -22908,17 +22908,17 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C677" t="inlineStr"/>
       <c r="D677" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E677" t="inlineStr"/>
@@ -22937,20 +22937,24 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C678" t="inlineStr"/>
       <c r="D678" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E678" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F678" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22966,7 +22970,7 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
@@ -22976,12 +22980,12 @@
       <c r="C679" t="inlineStr"/>
       <c r="D679" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E679" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F679" t="inlineStr">
@@ -22999,24 +23003,24 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C680" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D680" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E680" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr"/>
       <c r="F680" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23032,7 +23036,7 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
@@ -23041,12 +23045,12 @@
       </c>
       <c r="C681" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D681" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E681" t="inlineStr"/>
@@ -23065,7 +23069,7 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
@@ -23079,7 +23083,7 @@
       </c>
       <c r="D682" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E682" t="inlineStr"/>
@@ -23098,7 +23102,7 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
@@ -23112,10 +23116,14 @@
       </c>
       <c r="D683" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E683" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F683" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23131,7 +23139,7 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
@@ -23145,12 +23153,12 @@
       </c>
       <c r="D684" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E684" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F684" t="inlineStr">
@@ -23168,7 +23176,7 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
@@ -23182,14 +23190,10 @@
       </c>
       <c r="D685" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E685" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr"/>
       <c r="F685" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23205,24 +23209,24 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C686" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr"/>
       <c r="D686" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E686" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F686" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23238,24 +23242,20 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C687" t="inlineStr"/>
       <c r="D687" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E687" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr"/>
       <c r="F687" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23271,17 +23271,17 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C688" t="inlineStr"/>
       <c r="D688" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E688" t="inlineStr"/>
@@ -23300,7 +23300,7 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
@@ -23310,10 +23310,14 @@
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E689" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F689" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23329,24 +23333,20 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E690" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr"/>
       <c r="F690" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23362,7 +23362,7 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
@@ -23372,7 +23372,7 @@
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E691" t="inlineStr"/>
@@ -23391,7 +23391,7 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
@@ -23401,7 +23401,7 @@
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E692" t="inlineStr"/>
@@ -23420,17 +23420,17 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E693" t="inlineStr"/>
@@ -23449,7 +23449,7 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
@@ -23459,10 +23459,14 @@
       <c r="C694" t="inlineStr"/>
       <c r="D694" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="E694" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F694" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23478,7 +23482,7 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
@@ -23488,14 +23492,10 @@
       <c r="C695" t="inlineStr"/>
       <c r="D695" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E695" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr"/>
       <c r="F695" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23511,7 +23511,7 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
@@ -23521,10 +23521,14 @@
       <c r="C696" t="inlineStr"/>
       <c r="D696" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E696" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F696" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23540,7 +23544,7 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
@@ -23550,14 +23554,10 @@
       <c r="C697" t="inlineStr"/>
       <c r="D697" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E697" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr"/>
       <c r="F697" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23573,7 +23573,7 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
@@ -23583,7 +23583,7 @@
       <c r="C698" t="inlineStr"/>
       <c r="D698" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E698" t="inlineStr"/>
@@ -23602,7 +23602,7 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
@@ -23612,10 +23612,14 @@
       <c r="C699" t="inlineStr"/>
       <c r="D699" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E699" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F699" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23631,7 +23635,7 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
@@ -23641,12 +23645,12 @@
       <c r="C700" t="inlineStr"/>
       <c r="D700" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E700" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F700" t="inlineStr">
@@ -23664,7 +23668,7 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
@@ -23674,12 +23678,12 @@
       <c r="C701" t="inlineStr"/>
       <c r="D701" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E701" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F701" t="inlineStr">
@@ -23697,24 +23701,20 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E702" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr"/>
       <c r="F702" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23730,7 +23730,7 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
@@ -23740,10 +23740,14 @@
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E703" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F703" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23759,7 +23763,7 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
@@ -23769,12 +23773,12 @@
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E704" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F704" t="inlineStr">
@@ -23792,7 +23796,7 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
@@ -23802,14 +23806,10 @@
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E705" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr"/>
       <c r="F705" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23825,17 +23825,17 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E706" t="inlineStr"/>
@@ -23854,7 +23854,7 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
@@ -23864,7 +23864,7 @@
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E707" t="inlineStr"/>
@@ -23883,7 +23883,7 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
@@ -23893,10 +23893,14 @@
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E708" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F708" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23912,22 +23916,22 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C709" t="inlineStr"/>
       <c r="D709" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E709" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F709" t="inlineStr">
@@ -23945,7 +23949,7 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
@@ -23955,12 +23959,12 @@
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E710" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F710" t="inlineStr">
@@ -23978,24 +23982,20 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E711" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr"/>
       <c r="F711" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24011,23 +24011,27 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C712" t="inlineStr"/>
       <c r="D712" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E712" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F712" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G712" t="inlineStr"/>
@@ -24040,27 +24044,23 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C713" t="inlineStr"/>
       <c r="D713" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E713" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr"/>
       <c r="F713" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G713" t="inlineStr"/>
@@ -24073,7 +24073,7 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
@@ -24083,7 +24083,7 @@
       <c r="C714" t="inlineStr"/>
       <c r="D714" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E714" t="inlineStr"/>
@@ -24102,7 +24102,7 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
@@ -24112,7 +24112,7 @@
       <c r="C715" t="inlineStr"/>
       <c r="D715" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E715" t="inlineStr"/>
@@ -24131,7 +24131,7 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
@@ -24141,7 +24141,7 @@
       <c r="C716" t="inlineStr"/>
       <c r="D716" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E716" t="inlineStr"/>
@@ -24160,7 +24160,7 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
@@ -24170,10 +24170,14 @@
       <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E717" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F717" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24189,24 +24193,20 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C718" t="inlineStr"/>
       <c r="D718" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E718" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr"/>
       <c r="F718" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24222,7 +24222,7 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
@@ -24232,7 +24232,7 @@
       <c r="C719" t="inlineStr"/>
       <c r="D719" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E719" t="inlineStr"/>
@@ -24251,20 +24251,24 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C720" t="inlineStr"/>
       <c r="D720" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E720" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F720" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24280,27 +24284,23 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C721" t="inlineStr"/>
       <c r="D721" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E721" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr"/>
       <c r="F721" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G721" t="inlineStr"/>
@@ -24313,7 +24313,7 @@
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
@@ -24323,7 +24323,7 @@
       <c r="C722" t="inlineStr"/>
       <c r="D722" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E722" t="inlineStr"/>
@@ -24342,23 +24342,27 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C723" t="inlineStr"/>
       <c r="D723" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E723" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F723" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G723" t="inlineStr"/>
@@ -24371,27 +24375,31 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C724" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D724" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E724" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F724" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G724" t="inlineStr"/>
@@ -24404,11 +24412,11 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C725" t="inlineStr">
@@ -24418,12 +24426,12 @@
       </c>
       <c r="D725" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E725" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F725" t="inlineStr">
@@ -24441,26 +24449,26 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D726" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E726" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F726" t="inlineStr">
@@ -24478,31 +24486,27 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C727" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D727" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E727" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr"/>
       <c r="F727" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G727" t="inlineStr"/>
@@ -24515,27 +24519,27 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D728" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E728" t="inlineStr"/>
       <c r="F728" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G728" t="inlineStr"/>
@@ -24548,27 +24552,27 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C729" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D729" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E729" t="inlineStr"/>
       <c r="F729" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G729" t="inlineStr"/>
@@ -24581,27 +24585,27 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D730" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E730" t="inlineStr"/>
       <c r="F730" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G730" t="inlineStr"/>
@@ -24614,24 +24618,28 @@
     </row>
     <row r="731">
       <c r="A731" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C731" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D731" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E731" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F731" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -24647,11 +24655,11 @@
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C732" t="inlineStr">
@@ -24661,12 +24669,12 @@
       </c>
       <c r="D732" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E732" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F732" t="inlineStr">
@@ -24684,11 +24692,11 @@
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C733" t="inlineStr">
@@ -24698,7 +24706,7 @@
       </c>
       <c r="D733" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E733" t="inlineStr">
@@ -24721,31 +24729,31 @@
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C734" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D734" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E734" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F734" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G734" t="inlineStr"/>
@@ -24758,31 +24766,27 @@
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C735" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D735" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E735" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr"/>
       <c r="F735" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G735" t="inlineStr"/>
@@ -24795,27 +24799,31 @@
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C736" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E736" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F736" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G736" t="inlineStr"/>
@@ -24828,26 +24836,22 @@
     </row>
     <row r="737">
       <c r="A737" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C737" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr"/>
       <c r="D737" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E737" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F737" t="inlineStr">
@@ -24865,30 +24869,38 @@
     </row>
     <row r="738">
       <c r="A738" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C738" t="inlineStr"/>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D738" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E738" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F738" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G738" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G738" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H738" t="inlineStr"/>
       <c r="I738" t="inlineStr">
         <is>
@@ -24898,38 +24910,34 @@
     </row>
     <row r="739">
       <c r="A739" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C739" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D739" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E739" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F739" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G739" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G739" t="inlineStr"/>
       <c r="H739" t="inlineStr"/>
       <c r="I739" t="inlineStr">
         <is>
@@ -24939,26 +24947,26 @@
     </row>
     <row r="740">
       <c r="A740" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C740" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E740" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F740" t="inlineStr">
@@ -24966,7 +24974,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G740" t="inlineStr"/>
+      <c r="G740" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H740" t="inlineStr"/>
       <c r="I740" t="inlineStr">
         <is>
@@ -24976,11 +24988,11 @@
     </row>
     <row r="741">
       <c r="A741" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
@@ -24990,67 +25002,26 @@
       </c>
       <c r="D741" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E741" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F741" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G741" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H741" t="inlineStr"/>
       <c r="I741" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="742">
-      <c r="A742" t="n">
-        <v>763</v>
-      </c>
-      <c r="B742" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C742" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D742" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E742" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F742" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G742" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H742" t="inlineStr"/>
-      <c r="I742" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 686 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I741"/>
+  <dimension ref="A1:I740"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22676,15 +22676,19 @@
     </row>
     <row r="669">
       <c r="A669" t="n">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>714 226</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C669" t="inlineStr"/>
-      <c r="D669" t="inlineStr"/>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>výměna obrazovky Lokel na 914</t>
+        </is>
+      </c>
       <c r="E669" t="inlineStr"/>
       <c r="F669" t="inlineStr">
         <is>
@@ -22701,17 +22705,17 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C670" t="inlineStr"/>
       <c r="D670" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E670" t="inlineStr"/>
@@ -22730,17 +22734,17 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C671" t="inlineStr"/>
       <c r="D671" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="E671" t="inlineStr"/>
@@ -22759,17 +22763,17 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C672" t="inlineStr"/>
       <c r="D672" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E672" t="inlineStr"/>
@@ -22788,7 +22792,7 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
@@ -22798,10 +22802,14 @@
       <c r="C673" t="inlineStr"/>
       <c r="D673" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E673" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F673" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22817,24 +22825,20 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C674" t="inlineStr"/>
       <c r="D674" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E674" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr"/>
       <c r="F674" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22850,7 +22854,7 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
@@ -22860,7 +22864,7 @@
       <c r="C675" t="inlineStr"/>
       <c r="D675" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E675" t="inlineStr"/>
@@ -22879,17 +22883,17 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C676" t="inlineStr"/>
       <c r="D676" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E676" t="inlineStr"/>
@@ -22908,20 +22912,24 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C677" t="inlineStr"/>
       <c r="D677" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E677" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F677" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22937,7 +22945,7 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
@@ -22947,12 +22955,12 @@
       <c r="C678" t="inlineStr"/>
       <c r="D678" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E678" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F678" t="inlineStr">
@@ -22970,24 +22978,24 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C679" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D679" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E679" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr"/>
       <c r="F679" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23003,7 +23011,7 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
@@ -23012,12 +23020,12 @@
       </c>
       <c r="C680" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D680" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E680" t="inlineStr"/>
@@ -23036,7 +23044,7 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
@@ -23050,7 +23058,7 @@
       </c>
       <c r="D681" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E681" t="inlineStr"/>
@@ -23069,7 +23077,7 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
@@ -23083,10 +23091,14 @@
       </c>
       <c r="D682" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E682" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F682" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23102,7 +23114,7 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
@@ -23116,12 +23128,12 @@
       </c>
       <c r="D683" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E683" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F683" t="inlineStr">
@@ -23139,7 +23151,7 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
@@ -23153,14 +23165,10 @@
       </c>
       <c r="D684" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E684" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr"/>
       <c r="F684" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23176,24 +23184,24 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C685" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr"/>
       <c r="D685" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E685" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F685" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23209,24 +23217,20 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C686" t="inlineStr"/>
       <c r="D686" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E686" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr"/>
       <c r="F686" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23242,17 +23246,17 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C687" t="inlineStr"/>
       <c r="D687" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E687" t="inlineStr"/>
@@ -23271,7 +23275,7 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
@@ -23281,10 +23285,14 @@
       <c r="C688" t="inlineStr"/>
       <c r="D688" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E688" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F688" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23300,24 +23308,20 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E689" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr"/>
       <c r="F689" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23333,7 +23337,7 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
@@ -23343,7 +23347,7 @@
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E690" t="inlineStr"/>
@@ -23362,7 +23366,7 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
@@ -23372,7 +23376,7 @@
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E691" t="inlineStr"/>
@@ -23391,17 +23395,17 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E692" t="inlineStr"/>
@@ -23420,7 +23424,7 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
@@ -23430,10 +23434,14 @@
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="E693" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F693" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23449,7 +23457,7 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
@@ -23459,14 +23467,10 @@
       <c r="C694" t="inlineStr"/>
       <c r="D694" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E694" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr"/>
       <c r="F694" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23482,7 +23486,7 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
@@ -23492,10 +23496,14 @@
       <c r="C695" t="inlineStr"/>
       <c r="D695" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E695" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F695" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23511,7 +23519,7 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
@@ -23521,14 +23529,10 @@
       <c r="C696" t="inlineStr"/>
       <c r="D696" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E696" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr"/>
       <c r="F696" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23544,7 +23548,7 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
@@ -23554,7 +23558,7 @@
       <c r="C697" t="inlineStr"/>
       <c r="D697" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E697" t="inlineStr"/>
@@ -23573,7 +23577,7 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
@@ -23583,10 +23587,14 @@
       <c r="C698" t="inlineStr"/>
       <c r="D698" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E698" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F698" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23602,7 +23610,7 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
@@ -23612,12 +23620,12 @@
       <c r="C699" t="inlineStr"/>
       <c r="D699" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E699" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F699" t="inlineStr">
@@ -23635,7 +23643,7 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
@@ -23645,12 +23653,12 @@
       <c r="C700" t="inlineStr"/>
       <c r="D700" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E700" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F700" t="inlineStr">
@@ -23668,24 +23676,20 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C701" t="inlineStr"/>
       <c r="D701" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E701" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr"/>
       <c r="F701" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23701,7 +23705,7 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
@@ -23711,10 +23715,14 @@
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E702" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F702" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23730,7 +23738,7 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
@@ -23740,12 +23748,12 @@
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E703" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F703" t="inlineStr">
@@ -23763,7 +23771,7 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
@@ -23773,14 +23781,10 @@
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E704" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr"/>
       <c r="F704" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23796,17 +23800,17 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E705" t="inlineStr"/>
@@ -23825,7 +23829,7 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
@@ -23835,7 +23839,7 @@
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E706" t="inlineStr"/>
@@ -23854,7 +23858,7 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
@@ -23864,10 +23868,14 @@
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E707" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F707" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23883,22 +23891,22 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E708" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F708" t="inlineStr">
@@ -23916,7 +23924,7 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
@@ -23926,12 +23934,12 @@
       <c r="C709" t="inlineStr"/>
       <c r="D709" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E709" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F709" t="inlineStr">
@@ -23949,24 +23957,20 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E710" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr"/>
       <c r="F710" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23982,23 +23986,27 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E711" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F711" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G711" t="inlineStr"/>
@@ -24011,27 +24019,23 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C712" t="inlineStr"/>
       <c r="D712" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E712" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr"/>
       <c r="F712" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G712" t="inlineStr"/>
@@ -24044,7 +24048,7 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
@@ -24054,7 +24058,7 @@
       <c r="C713" t="inlineStr"/>
       <c r="D713" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E713" t="inlineStr"/>
@@ -24073,7 +24077,7 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
@@ -24083,7 +24087,7 @@
       <c r="C714" t="inlineStr"/>
       <c r="D714" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E714" t="inlineStr"/>
@@ -24102,7 +24106,7 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
@@ -24112,7 +24116,7 @@
       <c r="C715" t="inlineStr"/>
       <c r="D715" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E715" t="inlineStr"/>
@@ -24131,7 +24135,7 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
@@ -24141,10 +24145,14 @@
       <c r="C716" t="inlineStr"/>
       <c r="D716" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E716" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F716" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24160,24 +24168,20 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E717" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr"/>
       <c r="F717" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24193,7 +24197,7 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
@@ -24203,7 +24207,7 @@
       <c r="C718" t="inlineStr"/>
       <c r="D718" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E718" t="inlineStr"/>
@@ -24222,20 +24226,24 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C719" t="inlineStr"/>
       <c r="D719" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E719" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F719" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24251,27 +24259,23 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C720" t="inlineStr"/>
       <c r="D720" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E720" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr"/>
       <c r="F720" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G720" t="inlineStr"/>
@@ -24284,7 +24288,7 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
@@ -24294,7 +24298,7 @@
       <c r="C721" t="inlineStr"/>
       <c r="D721" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E721" t="inlineStr"/>
@@ -24313,23 +24317,27 @@
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C722" t="inlineStr"/>
       <c r="D722" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E722" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F722" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G722" t="inlineStr"/>
@@ -24342,27 +24350,31 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C723" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D723" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E723" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F723" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G723" t="inlineStr"/>
@@ -24375,11 +24387,11 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C724" t="inlineStr">
@@ -24389,12 +24401,12 @@
       </c>
       <c r="D724" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E724" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F724" t="inlineStr">
@@ -24412,26 +24424,26 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C725" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D725" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E725" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F725" t="inlineStr">
@@ -24449,31 +24461,27 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D726" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E726" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr"/>
       <c r="F726" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G726" t="inlineStr"/>
@@ -24486,27 +24494,27 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C727" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D727" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E727" t="inlineStr"/>
       <c r="F727" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G727" t="inlineStr"/>
@@ -24519,27 +24527,27 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D728" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E728" t="inlineStr"/>
       <c r="F728" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G728" t="inlineStr"/>
@@ -24552,27 +24560,27 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C729" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D729" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E729" t="inlineStr"/>
       <c r="F729" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G729" t="inlineStr"/>
@@ -24585,24 +24593,28 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D730" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E730" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F730" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -24618,11 +24630,11 @@
     </row>
     <row r="731">
       <c r="A731" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C731" t="inlineStr">
@@ -24632,12 +24644,12 @@
       </c>
       <c r="D731" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E731" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F731" t="inlineStr">
@@ -24655,11 +24667,11 @@
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C732" t="inlineStr">
@@ -24669,7 +24681,7 @@
       </c>
       <c r="D732" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E732" t="inlineStr">
@@ -24692,31 +24704,31 @@
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C733" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D733" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E733" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F733" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G733" t="inlineStr"/>
@@ -24729,31 +24741,27 @@
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C734" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D734" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E734" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr"/>
       <c r="F734" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G734" t="inlineStr"/>
@@ -24766,27 +24774,31 @@
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C735" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D735" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E735" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F735" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G735" t="inlineStr"/>
@@ -24799,26 +24811,22 @@
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C736" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr"/>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E736" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F736" t="inlineStr">
@@ -24836,30 +24844,38 @@
     </row>
     <row r="737">
       <c r="A737" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C737" t="inlineStr"/>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D737" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E737" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F737" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G737" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G737" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H737" t="inlineStr"/>
       <c r="I737" t="inlineStr">
         <is>
@@ -24869,38 +24885,34 @@
     </row>
     <row r="738">
       <c r="A738" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C738" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D738" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E738" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F738" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G738" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G738" t="inlineStr"/>
       <c r="H738" t="inlineStr"/>
       <c r="I738" t="inlineStr">
         <is>
@@ -24910,26 +24922,26 @@
     </row>
     <row r="739">
       <c r="A739" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C739" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D739" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E739" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F739" t="inlineStr">
@@ -24937,7 +24949,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G739" t="inlineStr"/>
+      <c r="G739" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H739" t="inlineStr"/>
       <c r="I739" t="inlineStr">
         <is>
@@ -24947,11 +24963,11 @@
     </row>
     <row r="740">
       <c r="A740" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C740" t="inlineStr">
@@ -24961,67 +24977,26 @@
       </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E740" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F740" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G740" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H740" t="inlineStr"/>
       <c r="I740" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="741">
-      <c r="A741" t="n">
-        <v>763</v>
-      </c>
-      <c r="B741" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C741" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D741" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E741" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F741" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G741" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H741" t="inlineStr"/>
-      <c r="I741" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 709 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I740"/>
+  <dimension ref="A1:I739"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23308,7 +23308,7 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
@@ -23318,7 +23318,7 @@
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E689" t="inlineStr"/>
@@ -23337,7 +23337,7 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
@@ -23347,7 +23347,7 @@
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E690" t="inlineStr"/>
@@ -23366,17 +23366,17 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E691" t="inlineStr"/>
@@ -23395,7 +23395,7 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
@@ -23405,10 +23405,14 @@
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="E692" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F692" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23424,7 +23428,7 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
@@ -23434,14 +23438,10 @@
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E693" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr"/>
       <c r="F693" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23457,7 +23457,7 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
@@ -23467,10 +23467,14 @@
       <c r="C694" t="inlineStr"/>
       <c r="D694" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E694" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F694" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23486,7 +23490,7 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
@@ -23496,14 +23500,10 @@
       <c r="C695" t="inlineStr"/>
       <c r="D695" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E695" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr"/>
       <c r="F695" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23519,7 +23519,7 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
@@ -23529,7 +23529,7 @@
       <c r="C696" t="inlineStr"/>
       <c r="D696" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E696" t="inlineStr"/>
@@ -23548,7 +23548,7 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
@@ -23558,10 +23558,14 @@
       <c r="C697" t="inlineStr"/>
       <c r="D697" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E697" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F697" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23577,7 +23581,7 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
@@ -23587,12 +23591,12 @@
       <c r="C698" t="inlineStr"/>
       <c r="D698" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E698" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F698" t="inlineStr">
@@ -23610,7 +23614,7 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
@@ -23620,12 +23624,12 @@
       <c r="C699" t="inlineStr"/>
       <c r="D699" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E699" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F699" t="inlineStr">
@@ -23643,24 +23647,20 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C700" t="inlineStr"/>
       <c r="D700" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E700" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr"/>
       <c r="F700" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23676,7 +23676,7 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
@@ -23686,10 +23686,14 @@
       <c r="C701" t="inlineStr"/>
       <c r="D701" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E701" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F701" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23705,7 +23709,7 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
@@ -23715,12 +23719,12 @@
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E702" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F702" t="inlineStr">
@@ -23738,7 +23742,7 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
@@ -23748,14 +23752,10 @@
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E703" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr"/>
       <c r="F703" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23771,17 +23771,17 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E704" t="inlineStr"/>
@@ -23800,7 +23800,7 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
@@ -23810,7 +23810,7 @@
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E705" t="inlineStr"/>
@@ -23829,7 +23829,7 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
@@ -23839,10 +23839,14 @@
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E706" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F706" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23858,22 +23862,22 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E707" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F707" t="inlineStr">
@@ -23891,7 +23895,7 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
@@ -23901,12 +23905,12 @@
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E708" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F708" t="inlineStr">
@@ -23924,24 +23928,20 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C709" t="inlineStr"/>
       <c r="D709" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E709" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr"/>
       <c r="F709" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23957,23 +23957,27 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E710" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F710" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G710" t="inlineStr"/>
@@ -23986,27 +23990,23 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E711" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr"/>
       <c r="F711" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G711" t="inlineStr"/>
@@ -24019,7 +24019,7 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
@@ -24029,7 +24029,7 @@
       <c r="C712" t="inlineStr"/>
       <c r="D712" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E712" t="inlineStr"/>
@@ -24048,7 +24048,7 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
@@ -24058,7 +24058,7 @@
       <c r="C713" t="inlineStr"/>
       <c r="D713" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E713" t="inlineStr"/>
@@ -24077,7 +24077,7 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
@@ -24087,7 +24087,7 @@
       <c r="C714" t="inlineStr"/>
       <c r="D714" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E714" t="inlineStr"/>
@@ -24106,7 +24106,7 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
@@ -24116,10 +24116,14 @@
       <c r="C715" t="inlineStr"/>
       <c r="D715" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E715" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F715" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24135,24 +24139,20 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C716" t="inlineStr"/>
       <c r="D716" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E716" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr"/>
       <c r="F716" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24168,7 +24168,7 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
@@ -24178,7 +24178,7 @@
       <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E717" t="inlineStr"/>
@@ -24197,20 +24197,24 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C718" t="inlineStr"/>
       <c r="D718" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E718" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F718" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24226,27 +24230,23 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C719" t="inlineStr"/>
       <c r="D719" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E719" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr"/>
       <c r="F719" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G719" t="inlineStr"/>
@@ -24259,7 +24259,7 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
@@ -24269,7 +24269,7 @@
       <c r="C720" t="inlineStr"/>
       <c r="D720" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E720" t="inlineStr"/>
@@ -24288,23 +24288,27 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C721" t="inlineStr"/>
       <c r="D721" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E721" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F721" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G721" t="inlineStr"/>
@@ -24317,27 +24321,31 @@
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C722" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D722" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E722" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F722" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G722" t="inlineStr"/>
@@ -24350,11 +24358,11 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C723" t="inlineStr">
@@ -24364,12 +24372,12 @@
       </c>
       <c r="D723" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E723" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F723" t="inlineStr">
@@ -24387,26 +24395,26 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C724" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D724" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E724" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F724" t="inlineStr">
@@ -24424,31 +24432,27 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C725" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D725" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E725" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr"/>
       <c r="F725" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G725" t="inlineStr"/>
@@ -24461,27 +24465,27 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D726" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E726" t="inlineStr"/>
       <c r="F726" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G726" t="inlineStr"/>
@@ -24494,27 +24498,27 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C727" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D727" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E727" t="inlineStr"/>
       <c r="F727" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G727" t="inlineStr"/>
@@ -24527,27 +24531,27 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D728" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E728" t="inlineStr"/>
       <c r="F728" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G728" t="inlineStr"/>
@@ -24560,24 +24564,28 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C729" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D729" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E729" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F729" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -24593,11 +24601,11 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
@@ -24607,12 +24615,12 @@
       </c>
       <c r="D730" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E730" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F730" t="inlineStr">
@@ -24630,11 +24638,11 @@
     </row>
     <row r="731">
       <c r="A731" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C731" t="inlineStr">
@@ -24644,7 +24652,7 @@
       </c>
       <c r="D731" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E731" t="inlineStr">
@@ -24667,31 +24675,31 @@
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C732" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D732" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E732" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F732" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G732" t="inlineStr"/>
@@ -24704,31 +24712,27 @@
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C733" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D733" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E733" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr"/>
       <c r="F733" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G733" t="inlineStr"/>
@@ -24741,27 +24745,31 @@
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C734" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D734" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E734" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F734" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G734" t="inlineStr"/>
@@ -24774,26 +24782,22 @@
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C735" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr"/>
       <c r="D735" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E735" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F735" t="inlineStr">
@@ -24811,30 +24815,38 @@
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C736" t="inlineStr"/>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E736" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F736" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G736" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H736" t="inlineStr"/>
       <c r="I736" t="inlineStr">
         <is>
@@ -24844,38 +24856,34 @@
     </row>
     <row r="737">
       <c r="A737" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C737" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D737" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E737" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F737" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G737" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G737" t="inlineStr"/>
       <c r="H737" t="inlineStr"/>
       <c r="I737" t="inlineStr">
         <is>
@@ -24885,26 +24893,26 @@
     </row>
     <row r="738">
       <c r="A738" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C738" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D738" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E738" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F738" t="inlineStr">
@@ -24912,7 +24920,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G738" t="inlineStr"/>
+      <c r="G738" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H738" t="inlineStr"/>
       <c r="I738" t="inlineStr">
         <is>
@@ -24922,11 +24934,11 @@
     </row>
     <row r="739">
       <c r="A739" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C739" t="inlineStr">
@@ -24936,67 +24948,26 @@
       </c>
       <c r="D739" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E739" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F739" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G739" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H739" t="inlineStr"/>
       <c r="I739" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="740">
-      <c r="A740" t="n">
-        <v>763</v>
-      </c>
-      <c r="B740" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C740" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D740" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E740" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F740" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G740" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H740" t="inlineStr"/>
-      <c r="I740" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 690 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I739"/>
+  <dimension ref="A1:I738"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22734,17 +22734,17 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C671" t="inlineStr"/>
       <c r="D671" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E671" t="inlineStr"/>
@@ -22763,7 +22763,7 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
@@ -22773,10 +22773,14 @@
       <c r="C672" t="inlineStr"/>
       <c r="D672" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E672" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F672" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22792,24 +22796,20 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C673" t="inlineStr"/>
       <c r="D673" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E673" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr"/>
       <c r="F673" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22825,7 +22825,7 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
@@ -22835,7 +22835,7 @@
       <c r="C674" t="inlineStr"/>
       <c r="D674" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E674" t="inlineStr"/>
@@ -22854,17 +22854,17 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C675" t="inlineStr"/>
       <c r="D675" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E675" t="inlineStr"/>
@@ -22883,20 +22883,24 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C676" t="inlineStr"/>
       <c r="D676" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E676" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F676" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22912,7 +22916,7 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
@@ -22922,12 +22926,12 @@
       <c r="C677" t="inlineStr"/>
       <c r="D677" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E677" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F677" t="inlineStr">
@@ -22945,24 +22949,24 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C678" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D678" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E678" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr"/>
       <c r="F678" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22978,7 +22982,7 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
@@ -22987,12 +22991,12 @@
       </c>
       <c r="C679" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D679" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E679" t="inlineStr"/>
@@ -23011,7 +23015,7 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
@@ -23025,7 +23029,7 @@
       </c>
       <c r="D680" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E680" t="inlineStr"/>
@@ -23044,7 +23048,7 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
@@ -23058,10 +23062,14 @@
       </c>
       <c r="D681" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E681" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F681" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23077,7 +23085,7 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
@@ -23091,12 +23099,12 @@
       </c>
       <c r="D682" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E682" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F682" t="inlineStr">
@@ -23114,7 +23122,7 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
@@ -23128,14 +23136,10 @@
       </c>
       <c r="D683" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E683" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr"/>
       <c r="F683" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23151,24 +23155,24 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C684" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr"/>
       <c r="D684" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E684" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F684" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23184,24 +23188,20 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C685" t="inlineStr"/>
       <c r="D685" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E685" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr"/>
       <c r="F685" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23217,17 +23217,17 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C686" t="inlineStr"/>
       <c r="D686" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E686" t="inlineStr"/>
@@ -23246,7 +23246,7 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
@@ -23256,10 +23256,14 @@
       <c r="C687" t="inlineStr"/>
       <c r="D687" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E687" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F687" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23275,24 +23279,20 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C688" t="inlineStr"/>
       <c r="D688" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E688" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr"/>
       <c r="F688" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23308,7 +23308,7 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
@@ -23318,7 +23318,7 @@
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E689" t="inlineStr"/>
@@ -23337,17 +23337,17 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E690" t="inlineStr"/>
@@ -23366,7 +23366,7 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
@@ -23376,10 +23376,14 @@
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="E691" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F691" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23395,7 +23399,7 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
@@ -23405,14 +23409,10 @@
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E692" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr"/>
       <c r="F692" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23428,7 +23428,7 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
@@ -23438,10 +23438,14 @@
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E693" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F693" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23457,7 +23461,7 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
@@ -23467,14 +23471,10 @@
       <c r="C694" t="inlineStr"/>
       <c r="D694" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E694" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr"/>
       <c r="F694" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23490,7 +23490,7 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
@@ -23500,7 +23500,7 @@
       <c r="C695" t="inlineStr"/>
       <c r="D695" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E695" t="inlineStr"/>
@@ -23519,7 +23519,7 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
@@ -23529,10 +23529,14 @@
       <c r="C696" t="inlineStr"/>
       <c r="D696" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E696" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F696" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23548,7 +23552,7 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
@@ -23558,12 +23562,12 @@
       <c r="C697" t="inlineStr"/>
       <c r="D697" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E697" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F697" t="inlineStr">
@@ -23581,7 +23585,7 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
@@ -23591,12 +23595,12 @@
       <c r="C698" t="inlineStr"/>
       <c r="D698" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E698" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F698" t="inlineStr">
@@ -23614,24 +23618,20 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C699" t="inlineStr"/>
       <c r="D699" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E699" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr"/>
       <c r="F699" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23647,7 +23647,7 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
@@ -23657,10 +23657,14 @@
       <c r="C700" t="inlineStr"/>
       <c r="D700" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E700" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F700" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23676,7 +23680,7 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
@@ -23686,12 +23690,12 @@
       <c r="C701" t="inlineStr"/>
       <c r="D701" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E701" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F701" t="inlineStr">
@@ -23709,7 +23713,7 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
@@ -23719,14 +23723,10 @@
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E702" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr"/>
       <c r="F702" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23742,17 +23742,17 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E703" t="inlineStr"/>
@@ -23771,7 +23771,7 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
@@ -23781,7 +23781,7 @@
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E704" t="inlineStr"/>
@@ -23800,7 +23800,7 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
@@ -23810,10 +23810,14 @@
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E705" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F705" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23829,22 +23833,22 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E706" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F706" t="inlineStr">
@@ -23862,7 +23866,7 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
@@ -23872,12 +23876,12 @@
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E707" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F707" t="inlineStr">
@@ -23895,24 +23899,20 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E708" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr"/>
       <c r="F708" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23928,23 +23928,27 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C709" t="inlineStr"/>
       <c r="D709" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E709" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F709" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G709" t="inlineStr"/>
@@ -23957,27 +23961,23 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E710" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr"/>
       <c r="F710" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G710" t="inlineStr"/>
@@ -23990,7 +23990,7 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
@@ -24000,7 +24000,7 @@
       <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E711" t="inlineStr"/>
@@ -24019,7 +24019,7 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
@@ -24029,7 +24029,7 @@
       <c r="C712" t="inlineStr"/>
       <c r="D712" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E712" t="inlineStr"/>
@@ -24048,7 +24048,7 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
@@ -24058,7 +24058,7 @@
       <c r="C713" t="inlineStr"/>
       <c r="D713" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E713" t="inlineStr"/>
@@ -24077,7 +24077,7 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
@@ -24087,10 +24087,14 @@
       <c r="C714" t="inlineStr"/>
       <c r="D714" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E714" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F714" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24106,24 +24110,20 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C715" t="inlineStr"/>
       <c r="D715" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E715" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr"/>
       <c r="F715" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24139,7 +24139,7 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
@@ -24149,7 +24149,7 @@
       <c r="C716" t="inlineStr"/>
       <c r="D716" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E716" t="inlineStr"/>
@@ -24168,20 +24168,24 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E717" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F717" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24197,27 +24201,23 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C718" t="inlineStr"/>
       <c r="D718" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E718" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr"/>
       <c r="F718" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G718" t="inlineStr"/>
@@ -24230,7 +24230,7 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
@@ -24240,7 +24240,7 @@
       <c r="C719" t="inlineStr"/>
       <c r="D719" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E719" t="inlineStr"/>
@@ -24259,23 +24259,27 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C720" t="inlineStr"/>
       <c r="D720" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E720" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F720" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G720" t="inlineStr"/>
@@ -24288,27 +24292,31 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C721" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D721" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E721" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F721" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G721" t="inlineStr"/>
@@ -24321,11 +24329,11 @@
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C722" t="inlineStr">
@@ -24335,12 +24343,12 @@
       </c>
       <c r="D722" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E722" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F722" t="inlineStr">
@@ -24358,26 +24366,26 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C723" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D723" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E723" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F723" t="inlineStr">
@@ -24395,31 +24403,27 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C724" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D724" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E724" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr"/>
       <c r="F724" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G724" t="inlineStr"/>
@@ -24432,27 +24436,27 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C725" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D725" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E725" t="inlineStr"/>
       <c r="F725" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G725" t="inlineStr"/>
@@ -24465,27 +24469,27 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D726" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E726" t="inlineStr"/>
       <c r="F726" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G726" t="inlineStr"/>
@@ -24498,27 +24502,27 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C727" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D727" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E727" t="inlineStr"/>
       <c r="F727" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G727" t="inlineStr"/>
@@ -24531,24 +24535,28 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D728" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E728" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F728" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -24564,11 +24572,11 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C729" t="inlineStr">
@@ -24578,12 +24586,12 @@
       </c>
       <c r="D729" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E729" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F729" t="inlineStr">
@@ -24601,11 +24609,11 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
@@ -24615,7 +24623,7 @@
       </c>
       <c r="D730" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E730" t="inlineStr">
@@ -24638,31 +24646,31 @@
     </row>
     <row r="731">
       <c r="A731" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C731" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D731" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E731" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F731" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G731" t="inlineStr"/>
@@ -24675,31 +24683,27 @@
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C732" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D732" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E732" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr"/>
       <c r="F732" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G732" t="inlineStr"/>
@@ -24712,27 +24716,31 @@
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C733" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D733" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E733" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F733" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G733" t="inlineStr"/>
@@ -24745,26 +24753,22 @@
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C734" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr"/>
       <c r="D734" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E734" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F734" t="inlineStr">
@@ -24782,30 +24786,38 @@
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C735" t="inlineStr"/>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D735" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E735" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F735" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G735" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G735" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H735" t="inlineStr"/>
       <c r="I735" t="inlineStr">
         <is>
@@ -24815,38 +24827,34 @@
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C736" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E736" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F736" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G736" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G736" t="inlineStr"/>
       <c r="H736" t="inlineStr"/>
       <c r="I736" t="inlineStr">
         <is>
@@ -24856,26 +24864,26 @@
     </row>
     <row r="737">
       <c r="A737" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C737" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D737" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E737" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F737" t="inlineStr">
@@ -24883,7 +24891,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G737" t="inlineStr"/>
+      <c r="G737" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H737" t="inlineStr"/>
       <c r="I737" t="inlineStr">
         <is>
@@ -24893,11 +24905,11 @@
     </row>
     <row r="738">
       <c r="A738" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C738" t="inlineStr">
@@ -24907,67 +24919,26 @@
       </c>
       <c r="D738" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E738" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F738" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G738" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H738" t="inlineStr"/>
       <c r="I738" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="739">
-      <c r="A739" t="n">
-        <v>763</v>
-      </c>
-      <c r="B739" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C739" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D739" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E739" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F739" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G739" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H739" t="inlineStr"/>
-      <c r="I739" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 712 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I738"/>
+  <dimension ref="A1:I737"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23337,7 +23337,7 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
@@ -23347,10 +23347,14 @@
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="E690" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F690" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23366,7 +23370,7 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
@@ -23376,14 +23380,10 @@
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E691" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr"/>
       <c r="F691" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23399,7 +23399,7 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
@@ -23409,10 +23409,14 @@
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E692" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F692" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23428,7 +23432,7 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
@@ -23438,14 +23442,10 @@
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E693" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr"/>
       <c r="F693" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23461,7 +23461,7 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
@@ -23471,7 +23471,7 @@
       <c r="C694" t="inlineStr"/>
       <c r="D694" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E694" t="inlineStr"/>
@@ -23490,7 +23490,7 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
@@ -23500,10 +23500,14 @@
       <c r="C695" t="inlineStr"/>
       <c r="D695" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E695" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F695" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23519,7 +23523,7 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
@@ -23529,12 +23533,12 @@
       <c r="C696" t="inlineStr"/>
       <c r="D696" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E696" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F696" t="inlineStr">
@@ -23552,7 +23556,7 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
@@ -23562,12 +23566,12 @@
       <c r="C697" t="inlineStr"/>
       <c r="D697" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E697" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F697" t="inlineStr">
@@ -23585,24 +23589,20 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C698" t="inlineStr"/>
       <c r="D698" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E698" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr"/>
       <c r="F698" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23618,7 +23618,7 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
@@ -23628,10 +23628,14 @@
       <c r="C699" t="inlineStr"/>
       <c r="D699" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E699" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F699" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23647,7 +23651,7 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
@@ -23657,12 +23661,12 @@
       <c r="C700" t="inlineStr"/>
       <c r="D700" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E700" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F700" t="inlineStr">
@@ -23680,7 +23684,7 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
@@ -23690,14 +23694,10 @@
       <c r="C701" t="inlineStr"/>
       <c r="D701" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E701" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr"/>
       <c r="F701" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23713,17 +23713,17 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E702" t="inlineStr"/>
@@ -23742,7 +23742,7 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
@@ -23752,7 +23752,7 @@
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E703" t="inlineStr"/>
@@ -23771,7 +23771,7 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
@@ -23781,10 +23781,14 @@
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E704" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F704" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23800,22 +23804,22 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E705" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F705" t="inlineStr">
@@ -23833,7 +23837,7 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
@@ -23843,12 +23847,12 @@
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E706" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F706" t="inlineStr">
@@ -23866,24 +23870,20 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E707" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr"/>
       <c r="F707" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23899,23 +23899,27 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E708" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F708" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G708" t="inlineStr"/>
@@ -23928,27 +23932,23 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C709" t="inlineStr"/>
       <c r="D709" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E709" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr"/>
       <c r="F709" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G709" t="inlineStr"/>
@@ -23961,7 +23961,7 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
@@ -23971,7 +23971,7 @@
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E710" t="inlineStr"/>
@@ -23990,7 +23990,7 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
@@ -24000,7 +24000,7 @@
       <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E711" t="inlineStr"/>
@@ -24019,7 +24019,7 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
@@ -24029,7 +24029,7 @@
       <c r="C712" t="inlineStr"/>
       <c r="D712" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E712" t="inlineStr"/>
@@ -24048,7 +24048,7 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
@@ -24058,10 +24058,14 @@
       <c r="C713" t="inlineStr"/>
       <c r="D713" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E713" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F713" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24077,24 +24081,20 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C714" t="inlineStr"/>
       <c r="D714" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E714" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr"/>
       <c r="F714" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24110,7 +24110,7 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
@@ -24120,7 +24120,7 @@
       <c r="C715" t="inlineStr"/>
       <c r="D715" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E715" t="inlineStr"/>
@@ -24139,20 +24139,24 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C716" t="inlineStr"/>
       <c r="D716" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E716" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F716" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24168,27 +24172,23 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E717" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr"/>
       <c r="F717" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G717" t="inlineStr"/>
@@ -24201,7 +24201,7 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
@@ -24211,7 +24211,7 @@
       <c r="C718" t="inlineStr"/>
       <c r="D718" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E718" t="inlineStr"/>
@@ -24230,23 +24230,27 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C719" t="inlineStr"/>
       <c r="D719" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E719" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F719" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G719" t="inlineStr"/>
@@ -24259,27 +24263,31 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C720" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D720" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E720" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F720" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G720" t="inlineStr"/>
@@ -24292,11 +24300,11 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C721" t="inlineStr">
@@ -24306,12 +24314,12 @@
       </c>
       <c r="D721" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E721" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F721" t="inlineStr">
@@ -24329,26 +24337,26 @@
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C722" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D722" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E722" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F722" t="inlineStr">
@@ -24366,31 +24374,27 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C723" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D723" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E723" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr"/>
       <c r="F723" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G723" t="inlineStr"/>
@@ -24403,27 +24407,27 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C724" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D724" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E724" t="inlineStr"/>
       <c r="F724" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G724" t="inlineStr"/>
@@ -24436,27 +24440,27 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C725" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D725" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E725" t="inlineStr"/>
       <c r="F725" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G725" t="inlineStr"/>
@@ -24469,27 +24473,27 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D726" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E726" t="inlineStr"/>
       <c r="F726" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G726" t="inlineStr"/>
@@ -24502,24 +24506,28 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C727" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D727" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E727" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F727" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -24535,11 +24543,11 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
@@ -24549,12 +24557,12 @@
       </c>
       <c r="D728" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E728" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F728" t="inlineStr">
@@ -24572,11 +24580,11 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C729" t="inlineStr">
@@ -24586,7 +24594,7 @@
       </c>
       <c r="D729" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E729" t="inlineStr">
@@ -24609,31 +24617,31 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D730" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E730" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F730" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G730" t="inlineStr"/>
@@ -24646,31 +24654,27 @@
     </row>
     <row r="731">
       <c r="A731" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C731" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D731" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E731" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr"/>
       <c r="F731" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G731" t="inlineStr"/>
@@ -24683,27 +24687,31 @@
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C732" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D732" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E732" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F732" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G732" t="inlineStr"/>
@@ -24716,26 +24724,22 @@
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C733" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr"/>
       <c r="D733" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E733" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F733" t="inlineStr">
@@ -24753,30 +24757,38 @@
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C734" t="inlineStr"/>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D734" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E734" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F734" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G734" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G734" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H734" t="inlineStr"/>
       <c r="I734" t="inlineStr">
         <is>
@@ -24786,38 +24798,34 @@
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C735" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D735" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E735" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F735" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G735" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G735" t="inlineStr"/>
       <c r="H735" t="inlineStr"/>
       <c r="I735" t="inlineStr">
         <is>
@@ -24827,26 +24835,26 @@
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C736" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E736" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F736" t="inlineStr">
@@ -24854,7 +24862,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G736" t="inlineStr"/>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H736" t="inlineStr"/>
       <c r="I736" t="inlineStr">
         <is>
@@ -24864,11 +24876,11 @@
     </row>
     <row r="737">
       <c r="A737" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C737" t="inlineStr">
@@ -24878,67 +24890,26 @@
       </c>
       <c r="D737" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E737" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F737" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G737" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H737" t="inlineStr"/>
       <c r="I737" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="738">
-      <c r="A738" t="n">
-        <v>763</v>
-      </c>
-      <c r="B738" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C738" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D738" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E738" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F738" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G738" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H738" t="inlineStr"/>
-      <c r="I738" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 725 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I737"/>
+  <dimension ref="A1:I736"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23713,7 +23713,7 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
@@ -23723,7 +23723,7 @@
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E702" t="inlineStr"/>
@@ -23742,7 +23742,7 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
@@ -23752,10 +23752,14 @@
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E703" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F703" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23771,22 +23775,22 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E704" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F704" t="inlineStr">
@@ -23804,7 +23808,7 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
@@ -23814,12 +23818,12 @@
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E705" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F705" t="inlineStr">
@@ -23837,24 +23841,20 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E706" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr"/>
       <c r="F706" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23870,23 +23870,27 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E707" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F707" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G707" t="inlineStr"/>
@@ -23899,27 +23903,23 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E708" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr"/>
       <c r="F708" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G708" t="inlineStr"/>
@@ -23932,7 +23932,7 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
@@ -23942,7 +23942,7 @@
       <c r="C709" t="inlineStr"/>
       <c r="D709" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E709" t="inlineStr"/>
@@ -23961,7 +23961,7 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
@@ -23971,7 +23971,7 @@
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E710" t="inlineStr"/>
@@ -23990,7 +23990,7 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
@@ -24000,7 +24000,7 @@
       <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E711" t="inlineStr"/>
@@ -24019,7 +24019,7 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
@@ -24029,10 +24029,14 @@
       <c r="C712" t="inlineStr"/>
       <c r="D712" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E712" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F712" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24048,24 +24052,20 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C713" t="inlineStr"/>
       <c r="D713" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E713" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr"/>
       <c r="F713" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24081,7 +24081,7 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
@@ -24091,7 +24091,7 @@
       <c r="C714" t="inlineStr"/>
       <c r="D714" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E714" t="inlineStr"/>
@@ -24110,20 +24110,24 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C715" t="inlineStr"/>
       <c r="D715" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E715" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F715" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -24139,27 +24143,23 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C716" t="inlineStr"/>
       <c r="D716" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E716" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr"/>
       <c r="F716" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G716" t="inlineStr"/>
@@ -24172,7 +24172,7 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
@@ -24182,7 +24182,7 @@
       <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E717" t="inlineStr"/>
@@ -24201,23 +24201,27 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C718" t="inlineStr"/>
       <c r="D718" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E718" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F718" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G718" t="inlineStr"/>
@@ -24230,27 +24234,31 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C719" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D719" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E719" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F719" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G719" t="inlineStr"/>
@@ -24263,11 +24271,11 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C720" t="inlineStr">
@@ -24277,12 +24285,12 @@
       </c>
       <c r="D720" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E720" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F720" t="inlineStr">
@@ -24300,26 +24308,26 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C721" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D721" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E721" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F721" t="inlineStr">
@@ -24337,31 +24345,27 @@
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C722" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D722" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E722" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr"/>
       <c r="F722" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G722" t="inlineStr"/>
@@ -24374,27 +24378,27 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C723" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D723" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E723" t="inlineStr"/>
       <c r="F723" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G723" t="inlineStr"/>
@@ -24407,27 +24411,27 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C724" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D724" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E724" t="inlineStr"/>
       <c r="F724" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G724" t="inlineStr"/>
@@ -24440,27 +24444,27 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C725" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D725" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E725" t="inlineStr"/>
       <c r="F725" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G725" t="inlineStr"/>
@@ -24473,24 +24477,28 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D726" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E726" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F726" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -24506,11 +24514,11 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C727" t="inlineStr">
@@ -24520,12 +24528,12 @@
       </c>
       <c r="D727" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E727" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F727" t="inlineStr">
@@ -24543,11 +24551,11 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
@@ -24557,7 +24565,7 @@
       </c>
       <c r="D728" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E728" t="inlineStr">
@@ -24580,31 +24588,31 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C729" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D729" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E729" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F729" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G729" t="inlineStr"/>
@@ -24617,31 +24625,27 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D730" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E730" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr"/>
       <c r="F730" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G730" t="inlineStr"/>
@@ -24654,27 +24658,31 @@
     </row>
     <row r="731">
       <c r="A731" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C731" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D731" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E731" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F731" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G731" t="inlineStr"/>
@@ -24687,26 +24695,22 @@
     </row>
     <row r="732">
       <c r="A732" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C732" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr"/>
       <c r="D732" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E732" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F732" t="inlineStr">
@@ -24724,30 +24728,38 @@
     </row>
     <row r="733">
       <c r="A733" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B733" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C733" t="inlineStr"/>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D733" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E733" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F733" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G733" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G733" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H733" t="inlineStr"/>
       <c r="I733" t="inlineStr">
         <is>
@@ -24757,38 +24769,34 @@
     </row>
     <row r="734">
       <c r="A734" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C734" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D734" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E734" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F734" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G734" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G734" t="inlineStr"/>
       <c r="H734" t="inlineStr"/>
       <c r="I734" t="inlineStr">
         <is>
@@ -24798,26 +24806,26 @@
     </row>
     <row r="735">
       <c r="A735" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C735" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D735" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E735" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F735" t="inlineStr">
@@ -24825,7 +24833,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G735" t="inlineStr"/>
+      <c r="G735" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H735" t="inlineStr"/>
       <c r="I735" t="inlineStr">
         <is>
@@ -24835,11 +24847,11 @@
     </row>
     <row r="736">
       <c r="A736" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C736" t="inlineStr">
@@ -24849,67 +24861,26 @@
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E736" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F736" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G736" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H736" t="inlineStr"/>
       <c r="I736" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="737">
-      <c r="A737" t="n">
-        <v>763</v>
-      </c>
-      <c r="B737" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C737" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D737" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E737" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F737" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G737" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H737" t="inlineStr"/>
-      <c r="I737" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Hromadná úprava z tabulky (Host) (autor: Host)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -492,7 +492,7 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1085,7 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1118,7 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1188,7 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -1645,7 +1645,7 @@
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3048,7 @@
       <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -3147,7 +3147,7 @@
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -3316,7 +3316,7 @@
       <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3345,7 @@
       <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -3481,7 +3481,7 @@
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -3514,7 +3514,7 @@
       <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -3613,7 +3613,7 @@
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -3959,7 +3959,7 @@
       <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       <c r="H102" t="inlineStr"/>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4124,7 +4124,7 @@
       <c r="H106" t="inlineStr"/>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4153,7 +4153,7 @@
       <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4355,7 +4355,7 @@
       <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4384,7 +4384,7 @@
       <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4413,7 +4413,7 @@
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4508,7 +4508,7 @@
       <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4595,7 +4595,7 @@
       <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4628,7 +4628,7 @@
       <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4661,7 @@
       <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4731,7 +4731,7 @@
       <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4834,7 +4834,7 @@
       <c r="H128" t="inlineStr"/>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -4863,7 +4863,7 @@
       <c r="H129" t="inlineStr"/>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -5073,7 +5073,7 @@
       <c r="H135" t="inlineStr"/>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -5436,7 +5436,7 @@
       <c r="H146" t="inlineStr"/>
       <c r="I146" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -5712,7 +5712,7 @@
       <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -5778,7 +5778,7 @@
       <c r="H156" t="inlineStr"/>
       <c r="I156" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -5951,7 +5951,7 @@
       <c r="H161" t="inlineStr"/>
       <c r="I161" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       <c r="H172" t="inlineStr"/>
       <c r="I172" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -6458,7 +6458,7 @@
       <c r="H176" t="inlineStr"/>
       <c r="I176" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -6520,7 +6520,7 @@
       <c r="H178" t="inlineStr"/>
       <c r="I178" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -6689,7 +6689,7 @@
       <c r="H183" t="inlineStr"/>
       <c r="I183" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       <c r="H193" t="inlineStr"/>
       <c r="I193" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7052,7 +7052,7 @@
       <c r="H194" t="inlineStr"/>
       <c r="I194" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7295,7 +7295,7 @@
       <c r="H201" t="inlineStr"/>
       <c r="I201" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7328,7 +7328,7 @@
       <c r="H202" t="inlineStr"/>
       <c r="I202" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7472,7 +7472,7 @@
       <c r="H206" t="inlineStr"/>
       <c r="I206" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7505,7 +7505,7 @@
       <c r="H207" t="inlineStr"/>
       <c r="I207" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7538,7 +7538,7 @@
       <c r="H208" t="inlineStr"/>
       <c r="I208" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7571,7 +7571,7 @@
       <c r="H209" t="inlineStr"/>
       <c r="I209" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7604,7 +7604,7 @@
       <c r="H210" t="inlineStr"/>
       <c r="I210" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7666,7 +7666,7 @@
       <c r="H212" t="inlineStr"/>
       <c r="I212" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7695,7 +7695,7 @@
       <c r="H213" t="inlineStr"/>
       <c r="I213" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7786,7 +7786,7 @@
       <c r="H216" t="inlineStr"/>
       <c r="I216" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7815,7 +7815,7 @@
       <c r="H217" t="inlineStr"/>
       <c r="I217" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7844,7 +7844,7 @@
       <c r="H218" t="inlineStr"/>
       <c r="I218" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7873,7 +7873,7 @@
       <c r="H219" t="inlineStr"/>
       <c r="I219" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7902,7 +7902,7 @@
       <c r="H220" t="inlineStr"/>
       <c r="I220" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7931,7 +7931,7 @@
       <c r="H221" t="inlineStr"/>
       <c r="I221" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -7993,7 +7993,7 @@
       <c r="H223" t="inlineStr"/>
       <c r="I223" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8022,7 +8022,7 @@
       <c r="H224" t="inlineStr"/>
       <c r="I224" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8084,7 +8084,7 @@
       <c r="H226" t="inlineStr"/>
       <c r="I226" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       <c r="H228" t="inlineStr"/>
       <c r="I228" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8175,7 +8175,7 @@
       <c r="H229" t="inlineStr"/>
       <c r="I229" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8307,7 +8307,7 @@
       <c r="H233" t="inlineStr"/>
       <c r="I233" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8340,7 +8340,7 @@
       <c r="H234" t="inlineStr"/>
       <c r="I234" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8373,7 +8373,7 @@
       <c r="H235" t="inlineStr"/>
       <c r="I235" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8406,7 +8406,7 @@
       <c r="H236" t="inlineStr"/>
       <c r="I236" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8439,7 +8439,7 @@
       <c r="H237" t="inlineStr"/>
       <c r="I237" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8472,7 +8472,7 @@
       <c r="H238" t="inlineStr"/>
       <c r="I238" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8542,7 +8542,7 @@
       <c r="H240" t="inlineStr"/>
       <c r="I240" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8612,7 +8612,7 @@
       <c r="H242" t="inlineStr"/>
       <c r="I242" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8645,7 +8645,7 @@
       <c r="H243" t="inlineStr"/>
       <c r="I243" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       <c r="H244" t="inlineStr"/>
       <c r="I244" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8773,7 +8773,7 @@
       <c r="H247" t="inlineStr"/>
       <c r="I247" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8872,7 +8872,7 @@
       <c r="H250" t="inlineStr"/>
       <c r="I250" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8905,7 +8905,7 @@
       <c r="H251" t="inlineStr"/>
       <c r="I251" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8934,7 +8934,7 @@
       <c r="H252" t="inlineStr"/>
       <c r="I252" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -8967,7 +8967,7 @@
       <c r="H253" t="inlineStr"/>
       <c r="I253" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9029,7 +9029,7 @@
       <c r="H255" t="inlineStr"/>
       <c r="I255" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9165,7 @@
       <c r="H259" t="inlineStr"/>
       <c r="I259" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9330,7 +9330,7 @@
       <c r="H264" t="inlineStr"/>
       <c r="I264" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9359,7 +9359,7 @@
       <c r="H265" t="inlineStr"/>
       <c r="I265" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9388,7 +9388,7 @@
       <c r="H266" t="inlineStr"/>
       <c r="I266" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9417,7 +9417,7 @@
       <c r="H267" t="inlineStr"/>
       <c r="I267" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9446,7 +9446,7 @@
       <c r="H268" t="inlineStr"/>
       <c r="I268" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9475,7 +9475,7 @@
       <c r="H269" t="inlineStr"/>
       <c r="I269" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9574,7 +9574,7 @@
       <c r="H272" t="inlineStr"/>
       <c r="I272" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9607,7 +9607,7 @@
       <c r="H273" t="inlineStr"/>
       <c r="I273" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9640,7 +9640,7 @@
       <c r="H274" t="inlineStr"/>
       <c r="I274" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9669,7 +9669,7 @@
       <c r="H275" t="inlineStr"/>
       <c r="I275" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9702,7 +9702,7 @@
       <c r="H276" t="inlineStr"/>
       <c r="I276" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9735,7 +9735,7 @@
       <c r="H277" t="inlineStr"/>
       <c r="I277" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9768,7 +9768,7 @@
       <c r="H278" t="inlineStr"/>
       <c r="I278" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9801,7 +9801,7 @@
       <c r="H279" t="inlineStr"/>
       <c r="I279" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9834,7 +9834,7 @@
       <c r="H280" t="inlineStr"/>
       <c r="I280" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9867,7 +9867,7 @@
       <c r="H281" t="inlineStr"/>
       <c r="I281" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9900,7 +9900,7 @@
       <c r="H282" t="inlineStr"/>
       <c r="I282" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9933,7 +9933,7 @@
       <c r="H283" t="inlineStr"/>
       <c r="I283" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -9999,7 +9999,7 @@
       <c r="H285" t="inlineStr"/>
       <c r="I285" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10028,7 +10028,7 @@
       <c r="H286" t="inlineStr"/>
       <c r="I286" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10090,7 +10090,7 @@
       <c r="H288" t="inlineStr"/>
       <c r="I288" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10152,7 +10152,7 @@
       <c r="H290" t="inlineStr"/>
       <c r="I290" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10181,7 +10181,7 @@
       <c r="H291" t="inlineStr"/>
       <c r="I291" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10210,7 +10210,7 @@
       <c r="H292" t="inlineStr"/>
       <c r="I292" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10305,7 +10305,7 @@
       <c r="H295" t="inlineStr"/>
       <c r="I295" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10334,7 +10334,7 @@
       <c r="H296" t="inlineStr"/>
       <c r="I296" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10363,7 +10363,7 @@
       <c r="H297" t="inlineStr"/>
       <c r="I297" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10392,7 +10392,7 @@
       <c r="H298" t="inlineStr"/>
       <c r="I298" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10421,7 +10421,7 @@
       <c r="H299" t="inlineStr"/>
       <c r="I299" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10450,7 +10450,7 @@
       <c r="H300" t="inlineStr"/>
       <c r="I300" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10479,7 +10479,7 @@
       <c r="H301" t="inlineStr"/>
       <c r="I301" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       <c r="H302" t="inlineStr"/>
       <c r="I302" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10537,7 +10537,7 @@
       <c r="H303" t="inlineStr"/>
       <c r="I303" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10566,7 +10566,7 @@
       <c r="H304" t="inlineStr"/>
       <c r="I304" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10661,7 +10661,7 @@
       <c r="H307" t="inlineStr"/>
       <c r="I307" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10690,7 +10690,7 @@
       <c r="H308" t="inlineStr"/>
       <c r="I308" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10719,7 +10719,7 @@
       <c r="H309" t="inlineStr"/>
       <c r="I309" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10748,7 +10748,7 @@
       <c r="H310" t="inlineStr"/>
       <c r="I310" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10777,7 +10777,7 @@
       <c r="H311" t="inlineStr"/>
       <c r="I311" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10806,7 +10806,7 @@
       <c r="H312" t="inlineStr"/>
       <c r="I312" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10835,7 +10835,7 @@
       <c r="H313" t="inlineStr"/>
       <c r="I313" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10901,7 +10901,7 @@
       <c r="H315" t="inlineStr"/>
       <c r="I315" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       <c r="H316" t="inlineStr"/>
       <c r="I316" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -10967,7 +10967,7 @@
       <c r="H317" t="inlineStr"/>
       <c r="I317" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -11000,7 +11000,7 @@
       <c r="H318" t="inlineStr"/>
       <c r="I318" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -11033,7 +11033,7 @@
       <c r="H319" t="inlineStr"/>
       <c r="I319" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -11066,7 +11066,7 @@
       <c r="H320" t="inlineStr"/>
       <c r="I320" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -11330,7 +11330,7 @@
       <c r="H328" t="inlineStr"/>
       <c r="I328" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -11528,7 +11528,7 @@
       <c r="H334" t="inlineStr"/>
       <c r="I334" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -11965,7 +11965,7 @@
       <c r="H347" t="inlineStr"/>
       <c r="I347" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -12146,7 +12146,7 @@
       <c r="H352" t="inlineStr"/>
       <c r="I352" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -12179,7 +12179,7 @@
       <c r="H353" t="inlineStr"/>
       <c r="I353" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -12323,7 +12323,7 @@
       <c r="H357" t="inlineStr"/>
       <c r="I357" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -12426,7 +12426,7 @@
       <c r="H360" t="inlineStr"/>
       <c r="I360" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -12587,7 +12587,7 @@
       <c r="H365" t="inlineStr"/>
       <c r="I365" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -12814,7 +12814,7 @@
       <c r="H372" t="inlineStr"/>
       <c r="I372" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -12843,7 +12843,7 @@
       <c r="H373" t="inlineStr"/>
       <c r="I373" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -12872,7 +12872,7 @@
       <c r="H374" t="inlineStr"/>
       <c r="I374" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -12934,7 +12934,7 @@
       <c r="H376" t="inlineStr"/>
       <c r="I376" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -13173,7 +13173,7 @@
       <c r="H383" t="inlineStr"/>
       <c r="I383" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -13470,7 +13470,7 @@
       <c r="H392" t="inlineStr"/>
       <c r="I392" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -13746,7 +13746,7 @@
       <c r="H400" t="inlineStr"/>
       <c r="I400" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -13808,7 +13808,7 @@
       <c r="H402" t="inlineStr"/>
       <c r="I402" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -13936,7 +13936,7 @@
       <c r="H406" t="inlineStr"/>
       <c r="I406" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -14196,7 +14196,7 @@
       <c r="H414" t="inlineStr"/>
       <c r="I414" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -14357,7 +14357,7 @@
       <c r="H419" t="inlineStr"/>
       <c r="I419" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -14452,7 +14452,7 @@
       <c r="H422" t="inlineStr"/>
       <c r="I422" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -14481,7 +14481,7 @@
       <c r="H423" t="inlineStr"/>
       <c r="I423" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -14576,7 +14576,7 @@
       <c r="H426" t="inlineStr"/>
       <c r="I426" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -15001,7 +15001,7 @@
       <c r="H439" t="inlineStr"/>
       <c r="I439" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -15071,7 +15071,7 @@
       <c r="H441" t="inlineStr"/>
       <c r="I441" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -15474,7 +15474,7 @@
       <c r="H452" t="inlineStr"/>
       <c r="I452" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -15898,7 +15898,7 @@
       <c r="H464" t="inlineStr"/>
       <c r="I464" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -16339,7 +16339,7 @@
       <c r="H477" t="inlineStr"/>
       <c r="I477" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -16368,7 +16368,7 @@
       <c r="H478" t="inlineStr"/>
       <c r="I478" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -16496,7 +16496,7 @@
       <c r="H482" t="inlineStr"/>
       <c r="I482" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -16525,7 +16525,7 @@
       <c r="H483" t="inlineStr"/>
       <c r="I483" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -16554,7 +16554,7 @@
       <c r="H484" t="inlineStr"/>
       <c r="I484" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -16616,7 +16616,7 @@
       <c r="H486" t="inlineStr"/>
       <c r="I486" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -16645,7 +16645,7 @@
       <c r="H487" t="inlineStr"/>
       <c r="I487" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -16674,7 +16674,7 @@
       <c r="H488" t="inlineStr"/>
       <c r="I488" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -16835,7 +16835,7 @@
       <c r="H493" t="inlineStr"/>
       <c r="I493" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -16897,7 +16897,7 @@
       <c r="H495" t="inlineStr"/>
       <c r="I495" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -16926,7 +16926,7 @@
       <c r="H496" t="inlineStr"/>
       <c r="I496" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -16955,7 +16955,7 @@
       <c r="H497" t="inlineStr"/>
       <c r="I497" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -17083,7 +17083,7 @@
       <c r="H501" t="inlineStr"/>
       <c r="I501" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -17112,7 +17112,7 @@
       <c r="H502" t="inlineStr"/>
       <c r="I502" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -17141,7 +17141,7 @@
       <c r="H503" t="inlineStr"/>
       <c r="I503" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -17421,7 +17421,7 @@
       <c r="H511" t="inlineStr"/>
       <c r="I511" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -17491,7 +17491,7 @@
       <c r="H513" t="inlineStr"/>
       <c r="I513" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -17561,7 +17561,7 @@
       <c r="H515" t="inlineStr"/>
       <c r="I515" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -17631,7 +17631,7 @@
       <c r="H517" t="inlineStr"/>
       <c r="I517" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -17664,7 +17664,7 @@
       <c r="H518" t="inlineStr"/>
       <c r="I518" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -17734,7 +17734,7 @@
       <c r="H520" t="inlineStr"/>
       <c r="I520" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -17841,7 +17841,7 @@
       <c r="H523" t="inlineStr"/>
       <c r="I523" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -17948,7 +17948,7 @@
       <c r="H526" t="inlineStr"/>
       <c r="I526" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -18129,7 +18129,7 @@
       <c r="H531" t="inlineStr"/>
       <c r="I531" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -18162,7 +18162,7 @@
       <c r="H532" t="inlineStr"/>
       <c r="I532" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -18689,7 +18689,7 @@
       <c r="H547" t="inlineStr"/>
       <c r="I547" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -18784,7 +18784,7 @@
       <c r="H550" t="inlineStr"/>
       <c r="I550" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -18846,7 +18846,7 @@
       <c r="H552" t="inlineStr"/>
       <c r="I552" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -19106,7 +19106,7 @@
       <c r="H560" t="inlineStr"/>
       <c r="I560" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -19168,7 +19168,7 @@
       <c r="H562" t="inlineStr"/>
       <c r="I562" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -19197,7 +19197,7 @@
       <c r="H563" t="inlineStr"/>
       <c r="I563" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -19391,7 +19391,7 @@
       <c r="H569" t="inlineStr"/>
       <c r="I569" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -19453,7 +19453,7 @@
       <c r="H571" t="inlineStr"/>
       <c r="I571" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -19552,7 +19552,7 @@
       <c r="H574" t="inlineStr"/>
       <c r="I574" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -20377,7 +20377,7 @@
       <c r="H599" t="inlineStr"/>
       <c r="I599" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -20410,7 +20410,7 @@
       <c r="H600" t="inlineStr"/>
       <c r="I600" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -20443,7 +20443,7 @@
       <c r="H601" t="inlineStr"/>
       <c r="I601" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -20550,7 +20550,7 @@
       <c r="H604" t="inlineStr"/>
       <c r="I604" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -20620,7 +20620,7 @@
       <c r="H606" t="inlineStr"/>
       <c r="I606" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -20949,7 +20949,7 @@
       <c r="H615" t="inlineStr"/>
       <c r="I615" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21019,7 +21019,7 @@
       <c r="H617" t="inlineStr"/>
       <c r="I617" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21052,7 +21052,7 @@
       <c r="H618" t="inlineStr"/>
       <c r="I618" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21081,7 +21081,7 @@
       <c r="H619" t="inlineStr"/>
       <c r="I619" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21110,7 +21110,7 @@
       <c r="H620" t="inlineStr"/>
       <c r="I620" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21139,7 +21139,7 @@
       <c r="H621" t="inlineStr"/>
       <c r="I621" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21234,7 +21234,7 @@
       <c r="H624" t="inlineStr"/>
       <c r="I624" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21333,7 +21333,7 @@
       <c r="H627" t="inlineStr"/>
       <c r="I627" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21362,7 +21362,7 @@
       <c r="H628" t="inlineStr"/>
       <c r="I628" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21391,7 +21391,7 @@
       <c r="H629" t="inlineStr"/>
       <c r="I629" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21420,7 +21420,7 @@
       <c r="H630" t="inlineStr"/>
       <c r="I630" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21453,7 +21453,7 @@
       <c r="H631" t="inlineStr"/>
       <c r="I631" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21486,7 +21486,7 @@
       <c r="H632" t="inlineStr"/>
       <c r="I632" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21548,7 +21548,7 @@
       <c r="H634" t="inlineStr"/>
       <c r="I634" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21581,7 +21581,7 @@
       <c r="H635" t="inlineStr"/>
       <c r="I635" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21614,7 +21614,7 @@
       <c r="H636" t="inlineStr"/>
       <c r="I636" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21709,7 +21709,7 @@
       <c r="H639" t="inlineStr"/>
       <c r="I639" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21742,7 +21742,7 @@
       <c r="H640" t="inlineStr"/>
       <c r="I640" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21771,7 +21771,7 @@
       <c r="H641" t="inlineStr"/>
       <c r="I641" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21800,7 +21800,7 @@
       <c r="H642" t="inlineStr"/>
       <c r="I642" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21829,7 +21829,7 @@
       <c r="H643" t="inlineStr"/>
       <c r="I643" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -21932,7 +21932,7 @@
       <c r="H646" t="inlineStr"/>
       <c r="I646" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -22068,7 +22068,7 @@
       <c r="H650" t="inlineStr"/>
       <c r="I650" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -22101,7 +22101,7 @@
       <c r="H651" t="inlineStr"/>
       <c r="I651" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -22208,7 +22208,7 @@
       <c r="H654" t="inlineStr"/>
       <c r="I654" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -22303,7 +22303,7 @@
       <c r="H657" t="inlineStr"/>
       <c r="I657" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -22641,7 +22641,7 @@
       <c r="H667" t="inlineStr"/>
       <c r="I667" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -22670,7 +22670,7 @@
       <c r="H668" t="inlineStr"/>
       <c r="I668" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -22699,7 +22699,7 @@
       <c r="H669" t="inlineStr"/>
       <c r="I669" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -22728,7 +22728,7 @@
       <c r="H670" t="inlineStr"/>
       <c r="I670" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -22790,7 +22790,7 @@
       <c r="H672" t="inlineStr"/>
       <c r="I672" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -22819,7 +22819,7 @@
       <c r="H673" t="inlineStr"/>
       <c r="I673" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -22848,7 +22848,7 @@
       <c r="H674" t="inlineStr"/>
       <c r="I674" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -22947,7 +22947,7 @@
       <c r="H677" t="inlineStr"/>
       <c r="I677" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -22973,14 +22973,14 @@
       <c r="E678" t="inlineStr"/>
       <c r="F678" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G678" t="inlineStr"/>
       <c r="H678" t="inlineStr"/>
       <c r="I678" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23013,7 +23013,7 @@
       <c r="H679" t="inlineStr"/>
       <c r="I679" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23120,7 +23120,7 @@
       <c r="H682" t="inlineStr"/>
       <c r="I682" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23182,7 +23182,7 @@
       <c r="H684" t="inlineStr"/>
       <c r="I684" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23211,7 +23211,7 @@
       <c r="H685" t="inlineStr"/>
       <c r="I685" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23273,7 +23273,7 @@
       <c r="H687" t="inlineStr"/>
       <c r="I687" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23302,7 +23302,7 @@
       <c r="H688" t="inlineStr"/>
       <c r="I688" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23364,7 +23364,7 @@
       <c r="H690" t="inlineStr"/>
       <c r="I690" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23426,7 +23426,7 @@
       <c r="H692" t="inlineStr"/>
       <c r="I692" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23455,7 +23455,7 @@
       <c r="H693" t="inlineStr"/>
       <c r="I693" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23583,7 +23583,7 @@
       <c r="H697" t="inlineStr"/>
       <c r="I697" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23678,7 +23678,7 @@
       <c r="H700" t="inlineStr"/>
       <c r="I700" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23707,7 +23707,7 @@
       <c r="H701" t="inlineStr"/>
       <c r="I701" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23835,7 +23835,7 @@
       <c r="H705" t="inlineStr"/>
       <c r="I705" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23897,7 +23897,7 @@
       <c r="H707" t="inlineStr"/>
       <c r="I707" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23926,7 +23926,7 @@
       <c r="H708" t="inlineStr"/>
       <c r="I708" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23955,7 +23955,7 @@
       <c r="H709" t="inlineStr"/>
       <c r="I709" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -23984,7 +23984,7 @@
       <c r="H710" t="inlineStr"/>
       <c r="I710" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -24046,7 +24046,7 @@
       <c r="H712" t="inlineStr"/>
       <c r="I712" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -24075,7 +24075,7 @@
       <c r="H713" t="inlineStr"/>
       <c r="I713" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -24137,7 +24137,7 @@
       <c r="H715" t="inlineStr"/>
       <c r="I715" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -24166,7 +24166,7 @@
       <c r="H716" t="inlineStr"/>
       <c r="I716" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -24343,7 +24343,7 @@
       <c r="H721" t="inlineStr"/>
       <c r="I721" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -24376,7 +24376,7 @@
       <c r="H722" t="inlineStr"/>
       <c r="I722" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -24409,7 +24409,7 @@
       <c r="H723" t="inlineStr"/>
       <c r="I723" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -24442,7 +24442,7 @@
       <c r="H724" t="inlineStr"/>
       <c r="I724" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>
@@ -24623,7 +24623,7 @@
       <c r="H729" t="inlineStr"/>
       <c r="I729" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Host</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Smazána závada ID 618 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I731"/>
+  <dimension ref="A1:I730"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20444,11 +20444,11 @@
     </row>
     <row r="601">
       <c r="A601" t="n">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>810 329</t>
+          <t>842 011</t>
         </is>
       </c>
       <c r="C601" t="inlineStr">
@@ -20458,14 +20458,10 @@
       </c>
       <c r="D601" t="inlineStr">
         <is>
-          <t>nejde rychloměr</t>
-        </is>
-      </c>
-      <c r="E601" t="inlineStr">
-        <is>
-          <t>výměna</t>
-        </is>
-      </c>
+          <t>udajně zateklo do pultu na 2st.(kontrola)</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr"/>
       <c r="F601" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20481,11 +20477,11 @@
     </row>
     <row r="602">
       <c r="A602" t="n">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>842 011</t>
+          <t>842 021</t>
         </is>
       </c>
       <c r="C602" t="inlineStr">
@@ -20495,10 +20491,14 @@
       </c>
       <c r="D602" t="inlineStr">
         <is>
-          <t>udajně zateklo do pultu na 2st.(kontrola)</t>
-        </is>
-      </c>
-      <c r="E602" t="inlineStr"/>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>vadné čidlo vody v míse</t>
+        </is>
+      </c>
       <c r="F602" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20514,26 +20514,26 @@
     </row>
     <row r="603">
       <c r="A603" t="n">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="B603" t="inlineStr">
         <is>
-          <t>842 021</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C603" t="inlineStr">
         <is>
-          <t>06.10.2023</t>
+          <t>06.09.2023</t>
         </is>
       </c>
       <c r="D603" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>Nejdou dvěře WC</t>
         </is>
       </c>
       <c r="E603" t="inlineStr">
         <is>
-          <t>vadné čidlo vody v míse</t>
+          <t>upadlý drát na přepínači funkce WC (zapnuto,bez dveří, vypnuto). Seřízení zámykání dveří. Frýdek</t>
         </is>
       </c>
       <c r="F603" t="inlineStr">
@@ -20551,11 +20551,11 @@
     </row>
     <row r="604">
       <c r="A604" t="n">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B604" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C604" t="inlineStr">
@@ -20565,12 +20565,12 @@
       </c>
       <c r="D604" t="inlineStr">
         <is>
-          <t>Nejdou dvěře WC</t>
+          <t>údajně nejdou někdy schody u levých dveří strany A</t>
         </is>
       </c>
       <c r="E604" t="inlineStr">
         <is>
-          <t>upadlý drát na přepínači funkce WC (zapnuto,bez dveří, vypnuto). Seřízení zámykání dveří. Frýdek</t>
+          <t>vyčištění od kamínků,odzkoušení-OK</t>
         </is>
       </c>
       <c r="F604" t="inlineStr">
@@ -20588,26 +20588,26 @@
     </row>
     <row r="605">
       <c r="A605" t="n">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C605" t="inlineStr">
         <is>
-          <t>06.09.2023</t>
+          <t>06.08.2023</t>
         </is>
       </c>
       <c r="D605" t="inlineStr">
         <is>
-          <t>údajně nejdou někdy schody u levých dveří strany A</t>
+          <t>zapůjčena z HB</t>
         </is>
       </c>
       <c r="E605" t="inlineStr">
         <is>
-          <t>vyčištění od kamínků,odzkoušení-OK</t>
+          <t>nahrány data IS ( funguje preš radiostanici)</t>
         </is>
       </c>
       <c r="F605" t="inlineStr">
@@ -20625,11 +20625,11 @@
     </row>
     <row r="606">
       <c r="A606" t="n">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B606" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C606" t="inlineStr">
@@ -20639,12 +20639,12 @@
       </c>
       <c r="D606" t="inlineStr">
         <is>
-          <t>zapůjčena z HB</t>
+          <t>Opět problémy se startováním</t>
         </is>
       </c>
       <c r="E606" t="inlineStr">
         <is>
-          <t>nahrány data IS ( funguje preš radiostanici)</t>
+          <t>(asi už vadný capos kondy)říkali veselani jak tu byli</t>
         </is>
       </c>
       <c r="F606" t="inlineStr">
@@ -20662,7 +20662,7 @@
     </row>
     <row r="607">
       <c r="A607" t="n">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B607" t="inlineStr">
         <is>
@@ -20676,12 +20676,12 @@
       </c>
       <c r="D607" t="inlineStr">
         <is>
-          <t>Opět problémy se startováním</t>
+          <t>oprava hlasitosti na stanovišti A</t>
         </is>
       </c>
       <c r="E607" t="inlineStr">
         <is>
-          <t>(asi už vadný capos kondy)říkali veselani jak tu byli</t>
+          <t>přechod na kontaktech u reproduktoru v pultě</t>
         </is>
       </c>
       <c r="F607" t="inlineStr">
@@ -20699,11 +20699,11 @@
     </row>
     <row r="608">
       <c r="A608" t="n">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B608" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C608" t="inlineStr">
@@ -20713,12 +20713,12 @@
       </c>
       <c r="D608" t="inlineStr">
         <is>
-          <t>oprava hlasitosti na stanovišti A</t>
+          <t>výměna ARR na B</t>
         </is>
       </c>
       <c r="E608" t="inlineStr">
         <is>
-          <t>přechod na kontaktech u reproduktoru v pultě</t>
+          <t>vadná linka CAN</t>
         </is>
       </c>
       <c r="F608" t="inlineStr">
@@ -20736,26 +20736,26 @@
     </row>
     <row r="609">
       <c r="A609" t="n">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>842 015</t>
         </is>
       </c>
       <c r="C609" t="inlineStr">
         <is>
-          <t>06.08.2023</t>
+          <t>06.07.2023</t>
         </is>
       </c>
       <c r="D609" t="inlineStr">
         <is>
-          <t>výměna ARR na B</t>
+          <t>někdy nejde brzda PB</t>
         </is>
       </c>
       <c r="E609" t="inlineStr">
         <is>
-          <t>vadná linka CAN</t>
+          <t>výměna karty DS a OUT z 842 025</t>
         </is>
       </c>
       <c r="F609" t="inlineStr">
@@ -20773,11 +20773,11 @@
     </row>
     <row r="610">
       <c r="A610" t="n">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B610" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C610" t="inlineStr">
@@ -20787,14 +20787,10 @@
       </c>
       <c r="D610" t="inlineStr">
         <is>
-          <t>někdy nejde brzda PB</t>
-        </is>
-      </c>
-      <c r="E610" t="inlineStr">
-        <is>
-          <t>výměna karty DS a OUT z 842 025</t>
-        </is>
-      </c>
+          <t>dosazeny karty z 842 015 (DS a OUT)</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr"/>
       <c r="F610" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20810,11 +20806,11 @@
     </row>
     <row r="611">
       <c r="A611" t="n">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B611" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C611" t="inlineStr">
@@ -20824,10 +20820,14 @@
       </c>
       <c r="D611" t="inlineStr">
         <is>
-          <t>dosazeny karty z 842 015 (DS a OUT)</t>
-        </is>
-      </c>
-      <c r="E611" t="inlineStr"/>
+          <t>dosazen asi 5 dobíječ na B funkční</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>ve skladu nefunkční jenom (má řešit asi Mlíčko)</t>
+        </is>
+      </c>
       <c r="F611" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20843,28 +20843,24 @@
     </row>
     <row r="612">
       <c r="A612" t="n">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="B612" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 076</t>
         </is>
       </c>
       <c r="C612" t="inlineStr">
         <is>
-          <t>06.07.2023</t>
+          <t>06.06.2023</t>
         </is>
       </c>
       <c r="D612" t="inlineStr">
         <is>
-          <t>dosazen asi 5 dobíječ na B funkční</t>
-        </is>
-      </c>
-      <c r="E612" t="inlineStr">
-        <is>
-          <t>ve skladu nefunkční jenom (má řešit asi Mlíčko)</t>
-        </is>
-      </c>
+          <t>NEHODA V HOLEŠOVĚ</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr"/>
       <c r="F612" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20880,21 +20876,21 @@
     </row>
     <row r="613">
       <c r="A613" t="n">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>814 076</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C613" t="inlineStr">
         <is>
-          <t>06.06.2023</t>
+          <t>06.05.2023</t>
         </is>
       </c>
       <c r="D613" t="inlineStr">
         <is>
-          <t>NEHODA V HOLEŠOVĚ</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E613" t="inlineStr"/>
@@ -20913,21 +20909,17 @@
     </row>
     <row r="614">
       <c r="A614" t="n">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="B614" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C614" t="inlineStr">
-        <is>
-          <t>06.05.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr"/>
       <c r="D614" t="inlineStr">
         <is>
-          <t>MM</t>
+          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
         </is>
       </c>
       <c r="E614" t="inlineStr"/>
@@ -20946,7 +20938,7 @@
     </row>
     <row r="615">
       <c r="A615" t="n">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="B615" t="inlineStr">
         <is>
@@ -20956,7 +20948,7 @@
       <c r="C615" t="inlineStr"/>
       <c r="D615" t="inlineStr">
         <is>
-          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
+          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
         </is>
       </c>
       <c r="E615" t="inlineStr"/>
@@ -20975,7 +20967,7 @@
     </row>
     <row r="616">
       <c r="A616" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B616" t="inlineStr">
         <is>
@@ -20985,7 +20977,7 @@
       <c r="C616" t="inlineStr"/>
       <c r="D616" t="inlineStr">
         <is>
-          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
+          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
         </is>
       </c>
       <c r="E616" t="inlineStr"/>
@@ -21004,20 +20996,24 @@
     </row>
     <row r="617">
       <c r="A617" t="n">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C617" t="inlineStr"/>
       <c r="D617" t="inlineStr">
         <is>
-          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
-        </is>
-      </c>
-      <c r="E617" t="inlineStr"/>
+          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>vyměnili dobíječ stacionární (Veselí)</t>
+        </is>
+      </c>
       <c r="F617" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21033,22 +21029,22 @@
     </row>
     <row r="618">
       <c r="A618" t="n">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B618" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C618" t="inlineStr"/>
       <c r="D618" t="inlineStr">
         <is>
-          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
         </is>
       </c>
       <c r="E618" t="inlineStr">
         <is>
-          <t>vyměnili dobíječ stacionární (Veselí)</t>
+          <t>jela ven</t>
         </is>
       </c>
       <c r="F618" t="inlineStr">
@@ -21066,24 +21062,20 @@
     </row>
     <row r="619">
       <c r="A619" t="n">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C619" t="inlineStr"/>
       <c r="D619" t="inlineStr">
         <is>
-          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
-        </is>
-      </c>
-      <c r="E619" t="inlineStr">
-        <is>
-          <t>jela ven</t>
-        </is>
-      </c>
+          <t>seřízení kamer přes program v notasu(obraz)</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr"/>
       <c r="F619" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21099,20 +21091,24 @@
     </row>
     <row r="620">
       <c r="A620" t="n">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C620" t="inlineStr"/>
       <c r="D620" t="inlineStr">
         <is>
-          <t>seřízení kamer přes program v notasu(obraz)</t>
-        </is>
-      </c>
-      <c r="E620" t="inlineStr"/>
+          <t>po startu někdy nenabíjí "B"</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+        </is>
+      </c>
       <c r="F620" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21128,22 +21124,22 @@
     </row>
     <row r="621">
       <c r="A621" t="n">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C621" t="inlineStr"/>
       <c r="D621" t="inlineStr">
         <is>
-          <t>po startu někdy nenabíjí "B"</t>
+          <t>2. motor korekce vody  vystup</t>
         </is>
       </c>
       <c r="E621" t="inlineStr">
         <is>
-          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
         </is>
       </c>
       <c r="F621" t="inlineStr">
@@ -21161,24 +21157,24 @@
     </row>
     <row r="622">
       <c r="A622" t="n">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>842 035</t>
-        </is>
-      </c>
-      <c r="C622" t="inlineStr"/>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>04.12.2023</t>
+        </is>
+      </c>
       <c r="D622" t="inlineStr">
         <is>
-          <t>2. motor korekce vody  vystup</t>
-        </is>
-      </c>
-      <c r="E622" t="inlineStr">
-        <is>
-          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
-        </is>
-      </c>
+          <t>Výměna motoru A</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr"/>
       <c r="F622" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21194,21 +21190,17 @@
     </row>
     <row r="623">
       <c r="A623" t="n">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B623" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C623" t="inlineStr">
-        <is>
-          <t>04.12.2023</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr"/>
       <c r="D623" t="inlineStr">
         <is>
-          <t>Výměna motoru A</t>
+          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
         </is>
       </c>
       <c r="E623" t="inlineStr"/>
@@ -21227,17 +21219,17 @@
     </row>
     <row r="624">
       <c r="A624" t="n">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C624" t="inlineStr"/>
       <c r="D624" t="inlineStr">
         <is>
-          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
+          <t>dosazena nahadni Mirelka + NO z 844 013</t>
         </is>
       </c>
       <c r="E624" t="inlineStr"/>
@@ -21256,17 +21248,17 @@
     </row>
     <row r="625">
       <c r="A625" t="n">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B625" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 062</t>
         </is>
       </c>
       <c r="C625" t="inlineStr"/>
       <c r="D625" t="inlineStr">
         <is>
-          <t>dosazena nahadni Mirelka + NO z 844 013</t>
+          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
         </is>
       </c>
       <c r="E625" t="inlineStr"/>
@@ -21285,17 +21277,21 @@
     </row>
     <row r="626">
       <c r="A626" t="n">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>814 062</t>
-        </is>
-      </c>
-      <c r="C626" t="inlineStr"/>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>03.03.2023</t>
+        </is>
+      </c>
       <c r="D626" t="inlineStr">
         <is>
-          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E626" t="inlineStr"/>
@@ -21314,11 +21310,11 @@
     </row>
     <row r="627">
       <c r="A627" t="n">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C627" t="inlineStr">
@@ -21328,7 +21324,7 @@
       </c>
       <c r="D627" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
+          <t>Dosazení ŘJ kamer</t>
         </is>
       </c>
       <c r="E627" t="inlineStr"/>
@@ -21347,24 +21343,24 @@
     </row>
     <row r="628">
       <c r="A628" t="n">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>844 013</t>
-        </is>
-      </c>
-      <c r="C628" t="inlineStr">
-        <is>
-          <t>03.03.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr"/>
       <c r="D628" t="inlineStr">
         <is>
-          <t>Dosazení ŘJ kamer</t>
-        </is>
-      </c>
-      <c r="E628" t="inlineStr"/>
+          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>hlášeno p. Škodovi</t>
+        </is>
+      </c>
       <c r="F628" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21380,24 +21376,20 @@
     </row>
     <row r="629">
       <c r="A629" t="n">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C629" t="inlineStr"/>
       <c r="D629" t="inlineStr">
         <is>
-          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
-        </is>
-      </c>
-      <c r="E629" t="inlineStr">
-        <is>
-          <t>hlášeno p. Škodovi</t>
-        </is>
-      </c>
+          <t>ŘJ kamer dosazena z 013</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr"/>
       <c r="F629" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21413,17 +21405,21 @@
     </row>
     <row r="630">
       <c r="A630" t="n">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B630" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C630" t="inlineStr"/>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>02.09.2023</t>
+        </is>
+      </c>
       <c r="D630" t="inlineStr">
         <is>
-          <t>ŘJ kamer dosazena z 013</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E630" t="inlineStr"/>
@@ -21442,21 +21438,21 @@
     </row>
     <row r="631">
       <c r="A631" t="n">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 072</t>
         </is>
       </c>
       <c r="C631" t="inlineStr">
         <is>
-          <t>02.09.2023</t>
+          <t>02.03.2023</t>
         </is>
       </c>
       <c r="D631" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E631" t="inlineStr"/>
@@ -21475,24 +21471,24 @@
     </row>
     <row r="632">
       <c r="A632" t="n">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>814 072</t>
-        </is>
-      </c>
-      <c r="C632" t="inlineStr">
-        <is>
-          <t>02.03.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr"/>
       <c r="D632" t="inlineStr">
         <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E632" t="inlineStr"/>
+          <t>dosazen opraveny MIREL</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+        </is>
+      </c>
       <c r="F632" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21508,22 +21504,22 @@
     </row>
     <row r="633">
       <c r="A633" t="n">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C633" t="inlineStr"/>
       <c r="D633" t="inlineStr">
         <is>
-          <t>dosazen opraveny MIREL</t>
+          <t>Odpojen trojcestný ventil na A i B</t>
         </is>
       </c>
       <c r="E633" t="inlineStr">
         <is>
-          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+          <t>Zapojeny zpět 24.2.2023</t>
         </is>
       </c>
       <c r="F633" t="inlineStr">
@@ -21541,24 +21537,20 @@
     </row>
     <row r="634">
       <c r="A634" t="n">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C634" t="inlineStr"/>
       <c r="D634" t="inlineStr">
         <is>
-          <t>Odpojen trojcestný ventil na A i B</t>
-        </is>
-      </c>
-      <c r="E634" t="inlineStr">
-        <is>
-          <t>Zapojeny zpět 24.2.2023</t>
-        </is>
-      </c>
+          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr"/>
       <c r="F634" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21574,17 +21566,21 @@
     </row>
     <row r="635">
       <c r="A635" t="n">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B635" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C635" t="inlineStr"/>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>01.10.2023</t>
+        </is>
+      </c>
       <c r="D635" t="inlineStr">
         <is>
-          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E635" t="inlineStr"/>
@@ -21603,21 +21599,17 @@
     </row>
     <row r="636">
       <c r="A636" t="n">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C636" t="inlineStr">
-        <is>
-          <t>01.10.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr"/>
       <c r="D636" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
         </is>
       </c>
       <c r="E636" t="inlineStr"/>
@@ -21636,17 +21628,17 @@
     </row>
     <row r="637">
       <c r="A637" t="n">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C637" t="inlineStr"/>
       <c r="D637" t="inlineStr">
         <is>
-          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
+          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
         </is>
       </c>
       <c r="E637" t="inlineStr"/>
@@ -21665,7 +21657,7 @@
     </row>
     <row r="638">
       <c r="A638" t="n">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B638" t="inlineStr">
         <is>
@@ -21675,7 +21667,7 @@
       <c r="C638" t="inlineStr"/>
       <c r="D638" t="inlineStr">
         <is>
-          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
+          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
         </is>
       </c>
       <c r="E638" t="inlineStr"/>
@@ -21694,20 +21686,24 @@
     </row>
     <row r="639">
       <c r="A639" t="n">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C639" t="inlineStr"/>
       <c r="D639" t="inlineStr">
         <is>
-          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
-        </is>
-      </c>
-      <c r="E639" t="inlineStr"/>
+          <t>Přišel opravený Mirel ve skladu</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>dosazen na 29.12.2022</t>
+        </is>
+      </c>
       <c r="F639" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21723,22 +21719,26 @@
     </row>
     <row r="640">
       <c r="A640" t="n">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C640" t="inlineStr"/>
+          <t>844 014</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>12.06.2022</t>
+        </is>
+      </c>
       <c r="D640" t="inlineStr">
         <is>
-          <t>Přišel opravený Mirel ve skladu</t>
+          <t>rychloměr do opravy hazí !!</t>
         </is>
       </c>
       <c r="E640" t="inlineStr">
         <is>
-          <t>dosazen na 29.12.2022</t>
+          <t>zapujcen z 844 028 z veselí</t>
         </is>
       </c>
       <c r="F640" t="inlineStr">
@@ -21756,11 +21756,11 @@
     </row>
     <row r="641">
       <c r="A641" t="n">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C641" t="inlineStr">
@@ -21770,14 +21770,10 @@
       </c>
       <c r="D641" t="inlineStr">
         <is>
-          <t>rychloměr do opravy hazí !!</t>
-        </is>
-      </c>
-      <c r="E641" t="inlineStr">
-        <is>
-          <t>zapujcen z 844 028 z veselí</t>
-        </is>
-      </c>
+          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr"/>
       <c r="F641" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21793,24 +21789,28 @@
     </row>
     <row r="642">
       <c r="A642" t="n">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C642" t="inlineStr">
         <is>
-          <t>12.06.2022</t>
+          <t>12.03.2022</t>
         </is>
       </c>
       <c r="D642" t="inlineStr">
         <is>
-          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
-        </is>
-      </c>
-      <c r="E642" t="inlineStr"/>
+          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>bude řešit Škoda</t>
+        </is>
+      </c>
       <c r="F642" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21826,26 +21826,22 @@
     </row>
     <row r="643">
       <c r="A643" t="n">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B643" t="inlineStr">
         <is>
           <t>844 003</t>
         </is>
       </c>
-      <c r="C643" t="inlineStr">
-        <is>
-          <t>12.03.2022</t>
-        </is>
-      </c>
+      <c r="C643" t="inlineStr"/>
       <c r="D643" t="inlineStr">
         <is>
-          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+          <t>na A strane asi vadna expanzní nadrz topení ?</t>
         </is>
       </c>
       <c r="E643" t="inlineStr">
         <is>
-          <t>bude řešit Škoda</t>
+          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
         </is>
       </c>
       <c r="F643" t="inlineStr">
@@ -21863,22 +21859,22 @@
     </row>
     <row r="644">
       <c r="A644" t="n">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C644" t="inlineStr"/>
       <c r="D644" t="inlineStr">
         <is>
-          <t>na A strane asi vadna expanzní nadrz topení ?</t>
+          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
         </is>
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
+          <t>nová obrazovka hazela vykricnik porad</t>
         </is>
       </c>
       <c r="F644" t="inlineStr">
@@ -21896,24 +21892,24 @@
     </row>
     <row r="645">
       <c r="A645" t="n">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C645" t="inlineStr"/>
+          <t>842 010</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>11.06.2022</t>
+        </is>
+      </c>
       <c r="D645" t="inlineStr">
         <is>
-          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
-        </is>
-      </c>
-      <c r="E645" t="inlineStr">
-        <is>
-          <t>nová obrazovka hazela vykricnik porad</t>
-        </is>
-      </c>
+          <t>Přehození karty TBA v DPV na 842 036</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr"/>
       <c r="F645" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21929,11 +21925,11 @@
     </row>
     <row r="646">
       <c r="A646" t="n">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>842 010</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
@@ -21943,7 +21939,7 @@
       </c>
       <c r="D646" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 036</t>
+          <t>Přehození karty TBA v DPV na 842 010</t>
         </is>
       </c>
       <c r="E646" t="inlineStr"/>
@@ -21962,11 +21958,11 @@
     </row>
     <row r="647">
       <c r="A647" t="n">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C647" t="inlineStr">
@@ -21976,10 +21972,14 @@
       </c>
       <c r="D647" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 010</t>
-        </is>
-      </c>
-      <c r="E647" t="inlineStr"/>
+          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>mirel byl špatný po opravě</t>
+        </is>
+      </c>
       <c r="F647" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21995,26 +21995,26 @@
     </row>
     <row r="648">
       <c r="A648" t="n">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C648" t="inlineStr">
         <is>
-          <t>11.06.2022</t>
+          <t>11.05.2022</t>
         </is>
       </c>
       <c r="D648" t="inlineStr">
         <is>
-          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
         </is>
       </c>
       <c r="E648" t="inlineStr">
         <is>
-          <t>mirel byl špatný po opravě</t>
+          <t>25.11. opraveno</t>
         </is>
       </c>
       <c r="F648" t="inlineStr">
@@ -22032,11 +22032,11 @@
     </row>
     <row r="649">
       <c r="A649" t="n">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C649" t="inlineStr">
@@ -22046,14 +22046,10 @@
       </c>
       <c r="D649" t="inlineStr">
         <is>
-          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
-        </is>
-      </c>
-      <c r="E649" t="inlineStr">
-        <is>
-          <t>25.11. opraveno</t>
-        </is>
-      </c>
+          <t>VESELÍ R3 (odjela)</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr"/>
       <c r="F649" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22069,24 +22065,24 @@
     </row>
     <row r="650">
       <c r="A650" t="n">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>844 020</t>
-        </is>
-      </c>
-      <c r="C650" t="inlineStr">
-        <is>
-          <t>11.05.2022</t>
-        </is>
-      </c>
+          <t>814 190</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr"/>
       <c r="D650" t="inlineStr">
         <is>
-          <t>VESELÍ R3 (odjela)</t>
-        </is>
-      </c>
-      <c r="E650" t="inlineStr"/>
+          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>hlášeno p.Škodovi</t>
+        </is>
+      </c>
       <c r="F650" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22102,22 +22098,22 @@
     </row>
     <row r="651">
       <c r="A651" t="n">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>814 190</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C651" t="inlineStr"/>
       <c r="D651" t="inlineStr">
         <is>
-          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
         </is>
       </c>
       <c r="E651" t="inlineStr">
         <is>
-          <t>hlášeno p.Škodovi</t>
+          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
         </is>
       </c>
       <c r="F651" t="inlineStr">
@@ -22135,24 +22131,20 @@
     </row>
     <row r="652">
       <c r="A652" t="n">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C652" t="inlineStr"/>
       <c r="D652" t="inlineStr">
         <is>
-          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
-        </is>
-      </c>
-      <c r="E652" t="inlineStr">
-        <is>
-          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
-        </is>
-      </c>
+          <t>dosazen předzesilovač linky</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr"/>
       <c r="F652" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22168,20 +22160,28 @@
     </row>
     <row r="653">
       <c r="A653" t="n">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B653" t="inlineStr">
         <is>
           <t>814 073</t>
         </is>
       </c>
-      <c r="C653" t="inlineStr"/>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>09.07.2022</t>
+        </is>
+      </c>
       <c r="D653" t="inlineStr">
         <is>
-          <t>dosazen předzesilovač linky</t>
-        </is>
-      </c>
-      <c r="E653" t="inlineStr"/>
+          <t>chybějící díl</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>předzasilovač linky - objednán nový</t>
+        </is>
+      </c>
       <c r="F653" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22197,26 +22197,26 @@
     </row>
     <row r="654">
       <c r="A654" t="n">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 003</t>
         </is>
       </c>
       <c r="C654" t="inlineStr">
         <is>
-          <t>09.07.2022</t>
+          <t>09.03.2022</t>
         </is>
       </c>
       <c r="D654" t="inlineStr">
         <is>
-          <t>chybějící díl</t>
+          <t>dosazen díl</t>
         </is>
       </c>
       <c r="E654" t="inlineStr">
         <is>
-          <t>předzasilovač linky - objednán nový</t>
+          <t>dosazen předzasilovač linky A23</t>
         </is>
       </c>
       <c r="F654" t="inlineStr">
@@ -22234,26 +22234,22 @@
     </row>
     <row r="655">
       <c r="A655" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C655" t="inlineStr">
-        <is>
-          <t>09.03.2022</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr"/>
       <c r="D655" t="inlineStr">
         <is>
-          <t>dosazen díl</t>
+          <t>oprava dveří na B pravé po směru jízdy</t>
         </is>
       </c>
       <c r="E655" t="inlineStr">
         <is>
-          <t>dosazen předzasilovač linky A23</t>
+          <t>vadný motorek</t>
         </is>
       </c>
       <c r="F655" t="inlineStr">
@@ -22271,22 +22267,22 @@
     </row>
     <row r="656">
       <c r="A656" t="n">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C656" t="inlineStr"/>
       <c r="D656" t="inlineStr">
         <is>
-          <t>oprava dveří na B pravé po směru jízdy</t>
+          <t>vadné čidlo množství písku M5</t>
         </is>
       </c>
       <c r="E656" t="inlineStr">
         <is>
-          <t>vadný motorek</t>
+          <t>2. osa pravo po smeru jizdy z B</t>
         </is>
       </c>
       <c r="F656" t="inlineStr">
@@ -22304,22 +22300,22 @@
     </row>
     <row r="657">
       <c r="A657" t="n">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C657" t="inlineStr"/>
       <c r="D657" t="inlineStr">
         <is>
-          <t>vadné čidlo množství písku M5</t>
+          <t>rychloměr dán do skladu na opravu</t>
         </is>
       </c>
       <c r="E657" t="inlineStr">
         <is>
-          <t>2. osa pravo po smeru jizdy z B</t>
+          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
         </is>
       </c>
       <c r="F657" t="inlineStr">
@@ -22337,22 +22333,22 @@
     </row>
     <row r="658">
       <c r="A658" t="n">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C658" t="inlineStr"/>
       <c r="D658" t="inlineStr">
         <is>
-          <t>rychloměr dán do skladu na opravu</t>
+          <t>rychloměr nekomunikuje</t>
         </is>
       </c>
       <c r="E658" t="inlineStr">
         <is>
-          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
+          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
         </is>
       </c>
       <c r="F658" t="inlineStr">
@@ -22370,22 +22366,26 @@
     </row>
     <row r="659">
       <c r="A659" t="n">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B659" t="inlineStr">
         <is>
-          <t>844 022</t>
-        </is>
-      </c>
-      <c r="C659" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>10.08.2021</t>
+        </is>
+      </c>
       <c r="D659" t="inlineStr">
         <is>
-          <t>rychloměr nekomunikuje</t>
+          <t>dosazeny díly</t>
         </is>
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
+          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
         </is>
       </c>
       <c r="F659" t="inlineStr">
@@ -22403,18 +22403,14 @@
     </row>
     <row r="660">
       <c r="A660" t="n">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B660" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C660" t="inlineStr">
-        <is>
-          <t>10.08.2021</t>
-        </is>
-      </c>
+      <c r="C660" t="inlineStr"/>
       <c r="D660" t="inlineStr">
         <is>
           <t>dosazeny díly</t>
@@ -22422,7 +22418,7 @@
       </c>
       <c r="E660" t="inlineStr">
         <is>
-          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
+          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
         </is>
       </c>
       <c r="F660" t="inlineStr">
@@ -22440,22 +22436,26 @@
     </row>
     <row r="661">
       <c r="A661" t="n">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B661" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C661" t="inlineStr"/>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>09.06.2021</t>
+        </is>
+      </c>
       <c r="D661" t="inlineStr">
         <is>
-          <t>dosazeny díly</t>
+          <t>Chybějící díly z důvodu použití na jinou lok.</t>
         </is>
       </c>
       <c r="E661" t="inlineStr">
         <is>
-          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
+          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
         </is>
       </c>
       <c r="F661" t="inlineStr">
@@ -22473,28 +22473,16 @@
     </row>
     <row r="662">
       <c r="A662" t="n">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B662" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C662" t="inlineStr">
-        <is>
-          <t>09.06.2021</t>
-        </is>
-      </c>
-      <c r="D662" t="inlineStr">
-        <is>
-          <t>Chybějící díly z důvodu použití na jinou lok.</t>
-        </is>
-      </c>
-      <c r="E662" t="inlineStr">
-        <is>
-          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
-        </is>
-      </c>
+          <t>842 015</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr"/>
+      <c r="D662" t="inlineStr"/>
+      <c r="E662" t="inlineStr"/>
       <c r="F662" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22510,15 +22498,19 @@
     </row>
     <row r="663">
       <c r="A663" t="n">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C663" t="inlineStr"/>
-      <c r="D663" t="inlineStr"/>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>výměna obrazovky Lokel na 914</t>
+        </is>
+      </c>
       <c r="E663" t="inlineStr"/>
       <c r="F663" t="inlineStr">
         <is>
@@ -22535,17 +22527,17 @@
     </row>
     <row r="664">
       <c r="A664" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C664" t="inlineStr"/>
       <c r="D664" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E664" t="inlineStr"/>
@@ -22564,17 +22556,17 @@
     </row>
     <row r="665">
       <c r="A665" t="n">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C665" t="inlineStr"/>
       <c r="D665" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E665" t="inlineStr"/>
@@ -22593,7 +22585,7 @@
     </row>
     <row r="666">
       <c r="A666" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B666" t="inlineStr">
         <is>
@@ -22603,10 +22595,14 @@
       <c r="C666" t="inlineStr"/>
       <c r="D666" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E666" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F666" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22622,24 +22618,20 @@
     </row>
     <row r="667">
       <c r="A667" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C667" t="inlineStr"/>
       <c r="D667" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E667" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr"/>
       <c r="F667" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22655,7 +22647,7 @@
     </row>
     <row r="668">
       <c r="A668" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B668" t="inlineStr">
         <is>
@@ -22665,7 +22657,7 @@
       <c r="C668" t="inlineStr"/>
       <c r="D668" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E668" t="inlineStr"/>
@@ -22684,17 +22676,17 @@
     </row>
     <row r="669">
       <c r="A669" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C669" t="inlineStr"/>
       <c r="D669" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E669" t="inlineStr"/>
@@ -22713,20 +22705,24 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C670" t="inlineStr"/>
       <c r="D670" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E670" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F670" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22742,7 +22738,7 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
@@ -22752,12 +22748,12 @@
       <c r="C671" t="inlineStr"/>
       <c r="D671" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E671" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F671" t="inlineStr">
@@ -22775,24 +22771,24 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C672" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D672" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E672" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr"/>
       <c r="F672" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22808,7 +22804,7 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
@@ -22817,12 +22813,12 @@
       </c>
       <c r="C673" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D673" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E673" t="inlineStr"/>
@@ -22841,7 +22837,7 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
@@ -22855,7 +22851,7 @@
       </c>
       <c r="D674" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E674" t="inlineStr"/>
@@ -22874,7 +22870,7 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
@@ -22888,10 +22884,14 @@
       </c>
       <c r="D675" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E675" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F675" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22907,7 +22907,7 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
@@ -22921,12 +22921,12 @@
       </c>
       <c r="D676" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E676" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F676" t="inlineStr">
@@ -22944,7 +22944,7 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
@@ -22958,14 +22958,10 @@
       </c>
       <c r="D677" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E677" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr"/>
       <c r="F677" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22981,24 +22977,24 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C678" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr"/>
       <c r="D678" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E678" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F678" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23014,24 +23010,20 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C679" t="inlineStr"/>
       <c r="D679" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E679" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr"/>
       <c r="F679" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23047,17 +23039,17 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C680" t="inlineStr"/>
       <c r="D680" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E680" t="inlineStr"/>
@@ -23076,7 +23068,7 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
@@ -23086,10 +23078,14 @@
       <c r="C681" t="inlineStr"/>
       <c r="D681" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E681" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F681" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23105,24 +23101,20 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C682" t="inlineStr"/>
       <c r="D682" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E682" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr"/>
       <c r="F682" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23138,7 +23130,7 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
@@ -23148,7 +23140,7 @@
       <c r="C683" t="inlineStr"/>
       <c r="D683" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E683" t="inlineStr"/>
@@ -23167,20 +23159,24 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C684" t="inlineStr"/>
       <c r="D684" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
-        </is>
-      </c>
-      <c r="E684" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F684" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23196,7 +23192,7 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
@@ -23206,14 +23202,10 @@
       <c r="C685" t="inlineStr"/>
       <c r="D685" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E685" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr"/>
       <c r="F685" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23229,7 +23221,7 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
@@ -23239,10 +23231,14 @@
       <c r="C686" t="inlineStr"/>
       <c r="D686" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E686" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F686" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23258,7 +23254,7 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
@@ -23268,14 +23264,10 @@
       <c r="C687" t="inlineStr"/>
       <c r="D687" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E687" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr"/>
       <c r="F687" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23291,7 +23283,7 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
@@ -23301,7 +23293,7 @@
       <c r="C688" t="inlineStr"/>
       <c r="D688" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E688" t="inlineStr"/>
@@ -23320,7 +23312,7 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
@@ -23330,10 +23322,14 @@
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E689" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F689" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23349,7 +23345,7 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
@@ -23359,12 +23355,12 @@
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E690" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F690" t="inlineStr">
@@ -23382,7 +23378,7 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
@@ -23392,12 +23388,12 @@
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E691" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F691" t="inlineStr">
@@ -23415,24 +23411,20 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E692" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr"/>
       <c r="F692" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23448,7 +23440,7 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
@@ -23458,10 +23450,14 @@
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E693" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F693" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23477,7 +23473,7 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
@@ -23487,12 +23483,12 @@
       <c r="C694" t="inlineStr"/>
       <c r="D694" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E694" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F694" t="inlineStr">
@@ -23510,7 +23506,7 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
@@ -23520,14 +23516,10 @@
       <c r="C695" t="inlineStr"/>
       <c r="D695" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E695" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr"/>
       <c r="F695" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23543,17 +23535,17 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C696" t="inlineStr"/>
       <c r="D696" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E696" t="inlineStr"/>
@@ -23572,7 +23564,7 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
@@ -23582,10 +23574,14 @@
       <c r="C697" t="inlineStr"/>
       <c r="D697" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E697" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F697" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23601,22 +23597,22 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C698" t="inlineStr"/>
       <c r="D698" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E698" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F698" t="inlineStr">
@@ -23634,7 +23630,7 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
@@ -23644,12 +23640,12 @@
       <c r="C699" t="inlineStr"/>
       <c r="D699" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E699" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F699" t="inlineStr">
@@ -23667,24 +23663,20 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C700" t="inlineStr"/>
       <c r="D700" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E700" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr"/>
       <c r="F700" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23700,23 +23692,27 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C701" t="inlineStr"/>
       <c r="D701" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E701" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F701" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G701" t="inlineStr"/>
@@ -23729,27 +23725,23 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E702" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr"/>
       <c r="F702" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G702" t="inlineStr"/>
@@ -23762,7 +23754,7 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
@@ -23772,7 +23764,7 @@
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E703" t="inlineStr"/>
@@ -23791,7 +23783,7 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
@@ -23801,7 +23793,7 @@
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E704" t="inlineStr"/>
@@ -23820,7 +23812,7 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
@@ -23830,7 +23822,7 @@
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E705" t="inlineStr"/>
@@ -23849,7 +23841,7 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
@@ -23859,10 +23851,14 @@
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E706" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F706" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23878,24 +23874,20 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E707" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr"/>
       <c r="F707" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23911,7 +23903,7 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
@@ -23921,7 +23913,7 @@
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E708" t="inlineStr"/>
@@ -23940,20 +23932,24 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C709" t="inlineStr"/>
       <c r="D709" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E709" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F709" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23969,27 +23965,23 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C710" t="inlineStr"/>
       <c r="D710" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E710" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr"/>
       <c r="F710" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G710" t="inlineStr"/>
@@ -24002,7 +23994,7 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
@@ -24012,7 +24004,7 @@
       <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E711" t="inlineStr"/>
@@ -24031,23 +24023,27 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C712" t="inlineStr"/>
       <c r="D712" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E712" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F712" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G712" t="inlineStr"/>
@@ -24060,27 +24056,31 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C713" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D713" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E713" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F713" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G713" t="inlineStr"/>
@@ -24093,11 +24093,11 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C714" t="inlineStr">
@@ -24107,12 +24107,12 @@
       </c>
       <c r="D714" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E714" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F714" t="inlineStr">
@@ -24130,26 +24130,26 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D715" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E715" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F715" t="inlineStr">
@@ -24167,31 +24167,27 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C716" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D716" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E716" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr"/>
       <c r="F716" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G716" t="inlineStr"/>
@@ -24204,27 +24200,27 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C717" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D717" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E717" t="inlineStr"/>
       <c r="F717" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G717" t="inlineStr"/>
@@ -24237,27 +24233,27 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C718" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D718" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E718" t="inlineStr"/>
       <c r="F718" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G718" t="inlineStr"/>
@@ -24270,27 +24266,27 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C719" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D719" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E719" t="inlineStr"/>
       <c r="F719" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G719" t="inlineStr"/>
@@ -24303,24 +24299,28 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C720" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D720" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E720" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F720" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -24336,11 +24336,11 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C721" t="inlineStr">
@@ -24350,12 +24350,12 @@
       </c>
       <c r="D721" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E721" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F721" t="inlineStr">
@@ -24373,11 +24373,11 @@
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C722" t="inlineStr">
@@ -24387,7 +24387,7 @@
       </c>
       <c r="D722" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E722" t="inlineStr">
@@ -24410,31 +24410,31 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C723" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D723" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E723" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F723" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G723" t="inlineStr"/>
@@ -24447,31 +24447,27 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C724" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D724" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E724" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr"/>
       <c r="F724" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G724" t="inlineStr"/>
@@ -24484,27 +24480,31 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C725" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D725" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E725" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F725" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G725" t="inlineStr"/>
@@ -24517,26 +24517,22 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C726" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr"/>
       <c r="D726" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E726" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F726" t="inlineStr">
@@ -24554,30 +24550,38 @@
     </row>
     <row r="727">
       <c r="A727" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B727" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C727" t="inlineStr"/>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D727" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E727" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F727" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G727" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G727" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H727" t="inlineStr"/>
       <c r="I727" t="inlineStr">
         <is>
@@ -24587,38 +24591,34 @@
     </row>
     <row r="728">
       <c r="A728" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D728" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E728" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F728" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G728" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G728" t="inlineStr"/>
       <c r="H728" t="inlineStr"/>
       <c r="I728" t="inlineStr">
         <is>
@@ -24628,26 +24628,26 @@
     </row>
     <row r="729">
       <c r="A729" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C729" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D729" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E729" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F729" t="inlineStr">
@@ -24655,7 +24655,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G729" t="inlineStr"/>
+      <c r="G729" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H729" t="inlineStr"/>
       <c r="I729" t="inlineStr">
         <is>
@@ -24665,11 +24669,11 @@
     </row>
     <row r="730">
       <c r="A730" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
@@ -24679,67 +24683,26 @@
       </c>
       <c r="D730" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E730" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F730" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G730" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H730" t="inlineStr"/>
       <c r="I730" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="731">
-      <c r="A731" t="n">
-        <v>763</v>
-      </c>
-      <c r="B731" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C731" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D731" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E731" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F731" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G731" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H731" t="inlineStr"/>
-      <c r="I731" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 586 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I727"/>
+  <dimension ref="A1:I726"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19314,18 +19314,22 @@
     </row>
     <row r="567">
       <c r="A567" t="n">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>810 329</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C567" t="inlineStr"/>
-      <c r="D567" t="inlineStr"/>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>levé schody  na A nejdou</t>
+        </is>
+      </c>
       <c r="E567" t="inlineStr">
         <is>
-          <t>oprava + vyčištění mincovníku, kontrola IS - OK</t>
+          <t>nečistoy kolem motoru+řemen</t>
         </is>
       </c>
       <c r="F567" t="inlineStr">
@@ -19343,22 +19347,22 @@
     </row>
     <row r="568">
       <c r="A568" t="n">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C568" t="inlineStr"/>
       <c r="D568" t="inlineStr">
         <is>
-          <t>levé schody  na A nejdou</t>
+          <t>údajne obrazovka IS v sekci B nad průchozími dveřmi ( směrem od WC) po tmě</t>
         </is>
       </c>
       <c r="E568" t="inlineStr">
         <is>
-          <t>nečistoy kolem motoru+řemen</t>
+          <t>neprojevilo se,kontrola konektorů,poklep obrazovka.Vše OK</t>
         </is>
       </c>
       <c r="F568" t="inlineStr">
@@ -19376,7 +19380,7 @@
     </row>
     <row r="569">
       <c r="A569" t="n">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B569" t="inlineStr">
         <is>
@@ -19386,12 +19390,12 @@
       <c r="C569" t="inlineStr"/>
       <c r="D569" t="inlineStr">
         <is>
-          <t>údajne obrazovka IS v sekci B nad průchozími dveřmi ( směrem od WC) po tmě</t>
+          <t>údajně problikává chyba čidla měření nafty</t>
         </is>
       </c>
       <c r="E569" t="inlineStr">
         <is>
-          <t>neprojevilo se,kontrola konektorů,poklep obrazovka.Vše OK</t>
+          <t>nenapsali jakého,neprojevilo se</t>
         </is>
       </c>
       <c r="F569" t="inlineStr">
@@ -19409,22 +19413,22 @@
     </row>
     <row r="570">
       <c r="A570" t="n">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C570" t="inlineStr"/>
       <c r="D570" t="inlineStr">
         <is>
-          <t>údajně problikává chyba čidla měření nafty</t>
+          <t>nechladí</t>
         </is>
       </c>
       <c r="E570" t="inlineStr">
         <is>
-          <t>nenapsali jakého,neprojevilo se</t>
+          <t>vydný proporcionální ventil,výměna</t>
         </is>
       </c>
       <c r="F570" t="inlineStr">
@@ -19442,22 +19446,22 @@
     </row>
     <row r="571">
       <c r="A571" t="n">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B571" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>842 015</t>
         </is>
       </c>
       <c r="C571" t="inlineStr"/>
       <c r="D571" t="inlineStr">
         <is>
-          <t>nechladí</t>
+          <t>někdy nejde brzda PB</t>
         </is>
       </c>
       <c r="E571" t="inlineStr">
         <is>
-          <t>vydný proporcionální ventil,výměna</t>
+          <t>výměna ventilu YV 61 včetně cívky</t>
         </is>
       </c>
       <c r="F571" t="inlineStr">
@@ -19475,22 +19479,22 @@
     </row>
     <row r="572">
       <c r="A572" t="n">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C572" t="inlineStr"/>
       <c r="D572" t="inlineStr">
         <is>
-          <t>někdy nejde brzda PB</t>
+          <t>v B salónu ukazuje prostřední čidlo 0°C</t>
         </is>
       </c>
       <c r="E572" t="inlineStr">
         <is>
-          <t>výměna ventilu YV 61 včetně cívky</t>
+          <t>po zahýbáním káblíku co vede ze stěny do svorkovnice čidla vše OK. Prodřený drát cca 5 cm od konce. Nasazení smršťovačky,přesvorkování dutinek</t>
         </is>
       </c>
       <c r="F572" t="inlineStr">
@@ -19508,22 +19512,22 @@
     </row>
     <row r="573">
       <c r="A573" t="n">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C573" t="inlineStr"/>
       <c r="D573" t="inlineStr">
         <is>
-          <t>v B salónu ukazuje prostřední čidlo 0°C</t>
+          <t>neukazuje vodoznak,pravá strana</t>
         </is>
       </c>
       <c r="E573" t="inlineStr">
         <is>
-          <t>po zahýbáním káblíku co vede ze stěny do svorkovnice čidla vše OK. Prodřený drát cca 5 cm od konce. Nasazení smršťovačky,přesvorkování dutinek</t>
+          <t>výměna</t>
         </is>
       </c>
       <c r="F573" t="inlineStr">
@@ -19541,22 +19545,22 @@
     </row>
     <row r="574">
       <c r="A574" t="n">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C574" t="inlineStr"/>
       <c r="D574" t="inlineStr">
         <is>
-          <t>neukazuje vodoznak,pravá strana</t>
+          <t>opět slabý výkon</t>
         </is>
       </c>
       <c r="E574" t="inlineStr">
         <is>
-          <t>výměna</t>
+          <t>byly "vyběhané" kloubky na táhlu AČ,výměna.Seřízení pákový,při 25% 930 otáček</t>
         </is>
       </c>
       <c r="F574" t="inlineStr">
@@ -19574,22 +19578,22 @@
     </row>
     <row r="575">
       <c r="A575" t="n">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="B575" t="inlineStr">
         <is>
-          <t>814 118</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C575" t="inlineStr"/>
       <c r="D575" t="inlineStr">
         <is>
-          <t>opět slabý výkon</t>
+          <t>údajně nejde ARR z B</t>
         </is>
       </c>
       <c r="E575" t="inlineStr">
         <is>
-          <t>byly "vyběhané" kloubky na táhlu AČ,výměna.Seřízení pákový,při 25% 930 otáček</t>
+          <t>neprojevilo se,neměněno</t>
         </is>
       </c>
       <c r="F575" t="inlineStr">
@@ -19607,7 +19611,7 @@
     </row>
     <row r="576">
       <c r="A576" t="n">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B576" t="inlineStr">
         <is>
@@ -19617,12 +19621,12 @@
       <c r="C576" t="inlineStr"/>
       <c r="D576" t="inlineStr">
         <is>
-          <t>údajně nejde ARR z B</t>
+          <t>v A salónu ukazuje prostřední čidlo -17°C</t>
         </is>
       </c>
       <c r="E576" t="inlineStr">
         <is>
-          <t>neprojevilo se,neměněno</t>
+          <t>ve skutečnosti se jedná o čidlo u měchů. 6.9.2021 se přehazovali vstupy do ŘJ mezi měchy a prostředkem. Chyba byla v prostředku. 2 roky pak byl klid. Proměření ohmicky cesty,vstupy dány zpět jak mají být. Pokud se vrátí zase v prostředku,chyba v ŘJ</t>
         </is>
       </c>
       <c r="F576" t="inlineStr">
@@ -19640,22 +19644,22 @@
     </row>
     <row r="577">
       <c r="A577" t="n">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>029 227</t>
         </is>
       </c>
       <c r="C577" t="inlineStr"/>
       <c r="D577" t="inlineStr">
         <is>
-          <t>v A salónu ukazuje prostřední čidlo -17°C</t>
+          <t>porucha dveří elektr.</t>
         </is>
       </c>
       <c r="E577" t="inlineStr">
         <is>
-          <t>ve skutečnosti se jedná o čidlo u měchů. 6.9.2021 se přehazovali vstupy do ŘJ mezi měchy a prostředkem. Chyba byla v prostředku. 2 roky pak byl klid. Proměření ohmicky cesty,vstupy dány zpět jak mají být. Pokud se vrátí zase v prostředku,chyba v ŘJ</t>
+          <t>neprojevilo se , přezkoušení stran</t>
         </is>
       </c>
       <c r="F577" t="inlineStr">
@@ -19673,22 +19677,22 @@
     </row>
     <row r="578">
       <c r="A578" t="n">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>029 227</t>
+          <t>742 263</t>
         </is>
       </c>
       <c r="C578" t="inlineStr"/>
       <c r="D578" t="inlineStr">
         <is>
-          <t>porucha dveří elektr.</t>
+          <t>při startu dlouho promázává, nejde zkrácený start</t>
         </is>
       </c>
       <c r="E578" t="inlineStr">
         <is>
-          <t>neprojevilo se , přezkoušení stran</t>
+          <t>vše bylo funkční , zkrácený start spíná při 49°C přesto výměna YCR7</t>
         </is>
       </c>
       <c r="F578" t="inlineStr">
@@ -19706,7 +19710,7 @@
     </row>
     <row r="579">
       <c r="A579" t="n">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B579" t="inlineStr">
         <is>
@@ -19716,12 +19720,12 @@
       <c r="C579" t="inlineStr"/>
       <c r="D579" t="inlineStr">
         <is>
-          <t>při startu dlouho promázává, nejde zkrácený start</t>
+          <t>porucha dveří elektr.</t>
         </is>
       </c>
       <c r="E579" t="inlineStr">
         <is>
-          <t>vše bylo funkční , zkrácený start spíná při 49°C přesto výměna YCR7</t>
+          <t>neprojevilo se , přezkoušení stran</t>
         </is>
       </c>
       <c r="F579" t="inlineStr">
@@ -19739,22 +19743,22 @@
     </row>
     <row r="580">
       <c r="A580" t="n">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B580" t="inlineStr">
         <is>
-          <t>742 263</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C580" t="inlineStr"/>
       <c r="D580" t="inlineStr">
         <is>
-          <t>porucha dveří elektr.</t>
+          <t>IS se rozpadá, ztráci komunikaci mezi stan.</t>
         </is>
       </c>
       <c r="E580" t="inlineStr">
         <is>
-          <t>neprojevilo se , přezkoušení stran</t>
+          <t>dotlační konektoru ale vše bylo funkční</t>
         </is>
       </c>
       <c r="F580" t="inlineStr">
@@ -19772,7 +19776,7 @@
     </row>
     <row r="581">
       <c r="A581" t="n">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B581" t="inlineStr">
         <is>
@@ -19782,12 +19786,12 @@
       <c r="C581" t="inlineStr"/>
       <c r="D581" t="inlineStr">
         <is>
-          <t>IS se rozpadá, ztráci komunikaci mezi stan.</t>
+          <t>parkovací brzda nevybaví KBS</t>
         </is>
       </c>
       <c r="E581" t="inlineStr">
         <is>
-          <t>dotlační konektoru ale vše bylo funkční</t>
+          <t>seřízení tlaku</t>
         </is>
       </c>
       <c r="F581" t="inlineStr">
@@ -19805,7 +19809,7 @@
     </row>
     <row r="582">
       <c r="A582" t="n">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="B582" t="inlineStr">
         <is>
@@ -19815,12 +19819,12 @@
       <c r="C582" t="inlineStr"/>
       <c r="D582" t="inlineStr">
         <is>
-          <t>parkovací brzda nevybaví KBS</t>
+          <t>únik oleje na 6. válci</t>
         </is>
       </c>
       <c r="E582" t="inlineStr">
         <is>
-          <t>seřízení tlaku</t>
+          <t>výměna</t>
         </is>
       </c>
       <c r="F582" t="inlineStr">
@@ -19838,7 +19842,7 @@
     </row>
     <row r="583">
       <c r="A583" t="n">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B583" t="inlineStr">
         <is>
@@ -19848,12 +19852,12 @@
       <c r="C583" t="inlineStr"/>
       <c r="D583" t="inlineStr">
         <is>
-          <t>únik oleje na 6. válci</t>
+          <t>nesvítí červené poziční světlo</t>
         </is>
       </c>
       <c r="E583" t="inlineStr">
         <is>
-          <t>výměna</t>
+          <t>zapojení vodiče 735 byl odpojený (výměna obou světel na stan 914)</t>
         </is>
       </c>
       <c r="F583" t="inlineStr">
@@ -19871,22 +19875,22 @@
     </row>
     <row r="584">
       <c r="A584" t="n">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="B584" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C584" t="inlineStr"/>
       <c r="D584" t="inlineStr">
         <is>
-          <t>nesvítí červené poziční světlo</t>
+          <t>nelze odbrzdit, tlak ve válcích zůstáva 0,3 bar závada jen z 914</t>
         </is>
       </c>
       <c r="E584" t="inlineStr">
         <is>
-          <t>zapojení vodiče 735 byl odpojený (výměna obou světel na stan 914)</t>
+          <t>zk. Jízda OK</t>
         </is>
       </c>
       <c r="F584" t="inlineStr">
@@ -19904,22 +19908,22 @@
     </row>
     <row r="585">
       <c r="A585" t="n">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B585" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C585" t="inlineStr"/>
       <c r="D585" t="inlineStr">
         <is>
-          <t>nelze odbrzdit, tlak ve válcích zůstáva 0,3 bar závada jen z 914</t>
+          <t>2.SM samovolně zvyšuje otáčky, seřízení GAC</t>
         </is>
       </c>
       <c r="E585" t="inlineStr">
         <is>
-          <t>zk. Jízda OK</t>
+          <t>přístě vyměnit GAC musela jet ven</t>
         </is>
       </c>
       <c r="F585" t="inlineStr">
@@ -19937,22 +19941,22 @@
     </row>
     <row r="586">
       <c r="A586" t="n">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="B586" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C586" t="inlineStr"/>
       <c r="D586" t="inlineStr">
         <is>
-          <t>2.SM samovolně zvyšuje otáčky, seřízení GAC</t>
+          <t>nehlási IS na stan. A</t>
         </is>
       </c>
       <c r="E586" t="inlineStr">
         <is>
-          <t>přístě vyměnit GAC musela jet ven</t>
+          <t>ztlumen potenciometr</t>
         </is>
       </c>
       <c r="F586" t="inlineStr">
@@ -19970,7 +19974,7 @@
     </row>
     <row r="587">
       <c r="A587" t="n">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B587" t="inlineStr">
         <is>
@@ -19980,12 +19984,12 @@
       <c r="C587" t="inlineStr"/>
       <c r="D587" t="inlineStr">
         <is>
-          <t>nehlási IS na stan. A</t>
+          <t>lednice nechladí</t>
         </is>
       </c>
       <c r="E587" t="inlineStr">
         <is>
-          <t>ztlumen potenciometr</t>
+          <t>odzkoušeno OK</t>
         </is>
       </c>
       <c r="F587" t="inlineStr">
@@ -20003,7 +20007,7 @@
     </row>
     <row r="588">
       <c r="A588" t="n">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B588" t="inlineStr">
         <is>
@@ -20013,12 +20017,12 @@
       <c r="C588" t="inlineStr"/>
       <c r="D588" t="inlineStr">
         <is>
-          <t>lednice nechladí</t>
+          <t>údajně rázy převodovky</t>
         </is>
       </c>
       <c r="E588" t="inlineStr">
         <is>
-          <t>odzkoušeno OK</t>
+          <t>řesí p. Šípek vyčítal jsi obě HMP</t>
         </is>
       </c>
       <c r="F588" t="inlineStr">
@@ -20036,22 +20040,22 @@
     </row>
     <row r="589">
       <c r="A589" t="n">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B589" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C589" t="inlineStr"/>
       <c r="D589" t="inlineStr">
         <is>
-          <t>údajně rázy převodovky</t>
+          <t>lok. Nejde nastartovat</t>
         </is>
       </c>
       <c r="E589" t="inlineStr">
         <is>
-          <t>řesí p. Šípek vyčítal jsi obě HMP</t>
+          <t>naftová netěsnost</t>
         </is>
       </c>
       <c r="F589" t="inlineStr">
@@ -20069,22 +20073,22 @@
     </row>
     <row r="590">
       <c r="A590" t="n">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B590" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C590" t="inlineStr"/>
       <c r="D590" t="inlineStr">
         <is>
-          <t>lok. Nejde nastartovat</t>
+          <t>izolačni stav odztraněny zkraty na vodiči 80 a 50</t>
         </is>
       </c>
       <c r="E590" t="inlineStr">
         <is>
-          <t>naftová netěsnost</t>
+          <t>startéry vyfoukany,ale nakonec výměna M2(volný pomocný vodič) seřízení GAC 2. SM , zkušební jízda se zdá v pořádku</t>
         </is>
       </c>
       <c r="F590" t="inlineStr">
@@ -20102,24 +20106,24 @@
     </row>
     <row r="591">
       <c r="A591" t="n">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B591" t="inlineStr">
         <is>
-          <t>842 035</t>
-        </is>
-      </c>
-      <c r="C591" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>06.12.2023</t>
+        </is>
+      </c>
       <c r="D591" t="inlineStr">
         <is>
-          <t>izolačni stav odztraněny zkraty na vodiči 80 a 50</t>
-        </is>
-      </c>
-      <c r="E591" t="inlineStr">
-        <is>
-          <t>startéry vyfoukany,ale nakonec výměna M2(volný pomocný vodič) seřízení GAC 2. SM , zkušební jízda se zdá v pořádku</t>
-        </is>
-      </c>
+          <t>Výměna obrazovky na 914 (občas zamrzá)</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr"/>
       <c r="F591" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20135,11 +20139,11 @@
     </row>
     <row r="592">
       <c r="A592" t="n">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>814 003</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C592" t="inlineStr">
@@ -20149,7 +20153,7 @@
       </c>
       <c r="D592" t="inlineStr">
         <is>
-          <t>Výměna obrazovky na 914 (občas zamrzá)</t>
+          <t>údajně se rozpadá IS přezkoušeno (kontrola konektoru)</t>
         </is>
       </c>
       <c r="E592" t="inlineStr"/>
@@ -20168,11 +20172,11 @@
     </row>
     <row r="593">
       <c r="A593" t="n">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 072</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
@@ -20182,7 +20186,7 @@
       </c>
       <c r="D593" t="inlineStr">
         <is>
-          <t>údajně se rozpadá IS přezkoušeno (kontrola konektoru)</t>
+          <t>tozpadáva se IS, oprava dispeleje na 914 byl volný</t>
         </is>
       </c>
       <c r="E593" t="inlineStr"/>
@@ -20201,24 +20205,28 @@
     </row>
     <row r="594">
       <c r="A594" t="n">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B594" t="inlineStr">
         <is>
-          <t>814 072</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C594" t="inlineStr">
         <is>
-          <t>06.12.2023</t>
+          <t>06.11.2023</t>
         </is>
       </c>
       <c r="D594" t="inlineStr">
         <is>
-          <t>tozpadáva se IS, oprava dispeleje na 914 byl volný</t>
-        </is>
-      </c>
-      <c r="E594" t="inlineStr"/>
+          <t>tabule vnitřní , venkovní nekomunikují</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>výměna konektoru C na 914</t>
+        </is>
+      </c>
       <c r="F594" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20234,11 +20242,11 @@
     </row>
     <row r="595">
       <c r="A595" t="n">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>814 118</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C595" t="inlineStr">
@@ -20248,12 +20256,12 @@
       </c>
       <c r="D595" t="inlineStr">
         <is>
-          <t>tabule vnitřní , venkovní nekomunikují</t>
+          <t>korekce vody 2</t>
         </is>
       </c>
       <c r="E595" t="inlineStr">
         <is>
-          <t>výměna konektoru C na 914</t>
+          <t>izolačni stav špatný  stáhlé zemni relé</t>
         </is>
       </c>
       <c r="F595" t="inlineStr">
@@ -20271,11 +20279,11 @@
     </row>
     <row r="596">
       <c r="A596" t="n">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B596" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C596" t="inlineStr">
@@ -20285,14 +20293,10 @@
       </c>
       <c r="D596" t="inlineStr">
         <is>
-          <t>korekce vody 2</t>
-        </is>
-      </c>
-      <c r="E596" t="inlineStr">
-        <is>
-          <t>izolačni stav špatný  stáhlé zemni relé</t>
-        </is>
-      </c>
+          <t>výměna ARR na B stan. Nefunkční</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr"/>
       <c r="F596" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20308,21 +20312,21 @@
     </row>
     <row r="597">
       <c r="A597" t="n">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="B597" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>842 011</t>
         </is>
       </c>
       <c r="C597" t="inlineStr">
         <is>
-          <t>06.11.2023</t>
+          <t>06.10.2023</t>
         </is>
       </c>
       <c r="D597" t="inlineStr">
         <is>
-          <t>výměna ARR na B stan. Nefunkční</t>
+          <t>udajně zateklo do pultu na 2st.(kontrola)</t>
         </is>
       </c>
       <c r="E597" t="inlineStr"/>
@@ -20341,11 +20345,11 @@
     </row>
     <row r="598">
       <c r="A598" t="n">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B598" t="inlineStr">
         <is>
-          <t>842 011</t>
+          <t>842 021</t>
         </is>
       </c>
       <c r="C598" t="inlineStr">
@@ -20355,10 +20359,14 @@
       </c>
       <c r="D598" t="inlineStr">
         <is>
-          <t>udajně zateklo do pultu na 2st.(kontrola)</t>
-        </is>
-      </c>
-      <c r="E598" t="inlineStr"/>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>vadné čidlo vody v míse</t>
+        </is>
+      </c>
       <c r="F598" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20374,26 +20382,26 @@
     </row>
     <row r="599">
       <c r="A599" t="n">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>842 021</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C599" t="inlineStr">
         <is>
-          <t>06.10.2023</t>
+          <t>06.09.2023</t>
         </is>
       </c>
       <c r="D599" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>Nejdou dvěře WC</t>
         </is>
       </c>
       <c r="E599" t="inlineStr">
         <is>
-          <t>vadné čidlo vody v míse</t>
+          <t>upadlý drát na přepínači funkce WC (zapnuto,bez dveří, vypnuto). Seřízení zámykání dveří. Frýdek</t>
         </is>
       </c>
       <c r="F599" t="inlineStr">
@@ -20411,11 +20419,11 @@
     </row>
     <row r="600">
       <c r="A600" t="n">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B600" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C600" t="inlineStr">
@@ -20425,12 +20433,12 @@
       </c>
       <c r="D600" t="inlineStr">
         <is>
-          <t>Nejdou dvěře WC</t>
+          <t>údajně nejdou někdy schody u levých dveří strany A</t>
         </is>
       </c>
       <c r="E600" t="inlineStr">
         <is>
-          <t>upadlý drát na přepínači funkce WC (zapnuto,bez dveří, vypnuto). Seřízení zámykání dveří. Frýdek</t>
+          <t>vyčištění od kamínků,odzkoušení-OK</t>
         </is>
       </c>
       <c r="F600" t="inlineStr">
@@ -20448,26 +20456,26 @@
     </row>
     <row r="601">
       <c r="A601" t="n">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C601" t="inlineStr">
         <is>
-          <t>06.09.2023</t>
+          <t>06.08.2023</t>
         </is>
       </c>
       <c r="D601" t="inlineStr">
         <is>
-          <t>údajně nejdou někdy schody u levých dveří strany A</t>
+          <t>zapůjčena z HB</t>
         </is>
       </c>
       <c r="E601" t="inlineStr">
         <is>
-          <t>vyčištění od kamínků,odzkoušení-OK</t>
+          <t>nahrány data IS ( funguje preš radiostanici)</t>
         </is>
       </c>
       <c r="F601" t="inlineStr">
@@ -20485,11 +20493,11 @@
     </row>
     <row r="602">
       <c r="A602" t="n">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C602" t="inlineStr">
@@ -20499,12 +20507,12 @@
       </c>
       <c r="D602" t="inlineStr">
         <is>
-          <t>zapůjčena z HB</t>
+          <t>Opět problémy se startováním</t>
         </is>
       </c>
       <c r="E602" t="inlineStr">
         <is>
-          <t>nahrány data IS ( funguje preš radiostanici)</t>
+          <t>(asi už vadný capos kondy)říkali veselani jak tu byli</t>
         </is>
       </c>
       <c r="F602" t="inlineStr">
@@ -20522,7 +20530,7 @@
     </row>
     <row r="603">
       <c r="A603" t="n">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B603" t="inlineStr">
         <is>
@@ -20536,12 +20544,12 @@
       </c>
       <c r="D603" t="inlineStr">
         <is>
-          <t>Opět problémy se startováním</t>
+          <t>oprava hlasitosti na stanovišti A</t>
         </is>
       </c>
       <c r="E603" t="inlineStr">
         <is>
-          <t>(asi už vadný capos kondy)říkali veselani jak tu byli</t>
+          <t>přechod na kontaktech u reproduktoru v pultě</t>
         </is>
       </c>
       <c r="F603" t="inlineStr">
@@ -20559,11 +20567,11 @@
     </row>
     <row r="604">
       <c r="A604" t="n">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B604" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C604" t="inlineStr">
@@ -20573,12 +20581,12 @@
       </c>
       <c r="D604" t="inlineStr">
         <is>
-          <t>oprava hlasitosti na stanovišti A</t>
+          <t>výměna ARR na B</t>
         </is>
       </c>
       <c r="E604" t="inlineStr">
         <is>
-          <t>přechod na kontaktech u reproduktoru v pultě</t>
+          <t>vadná linka CAN</t>
         </is>
       </c>
       <c r="F604" t="inlineStr">
@@ -20596,26 +20604,26 @@
     </row>
     <row r="605">
       <c r="A605" t="n">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>842 015</t>
         </is>
       </c>
       <c r="C605" t="inlineStr">
         <is>
-          <t>06.08.2023</t>
+          <t>06.07.2023</t>
         </is>
       </c>
       <c r="D605" t="inlineStr">
         <is>
-          <t>výměna ARR na B</t>
+          <t>někdy nejde brzda PB</t>
         </is>
       </c>
       <c r="E605" t="inlineStr">
         <is>
-          <t>vadná linka CAN</t>
+          <t>výměna karty DS a OUT z 842 025</t>
         </is>
       </c>
       <c r="F605" t="inlineStr">
@@ -20633,11 +20641,11 @@
     </row>
     <row r="606">
       <c r="A606" t="n">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B606" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C606" t="inlineStr">
@@ -20647,14 +20655,10 @@
       </c>
       <c r="D606" t="inlineStr">
         <is>
-          <t>někdy nejde brzda PB</t>
-        </is>
-      </c>
-      <c r="E606" t="inlineStr">
-        <is>
-          <t>výměna karty DS a OUT z 842 025</t>
-        </is>
-      </c>
+          <t>dosazeny karty z 842 015 (DS a OUT)</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr"/>
       <c r="F606" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20670,11 +20674,11 @@
     </row>
     <row r="607">
       <c r="A607" t="n">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B607" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C607" t="inlineStr">
@@ -20684,10 +20688,14 @@
       </c>
       <c r="D607" t="inlineStr">
         <is>
-          <t>dosazeny karty z 842 015 (DS a OUT)</t>
-        </is>
-      </c>
-      <c r="E607" t="inlineStr"/>
+          <t>dosazen asi 5 dobíječ na B funkční</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>ve skladu nefunkční jenom (má řešit asi Mlíčko)</t>
+        </is>
+      </c>
       <c r="F607" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20703,28 +20711,24 @@
     </row>
     <row r="608">
       <c r="A608" t="n">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="B608" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 076</t>
         </is>
       </c>
       <c r="C608" t="inlineStr">
         <is>
-          <t>06.07.2023</t>
+          <t>06.06.2023</t>
         </is>
       </c>
       <c r="D608" t="inlineStr">
         <is>
-          <t>dosazen asi 5 dobíječ na B funkční</t>
-        </is>
-      </c>
-      <c r="E608" t="inlineStr">
-        <is>
-          <t>ve skladu nefunkční jenom (má řešit asi Mlíčko)</t>
-        </is>
-      </c>
+          <t>NEHODA V HOLEŠOVĚ</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr"/>
       <c r="F608" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20740,21 +20744,21 @@
     </row>
     <row r="609">
       <c r="A609" t="n">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>814 076</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C609" t="inlineStr">
         <is>
-          <t>06.06.2023</t>
+          <t>06.05.2023</t>
         </is>
       </c>
       <c r="D609" t="inlineStr">
         <is>
-          <t>NEHODA V HOLEŠOVĚ</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E609" t="inlineStr"/>
@@ -20773,21 +20777,17 @@
     </row>
     <row r="610">
       <c r="A610" t="n">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="B610" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C610" t="inlineStr">
-        <is>
-          <t>06.05.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr"/>
       <c r="D610" t="inlineStr">
         <is>
-          <t>MM</t>
+          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
         </is>
       </c>
       <c r="E610" t="inlineStr"/>
@@ -20806,7 +20806,7 @@
     </row>
     <row r="611">
       <c r="A611" t="n">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="B611" t="inlineStr">
         <is>
@@ -20816,7 +20816,7 @@
       <c r="C611" t="inlineStr"/>
       <c r="D611" t="inlineStr">
         <is>
-          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
+          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
         </is>
       </c>
       <c r="E611" t="inlineStr"/>
@@ -20835,7 +20835,7 @@
     </row>
     <row r="612">
       <c r="A612" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B612" t="inlineStr">
         <is>
@@ -20845,7 +20845,7 @@
       <c r="C612" t="inlineStr"/>
       <c r="D612" t="inlineStr">
         <is>
-          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
+          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
         </is>
       </c>
       <c r="E612" t="inlineStr"/>
@@ -20864,20 +20864,24 @@
     </row>
     <row r="613">
       <c r="A613" t="n">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C613" t="inlineStr"/>
       <c r="D613" t="inlineStr">
         <is>
-          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
-        </is>
-      </c>
-      <c r="E613" t="inlineStr"/>
+          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>vyměnili dobíječ stacionární (Veselí)</t>
+        </is>
+      </c>
       <c r="F613" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20893,22 +20897,22 @@
     </row>
     <row r="614">
       <c r="A614" t="n">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B614" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C614" t="inlineStr"/>
       <c r="D614" t="inlineStr">
         <is>
-          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
         </is>
       </c>
       <c r="E614" t="inlineStr">
         <is>
-          <t>vyměnili dobíječ stacionární (Veselí)</t>
+          <t>jela ven</t>
         </is>
       </c>
       <c r="F614" t="inlineStr">
@@ -20926,24 +20930,20 @@
     </row>
     <row r="615">
       <c r="A615" t="n">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C615" t="inlineStr"/>
       <c r="D615" t="inlineStr">
         <is>
-          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
-        </is>
-      </c>
-      <c r="E615" t="inlineStr">
-        <is>
-          <t>jela ven</t>
-        </is>
-      </c>
+          <t>seřízení kamer přes program v notasu(obraz)</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr"/>
       <c r="F615" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20959,20 +20959,24 @@
     </row>
     <row r="616">
       <c r="A616" t="n">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B616" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C616" t="inlineStr"/>
       <c r="D616" t="inlineStr">
         <is>
-          <t>seřízení kamer přes program v notasu(obraz)</t>
-        </is>
-      </c>
-      <c r="E616" t="inlineStr"/>
+          <t>po startu někdy nenabíjí "B"</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+        </is>
+      </c>
       <c r="F616" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20988,22 +20992,22 @@
     </row>
     <row r="617">
       <c r="A617" t="n">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C617" t="inlineStr"/>
       <c r="D617" t="inlineStr">
         <is>
-          <t>po startu někdy nenabíjí "B"</t>
+          <t>2. motor korekce vody  vystup</t>
         </is>
       </c>
       <c r="E617" t="inlineStr">
         <is>
-          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
         </is>
       </c>
       <c r="F617" t="inlineStr">
@@ -21021,24 +21025,24 @@
     </row>
     <row r="618">
       <c r="A618" t="n">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B618" t="inlineStr">
         <is>
-          <t>842 035</t>
-        </is>
-      </c>
-      <c r="C618" t="inlineStr"/>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>04.12.2023</t>
+        </is>
+      </c>
       <c r="D618" t="inlineStr">
         <is>
-          <t>2. motor korekce vody  vystup</t>
-        </is>
-      </c>
-      <c r="E618" t="inlineStr">
-        <is>
-          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
-        </is>
-      </c>
+          <t>Výměna motoru A</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr"/>
       <c r="F618" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21054,21 +21058,17 @@
     </row>
     <row r="619">
       <c r="A619" t="n">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C619" t="inlineStr">
-        <is>
-          <t>04.12.2023</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr"/>
       <c r="D619" t="inlineStr">
         <is>
-          <t>Výměna motoru A</t>
+          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
         </is>
       </c>
       <c r="E619" t="inlineStr"/>
@@ -21087,17 +21087,17 @@
     </row>
     <row r="620">
       <c r="A620" t="n">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C620" t="inlineStr"/>
       <c r="D620" t="inlineStr">
         <is>
-          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
+          <t>dosazena nahadni Mirelka + NO z 844 013</t>
         </is>
       </c>
       <c r="E620" t="inlineStr"/>
@@ -21116,17 +21116,17 @@
     </row>
     <row r="621">
       <c r="A621" t="n">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 062</t>
         </is>
       </c>
       <c r="C621" t="inlineStr"/>
       <c r="D621" t="inlineStr">
         <is>
-          <t>dosazena nahadni Mirelka + NO z 844 013</t>
+          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
         </is>
       </c>
       <c r="E621" t="inlineStr"/>
@@ -21145,17 +21145,21 @@
     </row>
     <row r="622">
       <c r="A622" t="n">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>814 062</t>
-        </is>
-      </c>
-      <c r="C622" t="inlineStr"/>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>03.03.2023</t>
+        </is>
+      </c>
       <c r="D622" t="inlineStr">
         <is>
-          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E622" t="inlineStr"/>
@@ -21174,11 +21178,11 @@
     </row>
     <row r="623">
       <c r="A623" t="n">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B623" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C623" t="inlineStr">
@@ -21188,7 +21192,7 @@
       </c>
       <c r="D623" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
+          <t>Dosazení ŘJ kamer</t>
         </is>
       </c>
       <c r="E623" t="inlineStr"/>
@@ -21207,24 +21211,24 @@
     </row>
     <row r="624">
       <c r="A624" t="n">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>844 013</t>
-        </is>
-      </c>
-      <c r="C624" t="inlineStr">
-        <is>
-          <t>03.03.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr"/>
       <c r="D624" t="inlineStr">
         <is>
-          <t>Dosazení ŘJ kamer</t>
-        </is>
-      </c>
-      <c r="E624" t="inlineStr"/>
+          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>hlášeno p. Škodovi</t>
+        </is>
+      </c>
       <c r="F624" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21240,24 +21244,20 @@
     </row>
     <row r="625">
       <c r="A625" t="n">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="B625" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C625" t="inlineStr"/>
       <c r="D625" t="inlineStr">
         <is>
-          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
-        </is>
-      </c>
-      <c r="E625" t="inlineStr">
-        <is>
-          <t>hlášeno p. Škodovi</t>
-        </is>
-      </c>
+          <t>ŘJ kamer dosazena z 013</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr"/>
       <c r="F625" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21273,17 +21273,21 @@
     </row>
     <row r="626">
       <c r="A626" t="n">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B626" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C626" t="inlineStr"/>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>02.09.2023</t>
+        </is>
+      </c>
       <c r="D626" t="inlineStr">
         <is>
-          <t>ŘJ kamer dosazena z 013</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E626" t="inlineStr"/>
@@ -21302,21 +21306,21 @@
     </row>
     <row r="627">
       <c r="A627" t="n">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 072</t>
         </is>
       </c>
       <c r="C627" t="inlineStr">
         <is>
-          <t>02.09.2023</t>
+          <t>02.03.2023</t>
         </is>
       </c>
       <c r="D627" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E627" t="inlineStr"/>
@@ -21335,24 +21339,24 @@
     </row>
     <row r="628">
       <c r="A628" t="n">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>814 072</t>
-        </is>
-      </c>
-      <c r="C628" t="inlineStr">
-        <is>
-          <t>02.03.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr"/>
       <c r="D628" t="inlineStr">
         <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E628" t="inlineStr"/>
+          <t>dosazen opraveny MIREL</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+        </is>
+      </c>
       <c r="F628" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21368,22 +21372,22 @@
     </row>
     <row r="629">
       <c r="A629" t="n">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C629" t="inlineStr"/>
       <c r="D629" t="inlineStr">
         <is>
-          <t>dosazen opraveny MIREL</t>
+          <t>Odpojen trojcestný ventil na A i B</t>
         </is>
       </c>
       <c r="E629" t="inlineStr">
         <is>
-          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+          <t>Zapojeny zpět 24.2.2023</t>
         </is>
       </c>
       <c r="F629" t="inlineStr">
@@ -21401,24 +21405,20 @@
     </row>
     <row r="630">
       <c r="A630" t="n">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C630" t="inlineStr"/>
       <c r="D630" t="inlineStr">
         <is>
-          <t>Odpojen trojcestný ventil na A i B</t>
-        </is>
-      </c>
-      <c r="E630" t="inlineStr">
-        <is>
-          <t>Zapojeny zpět 24.2.2023</t>
-        </is>
-      </c>
+          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr"/>
       <c r="F630" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21434,17 +21434,21 @@
     </row>
     <row r="631">
       <c r="A631" t="n">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B631" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C631" t="inlineStr"/>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>01.10.2023</t>
+        </is>
+      </c>
       <c r="D631" t="inlineStr">
         <is>
-          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E631" t="inlineStr"/>
@@ -21463,21 +21467,17 @@
     </row>
     <row r="632">
       <c r="A632" t="n">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C632" t="inlineStr">
-        <is>
-          <t>01.10.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr"/>
       <c r="D632" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
         </is>
       </c>
       <c r="E632" t="inlineStr"/>
@@ -21496,17 +21496,17 @@
     </row>
     <row r="633">
       <c r="A633" t="n">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C633" t="inlineStr"/>
       <c r="D633" t="inlineStr">
         <is>
-          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
+          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
         </is>
       </c>
       <c r="E633" t="inlineStr"/>
@@ -21525,7 +21525,7 @@
     </row>
     <row r="634">
       <c r="A634" t="n">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B634" t="inlineStr">
         <is>
@@ -21535,7 +21535,7 @@
       <c r="C634" t="inlineStr"/>
       <c r="D634" t="inlineStr">
         <is>
-          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
+          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
         </is>
       </c>
       <c r="E634" t="inlineStr"/>
@@ -21554,20 +21554,24 @@
     </row>
     <row r="635">
       <c r="A635" t="n">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C635" t="inlineStr"/>
       <c r="D635" t="inlineStr">
         <is>
-          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
-        </is>
-      </c>
-      <c r="E635" t="inlineStr"/>
+          <t>Přišel opravený Mirel ve skladu</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>dosazen na 29.12.2022</t>
+        </is>
+      </c>
       <c r="F635" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21583,22 +21587,26 @@
     </row>
     <row r="636">
       <c r="A636" t="n">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C636" t="inlineStr"/>
+          <t>844 014</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>12.06.2022</t>
+        </is>
+      </c>
       <c r="D636" t="inlineStr">
         <is>
-          <t>Přišel opravený Mirel ve skladu</t>
+          <t>rychloměr do opravy hazí !!</t>
         </is>
       </c>
       <c r="E636" t="inlineStr">
         <is>
-          <t>dosazen na 29.12.2022</t>
+          <t>zapujcen z 844 028 z veselí</t>
         </is>
       </c>
       <c r="F636" t="inlineStr">
@@ -21616,11 +21624,11 @@
     </row>
     <row r="637">
       <c r="A637" t="n">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C637" t="inlineStr">
@@ -21630,14 +21638,10 @@
       </c>
       <c r="D637" t="inlineStr">
         <is>
-          <t>rychloměr do opravy hazí !!</t>
-        </is>
-      </c>
-      <c r="E637" t="inlineStr">
-        <is>
-          <t>zapujcen z 844 028 z veselí</t>
-        </is>
-      </c>
+          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr"/>
       <c r="F637" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21653,24 +21657,28 @@
     </row>
     <row r="638">
       <c r="A638" t="n">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C638" t="inlineStr">
         <is>
-          <t>12.06.2022</t>
+          <t>12.03.2022</t>
         </is>
       </c>
       <c r="D638" t="inlineStr">
         <is>
-          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
-        </is>
-      </c>
-      <c r="E638" t="inlineStr"/>
+          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>bude řešit Škoda</t>
+        </is>
+      </c>
       <c r="F638" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21686,26 +21694,22 @@
     </row>
     <row r="639">
       <c r="A639" t="n">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B639" t="inlineStr">
         <is>
           <t>844 003</t>
         </is>
       </c>
-      <c r="C639" t="inlineStr">
-        <is>
-          <t>12.03.2022</t>
-        </is>
-      </c>
+      <c r="C639" t="inlineStr"/>
       <c r="D639" t="inlineStr">
         <is>
-          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+          <t>na A strane asi vadna expanzní nadrz topení ?</t>
         </is>
       </c>
       <c r="E639" t="inlineStr">
         <is>
-          <t>bude řešit Škoda</t>
+          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
         </is>
       </c>
       <c r="F639" t="inlineStr">
@@ -21723,22 +21727,22 @@
     </row>
     <row r="640">
       <c r="A640" t="n">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C640" t="inlineStr"/>
       <c r="D640" t="inlineStr">
         <is>
-          <t>na A strane asi vadna expanzní nadrz topení ?</t>
+          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
         </is>
       </c>
       <c r="E640" t="inlineStr">
         <is>
-          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
+          <t>nová obrazovka hazela vykricnik porad</t>
         </is>
       </c>
       <c r="F640" t="inlineStr">
@@ -21756,24 +21760,24 @@
     </row>
     <row r="641">
       <c r="A641" t="n">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C641" t="inlineStr"/>
+          <t>842 010</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>11.06.2022</t>
+        </is>
+      </c>
       <c r="D641" t="inlineStr">
         <is>
-          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
-        </is>
-      </c>
-      <c r="E641" t="inlineStr">
-        <is>
-          <t>nová obrazovka hazela vykricnik porad</t>
-        </is>
-      </c>
+          <t>Přehození karty TBA v DPV na 842 036</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr"/>
       <c r="F641" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21789,11 +21793,11 @@
     </row>
     <row r="642">
       <c r="A642" t="n">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>842 010</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C642" t="inlineStr">
@@ -21803,7 +21807,7 @@
       </c>
       <c r="D642" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 036</t>
+          <t>Přehození karty TBA v DPV na 842 010</t>
         </is>
       </c>
       <c r="E642" t="inlineStr"/>
@@ -21822,11 +21826,11 @@
     </row>
     <row r="643">
       <c r="A643" t="n">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C643" t="inlineStr">
@@ -21836,10 +21840,14 @@
       </c>
       <c r="D643" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 010</t>
-        </is>
-      </c>
-      <c r="E643" t="inlineStr"/>
+          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>mirel byl špatný po opravě</t>
+        </is>
+      </c>
       <c r="F643" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21855,26 +21863,26 @@
     </row>
     <row r="644">
       <c r="A644" t="n">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C644" t="inlineStr">
         <is>
-          <t>11.06.2022</t>
+          <t>11.05.2022</t>
         </is>
       </c>
       <c r="D644" t="inlineStr">
         <is>
-          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
         </is>
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>mirel byl špatný po opravě</t>
+          <t>25.11. opraveno</t>
         </is>
       </c>
       <c r="F644" t="inlineStr">
@@ -21892,11 +21900,11 @@
     </row>
     <row r="645">
       <c r="A645" t="n">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C645" t="inlineStr">
@@ -21906,14 +21914,10 @@
       </c>
       <c r="D645" t="inlineStr">
         <is>
-          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
-        </is>
-      </c>
-      <c r="E645" t="inlineStr">
-        <is>
-          <t>25.11. opraveno</t>
-        </is>
-      </c>
+          <t>VESELÍ R3 (odjela)</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr"/>
       <c r="F645" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21929,24 +21933,24 @@
     </row>
     <row r="646">
       <c r="A646" t="n">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>844 020</t>
-        </is>
-      </c>
-      <c r="C646" t="inlineStr">
-        <is>
-          <t>11.05.2022</t>
-        </is>
-      </c>
+          <t>814 190</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr"/>
       <c r="D646" t="inlineStr">
         <is>
-          <t>VESELÍ R3 (odjela)</t>
-        </is>
-      </c>
-      <c r="E646" t="inlineStr"/>
+          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>hlášeno p.Škodovi</t>
+        </is>
+      </c>
       <c r="F646" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21962,22 +21966,22 @@
     </row>
     <row r="647">
       <c r="A647" t="n">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>814 190</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C647" t="inlineStr"/>
       <c r="D647" t="inlineStr">
         <is>
-          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
         </is>
       </c>
       <c r="E647" t="inlineStr">
         <is>
-          <t>hlášeno p.Škodovi</t>
+          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
         </is>
       </c>
       <c r="F647" t="inlineStr">
@@ -21995,24 +21999,20 @@
     </row>
     <row r="648">
       <c r="A648" t="n">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C648" t="inlineStr"/>
       <c r="D648" t="inlineStr">
         <is>
-          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
-        </is>
-      </c>
-      <c r="E648" t="inlineStr">
-        <is>
-          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
-        </is>
-      </c>
+          <t>dosazen předzesilovač linky</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr"/>
       <c r="F648" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22028,20 +22028,28 @@
     </row>
     <row r="649">
       <c r="A649" t="n">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B649" t="inlineStr">
         <is>
           <t>814 073</t>
         </is>
       </c>
-      <c r="C649" t="inlineStr"/>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>09.07.2022</t>
+        </is>
+      </c>
       <c r="D649" t="inlineStr">
         <is>
-          <t>dosazen předzesilovač linky</t>
-        </is>
-      </c>
-      <c r="E649" t="inlineStr"/>
+          <t>chybějící díl</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>předzasilovač linky - objednán nový</t>
+        </is>
+      </c>
       <c r="F649" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22057,26 +22065,26 @@
     </row>
     <row r="650">
       <c r="A650" t="n">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 003</t>
         </is>
       </c>
       <c r="C650" t="inlineStr">
         <is>
-          <t>09.07.2022</t>
+          <t>09.03.2022</t>
         </is>
       </c>
       <c r="D650" t="inlineStr">
         <is>
-          <t>chybějící díl</t>
+          <t>dosazen díl</t>
         </is>
       </c>
       <c r="E650" t="inlineStr">
         <is>
-          <t>předzasilovač linky - objednán nový</t>
+          <t>dosazen předzasilovač linky A23</t>
         </is>
       </c>
       <c r="F650" t="inlineStr">
@@ -22094,26 +22102,22 @@
     </row>
     <row r="651">
       <c r="A651" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C651" t="inlineStr">
-        <is>
-          <t>09.03.2022</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr"/>
       <c r="D651" t="inlineStr">
         <is>
-          <t>dosazen díl</t>
+          <t>oprava dveří na B pravé po směru jízdy</t>
         </is>
       </c>
       <c r="E651" t="inlineStr">
         <is>
-          <t>dosazen předzasilovač linky A23</t>
+          <t>vadný motorek</t>
         </is>
       </c>
       <c r="F651" t="inlineStr">
@@ -22131,22 +22135,22 @@
     </row>
     <row r="652">
       <c r="A652" t="n">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C652" t="inlineStr"/>
       <c r="D652" t="inlineStr">
         <is>
-          <t>oprava dveří na B pravé po směru jízdy</t>
+          <t>vadné čidlo množství písku M5</t>
         </is>
       </c>
       <c r="E652" t="inlineStr">
         <is>
-          <t>vadný motorek</t>
+          <t>2. osa pravo po smeru jizdy z B</t>
         </is>
       </c>
       <c r="F652" t="inlineStr">
@@ -22164,22 +22168,22 @@
     </row>
     <row r="653">
       <c r="A653" t="n">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C653" t="inlineStr"/>
       <c r="D653" t="inlineStr">
         <is>
-          <t>vadné čidlo množství písku M5</t>
+          <t>rychloměr dán do skladu na opravu</t>
         </is>
       </c>
       <c r="E653" t="inlineStr">
         <is>
-          <t>2. osa pravo po smeru jizdy z B</t>
+          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
         </is>
       </c>
       <c r="F653" t="inlineStr">
@@ -22197,22 +22201,22 @@
     </row>
     <row r="654">
       <c r="A654" t="n">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C654" t="inlineStr"/>
       <c r="D654" t="inlineStr">
         <is>
-          <t>rychloměr dán do skladu na opravu</t>
+          <t>rychloměr nekomunikuje</t>
         </is>
       </c>
       <c r="E654" t="inlineStr">
         <is>
-          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
+          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
         </is>
       </c>
       <c r="F654" t="inlineStr">
@@ -22230,22 +22234,26 @@
     </row>
     <row r="655">
       <c r="A655" t="n">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>844 022</t>
-        </is>
-      </c>
-      <c r="C655" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>10.08.2021</t>
+        </is>
+      </c>
       <c r="D655" t="inlineStr">
         <is>
-          <t>rychloměr nekomunikuje</t>
+          <t>dosazeny díly</t>
         </is>
       </c>
       <c r="E655" t="inlineStr">
         <is>
-          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
+          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
         </is>
       </c>
       <c r="F655" t="inlineStr">
@@ -22263,18 +22271,14 @@
     </row>
     <row r="656">
       <c r="A656" t="n">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B656" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C656" t="inlineStr">
-        <is>
-          <t>10.08.2021</t>
-        </is>
-      </c>
+      <c r="C656" t="inlineStr"/>
       <c r="D656" t="inlineStr">
         <is>
           <t>dosazeny díly</t>
@@ -22282,7 +22286,7 @@
       </c>
       <c r="E656" t="inlineStr">
         <is>
-          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
+          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
         </is>
       </c>
       <c r="F656" t="inlineStr">
@@ -22300,22 +22304,26 @@
     </row>
     <row r="657">
       <c r="A657" t="n">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B657" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C657" t="inlineStr"/>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>09.06.2021</t>
+        </is>
+      </c>
       <c r="D657" t="inlineStr">
         <is>
-          <t>dosazeny díly</t>
+          <t>Chybějící díly z důvodu použití na jinou lok.</t>
         </is>
       </c>
       <c r="E657" t="inlineStr">
         <is>
-          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
+          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
         </is>
       </c>
       <c r="F657" t="inlineStr">
@@ -22333,28 +22341,16 @@
     </row>
     <row r="658">
       <c r="A658" t="n">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C658" t="inlineStr">
-        <is>
-          <t>09.06.2021</t>
-        </is>
-      </c>
-      <c r="D658" t="inlineStr">
-        <is>
-          <t>Chybějící díly z důvodu použití na jinou lok.</t>
-        </is>
-      </c>
-      <c r="E658" t="inlineStr">
-        <is>
-          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
-        </is>
-      </c>
+          <t>842 015</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr"/>
+      <c r="D658" t="inlineStr"/>
+      <c r="E658" t="inlineStr"/>
       <c r="F658" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22370,15 +22366,19 @@
     </row>
     <row r="659">
       <c r="A659" t="n">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="B659" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C659" t="inlineStr"/>
-      <c r="D659" t="inlineStr"/>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>výměna obrazovky Lokel na 914</t>
+        </is>
+      </c>
       <c r="E659" t="inlineStr"/>
       <c r="F659" t="inlineStr">
         <is>
@@ -22395,17 +22395,17 @@
     </row>
     <row r="660">
       <c r="A660" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B660" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C660" t="inlineStr"/>
       <c r="D660" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E660" t="inlineStr"/>
@@ -22424,17 +22424,17 @@
     </row>
     <row r="661">
       <c r="A661" t="n">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="B661" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C661" t="inlineStr"/>
       <c r="D661" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E661" t="inlineStr"/>
@@ -22453,7 +22453,7 @@
     </row>
     <row r="662">
       <c r="A662" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B662" t="inlineStr">
         <is>
@@ -22463,10 +22463,14 @@
       <c r="C662" t="inlineStr"/>
       <c r="D662" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E662" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F662" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22482,24 +22486,20 @@
     </row>
     <row r="663">
       <c r="A663" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C663" t="inlineStr"/>
       <c r="D663" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E663" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr"/>
       <c r="F663" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22515,7 +22515,7 @@
     </row>
     <row r="664">
       <c r="A664" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B664" t="inlineStr">
         <is>
@@ -22525,7 +22525,7 @@
       <c r="C664" t="inlineStr"/>
       <c r="D664" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E664" t="inlineStr"/>
@@ -22544,17 +22544,17 @@
     </row>
     <row r="665">
       <c r="A665" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C665" t="inlineStr"/>
       <c r="D665" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E665" t="inlineStr"/>
@@ -22573,20 +22573,24 @@
     </row>
     <row r="666">
       <c r="A666" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C666" t="inlineStr"/>
       <c r="D666" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E666" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F666" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22602,7 +22606,7 @@
     </row>
     <row r="667">
       <c r="A667" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B667" t="inlineStr">
         <is>
@@ -22612,12 +22616,12 @@
       <c r="C667" t="inlineStr"/>
       <c r="D667" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E667" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F667" t="inlineStr">
@@ -22635,24 +22639,24 @@
     </row>
     <row r="668">
       <c r="A668" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B668" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C668" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D668" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E668" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr"/>
       <c r="F668" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22668,7 +22672,7 @@
     </row>
     <row r="669">
       <c r="A669" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B669" t="inlineStr">
         <is>
@@ -22677,12 +22681,12 @@
       </c>
       <c r="C669" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D669" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E669" t="inlineStr"/>
@@ -22701,7 +22705,7 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
@@ -22715,7 +22719,7 @@
       </c>
       <c r="D670" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E670" t="inlineStr"/>
@@ -22734,7 +22738,7 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
@@ -22748,10 +22752,14 @@
       </c>
       <c r="D671" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E671" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F671" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22767,7 +22775,7 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
@@ -22781,12 +22789,12 @@
       </c>
       <c r="D672" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E672" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F672" t="inlineStr">
@@ -22804,7 +22812,7 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
@@ -22818,14 +22826,10 @@
       </c>
       <c r="D673" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E673" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr"/>
       <c r="F673" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22841,24 +22845,24 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C674" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr"/>
       <c r="D674" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E674" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F674" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22874,24 +22878,20 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C675" t="inlineStr"/>
       <c r="D675" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E675" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr"/>
       <c r="F675" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22907,17 +22907,17 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C676" t="inlineStr"/>
       <c r="D676" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E676" t="inlineStr"/>
@@ -22936,7 +22936,7 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
@@ -22946,10 +22946,14 @@
       <c r="C677" t="inlineStr"/>
       <c r="D677" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E677" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F677" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22965,24 +22969,20 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C678" t="inlineStr"/>
       <c r="D678" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E678" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr"/>
       <c r="F678" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22998,7 +22998,7 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
@@ -23008,7 +23008,7 @@
       <c r="C679" t="inlineStr"/>
       <c r="D679" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E679" t="inlineStr"/>
@@ -23027,20 +23027,24 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C680" t="inlineStr"/>
       <c r="D680" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
-        </is>
-      </c>
-      <c r="E680" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F680" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23056,7 +23060,7 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
@@ -23066,14 +23070,10 @@
       <c r="C681" t="inlineStr"/>
       <c r="D681" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E681" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr"/>
       <c r="F681" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23089,7 +23089,7 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
@@ -23099,10 +23099,14 @@
       <c r="C682" t="inlineStr"/>
       <c r="D682" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E682" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F682" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23118,7 +23122,7 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
@@ -23128,14 +23132,10 @@
       <c r="C683" t="inlineStr"/>
       <c r="D683" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E683" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr"/>
       <c r="F683" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23151,7 +23151,7 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
@@ -23161,7 +23161,7 @@
       <c r="C684" t="inlineStr"/>
       <c r="D684" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E684" t="inlineStr"/>
@@ -23180,7 +23180,7 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
@@ -23190,10 +23190,14 @@
       <c r="C685" t="inlineStr"/>
       <c r="D685" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E685" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F685" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23209,7 +23213,7 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
@@ -23219,12 +23223,12 @@
       <c r="C686" t="inlineStr"/>
       <c r="D686" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E686" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F686" t="inlineStr">
@@ -23242,7 +23246,7 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
@@ -23252,12 +23256,12 @@
       <c r="C687" t="inlineStr"/>
       <c r="D687" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E687" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F687" t="inlineStr">
@@ -23275,24 +23279,20 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C688" t="inlineStr"/>
       <c r="D688" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E688" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr"/>
       <c r="F688" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23308,7 +23308,7 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
@@ -23318,10 +23318,14 @@
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E689" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F689" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23337,7 +23341,7 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
@@ -23347,12 +23351,12 @@
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E690" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F690" t="inlineStr">
@@ -23370,7 +23374,7 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
@@ -23380,14 +23384,10 @@
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E691" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr"/>
       <c r="F691" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23403,17 +23403,17 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E692" t="inlineStr"/>
@@ -23432,7 +23432,7 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
@@ -23442,10 +23442,14 @@
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E693" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F693" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23461,22 +23465,22 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C694" t="inlineStr"/>
       <c r="D694" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E694" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F694" t="inlineStr">
@@ -23494,7 +23498,7 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
@@ -23504,12 +23508,12 @@
       <c r="C695" t="inlineStr"/>
       <c r="D695" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E695" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F695" t="inlineStr">
@@ -23527,24 +23531,20 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C696" t="inlineStr"/>
       <c r="D696" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E696" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr"/>
       <c r="F696" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23560,23 +23560,27 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C697" t="inlineStr"/>
       <c r="D697" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E697" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F697" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G697" t="inlineStr"/>
@@ -23589,27 +23593,23 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C698" t="inlineStr"/>
       <c r="D698" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E698" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr"/>
       <c r="F698" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G698" t="inlineStr"/>
@@ -23622,7 +23622,7 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
@@ -23632,7 +23632,7 @@
       <c r="C699" t="inlineStr"/>
       <c r="D699" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E699" t="inlineStr"/>
@@ -23651,7 +23651,7 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
@@ -23661,7 +23661,7 @@
       <c r="C700" t="inlineStr"/>
       <c r="D700" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E700" t="inlineStr"/>
@@ -23680,7 +23680,7 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
@@ -23690,7 +23690,7 @@
       <c r="C701" t="inlineStr"/>
       <c r="D701" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E701" t="inlineStr"/>
@@ -23709,7 +23709,7 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
@@ -23719,10 +23719,14 @@
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E702" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F702" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23738,24 +23742,20 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E703" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr"/>
       <c r="F703" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23771,7 +23771,7 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
@@ -23781,7 +23781,7 @@
       <c r="C704" t="inlineStr"/>
       <c r="D704" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E704" t="inlineStr"/>
@@ -23800,20 +23800,24 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C705" t="inlineStr"/>
       <c r="D705" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E705" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F705" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23829,27 +23833,23 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C706" t="inlineStr"/>
       <c r="D706" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E706" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr"/>
       <c r="F706" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G706" t="inlineStr"/>
@@ -23862,7 +23862,7 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
@@ -23872,7 +23872,7 @@
       <c r="C707" t="inlineStr"/>
       <c r="D707" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E707" t="inlineStr"/>
@@ -23891,23 +23891,27 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C708" t="inlineStr"/>
       <c r="D708" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E708" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F708" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G708" t="inlineStr"/>
@@ -23920,27 +23924,31 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C709" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D709" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E709" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F709" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G709" t="inlineStr"/>
@@ -23953,11 +23961,11 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C710" t="inlineStr">
@@ -23967,12 +23975,12 @@
       </c>
       <c r="D710" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E710" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F710" t="inlineStr">
@@ -23990,26 +23998,26 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C711" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D711" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E711" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F711" t="inlineStr">
@@ -24027,31 +24035,27 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C712" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D712" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E712" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr"/>
       <c r="F712" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G712" t="inlineStr"/>
@@ -24064,27 +24068,27 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C713" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D713" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E713" t="inlineStr"/>
       <c r="F713" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G713" t="inlineStr"/>
@@ -24097,27 +24101,27 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C714" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D714" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E714" t="inlineStr"/>
       <c r="F714" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G714" t="inlineStr"/>
@@ -24130,27 +24134,27 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D715" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E715" t="inlineStr"/>
       <c r="F715" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G715" t="inlineStr"/>
@@ -24163,24 +24167,28 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C716" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D716" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E716" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F716" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -24196,11 +24204,11 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C717" t="inlineStr">
@@ -24210,12 +24218,12 @@
       </c>
       <c r="D717" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E717" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F717" t="inlineStr">
@@ -24233,11 +24241,11 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C718" t="inlineStr">
@@ -24247,7 +24255,7 @@
       </c>
       <c r="D718" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E718" t="inlineStr">
@@ -24270,31 +24278,31 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C719" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D719" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E719" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F719" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G719" t="inlineStr"/>
@@ -24307,31 +24315,27 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C720" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D720" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E720" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr"/>
       <c r="F720" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G720" t="inlineStr"/>
@@ -24344,27 +24348,31 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C721" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D721" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E721" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F721" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G721" t="inlineStr"/>
@@ -24377,26 +24385,22 @@
     </row>
     <row r="722">
       <c r="A722" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C722" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr"/>
       <c r="D722" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E722" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F722" t="inlineStr">
@@ -24414,30 +24418,38 @@
     </row>
     <row r="723">
       <c r="A723" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B723" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C723" t="inlineStr"/>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D723" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E723" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F723" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G723" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G723" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H723" t="inlineStr"/>
       <c r="I723" t="inlineStr">
         <is>
@@ -24447,38 +24459,34 @@
     </row>
     <row r="724">
       <c r="A724" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C724" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D724" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E724" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F724" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G724" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G724" t="inlineStr"/>
       <c r="H724" t="inlineStr"/>
       <c r="I724" t="inlineStr">
         <is>
@@ -24488,26 +24496,26 @@
     </row>
     <row r="725">
       <c r="A725" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C725" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D725" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E725" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F725" t="inlineStr">
@@ -24515,7 +24523,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G725" t="inlineStr"/>
+      <c r="G725" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H725" t="inlineStr"/>
       <c r="I725" t="inlineStr">
         <is>
@@ -24525,11 +24537,11 @@
     </row>
     <row r="726">
       <c r="A726" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
@@ -24539,67 +24551,26 @@
       </c>
       <c r="D726" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E726" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F726" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G726" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H726" t="inlineStr"/>
       <c r="I726" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="727">
-      <c r="A727" t="n">
-        <v>763</v>
-      </c>
-      <c r="B727" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C727" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D727" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E727" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F727" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G727" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H727" t="inlineStr"/>
-      <c r="I727" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 580 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I722"/>
+  <dimension ref="A1:I721"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18988,24 +18988,20 @@
     </row>
     <row r="557">
       <c r="A557" t="n">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>810 373</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C557" t="inlineStr"/>
       <c r="D557" t="inlineStr">
         <is>
-          <t>neseděli čísal jizdenek,řešil CAPSCH na dálku.Při vypnutí se automat hned vypl.Baterie měla 8,6V</t>
-        </is>
-      </c>
-      <c r="E557" t="inlineStr">
-        <is>
-          <t>výměna baterie</t>
-        </is>
-      </c>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr"/>
       <c r="F557" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19021,7 +19017,7 @@
     </row>
     <row r="558">
       <c r="A558" t="n">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B558" t="inlineStr">
         <is>
@@ -19031,10 +19027,14 @@
       <c r="C558" t="inlineStr"/>
       <c r="D558" t="inlineStr">
         <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E558" t="inlineStr"/>
+          <t>levé dveře na 914 se nezavírají</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>vadná optozávora - výměna</t>
+        </is>
+      </c>
       <c r="F558" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19050,22 +19050,18 @@
     </row>
     <row r="559">
       <c r="A559" t="n">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="B559" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>814 076</t>
         </is>
       </c>
       <c r="C559" t="inlineStr"/>
-      <c r="D559" t="inlineStr">
-        <is>
-          <t>levé dveře na 914 se nezavírají</t>
-        </is>
-      </c>
+      <c r="D559" t="inlineStr"/>
       <c r="E559" t="inlineStr">
         <is>
-          <t>vadná optozávora - výměna</t>
+          <t>vyčtení rychloměru</t>
         </is>
       </c>
       <c r="F559" t="inlineStr">
@@ -19083,18 +19079,26 @@
     </row>
     <row r="560">
       <c r="A560" t="n">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>814 076</t>
-        </is>
-      </c>
-      <c r="C560" t="inlineStr"/>
-      <c r="D560" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>22.06.2023</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>nasvěcuje se poruha mazání nákolků !MOK (přední stanoviště)</t>
+        </is>
+      </c>
       <c r="E560" t="inlineStr">
         <is>
-          <t>vyčtení rychloměru</t>
+          <t>při navolení přepínače SA90 do polohy plnění se závada cca 3x projevila,bohužel jsem nestihl doběhnout k obrazovce dřív než se zablokovala. Ale pravděpodobně nespína signál MOP (spíná ventil co pouští vzduch). Udělal jsem ještě profuk. Pravděpodobně to bylo někde přicpané a nedošlo ke změně tlaku na tlakáčích v bloku A61. Pro jistotu jsem ještě přehodil v DPV IN karty (první s druhou) a OUT karty.</t>
         </is>
       </c>
       <c r="F560" t="inlineStr">
@@ -19112,26 +19116,22 @@
     </row>
     <row r="561">
       <c r="A561" t="n">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="B561" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C561" t="inlineStr">
-        <is>
-          <t>22.06.2023</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr"/>
       <c r="D561" t="inlineStr">
         <is>
-          <t>nasvěcuje se poruha mazání nákolků !MOK (přední stanoviště)</t>
+          <t>často se navěcuje požár rozvaděče</t>
         </is>
       </c>
       <c r="E561" t="inlineStr">
         <is>
-          <t>při navolení přepínače SA90 do polohy plnění se závada cca 3x projevila,bohužel jsem nestihl doběhnout k obrazovce dřív než se zablokovala. Ale pravděpodobně nespína signál MOP (spíná ventil co pouští vzduch). Udělal jsem ještě profuk. Pravděpodobně to bylo někde přicpané a nedošlo ke změně tlaku na tlakáčích v bloku A61. Pro jistotu jsem ještě přehodil v DPV IN karty (první s druhou) a OUT karty.</t>
+          <t>neprojevilo se,výměna čidla požáru v RTO</t>
         </is>
       </c>
       <c r="F561" t="inlineStr">
@@ -19149,22 +19149,22 @@
     </row>
     <row r="562">
       <c r="A562" t="n">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C562" t="inlineStr"/>
       <c r="D562" t="inlineStr">
         <is>
-          <t>často se navěcuje požár rozvaděče</t>
+          <t>levé schody  na A nejdou</t>
         </is>
       </c>
       <c r="E562" t="inlineStr">
         <is>
-          <t>neprojevilo se,výměna čidla požáru v RTO</t>
+          <t>nečistoy kolem motoru+řemen</t>
         </is>
       </c>
       <c r="F562" t="inlineStr">
@@ -19182,22 +19182,22 @@
     </row>
     <row r="563">
       <c r="A563" t="n">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B563" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C563" t="inlineStr"/>
       <c r="D563" t="inlineStr">
         <is>
-          <t>levé schody  na A nejdou</t>
+          <t>údajne obrazovka IS v sekci B nad průchozími dveřmi ( směrem od WC) po tmě</t>
         </is>
       </c>
       <c r="E563" t="inlineStr">
         <is>
-          <t>nečistoy kolem motoru+řemen</t>
+          <t>neprojevilo se,kontrola konektorů,poklep obrazovka.Vše OK</t>
         </is>
       </c>
       <c r="F563" t="inlineStr">
@@ -19215,7 +19215,7 @@
     </row>
     <row r="564">
       <c r="A564" t="n">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B564" t="inlineStr">
         <is>
@@ -19225,12 +19225,12 @@
       <c r="C564" t="inlineStr"/>
       <c r="D564" t="inlineStr">
         <is>
-          <t>údajne obrazovka IS v sekci B nad průchozími dveřmi ( směrem od WC) po tmě</t>
+          <t>údajně problikává chyba čidla měření nafty</t>
         </is>
       </c>
       <c r="E564" t="inlineStr">
         <is>
-          <t>neprojevilo se,kontrola konektorů,poklep obrazovka.Vše OK</t>
+          <t>nenapsali jakého,neprojevilo se</t>
         </is>
       </c>
       <c r="F564" t="inlineStr">
@@ -19248,22 +19248,22 @@
     </row>
     <row r="565">
       <c r="A565" t="n">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B565" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C565" t="inlineStr"/>
       <c r="D565" t="inlineStr">
         <is>
-          <t>údajně problikává chyba čidla měření nafty</t>
+          <t>nechladí</t>
         </is>
       </c>
       <c r="E565" t="inlineStr">
         <is>
-          <t>nenapsali jakého,neprojevilo se</t>
+          <t>vydný proporcionální ventil,výměna</t>
         </is>
       </c>
       <c r="F565" t="inlineStr">
@@ -19281,22 +19281,22 @@
     </row>
     <row r="566">
       <c r="A566" t="n">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>842 015</t>
         </is>
       </c>
       <c r="C566" t="inlineStr"/>
       <c r="D566" t="inlineStr">
         <is>
-          <t>nechladí</t>
+          <t>někdy nejde brzda PB</t>
         </is>
       </c>
       <c r="E566" t="inlineStr">
         <is>
-          <t>vydný proporcionální ventil,výměna</t>
+          <t>výměna ventilu YV 61 včetně cívky</t>
         </is>
       </c>
       <c r="F566" t="inlineStr">
@@ -19314,22 +19314,22 @@
     </row>
     <row r="567">
       <c r="A567" t="n">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C567" t="inlineStr"/>
       <c r="D567" t="inlineStr">
         <is>
-          <t>někdy nejde brzda PB</t>
+          <t>v B salónu ukazuje prostřední čidlo 0°C</t>
         </is>
       </c>
       <c r="E567" t="inlineStr">
         <is>
-          <t>výměna ventilu YV 61 včetně cívky</t>
+          <t>po zahýbáním káblíku co vede ze stěny do svorkovnice čidla vše OK. Prodřený drát cca 5 cm od konce. Nasazení smršťovačky,přesvorkování dutinek</t>
         </is>
       </c>
       <c r="F567" t="inlineStr">
@@ -19347,22 +19347,22 @@
     </row>
     <row r="568">
       <c r="A568" t="n">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C568" t="inlineStr"/>
       <c r="D568" t="inlineStr">
         <is>
-          <t>v B salónu ukazuje prostřední čidlo 0°C</t>
+          <t>neukazuje vodoznak,pravá strana</t>
         </is>
       </c>
       <c r="E568" t="inlineStr">
         <is>
-          <t>po zahýbáním káblíku co vede ze stěny do svorkovnice čidla vše OK. Prodřený drát cca 5 cm od konce. Nasazení smršťovačky,přesvorkování dutinek</t>
+          <t>výměna</t>
         </is>
       </c>
       <c r="F568" t="inlineStr">
@@ -19380,22 +19380,22 @@
     </row>
     <row r="569">
       <c r="A569" t="n">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B569" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C569" t="inlineStr"/>
       <c r="D569" t="inlineStr">
         <is>
-          <t>neukazuje vodoznak,pravá strana</t>
+          <t>opět slabý výkon</t>
         </is>
       </c>
       <c r="E569" t="inlineStr">
         <is>
-          <t>výměna</t>
+          <t>byly "vyběhané" kloubky na táhlu AČ,výměna.Seřízení pákový,při 25% 930 otáček</t>
         </is>
       </c>
       <c r="F569" t="inlineStr">
@@ -19413,22 +19413,22 @@
     </row>
     <row r="570">
       <c r="A570" t="n">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>814 118</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C570" t="inlineStr"/>
       <c r="D570" t="inlineStr">
         <is>
-          <t>opět slabý výkon</t>
+          <t>údajně nejde ARR z B</t>
         </is>
       </c>
       <c r="E570" t="inlineStr">
         <is>
-          <t>byly "vyběhané" kloubky na táhlu AČ,výměna.Seřízení pákový,při 25% 930 otáček</t>
+          <t>neprojevilo se,neměněno</t>
         </is>
       </c>
       <c r="F570" t="inlineStr">
@@ -19446,7 +19446,7 @@
     </row>
     <row r="571">
       <c r="A571" t="n">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B571" t="inlineStr">
         <is>
@@ -19456,12 +19456,12 @@
       <c r="C571" t="inlineStr"/>
       <c r="D571" t="inlineStr">
         <is>
-          <t>údajně nejde ARR z B</t>
+          <t>v A salónu ukazuje prostřední čidlo -17°C</t>
         </is>
       </c>
       <c r="E571" t="inlineStr">
         <is>
-          <t>neprojevilo se,neměněno</t>
+          <t>ve skutečnosti se jedná o čidlo u měchů. 6.9.2021 se přehazovali vstupy do ŘJ mezi měchy a prostředkem. Chyba byla v prostředku. 2 roky pak byl klid. Proměření ohmicky cesty,vstupy dány zpět jak mají být. Pokud se vrátí zase v prostředku,chyba v ŘJ</t>
         </is>
       </c>
       <c r="F571" t="inlineStr">
@@ -19479,22 +19479,22 @@
     </row>
     <row r="572">
       <c r="A572" t="n">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>029 227</t>
         </is>
       </c>
       <c r="C572" t="inlineStr"/>
       <c r="D572" t="inlineStr">
         <is>
-          <t>v A salónu ukazuje prostřední čidlo -17°C</t>
+          <t>porucha dveří elektr.</t>
         </is>
       </c>
       <c r="E572" t="inlineStr">
         <is>
-          <t>ve skutečnosti se jedná o čidlo u měchů. 6.9.2021 se přehazovali vstupy do ŘJ mezi měchy a prostředkem. Chyba byla v prostředku. 2 roky pak byl klid. Proměření ohmicky cesty,vstupy dány zpět jak mají být. Pokud se vrátí zase v prostředku,chyba v ŘJ</t>
+          <t>neprojevilo se , přezkoušení stran</t>
         </is>
       </c>
       <c r="F572" t="inlineStr">
@@ -19512,22 +19512,22 @@
     </row>
     <row r="573">
       <c r="A573" t="n">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>029 227</t>
+          <t>742 263</t>
         </is>
       </c>
       <c r="C573" t="inlineStr"/>
       <c r="D573" t="inlineStr">
         <is>
-          <t>porucha dveří elektr.</t>
+          <t>při startu dlouho promázává, nejde zkrácený start</t>
         </is>
       </c>
       <c r="E573" t="inlineStr">
         <is>
-          <t>neprojevilo se , přezkoušení stran</t>
+          <t>vše bylo funkční , zkrácený start spíná při 49°C přesto výměna YCR7</t>
         </is>
       </c>
       <c r="F573" t="inlineStr">
@@ -19545,7 +19545,7 @@
     </row>
     <row r="574">
       <c r="A574" t="n">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B574" t="inlineStr">
         <is>
@@ -19555,12 +19555,12 @@
       <c r="C574" t="inlineStr"/>
       <c r="D574" t="inlineStr">
         <is>
-          <t>při startu dlouho promázává, nejde zkrácený start</t>
+          <t>porucha dveří elektr.</t>
         </is>
       </c>
       <c r="E574" t="inlineStr">
         <is>
-          <t>vše bylo funkční , zkrácený start spíná při 49°C přesto výměna YCR7</t>
+          <t>neprojevilo se , přezkoušení stran</t>
         </is>
       </c>
       <c r="F574" t="inlineStr">
@@ -19578,22 +19578,22 @@
     </row>
     <row r="575">
       <c r="A575" t="n">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B575" t="inlineStr">
         <is>
-          <t>742 263</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C575" t="inlineStr"/>
       <c r="D575" t="inlineStr">
         <is>
-          <t>porucha dveří elektr.</t>
+          <t>IS se rozpadá, ztráci komunikaci mezi stan.</t>
         </is>
       </c>
       <c r="E575" t="inlineStr">
         <is>
-          <t>neprojevilo se , přezkoušení stran</t>
+          <t>dotlační konektoru ale vše bylo funkční</t>
         </is>
       </c>
       <c r="F575" t="inlineStr">
@@ -19611,7 +19611,7 @@
     </row>
     <row r="576">
       <c r="A576" t="n">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B576" t="inlineStr">
         <is>
@@ -19621,12 +19621,12 @@
       <c r="C576" t="inlineStr"/>
       <c r="D576" t="inlineStr">
         <is>
-          <t>IS se rozpadá, ztráci komunikaci mezi stan.</t>
+          <t>parkovací brzda nevybaví KBS</t>
         </is>
       </c>
       <c r="E576" t="inlineStr">
         <is>
-          <t>dotlační konektoru ale vše bylo funkční</t>
+          <t>seřízení tlaku</t>
         </is>
       </c>
       <c r="F576" t="inlineStr">
@@ -19644,7 +19644,7 @@
     </row>
     <row r="577">
       <c r="A577" t="n">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="B577" t="inlineStr">
         <is>
@@ -19654,12 +19654,12 @@
       <c r="C577" t="inlineStr"/>
       <c r="D577" t="inlineStr">
         <is>
-          <t>parkovací brzda nevybaví KBS</t>
+          <t>únik oleje na 6. válci</t>
         </is>
       </c>
       <c r="E577" t="inlineStr">
         <is>
-          <t>seřízení tlaku</t>
+          <t>výměna</t>
         </is>
       </c>
       <c r="F577" t="inlineStr">
@@ -19677,7 +19677,7 @@
     </row>
     <row r="578">
       <c r="A578" t="n">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B578" t="inlineStr">
         <is>
@@ -19687,12 +19687,12 @@
       <c r="C578" t="inlineStr"/>
       <c r="D578" t="inlineStr">
         <is>
-          <t>únik oleje na 6. válci</t>
+          <t>nesvítí červené poziční světlo</t>
         </is>
       </c>
       <c r="E578" t="inlineStr">
         <is>
-          <t>výměna</t>
+          <t>zapojení vodiče 735 byl odpojený (výměna obou světel na stan 914)</t>
         </is>
       </c>
       <c r="F578" t="inlineStr">
@@ -19710,22 +19710,22 @@
     </row>
     <row r="579">
       <c r="A579" t="n">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="B579" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C579" t="inlineStr"/>
       <c r="D579" t="inlineStr">
         <is>
-          <t>nesvítí červené poziční světlo</t>
+          <t>nelze odbrzdit, tlak ve válcích zůstáva 0,3 bar závada jen z 914</t>
         </is>
       </c>
       <c r="E579" t="inlineStr">
         <is>
-          <t>zapojení vodiče 735 byl odpojený (výměna obou světel na stan 914)</t>
+          <t>zk. Jízda OK</t>
         </is>
       </c>
       <c r="F579" t="inlineStr">
@@ -19743,22 +19743,22 @@
     </row>
     <row r="580">
       <c r="A580" t="n">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B580" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C580" t="inlineStr"/>
       <c r="D580" t="inlineStr">
         <is>
-          <t>nelze odbrzdit, tlak ve válcích zůstáva 0,3 bar závada jen z 914</t>
+          <t>2.SM samovolně zvyšuje otáčky, seřízení GAC</t>
         </is>
       </c>
       <c r="E580" t="inlineStr">
         <is>
-          <t>zk. Jízda OK</t>
+          <t>přístě vyměnit GAC musela jet ven</t>
         </is>
       </c>
       <c r="F580" t="inlineStr">
@@ -19776,22 +19776,22 @@
     </row>
     <row r="581">
       <c r="A581" t="n">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="B581" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C581" t="inlineStr"/>
       <c r="D581" t="inlineStr">
         <is>
-          <t>2.SM samovolně zvyšuje otáčky, seřízení GAC</t>
+          <t>nehlási IS na stan. A</t>
         </is>
       </c>
       <c r="E581" t="inlineStr">
         <is>
-          <t>přístě vyměnit GAC musela jet ven</t>
+          <t>ztlumen potenciometr</t>
         </is>
       </c>
       <c r="F581" t="inlineStr">
@@ -19809,7 +19809,7 @@
     </row>
     <row r="582">
       <c r="A582" t="n">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B582" t="inlineStr">
         <is>
@@ -19819,12 +19819,12 @@
       <c r="C582" t="inlineStr"/>
       <c r="D582" t="inlineStr">
         <is>
-          <t>nehlási IS na stan. A</t>
+          <t>lednice nechladí</t>
         </is>
       </c>
       <c r="E582" t="inlineStr">
         <is>
-          <t>ztlumen potenciometr</t>
+          <t>odzkoušeno OK</t>
         </is>
       </c>
       <c r="F582" t="inlineStr">
@@ -19842,7 +19842,7 @@
     </row>
     <row r="583">
       <c r="A583" t="n">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B583" t="inlineStr">
         <is>
@@ -19852,12 +19852,12 @@
       <c r="C583" t="inlineStr"/>
       <c r="D583" t="inlineStr">
         <is>
-          <t>lednice nechladí</t>
+          <t>údajně rázy převodovky</t>
         </is>
       </c>
       <c r="E583" t="inlineStr">
         <is>
-          <t>odzkoušeno OK</t>
+          <t>řesí p. Šípek vyčítal jsi obě HMP</t>
         </is>
       </c>
       <c r="F583" t="inlineStr">
@@ -19875,22 +19875,22 @@
     </row>
     <row r="584">
       <c r="A584" t="n">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B584" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C584" t="inlineStr"/>
       <c r="D584" t="inlineStr">
         <is>
-          <t>údajně rázy převodovky</t>
+          <t>lok. Nejde nastartovat</t>
         </is>
       </c>
       <c r="E584" t="inlineStr">
         <is>
-          <t>řesí p. Šípek vyčítal jsi obě HMP</t>
+          <t>naftová netěsnost</t>
         </is>
       </c>
       <c r="F584" t="inlineStr">
@@ -19908,22 +19908,22 @@
     </row>
     <row r="585">
       <c r="A585" t="n">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B585" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C585" t="inlineStr"/>
       <c r="D585" t="inlineStr">
         <is>
-          <t>lok. Nejde nastartovat</t>
+          <t>izolačni stav odztraněny zkraty na vodiči 80 a 50</t>
         </is>
       </c>
       <c r="E585" t="inlineStr">
         <is>
-          <t>naftová netěsnost</t>
+          <t>startéry vyfoukany,ale nakonec výměna M2(volný pomocný vodič) seřízení GAC 2. SM , zkušební jízda se zdá v pořádku</t>
         </is>
       </c>
       <c r="F585" t="inlineStr">
@@ -19941,24 +19941,24 @@
     </row>
     <row r="586">
       <c r="A586" t="n">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B586" t="inlineStr">
         <is>
-          <t>842 035</t>
-        </is>
-      </c>
-      <c r="C586" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>06.12.2023</t>
+        </is>
+      </c>
       <c r="D586" t="inlineStr">
         <is>
-          <t>izolačni stav odztraněny zkraty na vodiči 80 a 50</t>
-        </is>
-      </c>
-      <c r="E586" t="inlineStr">
-        <is>
-          <t>startéry vyfoukany,ale nakonec výměna M2(volný pomocný vodič) seřízení GAC 2. SM , zkušební jízda se zdá v pořádku</t>
-        </is>
-      </c>
+          <t>Výměna obrazovky na 914 (občas zamrzá)</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr"/>
       <c r="F586" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19974,11 +19974,11 @@
     </row>
     <row r="587">
       <c r="A587" t="n">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B587" t="inlineStr">
         <is>
-          <t>814 003</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C587" t="inlineStr">
@@ -19988,7 +19988,7 @@
       </c>
       <c r="D587" t="inlineStr">
         <is>
-          <t>Výměna obrazovky na 914 (občas zamrzá)</t>
+          <t>údajně se rozpadá IS přezkoušeno (kontrola konektoru)</t>
         </is>
       </c>
       <c r="E587" t="inlineStr"/>
@@ -20007,11 +20007,11 @@
     </row>
     <row r="588">
       <c r="A588" t="n">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B588" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 072</t>
         </is>
       </c>
       <c r="C588" t="inlineStr">
@@ -20021,7 +20021,7 @@
       </c>
       <c r="D588" t="inlineStr">
         <is>
-          <t>údajně se rozpadá IS přezkoušeno (kontrola konektoru)</t>
+          <t>tozpadáva se IS, oprava dispeleje na 914 byl volný</t>
         </is>
       </c>
       <c r="E588" t="inlineStr"/>
@@ -20040,24 +20040,28 @@
     </row>
     <row r="589">
       <c r="A589" t="n">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B589" t="inlineStr">
         <is>
-          <t>814 072</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C589" t="inlineStr">
         <is>
-          <t>06.12.2023</t>
+          <t>06.11.2023</t>
         </is>
       </c>
       <c r="D589" t="inlineStr">
         <is>
-          <t>tozpadáva se IS, oprava dispeleje na 914 byl volný</t>
-        </is>
-      </c>
-      <c r="E589" t="inlineStr"/>
+          <t>tabule vnitřní , venkovní nekomunikují</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>výměna konektoru C na 914</t>
+        </is>
+      </c>
       <c r="F589" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20073,11 +20077,11 @@
     </row>
     <row r="590">
       <c r="A590" t="n">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B590" t="inlineStr">
         <is>
-          <t>814 118</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C590" t="inlineStr">
@@ -20087,12 +20091,12 @@
       </c>
       <c r="D590" t="inlineStr">
         <is>
-          <t>tabule vnitřní , venkovní nekomunikují</t>
+          <t>korekce vody 2</t>
         </is>
       </c>
       <c r="E590" t="inlineStr">
         <is>
-          <t>výměna konektoru C na 914</t>
+          <t>izolačni stav špatný  stáhlé zemni relé</t>
         </is>
       </c>
       <c r="F590" t="inlineStr">
@@ -20110,11 +20114,11 @@
     </row>
     <row r="591">
       <c r="A591" t="n">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B591" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C591" t="inlineStr">
@@ -20124,14 +20128,10 @@
       </c>
       <c r="D591" t="inlineStr">
         <is>
-          <t>korekce vody 2</t>
-        </is>
-      </c>
-      <c r="E591" t="inlineStr">
-        <is>
-          <t>izolačni stav špatný  stáhlé zemni relé</t>
-        </is>
-      </c>
+          <t>výměna ARR na B stan. Nefunkční</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr"/>
       <c r="F591" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20147,21 +20147,21 @@
     </row>
     <row r="592">
       <c r="A592" t="n">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>842 011</t>
         </is>
       </c>
       <c r="C592" t="inlineStr">
         <is>
-          <t>06.11.2023</t>
+          <t>06.10.2023</t>
         </is>
       </c>
       <c r="D592" t="inlineStr">
         <is>
-          <t>výměna ARR na B stan. Nefunkční</t>
+          <t>udajně zateklo do pultu na 2st.(kontrola)</t>
         </is>
       </c>
       <c r="E592" t="inlineStr"/>
@@ -20180,11 +20180,11 @@
     </row>
     <row r="593">
       <c r="A593" t="n">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>842 011</t>
+          <t>842 021</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
@@ -20194,10 +20194,14 @@
       </c>
       <c r="D593" t="inlineStr">
         <is>
-          <t>udajně zateklo do pultu na 2st.(kontrola)</t>
-        </is>
-      </c>
-      <c r="E593" t="inlineStr"/>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>vadné čidlo vody v míse</t>
+        </is>
+      </c>
       <c r="F593" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20213,26 +20217,26 @@
     </row>
     <row r="594">
       <c r="A594" t="n">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="B594" t="inlineStr">
         <is>
-          <t>842 021</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C594" t="inlineStr">
         <is>
-          <t>06.10.2023</t>
+          <t>06.09.2023</t>
         </is>
       </c>
       <c r="D594" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>Nejdou dvěře WC</t>
         </is>
       </c>
       <c r="E594" t="inlineStr">
         <is>
-          <t>vadné čidlo vody v míse</t>
+          <t>upadlý drát na přepínači funkce WC (zapnuto,bez dveří, vypnuto). Seřízení zámykání dveří. Frýdek</t>
         </is>
       </c>
       <c r="F594" t="inlineStr">
@@ -20250,11 +20254,11 @@
     </row>
     <row r="595">
       <c r="A595" t="n">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C595" t="inlineStr">
@@ -20264,12 +20268,12 @@
       </c>
       <c r="D595" t="inlineStr">
         <is>
-          <t>Nejdou dvěře WC</t>
+          <t>údajně nejdou někdy schody u levých dveří strany A</t>
         </is>
       </c>
       <c r="E595" t="inlineStr">
         <is>
-          <t>upadlý drát na přepínači funkce WC (zapnuto,bez dveří, vypnuto). Seřízení zámykání dveří. Frýdek</t>
+          <t>vyčištění od kamínků,odzkoušení-OK</t>
         </is>
       </c>
       <c r="F595" t="inlineStr">
@@ -20287,26 +20291,26 @@
     </row>
     <row r="596">
       <c r="A596" t="n">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="B596" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C596" t="inlineStr">
         <is>
-          <t>06.09.2023</t>
+          <t>06.08.2023</t>
         </is>
       </c>
       <c r="D596" t="inlineStr">
         <is>
-          <t>údajně nejdou někdy schody u levých dveří strany A</t>
+          <t>zapůjčena z HB</t>
         </is>
       </c>
       <c r="E596" t="inlineStr">
         <is>
-          <t>vyčištění od kamínků,odzkoušení-OK</t>
+          <t>nahrány data IS ( funguje preš radiostanici)</t>
         </is>
       </c>
       <c r="F596" t="inlineStr">
@@ -20324,11 +20328,11 @@
     </row>
     <row r="597">
       <c r="A597" t="n">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B597" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C597" t="inlineStr">
@@ -20338,12 +20342,12 @@
       </c>
       <c r="D597" t="inlineStr">
         <is>
-          <t>zapůjčena z HB</t>
+          <t>Opět problémy se startováním</t>
         </is>
       </c>
       <c r="E597" t="inlineStr">
         <is>
-          <t>nahrány data IS ( funguje preš radiostanici)</t>
+          <t>(asi už vadný capos kondy)říkali veselani jak tu byli</t>
         </is>
       </c>
       <c r="F597" t="inlineStr">
@@ -20361,7 +20365,7 @@
     </row>
     <row r="598">
       <c r="A598" t="n">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B598" t="inlineStr">
         <is>
@@ -20375,12 +20379,12 @@
       </c>
       <c r="D598" t="inlineStr">
         <is>
-          <t>Opět problémy se startováním</t>
+          <t>oprava hlasitosti na stanovišti A</t>
         </is>
       </c>
       <c r="E598" t="inlineStr">
         <is>
-          <t>(asi už vadný capos kondy)říkali veselani jak tu byli</t>
+          <t>přechod na kontaktech u reproduktoru v pultě</t>
         </is>
       </c>
       <c r="F598" t="inlineStr">
@@ -20398,11 +20402,11 @@
     </row>
     <row r="599">
       <c r="A599" t="n">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C599" t="inlineStr">
@@ -20412,12 +20416,12 @@
       </c>
       <c r="D599" t="inlineStr">
         <is>
-          <t>oprava hlasitosti na stanovišti A</t>
+          <t>výměna ARR na B</t>
         </is>
       </c>
       <c r="E599" t="inlineStr">
         <is>
-          <t>přechod na kontaktech u reproduktoru v pultě</t>
+          <t>vadná linka CAN</t>
         </is>
       </c>
       <c r="F599" t="inlineStr">
@@ -20435,26 +20439,26 @@
     </row>
     <row r="600">
       <c r="A600" t="n">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B600" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>842 015</t>
         </is>
       </c>
       <c r="C600" t="inlineStr">
         <is>
-          <t>06.08.2023</t>
+          <t>06.07.2023</t>
         </is>
       </c>
       <c r="D600" t="inlineStr">
         <is>
-          <t>výměna ARR na B</t>
+          <t>někdy nejde brzda PB</t>
         </is>
       </c>
       <c r="E600" t="inlineStr">
         <is>
-          <t>vadná linka CAN</t>
+          <t>výměna karty DS a OUT z 842 025</t>
         </is>
       </c>
       <c r="F600" t="inlineStr">
@@ -20472,11 +20476,11 @@
     </row>
     <row r="601">
       <c r="A601" t="n">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C601" t="inlineStr">
@@ -20486,14 +20490,10 @@
       </c>
       <c r="D601" t="inlineStr">
         <is>
-          <t>někdy nejde brzda PB</t>
-        </is>
-      </c>
-      <c r="E601" t="inlineStr">
-        <is>
-          <t>výměna karty DS a OUT z 842 025</t>
-        </is>
-      </c>
+          <t>dosazeny karty z 842 015 (DS a OUT)</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr"/>
       <c r="F601" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20509,11 +20509,11 @@
     </row>
     <row r="602">
       <c r="A602" t="n">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C602" t="inlineStr">
@@ -20523,10 +20523,14 @@
       </c>
       <c r="D602" t="inlineStr">
         <is>
-          <t>dosazeny karty z 842 015 (DS a OUT)</t>
-        </is>
-      </c>
-      <c r="E602" t="inlineStr"/>
+          <t>dosazen asi 5 dobíječ na B funkční</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>ve skladu nefunkční jenom (má řešit asi Mlíčko)</t>
+        </is>
+      </c>
       <c r="F602" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20542,28 +20546,24 @@
     </row>
     <row r="603">
       <c r="A603" t="n">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="B603" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 076</t>
         </is>
       </c>
       <c r="C603" t="inlineStr">
         <is>
-          <t>06.07.2023</t>
+          <t>06.06.2023</t>
         </is>
       </c>
       <c r="D603" t="inlineStr">
         <is>
-          <t>dosazen asi 5 dobíječ na B funkční</t>
-        </is>
-      </c>
-      <c r="E603" t="inlineStr">
-        <is>
-          <t>ve skladu nefunkční jenom (má řešit asi Mlíčko)</t>
-        </is>
-      </c>
+          <t>NEHODA V HOLEŠOVĚ</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr"/>
       <c r="F603" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20579,21 +20579,21 @@
     </row>
     <row r="604">
       <c r="A604" t="n">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="B604" t="inlineStr">
         <is>
-          <t>814 076</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C604" t="inlineStr">
         <is>
-          <t>06.06.2023</t>
+          <t>06.05.2023</t>
         </is>
       </c>
       <c r="D604" t="inlineStr">
         <is>
-          <t>NEHODA V HOLEŠOVĚ</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E604" t="inlineStr"/>
@@ -20612,21 +20612,17 @@
     </row>
     <row r="605">
       <c r="A605" t="n">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C605" t="inlineStr">
-        <is>
-          <t>06.05.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr"/>
       <c r="D605" t="inlineStr">
         <is>
-          <t>MM</t>
+          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
         </is>
       </c>
       <c r="E605" t="inlineStr"/>
@@ -20645,7 +20641,7 @@
     </row>
     <row r="606">
       <c r="A606" t="n">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="B606" t="inlineStr">
         <is>
@@ -20655,7 +20651,7 @@
       <c r="C606" t="inlineStr"/>
       <c r="D606" t="inlineStr">
         <is>
-          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
+          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
         </is>
       </c>
       <c r="E606" t="inlineStr"/>
@@ -20674,7 +20670,7 @@
     </row>
     <row r="607">
       <c r="A607" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B607" t="inlineStr">
         <is>
@@ -20684,7 +20680,7 @@
       <c r="C607" t="inlineStr"/>
       <c r="D607" t="inlineStr">
         <is>
-          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
+          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
         </is>
       </c>
       <c r="E607" t="inlineStr"/>
@@ -20703,20 +20699,24 @@
     </row>
     <row r="608">
       <c r="A608" t="n">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B608" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C608" t="inlineStr"/>
       <c r="D608" t="inlineStr">
         <is>
-          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
-        </is>
-      </c>
-      <c r="E608" t="inlineStr"/>
+          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>vyměnili dobíječ stacionární (Veselí)</t>
+        </is>
+      </c>
       <c r="F608" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20732,22 +20732,22 @@
     </row>
     <row r="609">
       <c r="A609" t="n">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C609" t="inlineStr"/>
       <c r="D609" t="inlineStr">
         <is>
-          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
         </is>
       </c>
       <c r="E609" t="inlineStr">
         <is>
-          <t>vyměnili dobíječ stacionární (Veselí)</t>
+          <t>jela ven</t>
         </is>
       </c>
       <c r="F609" t="inlineStr">
@@ -20765,24 +20765,20 @@
     </row>
     <row r="610">
       <c r="A610" t="n">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B610" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C610" t="inlineStr"/>
       <c r="D610" t="inlineStr">
         <is>
-          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
-        </is>
-      </c>
-      <c r="E610" t="inlineStr">
-        <is>
-          <t>jela ven</t>
-        </is>
-      </c>
+          <t>seřízení kamer přes program v notasu(obraz)</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr"/>
       <c r="F610" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20798,20 +20794,24 @@
     </row>
     <row r="611">
       <c r="A611" t="n">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B611" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C611" t="inlineStr"/>
       <c r="D611" t="inlineStr">
         <is>
-          <t>seřízení kamer přes program v notasu(obraz)</t>
-        </is>
-      </c>
-      <c r="E611" t="inlineStr"/>
+          <t>po startu někdy nenabíjí "B"</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+        </is>
+      </c>
       <c r="F611" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20827,22 +20827,22 @@
     </row>
     <row r="612">
       <c r="A612" t="n">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B612" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C612" t="inlineStr"/>
       <c r="D612" t="inlineStr">
         <is>
-          <t>po startu někdy nenabíjí "B"</t>
+          <t>2. motor korekce vody  vystup</t>
         </is>
       </c>
       <c r="E612" t="inlineStr">
         <is>
-          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
         </is>
       </c>
       <c r="F612" t="inlineStr">
@@ -20860,24 +20860,24 @@
     </row>
     <row r="613">
       <c r="A613" t="n">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>842 035</t>
-        </is>
-      </c>
-      <c r="C613" t="inlineStr"/>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>04.12.2023</t>
+        </is>
+      </c>
       <c r="D613" t="inlineStr">
         <is>
-          <t>2. motor korekce vody  vystup</t>
-        </is>
-      </c>
-      <c r="E613" t="inlineStr">
-        <is>
-          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
-        </is>
-      </c>
+          <t>Výměna motoru A</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr"/>
       <c r="F613" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20893,21 +20893,17 @@
     </row>
     <row r="614">
       <c r="A614" t="n">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B614" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C614" t="inlineStr">
-        <is>
-          <t>04.12.2023</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr"/>
       <c r="D614" t="inlineStr">
         <is>
-          <t>Výměna motoru A</t>
+          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
         </is>
       </c>
       <c r="E614" t="inlineStr"/>
@@ -20926,17 +20922,17 @@
     </row>
     <row r="615">
       <c r="A615" t="n">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C615" t="inlineStr"/>
       <c r="D615" t="inlineStr">
         <is>
-          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
+          <t>dosazena nahadni Mirelka + NO z 844 013</t>
         </is>
       </c>
       <c r="E615" t="inlineStr"/>
@@ -20955,17 +20951,17 @@
     </row>
     <row r="616">
       <c r="A616" t="n">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B616" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 062</t>
         </is>
       </c>
       <c r="C616" t="inlineStr"/>
       <c r="D616" t="inlineStr">
         <is>
-          <t>dosazena nahadni Mirelka + NO z 844 013</t>
+          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
         </is>
       </c>
       <c r="E616" t="inlineStr"/>
@@ -20984,17 +20980,21 @@
     </row>
     <row r="617">
       <c r="A617" t="n">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>814 062</t>
-        </is>
-      </c>
-      <c r="C617" t="inlineStr"/>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>03.03.2023</t>
+        </is>
+      </c>
       <c r="D617" t="inlineStr">
         <is>
-          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E617" t="inlineStr"/>
@@ -21013,11 +21013,11 @@
     </row>
     <row r="618">
       <c r="A618" t="n">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B618" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C618" t="inlineStr">
@@ -21027,7 +21027,7 @@
       </c>
       <c r="D618" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
+          <t>Dosazení ŘJ kamer</t>
         </is>
       </c>
       <c r="E618" t="inlineStr"/>
@@ -21046,24 +21046,24 @@
     </row>
     <row r="619">
       <c r="A619" t="n">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>844 013</t>
-        </is>
-      </c>
-      <c r="C619" t="inlineStr">
-        <is>
-          <t>03.03.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr"/>
       <c r="D619" t="inlineStr">
         <is>
-          <t>Dosazení ŘJ kamer</t>
-        </is>
-      </c>
-      <c r="E619" t="inlineStr"/>
+          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>hlášeno p. Škodovi</t>
+        </is>
+      </c>
       <c r="F619" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21079,24 +21079,20 @@
     </row>
     <row r="620">
       <c r="A620" t="n">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C620" t="inlineStr"/>
       <c r="D620" t="inlineStr">
         <is>
-          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
-        </is>
-      </c>
-      <c r="E620" t="inlineStr">
-        <is>
-          <t>hlášeno p. Škodovi</t>
-        </is>
-      </c>
+          <t>ŘJ kamer dosazena z 013</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr"/>
       <c r="F620" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21112,17 +21108,21 @@
     </row>
     <row r="621">
       <c r="A621" t="n">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B621" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C621" t="inlineStr"/>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>02.09.2023</t>
+        </is>
+      </c>
       <c r="D621" t="inlineStr">
         <is>
-          <t>ŘJ kamer dosazena z 013</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E621" t="inlineStr"/>
@@ -21141,21 +21141,21 @@
     </row>
     <row r="622">
       <c r="A622" t="n">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 072</t>
         </is>
       </c>
       <c r="C622" t="inlineStr">
         <is>
-          <t>02.09.2023</t>
+          <t>02.03.2023</t>
         </is>
       </c>
       <c r="D622" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E622" t="inlineStr"/>
@@ -21174,24 +21174,24 @@
     </row>
     <row r="623">
       <c r="A623" t="n">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B623" t="inlineStr">
         <is>
-          <t>814 072</t>
-        </is>
-      </c>
-      <c r="C623" t="inlineStr">
-        <is>
-          <t>02.03.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr"/>
       <c r="D623" t="inlineStr">
         <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E623" t="inlineStr"/>
+          <t>dosazen opraveny MIREL</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+        </is>
+      </c>
       <c r="F623" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21207,22 +21207,22 @@
     </row>
     <row r="624">
       <c r="A624" t="n">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C624" t="inlineStr"/>
       <c r="D624" t="inlineStr">
         <is>
-          <t>dosazen opraveny MIREL</t>
+          <t>Odpojen trojcestný ventil na A i B</t>
         </is>
       </c>
       <c r="E624" t="inlineStr">
         <is>
-          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+          <t>Zapojeny zpět 24.2.2023</t>
         </is>
       </c>
       <c r="F624" t="inlineStr">
@@ -21240,24 +21240,20 @@
     </row>
     <row r="625">
       <c r="A625" t="n">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B625" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C625" t="inlineStr"/>
       <c r="D625" t="inlineStr">
         <is>
-          <t>Odpojen trojcestný ventil na A i B</t>
-        </is>
-      </c>
-      <c r="E625" t="inlineStr">
-        <is>
-          <t>Zapojeny zpět 24.2.2023</t>
-        </is>
-      </c>
+          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr"/>
       <c r="F625" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21273,17 +21269,21 @@
     </row>
     <row r="626">
       <c r="A626" t="n">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B626" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C626" t="inlineStr"/>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>01.10.2023</t>
+        </is>
+      </c>
       <c r="D626" t="inlineStr">
         <is>
-          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E626" t="inlineStr"/>
@@ -21302,21 +21302,17 @@
     </row>
     <row r="627">
       <c r="A627" t="n">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C627" t="inlineStr">
-        <is>
-          <t>01.10.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr"/>
       <c r="D627" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
         </is>
       </c>
       <c r="E627" t="inlineStr"/>
@@ -21335,17 +21331,17 @@
     </row>
     <row r="628">
       <c r="A628" t="n">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C628" t="inlineStr"/>
       <c r="D628" t="inlineStr">
         <is>
-          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
+          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
         </is>
       </c>
       <c r="E628" t="inlineStr"/>
@@ -21364,7 +21360,7 @@
     </row>
     <row r="629">
       <c r="A629" t="n">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B629" t="inlineStr">
         <is>
@@ -21374,7 +21370,7 @@
       <c r="C629" t="inlineStr"/>
       <c r="D629" t="inlineStr">
         <is>
-          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
+          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
         </is>
       </c>
       <c r="E629" t="inlineStr"/>
@@ -21393,20 +21389,24 @@
     </row>
     <row r="630">
       <c r="A630" t="n">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C630" t="inlineStr"/>
       <c r="D630" t="inlineStr">
         <is>
-          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
-        </is>
-      </c>
-      <c r="E630" t="inlineStr"/>
+          <t>Přišel opravený Mirel ve skladu</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>dosazen na 29.12.2022</t>
+        </is>
+      </c>
       <c r="F630" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21422,22 +21422,26 @@
     </row>
     <row r="631">
       <c r="A631" t="n">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C631" t="inlineStr"/>
+          <t>844 014</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>12.06.2022</t>
+        </is>
+      </c>
       <c r="D631" t="inlineStr">
         <is>
-          <t>Přišel opravený Mirel ve skladu</t>
+          <t>rychloměr do opravy hazí !!</t>
         </is>
       </c>
       <c r="E631" t="inlineStr">
         <is>
-          <t>dosazen na 29.12.2022</t>
+          <t>zapujcen z 844 028 z veselí</t>
         </is>
       </c>
       <c r="F631" t="inlineStr">
@@ -21455,11 +21459,11 @@
     </row>
     <row r="632">
       <c r="A632" t="n">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C632" t="inlineStr">
@@ -21469,14 +21473,10 @@
       </c>
       <c r="D632" t="inlineStr">
         <is>
-          <t>rychloměr do opravy hazí !!</t>
-        </is>
-      </c>
-      <c r="E632" t="inlineStr">
-        <is>
-          <t>zapujcen z 844 028 z veselí</t>
-        </is>
-      </c>
+          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr"/>
       <c r="F632" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21492,24 +21492,28 @@
     </row>
     <row r="633">
       <c r="A633" t="n">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C633" t="inlineStr">
         <is>
-          <t>12.06.2022</t>
+          <t>12.03.2022</t>
         </is>
       </c>
       <c r="D633" t="inlineStr">
         <is>
-          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
-        </is>
-      </c>
-      <c r="E633" t="inlineStr"/>
+          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>bude řešit Škoda</t>
+        </is>
+      </c>
       <c r="F633" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21525,26 +21529,22 @@
     </row>
     <row r="634">
       <c r="A634" t="n">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B634" t="inlineStr">
         <is>
           <t>844 003</t>
         </is>
       </c>
-      <c r="C634" t="inlineStr">
-        <is>
-          <t>12.03.2022</t>
-        </is>
-      </c>
+      <c r="C634" t="inlineStr"/>
       <c r="D634" t="inlineStr">
         <is>
-          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+          <t>na A strane asi vadna expanzní nadrz topení ?</t>
         </is>
       </c>
       <c r="E634" t="inlineStr">
         <is>
-          <t>bude řešit Škoda</t>
+          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
         </is>
       </c>
       <c r="F634" t="inlineStr">
@@ -21562,22 +21562,22 @@
     </row>
     <row r="635">
       <c r="A635" t="n">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C635" t="inlineStr"/>
       <c r="D635" t="inlineStr">
         <is>
-          <t>na A strane asi vadna expanzní nadrz topení ?</t>
+          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
         </is>
       </c>
       <c r="E635" t="inlineStr">
         <is>
-          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
+          <t>nová obrazovka hazela vykricnik porad</t>
         </is>
       </c>
       <c r="F635" t="inlineStr">
@@ -21595,24 +21595,24 @@
     </row>
     <row r="636">
       <c r="A636" t="n">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C636" t="inlineStr"/>
+          <t>842 010</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>11.06.2022</t>
+        </is>
+      </c>
       <c r="D636" t="inlineStr">
         <is>
-          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
-        </is>
-      </c>
-      <c r="E636" t="inlineStr">
-        <is>
-          <t>nová obrazovka hazela vykricnik porad</t>
-        </is>
-      </c>
+          <t>Přehození karty TBA v DPV na 842 036</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr"/>
       <c r="F636" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21628,11 +21628,11 @@
     </row>
     <row r="637">
       <c r="A637" t="n">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>842 010</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C637" t="inlineStr">
@@ -21642,7 +21642,7 @@
       </c>
       <c r="D637" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 036</t>
+          <t>Přehození karty TBA v DPV na 842 010</t>
         </is>
       </c>
       <c r="E637" t="inlineStr"/>
@@ -21661,11 +21661,11 @@
     </row>
     <row r="638">
       <c r="A638" t="n">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C638" t="inlineStr">
@@ -21675,10 +21675,14 @@
       </c>
       <c r="D638" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 010</t>
-        </is>
-      </c>
-      <c r="E638" t="inlineStr"/>
+          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>mirel byl špatný po opravě</t>
+        </is>
+      </c>
       <c r="F638" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21694,26 +21698,26 @@
     </row>
     <row r="639">
       <c r="A639" t="n">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C639" t="inlineStr">
         <is>
-          <t>11.06.2022</t>
+          <t>11.05.2022</t>
         </is>
       </c>
       <c r="D639" t="inlineStr">
         <is>
-          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
         </is>
       </c>
       <c r="E639" t="inlineStr">
         <is>
-          <t>mirel byl špatný po opravě</t>
+          <t>25.11. opraveno</t>
         </is>
       </c>
       <c r="F639" t="inlineStr">
@@ -21731,11 +21735,11 @@
     </row>
     <row r="640">
       <c r="A640" t="n">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C640" t="inlineStr">
@@ -21745,14 +21749,10 @@
       </c>
       <c r="D640" t="inlineStr">
         <is>
-          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
-        </is>
-      </c>
-      <c r="E640" t="inlineStr">
-        <is>
-          <t>25.11. opraveno</t>
-        </is>
-      </c>
+          <t>VESELÍ R3 (odjela)</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr"/>
       <c r="F640" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21768,24 +21768,24 @@
     </row>
     <row r="641">
       <c r="A641" t="n">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>844 020</t>
-        </is>
-      </c>
-      <c r="C641" t="inlineStr">
-        <is>
-          <t>11.05.2022</t>
-        </is>
-      </c>
+          <t>814 190</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr"/>
       <c r="D641" t="inlineStr">
         <is>
-          <t>VESELÍ R3 (odjela)</t>
-        </is>
-      </c>
-      <c r="E641" t="inlineStr"/>
+          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>hlášeno p.Škodovi</t>
+        </is>
+      </c>
       <c r="F641" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21801,22 +21801,22 @@
     </row>
     <row r="642">
       <c r="A642" t="n">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>814 190</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C642" t="inlineStr"/>
       <c r="D642" t="inlineStr">
         <is>
-          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
         </is>
       </c>
       <c r="E642" t="inlineStr">
         <is>
-          <t>hlášeno p.Škodovi</t>
+          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
         </is>
       </c>
       <c r="F642" t="inlineStr">
@@ -21834,24 +21834,20 @@
     </row>
     <row r="643">
       <c r="A643" t="n">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C643" t="inlineStr"/>
       <c r="D643" t="inlineStr">
         <is>
-          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
-        </is>
-      </c>
-      <c r="E643" t="inlineStr">
-        <is>
-          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
-        </is>
-      </c>
+          <t>dosazen předzesilovač linky</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr"/>
       <c r="F643" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21867,20 +21863,28 @@
     </row>
     <row r="644">
       <c r="A644" t="n">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B644" t="inlineStr">
         <is>
           <t>814 073</t>
         </is>
       </c>
-      <c r="C644" t="inlineStr"/>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>09.07.2022</t>
+        </is>
+      </c>
       <c r="D644" t="inlineStr">
         <is>
-          <t>dosazen předzesilovač linky</t>
-        </is>
-      </c>
-      <c r="E644" t="inlineStr"/>
+          <t>chybějící díl</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>předzasilovač linky - objednán nový</t>
+        </is>
+      </c>
       <c r="F644" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21896,26 +21900,26 @@
     </row>
     <row r="645">
       <c r="A645" t="n">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 003</t>
         </is>
       </c>
       <c r="C645" t="inlineStr">
         <is>
-          <t>09.07.2022</t>
+          <t>09.03.2022</t>
         </is>
       </c>
       <c r="D645" t="inlineStr">
         <is>
-          <t>chybějící díl</t>
+          <t>dosazen díl</t>
         </is>
       </c>
       <c r="E645" t="inlineStr">
         <is>
-          <t>předzasilovač linky - objednán nový</t>
+          <t>dosazen předzasilovač linky A23</t>
         </is>
       </c>
       <c r="F645" t="inlineStr">
@@ -21933,26 +21937,22 @@
     </row>
     <row r="646">
       <c r="A646" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C646" t="inlineStr">
-        <is>
-          <t>09.03.2022</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr"/>
       <c r="D646" t="inlineStr">
         <is>
-          <t>dosazen díl</t>
+          <t>oprava dveří na B pravé po směru jízdy</t>
         </is>
       </c>
       <c r="E646" t="inlineStr">
         <is>
-          <t>dosazen předzasilovač linky A23</t>
+          <t>vadný motorek</t>
         </is>
       </c>
       <c r="F646" t="inlineStr">
@@ -21970,22 +21970,22 @@
     </row>
     <row r="647">
       <c r="A647" t="n">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C647" t="inlineStr"/>
       <c r="D647" t="inlineStr">
         <is>
-          <t>oprava dveří na B pravé po směru jízdy</t>
+          <t>vadné čidlo množství písku M5</t>
         </is>
       </c>
       <c r="E647" t="inlineStr">
         <is>
-          <t>vadný motorek</t>
+          <t>2. osa pravo po smeru jizdy z B</t>
         </is>
       </c>
       <c r="F647" t="inlineStr">
@@ -22003,22 +22003,22 @@
     </row>
     <row r="648">
       <c r="A648" t="n">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C648" t="inlineStr"/>
       <c r="D648" t="inlineStr">
         <is>
-          <t>vadné čidlo množství písku M5</t>
+          <t>rychloměr dán do skladu na opravu</t>
         </is>
       </c>
       <c r="E648" t="inlineStr">
         <is>
-          <t>2. osa pravo po smeru jizdy z B</t>
+          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
         </is>
       </c>
       <c r="F648" t="inlineStr">
@@ -22036,22 +22036,22 @@
     </row>
     <row r="649">
       <c r="A649" t="n">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C649" t="inlineStr"/>
       <c r="D649" t="inlineStr">
         <is>
-          <t>rychloměr dán do skladu na opravu</t>
+          <t>rychloměr nekomunikuje</t>
         </is>
       </c>
       <c r="E649" t="inlineStr">
         <is>
-          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
+          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
         </is>
       </c>
       <c r="F649" t="inlineStr">
@@ -22069,22 +22069,26 @@
     </row>
     <row r="650">
       <c r="A650" t="n">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>844 022</t>
-        </is>
-      </c>
-      <c r="C650" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>10.08.2021</t>
+        </is>
+      </c>
       <c r="D650" t="inlineStr">
         <is>
-          <t>rychloměr nekomunikuje</t>
+          <t>dosazeny díly</t>
         </is>
       </c>
       <c r="E650" t="inlineStr">
         <is>
-          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
+          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
         </is>
       </c>
       <c r="F650" t="inlineStr">
@@ -22102,18 +22106,14 @@
     </row>
     <row r="651">
       <c r="A651" t="n">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B651" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C651" t="inlineStr">
-        <is>
-          <t>10.08.2021</t>
-        </is>
-      </c>
+      <c r="C651" t="inlineStr"/>
       <c r="D651" t="inlineStr">
         <is>
           <t>dosazeny díly</t>
@@ -22121,7 +22121,7 @@
       </c>
       <c r="E651" t="inlineStr">
         <is>
-          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
+          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
         </is>
       </c>
       <c r="F651" t="inlineStr">
@@ -22139,22 +22139,26 @@
     </row>
     <row r="652">
       <c r="A652" t="n">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B652" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C652" t="inlineStr"/>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>09.06.2021</t>
+        </is>
+      </c>
       <c r="D652" t="inlineStr">
         <is>
-          <t>dosazeny díly</t>
+          <t>Chybějící díly z důvodu použití na jinou lok.</t>
         </is>
       </c>
       <c r="E652" t="inlineStr">
         <is>
-          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
+          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
         </is>
       </c>
       <c r="F652" t="inlineStr">
@@ -22172,28 +22176,16 @@
     </row>
     <row r="653">
       <c r="A653" t="n">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C653" t="inlineStr">
-        <is>
-          <t>09.06.2021</t>
-        </is>
-      </c>
-      <c r="D653" t="inlineStr">
-        <is>
-          <t>Chybějící díly z důvodu použití na jinou lok.</t>
-        </is>
-      </c>
-      <c r="E653" t="inlineStr">
-        <is>
-          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
-        </is>
-      </c>
+          <t>842 015</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr"/>
+      <c r="D653" t="inlineStr"/>
+      <c r="E653" t="inlineStr"/>
       <c r="F653" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22209,15 +22201,19 @@
     </row>
     <row r="654">
       <c r="A654" t="n">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C654" t="inlineStr"/>
-      <c r="D654" t="inlineStr"/>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>výměna obrazovky Lokel na 914</t>
+        </is>
+      </c>
       <c r="E654" t="inlineStr"/>
       <c r="F654" t="inlineStr">
         <is>
@@ -22234,17 +22230,17 @@
     </row>
     <row r="655">
       <c r="A655" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C655" t="inlineStr"/>
       <c r="D655" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E655" t="inlineStr"/>
@@ -22263,17 +22259,17 @@
     </row>
     <row r="656">
       <c r="A656" t="n">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C656" t="inlineStr"/>
       <c r="D656" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E656" t="inlineStr"/>
@@ -22292,7 +22288,7 @@
     </row>
     <row r="657">
       <c r="A657" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B657" t="inlineStr">
         <is>
@@ -22302,10 +22298,14 @@
       <c r="C657" t="inlineStr"/>
       <c r="D657" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E657" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F657" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22321,24 +22321,20 @@
     </row>
     <row r="658">
       <c r="A658" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C658" t="inlineStr"/>
       <c r="D658" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E658" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr"/>
       <c r="F658" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22354,7 +22350,7 @@
     </row>
     <row r="659">
       <c r="A659" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B659" t="inlineStr">
         <is>
@@ -22364,7 +22360,7 @@
       <c r="C659" t="inlineStr"/>
       <c r="D659" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E659" t="inlineStr"/>
@@ -22383,17 +22379,17 @@
     </row>
     <row r="660">
       <c r="A660" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B660" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C660" t="inlineStr"/>
       <c r="D660" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E660" t="inlineStr"/>
@@ -22412,20 +22408,24 @@
     </row>
     <row r="661">
       <c r="A661" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B661" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C661" t="inlineStr"/>
       <c r="D661" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E661" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F661" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22441,7 +22441,7 @@
     </row>
     <row r="662">
       <c r="A662" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B662" t="inlineStr">
         <is>
@@ -22451,12 +22451,12 @@
       <c r="C662" t="inlineStr"/>
       <c r="D662" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E662" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F662" t="inlineStr">
@@ -22474,24 +22474,24 @@
     </row>
     <row r="663">
       <c r="A663" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C663" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E663" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr"/>
       <c r="F663" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22507,7 +22507,7 @@
     </row>
     <row r="664">
       <c r="A664" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B664" t="inlineStr">
         <is>
@@ -22516,12 +22516,12 @@
       </c>
       <c r="C664" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D664" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E664" t="inlineStr"/>
@@ -22540,7 +22540,7 @@
     </row>
     <row r="665">
       <c r="A665" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B665" t="inlineStr">
         <is>
@@ -22554,7 +22554,7 @@
       </c>
       <c r="D665" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E665" t="inlineStr"/>
@@ -22573,7 +22573,7 @@
     </row>
     <row r="666">
       <c r="A666" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B666" t="inlineStr">
         <is>
@@ -22587,10 +22587,14 @@
       </c>
       <c r="D666" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E666" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F666" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22606,7 +22610,7 @@
     </row>
     <row r="667">
       <c r="A667" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B667" t="inlineStr">
         <is>
@@ -22620,12 +22624,12 @@
       </c>
       <c r="D667" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E667" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F667" t="inlineStr">
@@ -22643,7 +22647,7 @@
     </row>
     <row r="668">
       <c r="A668" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B668" t="inlineStr">
         <is>
@@ -22657,14 +22661,10 @@
       </c>
       <c r="D668" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E668" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr"/>
       <c r="F668" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22680,24 +22680,24 @@
     </row>
     <row r="669">
       <c r="A669" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C669" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr"/>
       <c r="D669" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E669" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F669" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22713,24 +22713,20 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C670" t="inlineStr"/>
       <c r="D670" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E670" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr"/>
       <c r="F670" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22746,17 +22742,17 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C671" t="inlineStr"/>
       <c r="D671" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E671" t="inlineStr"/>
@@ -22775,7 +22771,7 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
@@ -22785,10 +22781,14 @@
       <c r="C672" t="inlineStr"/>
       <c r="D672" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E672" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F672" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22804,24 +22804,20 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C673" t="inlineStr"/>
       <c r="D673" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E673" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr"/>
       <c r="F673" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22837,7 +22833,7 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
@@ -22847,7 +22843,7 @@
       <c r="C674" t="inlineStr"/>
       <c r="D674" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E674" t="inlineStr"/>
@@ -22866,20 +22862,24 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C675" t="inlineStr"/>
       <c r="D675" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
-        </is>
-      </c>
-      <c r="E675" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F675" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22895,7 +22895,7 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
@@ -22905,14 +22905,10 @@
       <c r="C676" t="inlineStr"/>
       <c r="D676" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E676" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr"/>
       <c r="F676" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22928,7 +22924,7 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
@@ -22938,10 +22934,14 @@
       <c r="C677" t="inlineStr"/>
       <c r="D677" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E677" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F677" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22957,7 +22957,7 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
@@ -22967,14 +22967,10 @@
       <c r="C678" t="inlineStr"/>
       <c r="D678" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E678" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr"/>
       <c r="F678" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22990,7 +22986,7 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
@@ -23000,7 +22996,7 @@
       <c r="C679" t="inlineStr"/>
       <c r="D679" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E679" t="inlineStr"/>
@@ -23019,7 +23015,7 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
@@ -23029,10 +23025,14 @@
       <c r="C680" t="inlineStr"/>
       <c r="D680" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E680" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F680" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23048,7 +23048,7 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
@@ -23058,12 +23058,12 @@
       <c r="C681" t="inlineStr"/>
       <c r="D681" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E681" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F681" t="inlineStr">
@@ -23081,7 +23081,7 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
@@ -23091,12 +23091,12 @@
       <c r="C682" t="inlineStr"/>
       <c r="D682" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E682" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F682" t="inlineStr">
@@ -23114,24 +23114,20 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C683" t="inlineStr"/>
       <c r="D683" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E683" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr"/>
       <c r="F683" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23147,7 +23143,7 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
@@ -23157,10 +23153,14 @@
       <c r="C684" t="inlineStr"/>
       <c r="D684" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E684" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F684" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23176,7 +23176,7 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
@@ -23186,12 +23186,12 @@
       <c r="C685" t="inlineStr"/>
       <c r="D685" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E685" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F685" t="inlineStr">
@@ -23209,7 +23209,7 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
@@ -23219,14 +23219,10 @@
       <c r="C686" t="inlineStr"/>
       <c r="D686" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E686" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr"/>
       <c r="F686" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23242,17 +23238,17 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C687" t="inlineStr"/>
       <c r="D687" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E687" t="inlineStr"/>
@@ -23271,7 +23267,7 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
@@ -23281,10 +23277,14 @@
       <c r="C688" t="inlineStr"/>
       <c r="D688" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E688" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F688" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23300,22 +23300,22 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E689" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F689" t="inlineStr">
@@ -23333,7 +23333,7 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
@@ -23343,12 +23343,12 @@
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E690" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F690" t="inlineStr">
@@ -23366,24 +23366,20 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E691" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr"/>
       <c r="F691" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23399,23 +23395,27 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E692" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F692" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G692" t="inlineStr"/>
@@ -23428,27 +23428,23 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E693" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr"/>
       <c r="F693" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G693" t="inlineStr"/>
@@ -23461,7 +23457,7 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
@@ -23471,7 +23467,7 @@
       <c r="C694" t="inlineStr"/>
       <c r="D694" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E694" t="inlineStr"/>
@@ -23490,7 +23486,7 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
@@ -23500,7 +23496,7 @@
       <c r="C695" t="inlineStr"/>
       <c r="D695" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E695" t="inlineStr"/>
@@ -23519,7 +23515,7 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
@@ -23529,7 +23525,7 @@
       <c r="C696" t="inlineStr"/>
       <c r="D696" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E696" t="inlineStr"/>
@@ -23548,7 +23544,7 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
@@ -23558,10 +23554,14 @@
       <c r="C697" t="inlineStr"/>
       <c r="D697" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E697" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F697" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23577,24 +23577,20 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C698" t="inlineStr"/>
       <c r="D698" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E698" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr"/>
       <c r="F698" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23610,7 +23606,7 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
@@ -23620,7 +23616,7 @@
       <c r="C699" t="inlineStr"/>
       <c r="D699" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E699" t="inlineStr"/>
@@ -23639,20 +23635,24 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C700" t="inlineStr"/>
       <c r="D700" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E700" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F700" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23668,27 +23668,23 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C701" t="inlineStr"/>
       <c r="D701" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E701" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr"/>
       <c r="F701" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G701" t="inlineStr"/>
@@ -23701,7 +23697,7 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
@@ -23711,7 +23707,7 @@
       <c r="C702" t="inlineStr"/>
       <c r="D702" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E702" t="inlineStr"/>
@@ -23730,23 +23726,27 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C703" t="inlineStr"/>
       <c r="D703" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E703" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F703" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G703" t="inlineStr"/>
@@ -23759,27 +23759,31 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C704" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D704" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E704" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F704" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G704" t="inlineStr"/>
@@ -23792,11 +23796,11 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C705" t="inlineStr">
@@ -23806,12 +23810,12 @@
       </c>
       <c r="D705" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E705" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F705" t="inlineStr">
@@ -23829,26 +23833,26 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C706" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D706" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E706" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F706" t="inlineStr">
@@ -23866,31 +23870,27 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C707" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D707" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E707" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr"/>
       <c r="F707" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G707" t="inlineStr"/>
@@ -23903,27 +23903,27 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C708" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D708" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E708" t="inlineStr"/>
       <c r="F708" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G708" t="inlineStr"/>
@@ -23936,27 +23936,27 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C709" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D709" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E709" t="inlineStr"/>
       <c r="F709" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G709" t="inlineStr"/>
@@ -23969,27 +23969,27 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C710" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D710" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E710" t="inlineStr"/>
       <c r="F710" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G710" t="inlineStr"/>
@@ -24002,24 +24002,28 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C711" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D711" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E711" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F711" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -24035,11 +24039,11 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C712" t="inlineStr">
@@ -24049,12 +24053,12 @@
       </c>
       <c r="D712" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E712" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F712" t="inlineStr">
@@ -24072,11 +24076,11 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C713" t="inlineStr">
@@ -24086,7 +24090,7 @@
       </c>
       <c r="D713" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E713" t="inlineStr">
@@ -24109,31 +24113,31 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C714" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D714" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E714" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F714" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G714" t="inlineStr"/>
@@ -24146,31 +24150,27 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D715" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E715" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr"/>
       <c r="F715" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G715" t="inlineStr"/>
@@ -24183,27 +24183,31 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C716" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D716" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E716" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F716" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G716" t="inlineStr"/>
@@ -24216,26 +24220,22 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C717" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr"/>
       <c r="D717" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E717" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F717" t="inlineStr">
@@ -24253,30 +24253,38 @@
     </row>
     <row r="718">
       <c r="A718" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B718" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C718" t="inlineStr"/>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D718" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E718" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F718" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G718" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G718" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H718" t="inlineStr"/>
       <c r="I718" t="inlineStr">
         <is>
@@ -24286,38 +24294,34 @@
     </row>
     <row r="719">
       <c r="A719" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C719" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D719" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E719" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F719" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G719" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G719" t="inlineStr"/>
       <c r="H719" t="inlineStr"/>
       <c r="I719" t="inlineStr">
         <is>
@@ -24327,26 +24331,26 @@
     </row>
     <row r="720">
       <c r="A720" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C720" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D720" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E720" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F720" t="inlineStr">
@@ -24354,7 +24358,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G720" t="inlineStr"/>
+      <c r="G720" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H720" t="inlineStr"/>
       <c r="I720" t="inlineStr">
         <is>
@@ -24364,11 +24372,11 @@
     </row>
     <row r="721">
       <c r="A721" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C721" t="inlineStr">
@@ -24378,67 +24386,26 @@
       </c>
       <c r="D721" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E721" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F721" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G721" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H721" t="inlineStr"/>
       <c r="I721" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="722">
-      <c r="A722" t="n">
-        <v>763</v>
-      </c>
-      <c r="B722" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C722" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D722" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E722" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F722" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G722" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H722" t="inlineStr"/>
-      <c r="I722" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 632 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I718"/>
+  <dimension ref="A1:I717"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20480,21 +20480,17 @@
     </row>
     <row r="601">
       <c r="A601" t="n">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C601" t="inlineStr">
-        <is>
-          <t>06.05.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr"/>
       <c r="D601" t="inlineStr">
         <is>
-          <t>MM</t>
+          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
         </is>
       </c>
       <c r="E601" t="inlineStr"/>
@@ -20513,7 +20509,7 @@
     </row>
     <row r="602">
       <c r="A602" t="n">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="B602" t="inlineStr">
         <is>
@@ -20523,7 +20519,7 @@
       <c r="C602" t="inlineStr"/>
       <c r="D602" t="inlineStr">
         <is>
-          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
+          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
         </is>
       </c>
       <c r="E602" t="inlineStr"/>
@@ -20542,7 +20538,7 @@
     </row>
     <row r="603">
       <c r="A603" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B603" t="inlineStr">
         <is>
@@ -20552,7 +20548,7 @@
       <c r="C603" t="inlineStr"/>
       <c r="D603" t="inlineStr">
         <is>
-          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
+          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
         </is>
       </c>
       <c r="E603" t="inlineStr"/>
@@ -20571,20 +20567,24 @@
     </row>
     <row r="604">
       <c r="A604" t="n">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B604" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C604" t="inlineStr"/>
       <c r="D604" t="inlineStr">
         <is>
-          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
-        </is>
-      </c>
-      <c r="E604" t="inlineStr"/>
+          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>vyměnili dobíječ stacionární (Veselí)</t>
+        </is>
+      </c>
       <c r="F604" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20600,22 +20600,22 @@
     </row>
     <row r="605">
       <c r="A605" t="n">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C605" t="inlineStr"/>
       <c r="D605" t="inlineStr">
         <is>
-          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
         </is>
       </c>
       <c r="E605" t="inlineStr">
         <is>
-          <t>vyměnili dobíječ stacionární (Veselí)</t>
+          <t>jela ven</t>
         </is>
       </c>
       <c r="F605" t="inlineStr">
@@ -20633,24 +20633,20 @@
     </row>
     <row r="606">
       <c r="A606" t="n">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B606" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C606" t="inlineStr"/>
       <c r="D606" t="inlineStr">
         <is>
-          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
-        </is>
-      </c>
-      <c r="E606" t="inlineStr">
-        <is>
-          <t>jela ven</t>
-        </is>
-      </c>
+          <t>seřízení kamer přes program v notasu(obraz)</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr"/>
       <c r="F606" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20666,20 +20662,24 @@
     </row>
     <row r="607">
       <c r="A607" t="n">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B607" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C607" t="inlineStr"/>
       <c r="D607" t="inlineStr">
         <is>
-          <t>seřízení kamer přes program v notasu(obraz)</t>
-        </is>
-      </c>
-      <c r="E607" t="inlineStr"/>
+          <t>po startu někdy nenabíjí "B"</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+        </is>
+      </c>
       <c r="F607" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20695,22 +20695,22 @@
     </row>
     <row r="608">
       <c r="A608" t="n">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B608" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C608" t="inlineStr"/>
       <c r="D608" t="inlineStr">
         <is>
-          <t>po startu někdy nenabíjí "B"</t>
+          <t>2. motor korekce vody  vystup</t>
         </is>
       </c>
       <c r="E608" t="inlineStr">
         <is>
-          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
         </is>
       </c>
       <c r="F608" t="inlineStr">
@@ -20728,24 +20728,24 @@
     </row>
     <row r="609">
       <c r="A609" t="n">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>842 035</t>
-        </is>
-      </c>
-      <c r="C609" t="inlineStr"/>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>04.12.2023</t>
+        </is>
+      </c>
       <c r="D609" t="inlineStr">
         <is>
-          <t>2. motor korekce vody  vystup</t>
-        </is>
-      </c>
-      <c r="E609" t="inlineStr">
-        <is>
-          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
-        </is>
-      </c>
+          <t>Výměna motoru A</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr"/>
       <c r="F609" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20761,21 +20761,17 @@
     </row>
     <row r="610">
       <c r="A610" t="n">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B610" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C610" t="inlineStr">
-        <is>
-          <t>04.12.2023</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr"/>
       <c r="D610" t="inlineStr">
         <is>
-          <t>Výměna motoru A</t>
+          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
         </is>
       </c>
       <c r="E610" t="inlineStr"/>
@@ -20794,17 +20790,17 @@
     </row>
     <row r="611">
       <c r="A611" t="n">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B611" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C611" t="inlineStr"/>
       <c r="D611" t="inlineStr">
         <is>
-          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
+          <t>dosazena nahadni Mirelka + NO z 844 013</t>
         </is>
       </c>
       <c r="E611" t="inlineStr"/>
@@ -20823,17 +20819,17 @@
     </row>
     <row r="612">
       <c r="A612" t="n">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B612" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 062</t>
         </is>
       </c>
       <c r="C612" t="inlineStr"/>
       <c r="D612" t="inlineStr">
         <is>
-          <t>dosazena nahadni Mirelka + NO z 844 013</t>
+          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
         </is>
       </c>
       <c r="E612" t="inlineStr"/>
@@ -20852,17 +20848,21 @@
     </row>
     <row r="613">
       <c r="A613" t="n">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>814 062</t>
-        </is>
-      </c>
-      <c r="C613" t="inlineStr"/>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>03.03.2023</t>
+        </is>
+      </c>
       <c r="D613" t="inlineStr">
         <is>
-          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E613" t="inlineStr"/>
@@ -20881,11 +20881,11 @@
     </row>
     <row r="614">
       <c r="A614" t="n">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B614" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C614" t="inlineStr">
@@ -20895,7 +20895,7 @@
       </c>
       <c r="D614" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
+          <t>Dosazení ŘJ kamer</t>
         </is>
       </c>
       <c r="E614" t="inlineStr"/>
@@ -20914,24 +20914,24 @@
     </row>
     <row r="615">
       <c r="A615" t="n">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>844 013</t>
-        </is>
-      </c>
-      <c r="C615" t="inlineStr">
-        <is>
-          <t>03.03.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr"/>
       <c r="D615" t="inlineStr">
         <is>
-          <t>Dosazení ŘJ kamer</t>
-        </is>
-      </c>
-      <c r="E615" t="inlineStr"/>
+          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>hlášeno p. Škodovi</t>
+        </is>
+      </c>
       <c r="F615" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20947,24 +20947,20 @@
     </row>
     <row r="616">
       <c r="A616" t="n">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="B616" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C616" t="inlineStr"/>
       <c r="D616" t="inlineStr">
         <is>
-          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
-        </is>
-      </c>
-      <c r="E616" t="inlineStr">
-        <is>
-          <t>hlášeno p. Škodovi</t>
-        </is>
-      </c>
+          <t>ŘJ kamer dosazena z 013</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr"/>
       <c r="F616" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20980,17 +20976,21 @@
     </row>
     <row r="617">
       <c r="A617" t="n">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B617" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C617" t="inlineStr"/>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>02.09.2023</t>
+        </is>
+      </c>
       <c r="D617" t="inlineStr">
         <is>
-          <t>ŘJ kamer dosazena z 013</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E617" t="inlineStr"/>
@@ -21009,21 +21009,21 @@
     </row>
     <row r="618">
       <c r="A618" t="n">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B618" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 072</t>
         </is>
       </c>
       <c r="C618" t="inlineStr">
         <is>
-          <t>02.09.2023</t>
+          <t>02.03.2023</t>
         </is>
       </c>
       <c r="D618" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>MM</t>
         </is>
       </c>
       <c r="E618" t="inlineStr"/>
@@ -21042,24 +21042,24 @@
     </row>
     <row r="619">
       <c r="A619" t="n">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>814 072</t>
-        </is>
-      </c>
-      <c r="C619" t="inlineStr">
-        <is>
-          <t>02.03.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr"/>
       <c r="D619" t="inlineStr">
         <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E619" t="inlineStr"/>
+          <t>dosazen opraveny MIREL</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+        </is>
+      </c>
       <c r="F619" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21075,22 +21075,22 @@
     </row>
     <row r="620">
       <c r="A620" t="n">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C620" t="inlineStr"/>
       <c r="D620" t="inlineStr">
         <is>
-          <t>dosazen opraveny MIREL</t>
+          <t>Odpojen trojcestný ventil na A i B</t>
         </is>
       </c>
       <c r="E620" t="inlineStr">
         <is>
-          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+          <t>Zapojeny zpět 24.2.2023</t>
         </is>
       </c>
       <c r="F620" t="inlineStr">
@@ -21108,24 +21108,20 @@
     </row>
     <row r="621">
       <c r="A621" t="n">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C621" t="inlineStr"/>
       <c r="D621" t="inlineStr">
         <is>
-          <t>Odpojen trojcestný ventil na A i B</t>
-        </is>
-      </c>
-      <c r="E621" t="inlineStr">
-        <is>
-          <t>Zapojeny zpět 24.2.2023</t>
-        </is>
-      </c>
+          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr"/>
       <c r="F621" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21141,17 +21137,21 @@
     </row>
     <row r="622">
       <c r="A622" t="n">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B622" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C622" t="inlineStr"/>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>01.10.2023</t>
+        </is>
+      </c>
       <c r="D622" t="inlineStr">
         <is>
-          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E622" t="inlineStr"/>
@@ -21170,21 +21170,17 @@
     </row>
     <row r="623">
       <c r="A623" t="n">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="B623" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C623" t="inlineStr">
-        <is>
-          <t>01.10.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr"/>
       <c r="D623" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
         </is>
       </c>
       <c r="E623" t="inlineStr"/>
@@ -21203,17 +21199,17 @@
     </row>
     <row r="624">
       <c r="A624" t="n">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C624" t="inlineStr"/>
       <c r="D624" t="inlineStr">
         <is>
-          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
+          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
         </is>
       </c>
       <c r="E624" t="inlineStr"/>
@@ -21232,7 +21228,7 @@
     </row>
     <row r="625">
       <c r="A625" t="n">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B625" t="inlineStr">
         <is>
@@ -21242,7 +21238,7 @@
       <c r="C625" t="inlineStr"/>
       <c r="D625" t="inlineStr">
         <is>
-          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
+          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
         </is>
       </c>
       <c r="E625" t="inlineStr"/>
@@ -21261,20 +21257,24 @@
     </row>
     <row r="626">
       <c r="A626" t="n">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C626" t="inlineStr"/>
       <c r="D626" t="inlineStr">
         <is>
-          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
-        </is>
-      </c>
-      <c r="E626" t="inlineStr"/>
+          <t>Přišel opravený Mirel ve skladu</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>dosazen na 29.12.2022</t>
+        </is>
+      </c>
       <c r="F626" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21290,22 +21290,26 @@
     </row>
     <row r="627">
       <c r="A627" t="n">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C627" t="inlineStr"/>
+          <t>844 014</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>12.06.2022</t>
+        </is>
+      </c>
       <c r="D627" t="inlineStr">
         <is>
-          <t>Přišel opravený Mirel ve skladu</t>
+          <t>rychloměr do opravy hazí !!</t>
         </is>
       </c>
       <c r="E627" t="inlineStr">
         <is>
-          <t>dosazen na 29.12.2022</t>
+          <t>zapujcen z 844 028 z veselí</t>
         </is>
       </c>
       <c r="F627" t="inlineStr">
@@ -21323,11 +21327,11 @@
     </row>
     <row r="628">
       <c r="A628" t="n">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C628" t="inlineStr">
@@ -21337,14 +21341,10 @@
       </c>
       <c r="D628" t="inlineStr">
         <is>
-          <t>rychloměr do opravy hazí !!</t>
-        </is>
-      </c>
-      <c r="E628" t="inlineStr">
-        <is>
-          <t>zapujcen z 844 028 z veselí</t>
-        </is>
-      </c>
+          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr"/>
       <c r="F628" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21360,24 +21360,28 @@
     </row>
     <row r="629">
       <c r="A629" t="n">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>12.06.2022</t>
+          <t>12.03.2022</t>
         </is>
       </c>
       <c r="D629" t="inlineStr">
         <is>
-          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
-        </is>
-      </c>
-      <c r="E629" t="inlineStr"/>
+          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>bude řešit Škoda</t>
+        </is>
+      </c>
       <c r="F629" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21393,26 +21397,22 @@
     </row>
     <row r="630">
       <c r="A630" t="n">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B630" t="inlineStr">
         <is>
           <t>844 003</t>
         </is>
       </c>
-      <c r="C630" t="inlineStr">
-        <is>
-          <t>12.03.2022</t>
-        </is>
-      </c>
+      <c r="C630" t="inlineStr"/>
       <c r="D630" t="inlineStr">
         <is>
-          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+          <t>na A strane asi vadna expanzní nadrz topení ?</t>
         </is>
       </c>
       <c r="E630" t="inlineStr">
         <is>
-          <t>bude řešit Škoda</t>
+          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
         </is>
       </c>
       <c r="F630" t="inlineStr">
@@ -21430,22 +21430,22 @@
     </row>
     <row r="631">
       <c r="A631" t="n">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C631" t="inlineStr"/>
       <c r="D631" t="inlineStr">
         <is>
-          <t>na A strane asi vadna expanzní nadrz topení ?</t>
+          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
         </is>
       </c>
       <c r="E631" t="inlineStr">
         <is>
-          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
+          <t>nová obrazovka hazela vykricnik porad</t>
         </is>
       </c>
       <c r="F631" t="inlineStr">
@@ -21463,24 +21463,24 @@
     </row>
     <row r="632">
       <c r="A632" t="n">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C632" t="inlineStr"/>
+          <t>842 010</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>11.06.2022</t>
+        </is>
+      </c>
       <c r="D632" t="inlineStr">
         <is>
-          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
-        </is>
-      </c>
-      <c r="E632" t="inlineStr">
-        <is>
-          <t>nová obrazovka hazela vykricnik porad</t>
-        </is>
-      </c>
+          <t>Přehození karty TBA v DPV na 842 036</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr"/>
       <c r="F632" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21496,11 +21496,11 @@
     </row>
     <row r="633">
       <c r="A633" t="n">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>842 010</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C633" t="inlineStr">
@@ -21510,7 +21510,7 @@
       </c>
       <c r="D633" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 036</t>
+          <t>Přehození karty TBA v DPV na 842 010</t>
         </is>
       </c>
       <c r="E633" t="inlineStr"/>
@@ -21529,11 +21529,11 @@
     </row>
     <row r="634">
       <c r="A634" t="n">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C634" t="inlineStr">
@@ -21543,10 +21543,14 @@
       </c>
       <c r="D634" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 010</t>
-        </is>
-      </c>
-      <c r="E634" t="inlineStr"/>
+          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>mirel byl špatný po opravě</t>
+        </is>
+      </c>
       <c r="F634" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21562,26 +21566,26 @@
     </row>
     <row r="635">
       <c r="A635" t="n">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C635" t="inlineStr">
         <is>
-          <t>11.06.2022</t>
+          <t>11.05.2022</t>
         </is>
       </c>
       <c r="D635" t="inlineStr">
         <is>
-          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
         </is>
       </c>
       <c r="E635" t="inlineStr">
         <is>
-          <t>mirel byl špatný po opravě</t>
+          <t>25.11. opraveno</t>
         </is>
       </c>
       <c r="F635" t="inlineStr">
@@ -21599,11 +21603,11 @@
     </row>
     <row r="636">
       <c r="A636" t="n">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C636" t="inlineStr">
@@ -21613,14 +21617,10 @@
       </c>
       <c r="D636" t="inlineStr">
         <is>
-          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
-        </is>
-      </c>
-      <c r="E636" t="inlineStr">
-        <is>
-          <t>25.11. opraveno</t>
-        </is>
-      </c>
+          <t>VESELÍ R3 (odjela)</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr"/>
       <c r="F636" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21636,24 +21636,24 @@
     </row>
     <row r="637">
       <c r="A637" t="n">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>844 020</t>
-        </is>
-      </c>
-      <c r="C637" t="inlineStr">
-        <is>
-          <t>11.05.2022</t>
-        </is>
-      </c>
+          <t>814 190</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr"/>
       <c r="D637" t="inlineStr">
         <is>
-          <t>VESELÍ R3 (odjela)</t>
-        </is>
-      </c>
-      <c r="E637" t="inlineStr"/>
+          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>hlášeno p.Škodovi</t>
+        </is>
+      </c>
       <c r="F637" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21669,22 +21669,22 @@
     </row>
     <row r="638">
       <c r="A638" t="n">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>814 190</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C638" t="inlineStr"/>
       <c r="D638" t="inlineStr">
         <is>
-          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
         </is>
       </c>
       <c r="E638" t="inlineStr">
         <is>
-          <t>hlášeno p.Škodovi</t>
+          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
         </is>
       </c>
       <c r="F638" t="inlineStr">
@@ -21702,24 +21702,20 @@
     </row>
     <row r="639">
       <c r="A639" t="n">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C639" t="inlineStr"/>
       <c r="D639" t="inlineStr">
         <is>
-          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
-        </is>
-      </c>
-      <c r="E639" t="inlineStr">
-        <is>
-          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
-        </is>
-      </c>
+          <t>dosazen předzesilovač linky</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr"/>
       <c r="F639" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21735,20 +21731,28 @@
     </row>
     <row r="640">
       <c r="A640" t="n">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B640" t="inlineStr">
         <is>
           <t>814 073</t>
         </is>
       </c>
-      <c r="C640" t="inlineStr"/>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>09.07.2022</t>
+        </is>
+      </c>
       <c r="D640" t="inlineStr">
         <is>
-          <t>dosazen předzesilovač linky</t>
-        </is>
-      </c>
-      <c r="E640" t="inlineStr"/>
+          <t>chybějící díl</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>předzasilovač linky - objednán nový</t>
+        </is>
+      </c>
       <c r="F640" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21764,26 +21768,26 @@
     </row>
     <row r="641">
       <c r="A641" t="n">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 003</t>
         </is>
       </c>
       <c r="C641" t="inlineStr">
         <is>
-          <t>09.07.2022</t>
+          <t>09.03.2022</t>
         </is>
       </c>
       <c r="D641" t="inlineStr">
         <is>
-          <t>chybějící díl</t>
+          <t>dosazen díl</t>
         </is>
       </c>
       <c r="E641" t="inlineStr">
         <is>
-          <t>předzasilovač linky - objednán nový</t>
+          <t>dosazen předzasilovač linky A23</t>
         </is>
       </c>
       <c r="F641" t="inlineStr">
@@ -21801,26 +21805,22 @@
     </row>
     <row r="642">
       <c r="A642" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C642" t="inlineStr">
-        <is>
-          <t>09.03.2022</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr"/>
       <c r="D642" t="inlineStr">
         <is>
-          <t>dosazen díl</t>
+          <t>oprava dveří na B pravé po směru jízdy</t>
         </is>
       </c>
       <c r="E642" t="inlineStr">
         <is>
-          <t>dosazen předzasilovač linky A23</t>
+          <t>vadný motorek</t>
         </is>
       </c>
       <c r="F642" t="inlineStr">
@@ -21838,22 +21838,22 @@
     </row>
     <row r="643">
       <c r="A643" t="n">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C643" t="inlineStr"/>
       <c r="D643" t="inlineStr">
         <is>
-          <t>oprava dveří na B pravé po směru jízdy</t>
+          <t>vadné čidlo množství písku M5</t>
         </is>
       </c>
       <c r="E643" t="inlineStr">
         <is>
-          <t>vadný motorek</t>
+          <t>2. osa pravo po smeru jizdy z B</t>
         </is>
       </c>
       <c r="F643" t="inlineStr">
@@ -21871,22 +21871,22 @@
     </row>
     <row r="644">
       <c r="A644" t="n">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C644" t="inlineStr"/>
       <c r="D644" t="inlineStr">
         <is>
-          <t>vadné čidlo množství písku M5</t>
+          <t>rychloměr dán do skladu na opravu</t>
         </is>
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>2. osa pravo po smeru jizdy z B</t>
+          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
         </is>
       </c>
       <c r="F644" t="inlineStr">
@@ -21904,22 +21904,22 @@
     </row>
     <row r="645">
       <c r="A645" t="n">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C645" t="inlineStr"/>
       <c r="D645" t="inlineStr">
         <is>
-          <t>rychloměr dán do skladu na opravu</t>
+          <t>rychloměr nekomunikuje</t>
         </is>
       </c>
       <c r="E645" t="inlineStr">
         <is>
-          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
+          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
         </is>
       </c>
       <c r="F645" t="inlineStr">
@@ -21937,22 +21937,26 @@
     </row>
     <row r="646">
       <c r="A646" t="n">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>844 022</t>
-        </is>
-      </c>
-      <c r="C646" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>10.08.2021</t>
+        </is>
+      </c>
       <c r="D646" t="inlineStr">
         <is>
-          <t>rychloměr nekomunikuje</t>
+          <t>dosazeny díly</t>
         </is>
       </c>
       <c r="E646" t="inlineStr">
         <is>
-          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
+          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
         </is>
       </c>
       <c r="F646" t="inlineStr">
@@ -21970,18 +21974,14 @@
     </row>
     <row r="647">
       <c r="A647" t="n">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B647" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C647" t="inlineStr">
-        <is>
-          <t>10.08.2021</t>
-        </is>
-      </c>
+      <c r="C647" t="inlineStr"/>
       <c r="D647" t="inlineStr">
         <is>
           <t>dosazeny díly</t>
@@ -21989,7 +21989,7 @@
       </c>
       <c r="E647" t="inlineStr">
         <is>
-          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
+          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
         </is>
       </c>
       <c r="F647" t="inlineStr">
@@ -22007,22 +22007,26 @@
     </row>
     <row r="648">
       <c r="A648" t="n">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B648" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C648" t="inlineStr"/>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>09.06.2021</t>
+        </is>
+      </c>
       <c r="D648" t="inlineStr">
         <is>
-          <t>dosazeny díly</t>
+          <t>Chybějící díly z důvodu použití na jinou lok.</t>
         </is>
       </c>
       <c r="E648" t="inlineStr">
         <is>
-          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
+          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
         </is>
       </c>
       <c r="F648" t="inlineStr">
@@ -22040,28 +22044,16 @@
     </row>
     <row r="649">
       <c r="A649" t="n">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C649" t="inlineStr">
-        <is>
-          <t>09.06.2021</t>
-        </is>
-      </c>
-      <c r="D649" t="inlineStr">
-        <is>
-          <t>Chybějící díly z důvodu použití na jinou lok.</t>
-        </is>
-      </c>
-      <c r="E649" t="inlineStr">
-        <is>
-          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
-        </is>
-      </c>
+          <t>842 015</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr"/>
+      <c r="D649" t="inlineStr"/>
+      <c r="E649" t="inlineStr"/>
       <c r="F649" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22077,15 +22069,19 @@
     </row>
     <row r="650">
       <c r="A650" t="n">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C650" t="inlineStr"/>
-      <c r="D650" t="inlineStr"/>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>výměna obrazovky Lokel na 914</t>
+        </is>
+      </c>
       <c r="E650" t="inlineStr"/>
       <c r="F650" t="inlineStr">
         <is>
@@ -22102,17 +22098,17 @@
     </row>
     <row r="651">
       <c r="A651" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C651" t="inlineStr"/>
       <c r="D651" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E651" t="inlineStr"/>
@@ -22131,17 +22127,17 @@
     </row>
     <row r="652">
       <c r="A652" t="n">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C652" t="inlineStr"/>
       <c r="D652" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E652" t="inlineStr"/>
@@ -22160,7 +22156,7 @@
     </row>
     <row r="653">
       <c r="A653" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B653" t="inlineStr">
         <is>
@@ -22170,10 +22166,14 @@
       <c r="C653" t="inlineStr"/>
       <c r="D653" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E653" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F653" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22189,24 +22189,20 @@
     </row>
     <row r="654">
       <c r="A654" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C654" t="inlineStr"/>
       <c r="D654" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E654" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr"/>
       <c r="F654" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22222,7 +22218,7 @@
     </row>
     <row r="655">
       <c r="A655" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B655" t="inlineStr">
         <is>
@@ -22232,7 +22228,7 @@
       <c r="C655" t="inlineStr"/>
       <c r="D655" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E655" t="inlineStr"/>
@@ -22251,17 +22247,17 @@
     </row>
     <row r="656">
       <c r="A656" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C656" t="inlineStr"/>
       <c r="D656" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E656" t="inlineStr"/>
@@ -22280,20 +22276,24 @@
     </row>
     <row r="657">
       <c r="A657" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C657" t="inlineStr"/>
       <c r="D657" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E657" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F657" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22309,7 +22309,7 @@
     </row>
     <row r="658">
       <c r="A658" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B658" t="inlineStr">
         <is>
@@ -22319,12 +22319,12 @@
       <c r="C658" t="inlineStr"/>
       <c r="D658" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E658" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F658" t="inlineStr">
@@ -22342,24 +22342,24 @@
     </row>
     <row r="659">
       <c r="A659" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B659" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C659" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D659" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E659" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr"/>
       <c r="F659" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22375,7 +22375,7 @@
     </row>
     <row r="660">
       <c r="A660" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B660" t="inlineStr">
         <is>
@@ -22384,12 +22384,12 @@
       </c>
       <c r="C660" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D660" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E660" t="inlineStr"/>
@@ -22408,7 +22408,7 @@
     </row>
     <row r="661">
       <c r="A661" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B661" t="inlineStr">
         <is>
@@ -22422,7 +22422,7 @@
       </c>
       <c r="D661" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E661" t="inlineStr"/>
@@ -22441,7 +22441,7 @@
     </row>
     <row r="662">
       <c r="A662" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B662" t="inlineStr">
         <is>
@@ -22455,10 +22455,14 @@
       </c>
       <c r="D662" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E662" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F662" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22474,7 +22478,7 @@
     </row>
     <row r="663">
       <c r="A663" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B663" t="inlineStr">
         <is>
@@ -22488,12 +22492,12 @@
       </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E663" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F663" t="inlineStr">
@@ -22511,7 +22515,7 @@
     </row>
     <row r="664">
       <c r="A664" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B664" t="inlineStr">
         <is>
@@ -22525,14 +22529,10 @@
       </c>
       <c r="D664" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E664" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr"/>
       <c r="F664" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22548,24 +22548,24 @@
     </row>
     <row r="665">
       <c r="A665" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C665" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr"/>
       <c r="D665" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E665" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F665" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22581,24 +22581,20 @@
     </row>
     <row r="666">
       <c r="A666" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C666" t="inlineStr"/>
       <c r="D666" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E666" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr"/>
       <c r="F666" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22614,17 +22610,17 @@
     </row>
     <row r="667">
       <c r="A667" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C667" t="inlineStr"/>
       <c r="D667" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E667" t="inlineStr"/>
@@ -22643,7 +22639,7 @@
     </row>
     <row r="668">
       <c r="A668" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B668" t="inlineStr">
         <is>
@@ -22653,10 +22649,14 @@
       <c r="C668" t="inlineStr"/>
       <c r="D668" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E668" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F668" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22672,24 +22672,20 @@
     </row>
     <row r="669">
       <c r="A669" t="n">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C669" t="inlineStr"/>
       <c r="D669" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E669" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr"/>
       <c r="F669" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22705,7 +22701,7 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
@@ -22715,7 +22711,7 @@
       <c r="C670" t="inlineStr"/>
       <c r="D670" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E670" t="inlineStr"/>
@@ -22734,20 +22730,24 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C671" t="inlineStr"/>
       <c r="D671" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
-        </is>
-      </c>
-      <c r="E671" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F671" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22763,7 +22763,7 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
@@ -22773,14 +22773,10 @@
       <c r="C672" t="inlineStr"/>
       <c r="D672" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E672" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr"/>
       <c r="F672" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22796,7 +22792,7 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
@@ -22806,10 +22802,14 @@
       <c r="C673" t="inlineStr"/>
       <c r="D673" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E673" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F673" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22825,7 +22825,7 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
@@ -22835,14 +22835,10 @@
       <c r="C674" t="inlineStr"/>
       <c r="D674" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E674" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr"/>
       <c r="F674" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22858,7 +22854,7 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
@@ -22868,7 +22864,7 @@
       <c r="C675" t="inlineStr"/>
       <c r="D675" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E675" t="inlineStr"/>
@@ -22887,7 +22883,7 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
@@ -22897,10 +22893,14 @@
       <c r="C676" t="inlineStr"/>
       <c r="D676" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E676" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F676" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22916,7 +22916,7 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
@@ -22926,12 +22926,12 @@
       <c r="C677" t="inlineStr"/>
       <c r="D677" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E677" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F677" t="inlineStr">
@@ -22949,7 +22949,7 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
@@ -22959,12 +22959,12 @@
       <c r="C678" t="inlineStr"/>
       <c r="D678" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E678" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F678" t="inlineStr">
@@ -22982,24 +22982,20 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C679" t="inlineStr"/>
       <c r="D679" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E679" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr"/>
       <c r="F679" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23015,7 +23011,7 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
@@ -23025,10 +23021,14 @@
       <c r="C680" t="inlineStr"/>
       <c r="D680" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E680" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F680" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23044,7 +23044,7 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
@@ -23054,12 +23054,12 @@
       <c r="C681" t="inlineStr"/>
       <c r="D681" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E681" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F681" t="inlineStr">
@@ -23077,7 +23077,7 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
@@ -23087,14 +23087,10 @@
       <c r="C682" t="inlineStr"/>
       <c r="D682" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E682" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr"/>
       <c r="F682" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23110,17 +23106,17 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C683" t="inlineStr"/>
       <c r="D683" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E683" t="inlineStr"/>
@@ -23139,7 +23135,7 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
@@ -23149,10 +23145,14 @@
       <c r="C684" t="inlineStr"/>
       <c r="D684" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E684" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F684" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23168,22 +23168,22 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C685" t="inlineStr"/>
       <c r="D685" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E685" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F685" t="inlineStr">
@@ -23201,7 +23201,7 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
@@ -23211,12 +23211,12 @@
       <c r="C686" t="inlineStr"/>
       <c r="D686" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E686" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F686" t="inlineStr">
@@ -23234,24 +23234,20 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C687" t="inlineStr"/>
       <c r="D687" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E687" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr"/>
       <c r="F687" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23267,23 +23263,27 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C688" t="inlineStr"/>
       <c r="D688" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E688" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F688" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G688" t="inlineStr"/>
@@ -23296,27 +23296,23 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E689" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr"/>
       <c r="F689" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G689" t="inlineStr"/>
@@ -23329,7 +23325,7 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
@@ -23339,7 +23335,7 @@
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E690" t="inlineStr"/>
@@ -23358,7 +23354,7 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
@@ -23368,7 +23364,7 @@
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E691" t="inlineStr"/>
@@ -23387,7 +23383,7 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
@@ -23397,7 +23393,7 @@
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E692" t="inlineStr"/>
@@ -23416,7 +23412,7 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
@@ -23426,10 +23422,14 @@
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E693" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F693" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23445,24 +23445,20 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C694" t="inlineStr"/>
       <c r="D694" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E694" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr"/>
       <c r="F694" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23478,7 +23474,7 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
@@ -23488,7 +23484,7 @@
       <c r="C695" t="inlineStr"/>
       <c r="D695" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E695" t="inlineStr"/>
@@ -23507,20 +23503,24 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C696" t="inlineStr"/>
       <c r="D696" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E696" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F696" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23536,27 +23536,23 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C697" t="inlineStr"/>
       <c r="D697" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E697" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr"/>
       <c r="F697" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G697" t="inlineStr"/>
@@ -23569,7 +23565,7 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
@@ -23579,7 +23575,7 @@
       <c r="C698" t="inlineStr"/>
       <c r="D698" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E698" t="inlineStr"/>
@@ -23598,23 +23594,27 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C699" t="inlineStr"/>
       <c r="D699" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E699" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F699" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G699" t="inlineStr"/>
@@ -23627,27 +23627,31 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C700" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D700" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E700" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F700" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G700" t="inlineStr"/>
@@ -23660,11 +23664,11 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C701" t="inlineStr">
@@ -23674,12 +23678,12 @@
       </c>
       <c r="D701" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E701" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F701" t="inlineStr">
@@ -23697,26 +23701,26 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C702" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D702" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E702" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F702" t="inlineStr">
@@ -23734,31 +23738,27 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C703" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D703" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E703" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr"/>
       <c r="F703" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G703" t="inlineStr"/>
@@ -23771,27 +23771,27 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C704" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D704" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E704" t="inlineStr"/>
       <c r="F704" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G704" t="inlineStr"/>
@@ -23804,27 +23804,27 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C705" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D705" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E705" t="inlineStr"/>
       <c r="F705" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G705" t="inlineStr"/>
@@ -23837,27 +23837,27 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C706" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D706" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E706" t="inlineStr"/>
       <c r="F706" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G706" t="inlineStr"/>
@@ -23870,24 +23870,28 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C707" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D707" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E707" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F707" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -23903,11 +23907,11 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C708" t="inlineStr">
@@ -23917,12 +23921,12 @@
       </c>
       <c r="D708" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E708" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F708" t="inlineStr">
@@ -23940,11 +23944,11 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C709" t="inlineStr">
@@ -23954,7 +23958,7 @@
       </c>
       <c r="D709" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E709" t="inlineStr">
@@ -23977,31 +23981,31 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C710" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D710" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E710" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F710" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G710" t="inlineStr"/>
@@ -24014,31 +24018,27 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C711" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D711" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E711" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr"/>
       <c r="F711" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G711" t="inlineStr"/>
@@ -24051,27 +24051,31 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C712" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D712" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E712" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F712" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G712" t="inlineStr"/>
@@ -24084,26 +24088,22 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C713" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr"/>
       <c r="D713" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E713" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F713" t="inlineStr">
@@ -24121,30 +24121,38 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C714" t="inlineStr"/>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D714" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E714" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F714" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G714" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H714" t="inlineStr"/>
       <c r="I714" t="inlineStr">
         <is>
@@ -24154,38 +24162,34 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D715" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E715" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F715" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G715" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G715" t="inlineStr"/>
       <c r="H715" t="inlineStr"/>
       <c r="I715" t="inlineStr">
         <is>
@@ -24195,26 +24199,26 @@
     </row>
     <row r="716">
       <c r="A716" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C716" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D716" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E716" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F716" t="inlineStr">
@@ -24222,7 +24226,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G716" t="inlineStr"/>
+      <c r="G716" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H716" t="inlineStr"/>
       <c r="I716" t="inlineStr">
         <is>
@@ -24232,11 +24240,11 @@
     </row>
     <row r="717">
       <c r="A717" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C717" t="inlineStr">
@@ -24246,67 +24254,26 @@
       </c>
       <c r="D717" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E717" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F717" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G717" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H717" t="inlineStr"/>
       <c r="I717" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="718">
-      <c r="A718" t="n">
-        <v>763</v>
-      </c>
-      <c r="B718" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C718" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D718" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E718" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F718" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G718" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H718" t="inlineStr"/>
-      <c r="I718" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 650 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I716"/>
+  <dimension ref="A1:I715"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20972,24 +20972,24 @@
     </row>
     <row r="617">
       <c r="A617" t="n">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>814 072</t>
-        </is>
-      </c>
-      <c r="C617" t="inlineStr">
-        <is>
-          <t>02.03.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr"/>
       <c r="D617" t="inlineStr">
         <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E617" t="inlineStr"/>
+          <t>dosazen opraveny MIREL</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+        </is>
+      </c>
       <c r="F617" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21005,22 +21005,22 @@
     </row>
     <row r="618">
       <c r="A618" t="n">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B618" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C618" t="inlineStr"/>
       <c r="D618" t="inlineStr">
         <is>
-          <t>dosazen opraveny MIREL</t>
+          <t>Odpojen trojcestný ventil na A i B</t>
         </is>
       </c>
       <c r="E618" t="inlineStr">
         <is>
-          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+          <t>Zapojeny zpět 24.2.2023</t>
         </is>
       </c>
       <c r="F618" t="inlineStr">
@@ -21038,24 +21038,20 @@
     </row>
     <row r="619">
       <c r="A619" t="n">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C619" t="inlineStr"/>
       <c r="D619" t="inlineStr">
         <is>
-          <t>Odpojen trojcestný ventil na A i B</t>
-        </is>
-      </c>
-      <c r="E619" t="inlineStr">
-        <is>
-          <t>Zapojeny zpět 24.2.2023</t>
-        </is>
-      </c>
+          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr"/>
       <c r="F619" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21071,17 +21067,21 @@
     </row>
     <row r="620">
       <c r="A620" t="n">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B620" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C620" t="inlineStr"/>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>01.10.2023</t>
+        </is>
+      </c>
       <c r="D620" t="inlineStr">
         <is>
-          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E620" t="inlineStr"/>
@@ -21100,21 +21100,17 @@
     </row>
     <row r="621">
       <c r="A621" t="n">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C621" t="inlineStr">
-        <is>
-          <t>01.10.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr"/>
       <c r="D621" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
         </is>
       </c>
       <c r="E621" t="inlineStr"/>
@@ -21133,17 +21129,17 @@
     </row>
     <row r="622">
       <c r="A622" t="n">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C622" t="inlineStr"/>
       <c r="D622" t="inlineStr">
         <is>
-          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
+          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
         </is>
       </c>
       <c r="E622" t="inlineStr"/>
@@ -21162,7 +21158,7 @@
     </row>
     <row r="623">
       <c r="A623" t="n">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B623" t="inlineStr">
         <is>
@@ -21172,7 +21168,7 @@
       <c r="C623" t="inlineStr"/>
       <c r="D623" t="inlineStr">
         <is>
-          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
+          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
         </is>
       </c>
       <c r="E623" t="inlineStr"/>
@@ -21191,20 +21187,24 @@
     </row>
     <row r="624">
       <c r="A624" t="n">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C624" t="inlineStr"/>
       <c r="D624" t="inlineStr">
         <is>
-          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
-        </is>
-      </c>
-      <c r="E624" t="inlineStr"/>
+          <t>Přišel opravený Mirel ve skladu</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>dosazen na 29.12.2022</t>
+        </is>
+      </c>
       <c r="F624" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21220,22 +21220,26 @@
     </row>
     <row r="625">
       <c r="A625" t="n">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B625" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C625" t="inlineStr"/>
+          <t>844 014</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>12.06.2022</t>
+        </is>
+      </c>
       <c r="D625" t="inlineStr">
         <is>
-          <t>Přišel opravený Mirel ve skladu</t>
+          <t>rychloměr do opravy hazí !!</t>
         </is>
       </c>
       <c r="E625" t="inlineStr">
         <is>
-          <t>dosazen na 29.12.2022</t>
+          <t>zapujcen z 844 028 z veselí</t>
         </is>
       </c>
       <c r="F625" t="inlineStr">
@@ -21253,11 +21257,11 @@
     </row>
     <row r="626">
       <c r="A626" t="n">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C626" t="inlineStr">
@@ -21267,14 +21271,10 @@
       </c>
       <c r="D626" t="inlineStr">
         <is>
-          <t>rychloměr do opravy hazí !!</t>
-        </is>
-      </c>
-      <c r="E626" t="inlineStr">
-        <is>
-          <t>zapujcen z 844 028 z veselí</t>
-        </is>
-      </c>
+          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr"/>
       <c r="F626" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21290,24 +21290,28 @@
     </row>
     <row r="627">
       <c r="A627" t="n">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C627" t="inlineStr">
         <is>
-          <t>12.06.2022</t>
+          <t>12.03.2022</t>
         </is>
       </c>
       <c r="D627" t="inlineStr">
         <is>
-          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
-        </is>
-      </c>
-      <c r="E627" t="inlineStr"/>
+          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>bude řešit Škoda</t>
+        </is>
+      </c>
       <c r="F627" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21323,26 +21327,22 @@
     </row>
     <row r="628">
       <c r="A628" t="n">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B628" t="inlineStr">
         <is>
           <t>844 003</t>
         </is>
       </c>
-      <c r="C628" t="inlineStr">
-        <is>
-          <t>12.03.2022</t>
-        </is>
-      </c>
+      <c r="C628" t="inlineStr"/>
       <c r="D628" t="inlineStr">
         <is>
-          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+          <t>na A strane asi vadna expanzní nadrz topení ?</t>
         </is>
       </c>
       <c r="E628" t="inlineStr">
         <is>
-          <t>bude řešit Škoda</t>
+          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
         </is>
       </c>
       <c r="F628" t="inlineStr">
@@ -21360,22 +21360,22 @@
     </row>
     <row r="629">
       <c r="A629" t="n">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C629" t="inlineStr"/>
       <c r="D629" t="inlineStr">
         <is>
-          <t>na A strane asi vadna expanzní nadrz topení ?</t>
+          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
         </is>
       </c>
       <c r="E629" t="inlineStr">
         <is>
-          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
+          <t>nová obrazovka hazela vykricnik porad</t>
         </is>
       </c>
       <c r="F629" t="inlineStr">
@@ -21393,24 +21393,24 @@
     </row>
     <row r="630">
       <c r="A630" t="n">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C630" t="inlineStr"/>
+          <t>842 010</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>11.06.2022</t>
+        </is>
+      </c>
       <c r="D630" t="inlineStr">
         <is>
-          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
-        </is>
-      </c>
-      <c r="E630" t="inlineStr">
-        <is>
-          <t>nová obrazovka hazela vykricnik porad</t>
-        </is>
-      </c>
+          <t>Přehození karty TBA v DPV na 842 036</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr"/>
       <c r="F630" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21426,11 +21426,11 @@
     </row>
     <row r="631">
       <c r="A631" t="n">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>842 010</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C631" t="inlineStr">
@@ -21440,7 +21440,7 @@
       </c>
       <c r="D631" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 036</t>
+          <t>Přehození karty TBA v DPV na 842 010</t>
         </is>
       </c>
       <c r="E631" t="inlineStr"/>
@@ -21459,11 +21459,11 @@
     </row>
     <row r="632">
       <c r="A632" t="n">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C632" t="inlineStr">
@@ -21473,10 +21473,14 @@
       </c>
       <c r="D632" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 010</t>
-        </is>
-      </c>
-      <c r="E632" t="inlineStr"/>
+          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>mirel byl špatný po opravě</t>
+        </is>
+      </c>
       <c r="F632" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21492,26 +21496,26 @@
     </row>
     <row r="633">
       <c r="A633" t="n">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C633" t="inlineStr">
         <is>
-          <t>11.06.2022</t>
+          <t>11.05.2022</t>
         </is>
       </c>
       <c r="D633" t="inlineStr">
         <is>
-          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
         </is>
       </c>
       <c r="E633" t="inlineStr">
         <is>
-          <t>mirel byl špatný po opravě</t>
+          <t>25.11. opraveno</t>
         </is>
       </c>
       <c r="F633" t="inlineStr">
@@ -21529,11 +21533,11 @@
     </row>
     <row r="634">
       <c r="A634" t="n">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C634" t="inlineStr">
@@ -21543,14 +21547,10 @@
       </c>
       <c r="D634" t="inlineStr">
         <is>
-          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
-        </is>
-      </c>
-      <c r="E634" t="inlineStr">
-        <is>
-          <t>25.11. opraveno</t>
-        </is>
-      </c>
+          <t>VESELÍ R3 (odjela)</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr"/>
       <c r="F634" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21566,24 +21566,24 @@
     </row>
     <row r="635">
       <c r="A635" t="n">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>844 020</t>
-        </is>
-      </c>
-      <c r="C635" t="inlineStr">
-        <is>
-          <t>11.05.2022</t>
-        </is>
-      </c>
+          <t>814 190</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr"/>
       <c r="D635" t="inlineStr">
         <is>
-          <t>VESELÍ R3 (odjela)</t>
-        </is>
-      </c>
-      <c r="E635" t="inlineStr"/>
+          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>hlášeno p.Škodovi</t>
+        </is>
+      </c>
       <c r="F635" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21599,22 +21599,22 @@
     </row>
     <row r="636">
       <c r="A636" t="n">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>814 190</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C636" t="inlineStr"/>
       <c r="D636" t="inlineStr">
         <is>
-          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
         </is>
       </c>
       <c r="E636" t="inlineStr">
         <is>
-          <t>hlášeno p.Škodovi</t>
+          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
         </is>
       </c>
       <c r="F636" t="inlineStr">
@@ -21632,24 +21632,20 @@
     </row>
     <row r="637">
       <c r="A637" t="n">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C637" t="inlineStr"/>
       <c r="D637" t="inlineStr">
         <is>
-          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
-        </is>
-      </c>
-      <c r="E637" t="inlineStr">
-        <is>
-          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
-        </is>
-      </c>
+          <t>dosazen předzesilovač linky</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr"/>
       <c r="F637" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21665,20 +21661,28 @@
     </row>
     <row r="638">
       <c r="A638" t="n">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B638" t="inlineStr">
         <is>
           <t>814 073</t>
         </is>
       </c>
-      <c r="C638" t="inlineStr"/>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>09.07.2022</t>
+        </is>
+      </c>
       <c r="D638" t="inlineStr">
         <is>
-          <t>dosazen předzesilovač linky</t>
-        </is>
-      </c>
-      <c r="E638" t="inlineStr"/>
+          <t>chybějící díl</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>předzasilovač linky - objednán nový</t>
+        </is>
+      </c>
       <c r="F638" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21694,26 +21698,26 @@
     </row>
     <row r="639">
       <c r="A639" t="n">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 003</t>
         </is>
       </c>
       <c r="C639" t="inlineStr">
         <is>
-          <t>09.07.2022</t>
+          <t>09.03.2022</t>
         </is>
       </c>
       <c r="D639" t="inlineStr">
         <is>
-          <t>chybějící díl</t>
+          <t>dosazen díl</t>
         </is>
       </c>
       <c r="E639" t="inlineStr">
         <is>
-          <t>předzasilovač linky - objednán nový</t>
+          <t>dosazen předzasilovač linky A23</t>
         </is>
       </c>
       <c r="F639" t="inlineStr">
@@ -21731,26 +21735,22 @@
     </row>
     <row r="640">
       <c r="A640" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C640" t="inlineStr">
-        <is>
-          <t>09.03.2022</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr"/>
       <c r="D640" t="inlineStr">
         <is>
-          <t>dosazen díl</t>
+          <t>oprava dveří na B pravé po směru jízdy</t>
         </is>
       </c>
       <c r="E640" t="inlineStr">
         <is>
-          <t>dosazen předzasilovač linky A23</t>
+          <t>vadný motorek</t>
         </is>
       </c>
       <c r="F640" t="inlineStr">
@@ -21768,22 +21768,22 @@
     </row>
     <row r="641">
       <c r="A641" t="n">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C641" t="inlineStr"/>
       <c r="D641" t="inlineStr">
         <is>
-          <t>oprava dveří na B pravé po směru jízdy</t>
+          <t>vadné čidlo množství písku M5</t>
         </is>
       </c>
       <c r="E641" t="inlineStr">
         <is>
-          <t>vadný motorek</t>
+          <t>2. osa pravo po smeru jizdy z B</t>
         </is>
       </c>
       <c r="F641" t="inlineStr">
@@ -21801,22 +21801,22 @@
     </row>
     <row r="642">
       <c r="A642" t="n">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C642" t="inlineStr"/>
       <c r="D642" t="inlineStr">
         <is>
-          <t>vadné čidlo množství písku M5</t>
+          <t>rychloměr dán do skladu na opravu</t>
         </is>
       </c>
       <c r="E642" t="inlineStr">
         <is>
-          <t>2. osa pravo po smeru jizdy z B</t>
+          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
         </is>
       </c>
       <c r="F642" t="inlineStr">
@@ -21834,22 +21834,22 @@
     </row>
     <row r="643">
       <c r="A643" t="n">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C643" t="inlineStr"/>
       <c r="D643" t="inlineStr">
         <is>
-          <t>rychloměr dán do skladu na opravu</t>
+          <t>rychloměr nekomunikuje</t>
         </is>
       </c>
       <c r="E643" t="inlineStr">
         <is>
-          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
+          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
         </is>
       </c>
       <c r="F643" t="inlineStr">
@@ -21867,22 +21867,26 @@
     </row>
     <row r="644">
       <c r="A644" t="n">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>844 022</t>
-        </is>
-      </c>
-      <c r="C644" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>10.08.2021</t>
+        </is>
+      </c>
       <c r="D644" t="inlineStr">
         <is>
-          <t>rychloměr nekomunikuje</t>
+          <t>dosazeny díly</t>
         </is>
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
+          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
         </is>
       </c>
       <c r="F644" t="inlineStr">
@@ -21900,18 +21904,14 @@
     </row>
     <row r="645">
       <c r="A645" t="n">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B645" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C645" t="inlineStr">
-        <is>
-          <t>10.08.2021</t>
-        </is>
-      </c>
+      <c r="C645" t="inlineStr"/>
       <c r="D645" t="inlineStr">
         <is>
           <t>dosazeny díly</t>
@@ -21919,7 +21919,7 @@
       </c>
       <c r="E645" t="inlineStr">
         <is>
-          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
+          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
         </is>
       </c>
       <c r="F645" t="inlineStr">
@@ -21937,22 +21937,26 @@
     </row>
     <row r="646">
       <c r="A646" t="n">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B646" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C646" t="inlineStr"/>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>09.06.2021</t>
+        </is>
+      </c>
       <c r="D646" t="inlineStr">
         <is>
-          <t>dosazeny díly</t>
+          <t>Chybějící díly z důvodu použití na jinou lok.</t>
         </is>
       </c>
       <c r="E646" t="inlineStr">
         <is>
-          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
+          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
         </is>
       </c>
       <c r="F646" t="inlineStr">
@@ -21970,28 +21974,16 @@
     </row>
     <row r="647">
       <c r="A647" t="n">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C647" t="inlineStr">
-        <is>
-          <t>09.06.2021</t>
-        </is>
-      </c>
-      <c r="D647" t="inlineStr">
-        <is>
-          <t>Chybějící díly z důvodu použití na jinou lok.</t>
-        </is>
-      </c>
-      <c r="E647" t="inlineStr">
-        <is>
-          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
-        </is>
-      </c>
+          <t>842 015</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr"/>
+      <c r="D647" t="inlineStr"/>
+      <c r="E647" t="inlineStr"/>
       <c r="F647" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22007,15 +21999,19 @@
     </row>
     <row r="648">
       <c r="A648" t="n">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C648" t="inlineStr"/>
-      <c r="D648" t="inlineStr"/>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>výměna obrazovky Lokel na 914</t>
+        </is>
+      </c>
       <c r="E648" t="inlineStr"/>
       <c r="F648" t="inlineStr">
         <is>
@@ -22032,17 +22028,17 @@
     </row>
     <row r="649">
       <c r="A649" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C649" t="inlineStr"/>
       <c r="D649" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E649" t="inlineStr"/>
@@ -22061,17 +22057,17 @@
     </row>
     <row r="650">
       <c r="A650" t="n">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C650" t="inlineStr"/>
       <c r="D650" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E650" t="inlineStr"/>
@@ -22090,7 +22086,7 @@
     </row>
     <row r="651">
       <c r="A651" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B651" t="inlineStr">
         <is>
@@ -22100,10 +22096,14 @@
       <c r="C651" t="inlineStr"/>
       <c r="D651" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E651" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F651" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22119,24 +22119,20 @@
     </row>
     <row r="652">
       <c r="A652" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C652" t="inlineStr"/>
       <c r="D652" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E652" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr"/>
       <c r="F652" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22152,7 +22148,7 @@
     </row>
     <row r="653">
       <c r="A653" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B653" t="inlineStr">
         <is>
@@ -22162,7 +22158,7 @@
       <c r="C653" t="inlineStr"/>
       <c r="D653" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E653" t="inlineStr"/>
@@ -22181,17 +22177,17 @@
     </row>
     <row r="654">
       <c r="A654" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C654" t="inlineStr"/>
       <c r="D654" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E654" t="inlineStr"/>
@@ -22210,20 +22206,24 @@
     </row>
     <row r="655">
       <c r="A655" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C655" t="inlineStr"/>
       <c r="D655" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E655" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F655" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22239,7 +22239,7 @@
     </row>
     <row r="656">
       <c r="A656" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B656" t="inlineStr">
         <is>
@@ -22249,12 +22249,12 @@
       <c r="C656" t="inlineStr"/>
       <c r="D656" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E656" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F656" t="inlineStr">
@@ -22272,24 +22272,24 @@
     </row>
     <row r="657">
       <c r="A657" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C657" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D657" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E657" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr"/>
       <c r="F657" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22305,7 +22305,7 @@
     </row>
     <row r="658">
       <c r="A658" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B658" t="inlineStr">
         <is>
@@ -22314,12 +22314,12 @@
       </c>
       <c r="C658" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D658" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E658" t="inlineStr"/>
@@ -22338,7 +22338,7 @@
     </row>
     <row r="659">
       <c r="A659" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B659" t="inlineStr">
         <is>
@@ -22352,7 +22352,7 @@
       </c>
       <c r="D659" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E659" t="inlineStr"/>
@@ -22371,7 +22371,7 @@
     </row>
     <row r="660">
       <c r="A660" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B660" t="inlineStr">
         <is>
@@ -22385,10 +22385,14 @@
       </c>
       <c r="D660" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E660" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F660" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22404,7 +22408,7 @@
     </row>
     <row r="661">
       <c r="A661" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B661" t="inlineStr">
         <is>
@@ -22418,12 +22422,12 @@
       </c>
       <c r="D661" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E661" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F661" t="inlineStr">
@@ -22441,7 +22445,7 @@
     </row>
     <row r="662">
       <c r="A662" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B662" t="inlineStr">
         <is>
@@ -22455,14 +22459,10 @@
       </c>
       <c r="D662" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E662" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr"/>
       <c r="F662" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22478,24 +22478,24 @@
     </row>
     <row r="663">
       <c r="A663" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C663" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr"/>
       <c r="D663" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E663" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F663" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22511,24 +22511,20 @@
     </row>
     <row r="664">
       <c r="A664" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C664" t="inlineStr"/>
       <c r="D664" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E664" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr"/>
       <c r="F664" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22544,17 +22540,17 @@
     </row>
     <row r="665">
       <c r="A665" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C665" t="inlineStr"/>
       <c r="D665" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E665" t="inlineStr"/>
@@ -22573,7 +22569,7 @@
     </row>
     <row r="666">
       <c r="A666" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B666" t="inlineStr">
         <is>
@@ -22583,10 +22579,14 @@
       <c r="C666" t="inlineStr"/>
       <c r="D666" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E666" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F666" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22602,24 +22602,20 @@
     </row>
     <row r="667">
       <c r="A667" t="n">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C667" t="inlineStr"/>
       <c r="D667" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E667" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr"/>
       <c r="F667" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22635,7 +22631,7 @@
     </row>
     <row r="668">
       <c r="A668" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B668" t="inlineStr">
         <is>
@@ -22645,7 +22641,7 @@
       <c r="C668" t="inlineStr"/>
       <c r="D668" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E668" t="inlineStr"/>
@@ -22664,20 +22660,24 @@
     </row>
     <row r="669">
       <c r="A669" t="n">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C669" t="inlineStr"/>
       <c r="D669" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
-        </is>
-      </c>
-      <c r="E669" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F669" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22693,7 +22693,7 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
@@ -22703,14 +22703,10 @@
       <c r="C670" t="inlineStr"/>
       <c r="D670" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E670" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr"/>
       <c r="F670" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22726,7 +22722,7 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
@@ -22736,10 +22732,14 @@
       <c r="C671" t="inlineStr"/>
       <c r="D671" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E671" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F671" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22755,7 +22755,7 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
@@ -22765,14 +22765,10 @@
       <c r="C672" t="inlineStr"/>
       <c r="D672" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E672" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr"/>
       <c r="F672" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22788,7 +22784,7 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
@@ -22798,7 +22794,7 @@
       <c r="C673" t="inlineStr"/>
       <c r="D673" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E673" t="inlineStr"/>
@@ -22817,7 +22813,7 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
@@ -22827,10 +22823,14 @@
       <c r="C674" t="inlineStr"/>
       <c r="D674" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E674" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F674" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22846,7 +22846,7 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
@@ -22856,12 +22856,12 @@
       <c r="C675" t="inlineStr"/>
       <c r="D675" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E675" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F675" t="inlineStr">
@@ -22879,7 +22879,7 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
@@ -22889,12 +22889,12 @@
       <c r="C676" t="inlineStr"/>
       <c r="D676" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E676" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F676" t="inlineStr">
@@ -22912,24 +22912,20 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C677" t="inlineStr"/>
       <c r="D677" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E677" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr"/>
       <c r="F677" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22945,7 +22941,7 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
@@ -22955,10 +22951,14 @@
       <c r="C678" t="inlineStr"/>
       <c r="D678" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E678" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F678" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22974,7 +22974,7 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
@@ -22984,12 +22984,12 @@
       <c r="C679" t="inlineStr"/>
       <c r="D679" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E679" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F679" t="inlineStr">
@@ -23007,7 +23007,7 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
@@ -23017,14 +23017,10 @@
       <c r="C680" t="inlineStr"/>
       <c r="D680" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E680" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr"/>
       <c r="F680" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23040,17 +23036,17 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C681" t="inlineStr"/>
       <c r="D681" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E681" t="inlineStr"/>
@@ -23069,7 +23065,7 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
@@ -23079,10 +23075,14 @@
       <c r="C682" t="inlineStr"/>
       <c r="D682" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E682" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F682" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23098,22 +23098,22 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C683" t="inlineStr"/>
       <c r="D683" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E683" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F683" t="inlineStr">
@@ -23131,7 +23131,7 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
@@ -23141,12 +23141,12 @@
       <c r="C684" t="inlineStr"/>
       <c r="D684" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E684" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F684" t="inlineStr">
@@ -23164,24 +23164,20 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C685" t="inlineStr"/>
       <c r="D685" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E685" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr"/>
       <c r="F685" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23197,23 +23193,27 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C686" t="inlineStr"/>
       <c r="D686" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E686" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F686" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G686" t="inlineStr"/>
@@ -23226,27 +23226,23 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C687" t="inlineStr"/>
       <c r="D687" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E687" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr"/>
       <c r="F687" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G687" t="inlineStr"/>
@@ -23259,7 +23255,7 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
@@ -23269,7 +23265,7 @@
       <c r="C688" t="inlineStr"/>
       <c r="D688" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E688" t="inlineStr"/>
@@ -23288,7 +23284,7 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
@@ -23298,7 +23294,7 @@
       <c r="C689" t="inlineStr"/>
       <c r="D689" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E689" t="inlineStr"/>
@@ -23317,7 +23313,7 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
@@ -23327,7 +23323,7 @@
       <c r="C690" t="inlineStr"/>
       <c r="D690" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E690" t="inlineStr"/>
@@ -23346,7 +23342,7 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
@@ -23356,10 +23352,14 @@
       <c r="C691" t="inlineStr"/>
       <c r="D691" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E691" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F691" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23375,24 +23375,20 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C692" t="inlineStr"/>
       <c r="D692" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E692" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr"/>
       <c r="F692" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23408,7 +23404,7 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
@@ -23418,7 +23414,7 @@
       <c r="C693" t="inlineStr"/>
       <c r="D693" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E693" t="inlineStr"/>
@@ -23437,20 +23433,24 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C694" t="inlineStr"/>
       <c r="D694" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E694" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F694" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23466,27 +23466,23 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C695" t="inlineStr"/>
       <c r="D695" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E695" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr"/>
       <c r="F695" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G695" t="inlineStr"/>
@@ -23499,7 +23495,7 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
@@ -23509,7 +23505,7 @@
       <c r="C696" t="inlineStr"/>
       <c r="D696" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E696" t="inlineStr"/>
@@ -23528,23 +23524,27 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C697" t="inlineStr"/>
       <c r="D697" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E697" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F697" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G697" t="inlineStr"/>
@@ -23557,27 +23557,31 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C698" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D698" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E698" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F698" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G698" t="inlineStr"/>
@@ -23590,11 +23594,11 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C699" t="inlineStr">
@@ -23604,12 +23608,12 @@
       </c>
       <c r="D699" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E699" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F699" t="inlineStr">
@@ -23627,26 +23631,26 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C700" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D700" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E700" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F700" t="inlineStr">
@@ -23664,31 +23668,27 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C701" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D701" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E701" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr"/>
       <c r="F701" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G701" t="inlineStr"/>
@@ -23701,27 +23701,27 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C702" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D702" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E702" t="inlineStr"/>
       <c r="F702" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G702" t="inlineStr"/>
@@ -23734,27 +23734,27 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C703" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D703" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E703" t="inlineStr"/>
       <c r="F703" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G703" t="inlineStr"/>
@@ -23767,27 +23767,27 @@
     </row>
     <row r="704">
       <c r="A704" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C704" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D704" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E704" t="inlineStr"/>
       <c r="F704" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G704" t="inlineStr"/>
@@ -23800,24 +23800,28 @@
     </row>
     <row r="705">
       <c r="A705" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B705" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C705" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D705" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E705" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F705" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -23833,11 +23837,11 @@
     </row>
     <row r="706">
       <c r="A706" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B706" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C706" t="inlineStr">
@@ -23847,12 +23851,12 @@
       </c>
       <c r="D706" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E706" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F706" t="inlineStr">
@@ -23870,11 +23874,11 @@
     </row>
     <row r="707">
       <c r="A707" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B707" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C707" t="inlineStr">
@@ -23884,7 +23888,7 @@
       </c>
       <c r="D707" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E707" t="inlineStr">
@@ -23907,31 +23911,31 @@
     </row>
     <row r="708">
       <c r="A708" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C708" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D708" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E708" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F708" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G708" t="inlineStr"/>
@@ -23944,31 +23948,27 @@
     </row>
     <row r="709">
       <c r="A709" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C709" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D709" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E709" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr"/>
       <c r="F709" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G709" t="inlineStr"/>
@@ -23981,27 +23981,31 @@
     </row>
     <row r="710">
       <c r="A710" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C710" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D710" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E710" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F710" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G710" t="inlineStr"/>
@@ -24014,26 +24018,22 @@
     </row>
     <row r="711">
       <c r="A711" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C711" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr"/>
       <c r="D711" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E711" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F711" t="inlineStr">
@@ -24051,30 +24051,38 @@
     </row>
     <row r="712">
       <c r="A712" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B712" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C712" t="inlineStr"/>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D712" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E712" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F712" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G712" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G712" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H712" t="inlineStr"/>
       <c r="I712" t="inlineStr">
         <is>
@@ -24084,38 +24092,34 @@
     </row>
     <row r="713">
       <c r="A713" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C713" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D713" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E713" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F713" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G713" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G713" t="inlineStr"/>
       <c r="H713" t="inlineStr"/>
       <c r="I713" t="inlineStr">
         <is>
@@ -24125,26 +24129,26 @@
     </row>
     <row r="714">
       <c r="A714" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B714" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C714" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D714" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E714" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F714" t="inlineStr">
@@ -24152,7 +24156,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G714" t="inlineStr"/>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H714" t="inlineStr"/>
       <c r="I714" t="inlineStr">
         <is>
@@ -24162,11 +24170,11 @@
     </row>
     <row r="715">
       <c r="A715" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C715" t="inlineStr">
@@ -24176,67 +24184,26 @@
       </c>
       <c r="D715" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E715" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F715" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G715" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H715" t="inlineStr"/>
       <c r="I715" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="716">
-      <c r="A716" t="n">
-        <v>763</v>
-      </c>
-      <c r="B716" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C716" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D716" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E716" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F716" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G716" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H716" t="inlineStr"/>
-      <c r="I716" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 574 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I704"/>
+  <dimension ref="A1:I703"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18327,7 +18327,7 @@
     </row>
     <row r="536">
       <c r="A536" t="n">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B536" t="inlineStr">
         <is>
@@ -18338,7 +18338,7 @@
       <c r="D536" t="inlineStr"/>
       <c r="E536" t="inlineStr">
         <is>
-          <t>MM</t>
+          <t>nahrání nových dat IS</t>
         </is>
       </c>
       <c r="F536" t="inlineStr">
@@ -18356,18 +18356,22 @@
     </row>
     <row r="537">
       <c r="A537" t="n">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>814 028</t>
+          <t>814 072</t>
         </is>
       </c>
       <c r="C537" t="inlineStr"/>
-      <c r="D537" t="inlineStr"/>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>Tempo na 814 nedrží čas</t>
+        </is>
+      </c>
       <c r="E537" t="inlineStr">
         <is>
-          <t>nahrání nových dat IS</t>
+          <t>výměna Tempa</t>
         </is>
       </c>
       <c r="F537" t="inlineStr">
@@ -18385,22 +18389,22 @@
     </row>
     <row r="538">
       <c r="A538" t="n">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>814 072</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C538" t="inlineStr"/>
       <c r="D538" t="inlineStr">
         <is>
-          <t>Tempo na 814 nedrží čas</t>
+          <t>na 814 se samovolně restartuje Tempo</t>
         </is>
       </c>
       <c r="E538" t="inlineStr">
         <is>
-          <t>výměna Tempa</t>
+          <t>neděláno,nebyla tu</t>
         </is>
       </c>
       <c r="F538" t="inlineStr">
@@ -18418,22 +18422,22 @@
     </row>
     <row r="539">
       <c r="A539" t="n">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 191</t>
         </is>
       </c>
       <c r="C539" t="inlineStr"/>
       <c r="D539" t="inlineStr">
         <is>
-          <t>na 814 se samovolně restartuje Tempo</t>
+          <t>někdy nejdou zavřít dvojité dveře (obě strany)</t>
         </is>
       </c>
       <c r="E539" t="inlineStr">
         <is>
-          <t>neděláno,nebyla tu</t>
+          <t>obě optozávory byly nastaveny až nazábradlí a jak posvítilo slunce asi to trochu zkreslilo a reagovaly. Nastavení cca 20cm od zábradlí</t>
         </is>
       </c>
       <c r="F539" t="inlineStr">
@@ -18451,22 +18455,22 @@
     </row>
     <row r="540">
       <c r="A540" t="n">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>814 191</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C540" t="inlineStr"/>
       <c r="D540" t="inlineStr">
         <is>
-          <t>někdy nejdou zavřít dvojité dveře (obě strany)</t>
+          <t>levé schody  na A nejdou</t>
         </is>
       </c>
       <c r="E540" t="inlineStr">
         <is>
-          <t>obě optozávory byly nastaveny až nazábradlí a jak posvítilo slunce asi to trochu zkreslilo a reagovaly. Nastavení cca 20cm od zábradlí</t>
+          <t>výměna motorku</t>
         </is>
       </c>
       <c r="F540" t="inlineStr">
@@ -18484,24 +18488,20 @@
     </row>
     <row r="541">
       <c r="A541" t="n">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C541" t="inlineStr"/>
       <c r="D541" t="inlineStr">
         <is>
-          <t>levé schody  na A nejdou</t>
-        </is>
-      </c>
-      <c r="E541" t="inlineStr">
-        <is>
-          <t>výměna motorku</t>
-        </is>
-      </c>
+          <t>MM</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr"/>
       <c r="F541" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -18517,7 +18517,7 @@
     </row>
     <row r="542">
       <c r="A542" t="n">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B542" t="inlineStr">
         <is>
@@ -18527,10 +18527,14 @@
       <c r="C542" t="inlineStr"/>
       <c r="D542" t="inlineStr">
         <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E542" t="inlineStr"/>
+          <t>levé dveře na 914 se nezavírají</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>vadná optozávora - výměna</t>
+        </is>
+      </c>
       <c r="F542" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -18546,22 +18550,18 @@
     </row>
     <row r="543">
       <c r="A543" t="n">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>814 076</t>
         </is>
       </c>
       <c r="C543" t="inlineStr"/>
-      <c r="D543" t="inlineStr">
-        <is>
-          <t>levé dveře na 914 se nezavírají</t>
-        </is>
-      </c>
+      <c r="D543" t="inlineStr"/>
       <c r="E543" t="inlineStr">
         <is>
-          <t>vadná optozávora - výměna</t>
+          <t>vyčtení rychloměru</t>
         </is>
       </c>
       <c r="F543" t="inlineStr">
@@ -18579,18 +18579,26 @@
     </row>
     <row r="544">
       <c r="A544" t="n">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>814 076</t>
-        </is>
-      </c>
-      <c r="C544" t="inlineStr"/>
-      <c r="D544" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>22.06.2023</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>nasvěcuje se poruha mazání nákolků !MOK (přední stanoviště)</t>
+        </is>
+      </c>
       <c r="E544" t="inlineStr">
         <is>
-          <t>vyčtení rychloměru</t>
+          <t>při navolení přepínače SA90 do polohy plnění se závada cca 3x projevila,bohužel jsem nestihl doběhnout k obrazovce dřív než se zablokovala. Ale pravděpodobně nespína signál MOP (spíná ventil co pouští vzduch). Udělal jsem ještě profuk. Pravděpodobně to bylo někde přicpané a nedošlo ke změně tlaku na tlakáčích v bloku A61. Pro jistotu jsem ještě přehodil v DPV IN karty (první s druhou) a OUT karty.</t>
         </is>
       </c>
       <c r="F544" t="inlineStr">
@@ -18608,26 +18616,22 @@
     </row>
     <row r="545">
       <c r="A545" t="n">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C545" t="inlineStr">
-        <is>
-          <t>22.06.2023</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr"/>
       <c r="D545" t="inlineStr">
         <is>
-          <t>nasvěcuje se poruha mazání nákolků !MOK (přední stanoviště)</t>
+          <t>často se navěcuje požár rozvaděče</t>
         </is>
       </c>
       <c r="E545" t="inlineStr">
         <is>
-          <t>při navolení přepínače SA90 do polohy plnění se závada cca 3x projevila,bohužel jsem nestihl doběhnout k obrazovce dřív než se zablokovala. Ale pravděpodobně nespína signál MOP (spíná ventil co pouští vzduch). Udělal jsem ještě profuk. Pravděpodobně to bylo někde přicpané a nedošlo ke změně tlaku na tlakáčích v bloku A61. Pro jistotu jsem ještě přehodil v DPV IN karty (první s druhou) a OUT karty.</t>
+          <t>neprojevilo se,výměna čidla požáru v RTO</t>
         </is>
       </c>
       <c r="F545" t="inlineStr">
@@ -18645,22 +18649,22 @@
     </row>
     <row r="546">
       <c r="A546" t="n">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C546" t="inlineStr"/>
       <c r="D546" t="inlineStr">
         <is>
-          <t>často se navěcuje požár rozvaděče</t>
+          <t>levé schody  na A nejdou</t>
         </is>
       </c>
       <c r="E546" t="inlineStr">
         <is>
-          <t>neprojevilo se,výměna čidla požáru v RTO</t>
+          <t>nečistoy kolem motoru+řemen</t>
         </is>
       </c>
       <c r="F546" t="inlineStr">
@@ -18678,22 +18682,22 @@
     </row>
     <row r="547">
       <c r="A547" t="n">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B547" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C547" t="inlineStr"/>
       <c r="D547" t="inlineStr">
         <is>
-          <t>levé schody  na A nejdou</t>
+          <t>údajne obrazovka IS v sekci B nad průchozími dveřmi ( směrem od WC) po tmě</t>
         </is>
       </c>
       <c r="E547" t="inlineStr">
         <is>
-          <t>nečistoy kolem motoru+řemen</t>
+          <t>neprojevilo se,kontrola konektorů,poklep obrazovka.Vše OK</t>
         </is>
       </c>
       <c r="F547" t="inlineStr">
@@ -18711,7 +18715,7 @@
     </row>
     <row r="548">
       <c r="A548" t="n">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B548" t="inlineStr">
         <is>
@@ -18721,12 +18725,12 @@
       <c r="C548" t="inlineStr"/>
       <c r="D548" t="inlineStr">
         <is>
-          <t>údajne obrazovka IS v sekci B nad průchozími dveřmi ( směrem od WC) po tmě</t>
+          <t>údajně problikává chyba čidla měření nafty</t>
         </is>
       </c>
       <c r="E548" t="inlineStr">
         <is>
-          <t>neprojevilo se,kontrola konektorů,poklep obrazovka.Vše OK</t>
+          <t>nenapsali jakého,neprojevilo se</t>
         </is>
       </c>
       <c r="F548" t="inlineStr">
@@ -18744,22 +18748,22 @@
     </row>
     <row r="549">
       <c r="A549" t="n">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C549" t="inlineStr"/>
       <c r="D549" t="inlineStr">
         <is>
-          <t>údajně problikává chyba čidla měření nafty</t>
+          <t>nechladí</t>
         </is>
       </c>
       <c r="E549" t="inlineStr">
         <is>
-          <t>nenapsali jakého,neprojevilo se</t>
+          <t>vydný proporcionální ventil,výměna</t>
         </is>
       </c>
       <c r="F549" t="inlineStr">
@@ -18777,22 +18781,22 @@
     </row>
     <row r="550">
       <c r="A550" t="n">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>842 015</t>
         </is>
       </c>
       <c r="C550" t="inlineStr"/>
       <c r="D550" t="inlineStr">
         <is>
-          <t>nechladí</t>
+          <t>někdy nejde brzda PB</t>
         </is>
       </c>
       <c r="E550" t="inlineStr">
         <is>
-          <t>vydný proporcionální ventil,výměna</t>
+          <t>výměna ventilu YV 61 včetně cívky</t>
         </is>
       </c>
       <c r="F550" t="inlineStr">
@@ -18810,22 +18814,22 @@
     </row>
     <row r="551">
       <c r="A551" t="n">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C551" t="inlineStr"/>
       <c r="D551" t="inlineStr">
         <is>
-          <t>někdy nejde brzda PB</t>
+          <t>v B salónu ukazuje prostřední čidlo 0°C</t>
         </is>
       </c>
       <c r="E551" t="inlineStr">
         <is>
-          <t>výměna ventilu YV 61 včetně cívky</t>
+          <t>po zahýbáním káblíku co vede ze stěny do svorkovnice čidla vše OK. Prodřený drát cca 5 cm od konce. Nasazení smršťovačky,přesvorkování dutinek</t>
         </is>
       </c>
       <c r="F551" t="inlineStr">
@@ -18843,22 +18847,22 @@
     </row>
     <row r="552">
       <c r="A552" t="n">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B552" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C552" t="inlineStr"/>
       <c r="D552" t="inlineStr">
         <is>
-          <t>v B salónu ukazuje prostřední čidlo 0°C</t>
+          <t>neukazuje vodoznak,pravá strana</t>
         </is>
       </c>
       <c r="E552" t="inlineStr">
         <is>
-          <t>po zahýbáním káblíku co vede ze stěny do svorkovnice čidla vše OK. Prodřený drát cca 5 cm od konce. Nasazení smršťovačky,přesvorkování dutinek</t>
+          <t>výměna</t>
         </is>
       </c>
       <c r="F552" t="inlineStr">
@@ -18876,22 +18880,22 @@
     </row>
     <row r="553">
       <c r="A553" t="n">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C553" t="inlineStr"/>
       <c r="D553" t="inlineStr">
         <is>
-          <t>neukazuje vodoznak,pravá strana</t>
+          <t>opět slabý výkon</t>
         </is>
       </c>
       <c r="E553" t="inlineStr">
         <is>
-          <t>výměna</t>
+          <t>byly "vyběhané" kloubky na táhlu AČ,výměna.Seřízení pákový,při 25% 930 otáček</t>
         </is>
       </c>
       <c r="F553" t="inlineStr">
@@ -18909,22 +18913,22 @@
     </row>
     <row r="554">
       <c r="A554" t="n">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="B554" t="inlineStr">
         <is>
-          <t>814 118</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C554" t="inlineStr"/>
       <c r="D554" t="inlineStr">
         <is>
-          <t>opět slabý výkon</t>
+          <t>údajně nejde ARR z B</t>
         </is>
       </c>
       <c r="E554" t="inlineStr">
         <is>
-          <t>byly "vyběhané" kloubky na táhlu AČ,výměna.Seřízení pákový,při 25% 930 otáček</t>
+          <t>neprojevilo se,neměněno</t>
         </is>
       </c>
       <c r="F554" t="inlineStr">
@@ -18942,7 +18946,7 @@
     </row>
     <row r="555">
       <c r="A555" t="n">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B555" t="inlineStr">
         <is>
@@ -18952,12 +18956,12 @@
       <c r="C555" t="inlineStr"/>
       <c r="D555" t="inlineStr">
         <is>
-          <t>údajně nejde ARR z B</t>
+          <t>v A salónu ukazuje prostřední čidlo -17°C</t>
         </is>
       </c>
       <c r="E555" t="inlineStr">
         <is>
-          <t>neprojevilo se,neměněno</t>
+          <t>ve skutečnosti se jedná o čidlo u měchů. 6.9.2021 se přehazovali vstupy do ŘJ mezi měchy a prostředkem. Chyba byla v prostředku. 2 roky pak byl klid. Proměření ohmicky cesty,vstupy dány zpět jak mají být. Pokud se vrátí zase v prostředku,chyba v ŘJ</t>
         </is>
       </c>
       <c r="F555" t="inlineStr">
@@ -18975,22 +18979,22 @@
     </row>
     <row r="556">
       <c r="A556" t="n">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="B556" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>029 227</t>
         </is>
       </c>
       <c r="C556" t="inlineStr"/>
       <c r="D556" t="inlineStr">
         <is>
-          <t>v A salónu ukazuje prostřední čidlo -17°C</t>
+          <t>porucha dveří elektr.</t>
         </is>
       </c>
       <c r="E556" t="inlineStr">
         <is>
-          <t>ve skutečnosti se jedná o čidlo u měchů. 6.9.2021 se přehazovali vstupy do ŘJ mezi měchy a prostředkem. Chyba byla v prostředku. 2 roky pak byl klid. Proměření ohmicky cesty,vstupy dány zpět jak mají být. Pokud se vrátí zase v prostředku,chyba v ŘJ</t>
+          <t>neprojevilo se , přezkoušení stran</t>
         </is>
       </c>
       <c r="F556" t="inlineStr">
@@ -19008,22 +19012,22 @@
     </row>
     <row r="557">
       <c r="A557" t="n">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>029 227</t>
+          <t>742 263</t>
         </is>
       </c>
       <c r="C557" t="inlineStr"/>
       <c r="D557" t="inlineStr">
         <is>
-          <t>porucha dveří elektr.</t>
+          <t>při startu dlouho promázává, nejde zkrácený start</t>
         </is>
       </c>
       <c r="E557" t="inlineStr">
         <is>
-          <t>neprojevilo se , přezkoušení stran</t>
+          <t>vše bylo funkční , zkrácený start spíná při 49°C přesto výměna YCR7</t>
         </is>
       </c>
       <c r="F557" t="inlineStr">
@@ -19041,7 +19045,7 @@
     </row>
     <row r="558">
       <c r="A558" t="n">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B558" t="inlineStr">
         <is>
@@ -19051,12 +19055,12 @@
       <c r="C558" t="inlineStr"/>
       <c r="D558" t="inlineStr">
         <is>
-          <t>při startu dlouho promázává, nejde zkrácený start</t>
+          <t>porucha dveří elektr.</t>
         </is>
       </c>
       <c r="E558" t="inlineStr">
         <is>
-          <t>vše bylo funkční , zkrácený start spíná při 49°C přesto výměna YCR7</t>
+          <t>neprojevilo se , přezkoušení stran</t>
         </is>
       </c>
       <c r="F558" t="inlineStr">
@@ -19074,22 +19078,22 @@
     </row>
     <row r="559">
       <c r="A559" t="n">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B559" t="inlineStr">
         <is>
-          <t>742 263</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C559" t="inlineStr"/>
       <c r="D559" t="inlineStr">
         <is>
-          <t>porucha dveří elektr.</t>
+          <t>IS se rozpadá, ztráci komunikaci mezi stan.</t>
         </is>
       </c>
       <c r="E559" t="inlineStr">
         <is>
-          <t>neprojevilo se , přezkoušení stran</t>
+          <t>dotlační konektoru ale vše bylo funkční</t>
         </is>
       </c>
       <c r="F559" t="inlineStr">
@@ -19107,7 +19111,7 @@
     </row>
     <row r="560">
       <c r="A560" t="n">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B560" t="inlineStr">
         <is>
@@ -19117,12 +19121,12 @@
       <c r="C560" t="inlineStr"/>
       <c r="D560" t="inlineStr">
         <is>
-          <t>IS se rozpadá, ztráci komunikaci mezi stan.</t>
+          <t>parkovací brzda nevybaví KBS</t>
         </is>
       </c>
       <c r="E560" t="inlineStr">
         <is>
-          <t>dotlační konektoru ale vše bylo funkční</t>
+          <t>seřízení tlaku</t>
         </is>
       </c>
       <c r="F560" t="inlineStr">
@@ -19140,7 +19144,7 @@
     </row>
     <row r="561">
       <c r="A561" t="n">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="B561" t="inlineStr">
         <is>
@@ -19150,12 +19154,12 @@
       <c r="C561" t="inlineStr"/>
       <c r="D561" t="inlineStr">
         <is>
-          <t>parkovací brzda nevybaví KBS</t>
+          <t>únik oleje na 6. válci</t>
         </is>
       </c>
       <c r="E561" t="inlineStr">
         <is>
-          <t>seřízení tlaku</t>
+          <t>výměna</t>
         </is>
       </c>
       <c r="F561" t="inlineStr">
@@ -19173,7 +19177,7 @@
     </row>
     <row r="562">
       <c r="A562" t="n">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B562" t="inlineStr">
         <is>
@@ -19183,12 +19187,12 @@
       <c r="C562" t="inlineStr"/>
       <c r="D562" t="inlineStr">
         <is>
-          <t>únik oleje na 6. válci</t>
+          <t>nesvítí červené poziční světlo</t>
         </is>
       </c>
       <c r="E562" t="inlineStr">
         <is>
-          <t>výměna</t>
+          <t>zapojení vodiče 735 byl odpojený (výměna obou světel na stan 914)</t>
         </is>
       </c>
       <c r="F562" t="inlineStr">
@@ -19206,22 +19210,22 @@
     </row>
     <row r="563">
       <c r="A563" t="n">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="B563" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C563" t="inlineStr"/>
       <c r="D563" t="inlineStr">
         <is>
-          <t>nesvítí červené poziční světlo</t>
+          <t>nelze odbrzdit, tlak ve válcích zůstáva 0,3 bar závada jen z 914</t>
         </is>
       </c>
       <c r="E563" t="inlineStr">
         <is>
-          <t>zapojení vodiče 735 byl odpojený (výměna obou světel na stan 914)</t>
+          <t>zk. Jízda OK</t>
         </is>
       </c>
       <c r="F563" t="inlineStr">
@@ -19239,22 +19243,22 @@
     </row>
     <row r="564">
       <c r="A564" t="n">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B564" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C564" t="inlineStr"/>
       <c r="D564" t="inlineStr">
         <is>
-          <t>nelze odbrzdit, tlak ve válcích zůstáva 0,3 bar závada jen z 914</t>
+          <t>2.SM samovolně zvyšuje otáčky, seřízení GAC</t>
         </is>
       </c>
       <c r="E564" t="inlineStr">
         <is>
-          <t>zk. Jízda OK</t>
+          <t>přístě vyměnit GAC musela jet ven</t>
         </is>
       </c>
       <c r="F564" t="inlineStr">
@@ -19272,22 +19276,22 @@
     </row>
     <row r="565">
       <c r="A565" t="n">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="B565" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C565" t="inlineStr"/>
       <c r="D565" t="inlineStr">
         <is>
-          <t>2.SM samovolně zvyšuje otáčky, seřízení GAC</t>
+          <t>nehlási IS na stan. A</t>
         </is>
       </c>
       <c r="E565" t="inlineStr">
         <is>
-          <t>přístě vyměnit GAC musela jet ven</t>
+          <t>ztlumen potenciometr</t>
         </is>
       </c>
       <c r="F565" t="inlineStr">
@@ -19305,7 +19309,7 @@
     </row>
     <row r="566">
       <c r="A566" t="n">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B566" t="inlineStr">
         <is>
@@ -19315,12 +19319,12 @@
       <c r="C566" t="inlineStr"/>
       <c r="D566" t="inlineStr">
         <is>
-          <t>nehlási IS na stan. A</t>
+          <t>lednice nechladí</t>
         </is>
       </c>
       <c r="E566" t="inlineStr">
         <is>
-          <t>ztlumen potenciometr</t>
+          <t>odzkoušeno OK</t>
         </is>
       </c>
       <c r="F566" t="inlineStr">
@@ -19338,7 +19342,7 @@
     </row>
     <row r="567">
       <c r="A567" t="n">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B567" t="inlineStr">
         <is>
@@ -19348,12 +19352,12 @@
       <c r="C567" t="inlineStr"/>
       <c r="D567" t="inlineStr">
         <is>
-          <t>lednice nechladí</t>
+          <t>údajně rázy převodovky</t>
         </is>
       </c>
       <c r="E567" t="inlineStr">
         <is>
-          <t>odzkoušeno OK</t>
+          <t>řesí p. Šípek vyčítal jsi obě HMP</t>
         </is>
       </c>
       <c r="F567" t="inlineStr">
@@ -19371,22 +19375,22 @@
     </row>
     <row r="568">
       <c r="A568" t="n">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C568" t="inlineStr"/>
       <c r="D568" t="inlineStr">
         <is>
-          <t>údajně rázy převodovky</t>
+          <t>lok. Nejde nastartovat</t>
         </is>
       </c>
       <c r="E568" t="inlineStr">
         <is>
-          <t>řesí p. Šípek vyčítal jsi obě HMP</t>
+          <t>naftová netěsnost</t>
         </is>
       </c>
       <c r="F568" t="inlineStr">
@@ -19404,22 +19408,22 @@
     </row>
     <row r="569">
       <c r="A569" t="n">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B569" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C569" t="inlineStr"/>
       <c r="D569" t="inlineStr">
         <is>
-          <t>lok. Nejde nastartovat</t>
+          <t>izolačni stav odztraněny zkraty na vodiči 80 a 50</t>
         </is>
       </c>
       <c r="E569" t="inlineStr">
         <is>
-          <t>naftová netěsnost</t>
+          <t>startéry vyfoukany,ale nakonec výměna M2(volný pomocný vodič) seřízení GAC 2. SM , zkušební jízda se zdá v pořádku</t>
         </is>
       </c>
       <c r="F569" t="inlineStr">
@@ -19437,24 +19441,24 @@
     </row>
     <row r="570">
       <c r="A570" t="n">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>842 035</t>
-        </is>
-      </c>
-      <c r="C570" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>06.12.2023</t>
+        </is>
+      </c>
       <c r="D570" t="inlineStr">
         <is>
-          <t>izolačni stav odztraněny zkraty na vodiči 80 a 50</t>
-        </is>
-      </c>
-      <c r="E570" t="inlineStr">
-        <is>
-          <t>startéry vyfoukany,ale nakonec výměna M2(volný pomocný vodič) seřízení GAC 2. SM , zkušební jízda se zdá v pořádku</t>
-        </is>
-      </c>
+          <t>Výměna obrazovky na 914 (občas zamrzá)</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr"/>
       <c r="F570" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19470,11 +19474,11 @@
     </row>
     <row r="571">
       <c r="A571" t="n">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B571" t="inlineStr">
         <is>
-          <t>814 003</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C571" t="inlineStr">
@@ -19484,7 +19488,7 @@
       </c>
       <c r="D571" t="inlineStr">
         <is>
-          <t>Výměna obrazovky na 914 (občas zamrzá)</t>
+          <t>údajně se rozpadá IS přezkoušeno (kontrola konektoru)</t>
         </is>
       </c>
       <c r="E571" t="inlineStr"/>
@@ -19503,11 +19507,11 @@
     </row>
     <row r="572">
       <c r="A572" t="n">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 072</t>
         </is>
       </c>
       <c r="C572" t="inlineStr">
@@ -19517,7 +19521,7 @@
       </c>
       <c r="D572" t="inlineStr">
         <is>
-          <t>údajně se rozpadá IS přezkoušeno (kontrola konektoru)</t>
+          <t>tozpadáva se IS, oprava dispeleje na 914 byl volný</t>
         </is>
       </c>
       <c r="E572" t="inlineStr"/>
@@ -19536,24 +19540,28 @@
     </row>
     <row r="573">
       <c r="A573" t="n">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>814 072</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C573" t="inlineStr">
         <is>
-          <t>06.12.2023</t>
+          <t>06.11.2023</t>
         </is>
       </c>
       <c r="D573" t="inlineStr">
         <is>
-          <t>tozpadáva se IS, oprava dispeleje na 914 byl volný</t>
-        </is>
-      </c>
-      <c r="E573" t="inlineStr"/>
+          <t>tabule vnitřní , venkovní nekomunikují</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>výměna konektoru C na 914</t>
+        </is>
+      </c>
       <c r="F573" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19569,11 +19577,11 @@
     </row>
     <row r="574">
       <c r="A574" t="n">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>814 118</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C574" t="inlineStr">
@@ -19583,12 +19591,12 @@
       </c>
       <c r="D574" t="inlineStr">
         <is>
-          <t>tabule vnitřní , venkovní nekomunikují</t>
+          <t>korekce vody 2</t>
         </is>
       </c>
       <c r="E574" t="inlineStr">
         <is>
-          <t>výměna konektoru C na 914</t>
+          <t>izolačni stav špatný  stáhlé zemni relé</t>
         </is>
       </c>
       <c r="F574" t="inlineStr">
@@ -19606,11 +19614,11 @@
     </row>
     <row r="575">
       <c r="A575" t="n">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B575" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C575" t="inlineStr">
@@ -19620,14 +19628,10 @@
       </c>
       <c r="D575" t="inlineStr">
         <is>
-          <t>korekce vody 2</t>
-        </is>
-      </c>
-      <c r="E575" t="inlineStr">
-        <is>
-          <t>izolačni stav špatný  stáhlé zemni relé</t>
-        </is>
-      </c>
+          <t>výměna ARR na B stan. Nefunkční</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr"/>
       <c r="F575" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19643,21 +19647,21 @@
     </row>
     <row r="576">
       <c r="A576" t="n">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="B576" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>842 011</t>
         </is>
       </c>
       <c r="C576" t="inlineStr">
         <is>
-          <t>06.11.2023</t>
+          <t>06.10.2023</t>
         </is>
       </c>
       <c r="D576" t="inlineStr">
         <is>
-          <t>výměna ARR na B stan. Nefunkční</t>
+          <t>udajně zateklo do pultu na 2st.(kontrola)</t>
         </is>
       </c>
       <c r="E576" t="inlineStr"/>
@@ -19676,11 +19680,11 @@
     </row>
     <row r="577">
       <c r="A577" t="n">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>842 011</t>
+          <t>842 021</t>
         </is>
       </c>
       <c r="C577" t="inlineStr">
@@ -19690,10 +19694,14 @@
       </c>
       <c r="D577" t="inlineStr">
         <is>
-          <t>udajně zateklo do pultu na 2st.(kontrola)</t>
-        </is>
-      </c>
-      <c r="E577" t="inlineStr"/>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>vadné čidlo vody v míse</t>
+        </is>
+      </c>
       <c r="F577" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19709,26 +19717,26 @@
     </row>
     <row r="578">
       <c r="A578" t="n">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>842 021</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C578" t="inlineStr">
         <is>
-          <t>06.10.2023</t>
+          <t>06.09.2023</t>
         </is>
       </c>
       <c r="D578" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>Nejdou dvěře WC</t>
         </is>
       </c>
       <c r="E578" t="inlineStr">
         <is>
-          <t>vadné čidlo vody v míse</t>
+          <t>upadlý drát na přepínači funkce WC (zapnuto,bez dveří, vypnuto). Seřízení zámykání dveří. Frýdek</t>
         </is>
       </c>
       <c r="F578" t="inlineStr">
@@ -19746,11 +19754,11 @@
     </row>
     <row r="579">
       <c r="A579" t="n">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B579" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C579" t="inlineStr">
@@ -19760,12 +19768,12 @@
       </c>
       <c r="D579" t="inlineStr">
         <is>
-          <t>Nejdou dvěře WC</t>
+          <t>údajně nejdou někdy schody u levých dveří strany A</t>
         </is>
       </c>
       <c r="E579" t="inlineStr">
         <is>
-          <t>upadlý drát na přepínači funkce WC (zapnuto,bez dveří, vypnuto). Seřízení zámykání dveří. Frýdek</t>
+          <t>vyčištění od kamínků,odzkoušení-OK</t>
         </is>
       </c>
       <c r="F579" t="inlineStr">
@@ -19783,26 +19791,26 @@
     </row>
     <row r="580">
       <c r="A580" t="n">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="B580" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C580" t="inlineStr">
         <is>
-          <t>06.09.2023</t>
+          <t>06.08.2023</t>
         </is>
       </c>
       <c r="D580" t="inlineStr">
         <is>
-          <t>údajně nejdou někdy schody u levých dveří strany A</t>
+          <t>zapůjčena z HB</t>
         </is>
       </c>
       <c r="E580" t="inlineStr">
         <is>
-          <t>vyčištění od kamínků,odzkoušení-OK</t>
+          <t>nahrány data IS ( funguje preš radiostanici)</t>
         </is>
       </c>
       <c r="F580" t="inlineStr">
@@ -19820,11 +19828,11 @@
     </row>
     <row r="581">
       <c r="A581" t="n">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B581" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C581" t="inlineStr">
@@ -19834,12 +19842,12 @@
       </c>
       <c r="D581" t="inlineStr">
         <is>
-          <t>zapůjčena z HB</t>
+          <t>Opět problémy se startováním</t>
         </is>
       </c>
       <c r="E581" t="inlineStr">
         <is>
-          <t>nahrány data IS ( funguje preš radiostanici)</t>
+          <t>(asi už vadný capos kondy)říkali veselani jak tu byli</t>
         </is>
       </c>
       <c r="F581" t="inlineStr">
@@ -19857,7 +19865,7 @@
     </row>
     <row r="582">
       <c r="A582" t="n">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B582" t="inlineStr">
         <is>
@@ -19871,12 +19879,12 @@
       </c>
       <c r="D582" t="inlineStr">
         <is>
-          <t>Opět problémy se startováním</t>
+          <t>oprava hlasitosti na stanovišti A</t>
         </is>
       </c>
       <c r="E582" t="inlineStr">
         <is>
-          <t>(asi už vadný capos kondy)říkali veselani jak tu byli</t>
+          <t>přechod na kontaktech u reproduktoru v pultě</t>
         </is>
       </c>
       <c r="F582" t="inlineStr">
@@ -19894,11 +19902,11 @@
     </row>
     <row r="583">
       <c r="A583" t="n">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B583" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C583" t="inlineStr">
@@ -19908,12 +19916,12 @@
       </c>
       <c r="D583" t="inlineStr">
         <is>
-          <t>oprava hlasitosti na stanovišti A</t>
+          <t>výměna ARR na B</t>
         </is>
       </c>
       <c r="E583" t="inlineStr">
         <is>
-          <t>přechod na kontaktech u reproduktoru v pultě</t>
+          <t>vadná linka CAN</t>
         </is>
       </c>
       <c r="F583" t="inlineStr">
@@ -19931,26 +19939,26 @@
     </row>
     <row r="584">
       <c r="A584" t="n">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B584" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>842 015</t>
         </is>
       </c>
       <c r="C584" t="inlineStr">
         <is>
-          <t>06.08.2023</t>
+          <t>06.07.2023</t>
         </is>
       </c>
       <c r="D584" t="inlineStr">
         <is>
-          <t>výměna ARR na B</t>
+          <t>někdy nejde brzda PB</t>
         </is>
       </c>
       <c r="E584" t="inlineStr">
         <is>
-          <t>vadná linka CAN</t>
+          <t>výměna karty DS a OUT z 842 025</t>
         </is>
       </c>
       <c r="F584" t="inlineStr">
@@ -19968,11 +19976,11 @@
     </row>
     <row r="585">
       <c r="A585" t="n">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B585" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C585" t="inlineStr">
@@ -19982,14 +19990,10 @@
       </c>
       <c r="D585" t="inlineStr">
         <is>
-          <t>někdy nejde brzda PB</t>
-        </is>
-      </c>
-      <c r="E585" t="inlineStr">
-        <is>
-          <t>výměna karty DS a OUT z 842 025</t>
-        </is>
-      </c>
+          <t>dosazeny karty z 842 015 (DS a OUT)</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr"/>
       <c r="F585" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20005,11 +20009,11 @@
     </row>
     <row r="586">
       <c r="A586" t="n">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B586" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C586" t="inlineStr">
@@ -20019,10 +20023,14 @@
       </c>
       <c r="D586" t="inlineStr">
         <is>
-          <t>dosazeny karty z 842 015 (DS a OUT)</t>
-        </is>
-      </c>
-      <c r="E586" t="inlineStr"/>
+          <t>dosazen asi 5 dobíječ na B funkční</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>ve skladu nefunkční jenom (má řešit asi Mlíčko)</t>
+        </is>
+      </c>
       <c r="F586" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20038,28 +20046,24 @@
     </row>
     <row r="587">
       <c r="A587" t="n">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="B587" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 076</t>
         </is>
       </c>
       <c r="C587" t="inlineStr">
         <is>
-          <t>06.07.2023</t>
+          <t>06.06.2023</t>
         </is>
       </c>
       <c r="D587" t="inlineStr">
         <is>
-          <t>dosazen asi 5 dobíječ na B funkční</t>
-        </is>
-      </c>
-      <c r="E587" t="inlineStr">
-        <is>
-          <t>ve skladu nefunkční jenom (má řešit asi Mlíčko)</t>
-        </is>
-      </c>
+          <t>NEHODA V HOLEŠOVĚ</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr"/>
       <c r="F587" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20075,21 +20079,17 @@
     </row>
     <row r="588">
       <c r="A588" t="n">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="B588" t="inlineStr">
         <is>
-          <t>814 076</t>
-        </is>
-      </c>
-      <c r="C588" t="inlineStr">
-        <is>
-          <t>06.06.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr"/>
       <c r="D588" t="inlineStr">
         <is>
-          <t>NEHODA V HOLEŠOVĚ</t>
+          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
         </is>
       </c>
       <c r="E588" t="inlineStr"/>
@@ -20108,7 +20108,7 @@
     </row>
     <row r="589">
       <c r="A589" t="n">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="B589" t="inlineStr">
         <is>
@@ -20118,7 +20118,7 @@
       <c r="C589" t="inlineStr"/>
       <c r="D589" t="inlineStr">
         <is>
-          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
+          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
         </is>
       </c>
       <c r="E589" t="inlineStr"/>
@@ -20137,7 +20137,7 @@
     </row>
     <row r="590">
       <c r="A590" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B590" t="inlineStr">
         <is>
@@ -20147,7 +20147,7 @@
       <c r="C590" t="inlineStr"/>
       <c r="D590" t="inlineStr">
         <is>
-          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
+          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
         </is>
       </c>
       <c r="E590" t="inlineStr"/>
@@ -20166,20 +20166,24 @@
     </row>
     <row r="591">
       <c r="A591" t="n">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B591" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C591" t="inlineStr"/>
       <c r="D591" t="inlineStr">
         <is>
-          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
-        </is>
-      </c>
-      <c r="E591" t="inlineStr"/>
+          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>vyměnili dobíječ stacionární (Veselí)</t>
+        </is>
+      </c>
       <c r="F591" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20195,22 +20199,22 @@
     </row>
     <row r="592">
       <c r="A592" t="n">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C592" t="inlineStr"/>
       <c r="D592" t="inlineStr">
         <is>
-          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
         </is>
       </c>
       <c r="E592" t="inlineStr">
         <is>
-          <t>vyměnili dobíječ stacionární (Veselí)</t>
+          <t>jela ven</t>
         </is>
       </c>
       <c r="F592" t="inlineStr">
@@ -20228,24 +20232,20 @@
     </row>
     <row r="593">
       <c r="A593" t="n">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C593" t="inlineStr"/>
       <c r="D593" t="inlineStr">
         <is>
-          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
-        </is>
-      </c>
-      <c r="E593" t="inlineStr">
-        <is>
-          <t>jela ven</t>
-        </is>
-      </c>
+          <t>seřízení kamer přes program v notasu(obraz)</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr"/>
       <c r="F593" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20261,20 +20261,24 @@
     </row>
     <row r="594">
       <c r="A594" t="n">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B594" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C594" t="inlineStr"/>
       <c r="D594" t="inlineStr">
         <is>
-          <t>seřízení kamer přes program v notasu(obraz)</t>
-        </is>
-      </c>
-      <c r="E594" t="inlineStr"/>
+          <t>po startu někdy nenabíjí "B"</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+        </is>
+      </c>
       <c r="F594" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20290,22 +20294,22 @@
     </row>
     <row r="595">
       <c r="A595" t="n">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C595" t="inlineStr"/>
       <c r="D595" t="inlineStr">
         <is>
-          <t>po startu někdy nenabíjí "B"</t>
+          <t>2. motor korekce vody  vystup</t>
         </is>
       </c>
       <c r="E595" t="inlineStr">
         <is>
-          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
         </is>
       </c>
       <c r="F595" t="inlineStr">
@@ -20323,24 +20327,24 @@
     </row>
     <row r="596">
       <c r="A596" t="n">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B596" t="inlineStr">
         <is>
-          <t>842 035</t>
-        </is>
-      </c>
-      <c r="C596" t="inlineStr"/>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>04.12.2023</t>
+        </is>
+      </c>
       <c r="D596" t="inlineStr">
         <is>
-          <t>2. motor korekce vody  vystup</t>
-        </is>
-      </c>
-      <c r="E596" t="inlineStr">
-        <is>
-          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
-        </is>
-      </c>
+          <t>Výměna motoru A</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr"/>
       <c r="F596" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20356,21 +20360,17 @@
     </row>
     <row r="597">
       <c r="A597" t="n">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B597" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C597" t="inlineStr">
-        <is>
-          <t>04.12.2023</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr"/>
       <c r="D597" t="inlineStr">
         <is>
-          <t>Výměna motoru A</t>
+          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
         </is>
       </c>
       <c r="E597" t="inlineStr"/>
@@ -20389,17 +20389,17 @@
     </row>
     <row r="598">
       <c r="A598" t="n">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B598" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C598" t="inlineStr"/>
       <c r="D598" t="inlineStr">
         <is>
-          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
+          <t>dosazena nahadni Mirelka + NO z 844 013</t>
         </is>
       </c>
       <c r="E598" t="inlineStr"/>
@@ -20418,17 +20418,17 @@
     </row>
     <row r="599">
       <c r="A599" t="n">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 062</t>
         </is>
       </c>
       <c r="C599" t="inlineStr"/>
       <c r="D599" t="inlineStr">
         <is>
-          <t>dosazena nahadni Mirelka + NO z 844 013</t>
+          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
         </is>
       </c>
       <c r="E599" t="inlineStr"/>
@@ -20447,17 +20447,21 @@
     </row>
     <row r="600">
       <c r="A600" t="n">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B600" t="inlineStr">
         <is>
-          <t>814 062</t>
-        </is>
-      </c>
-      <c r="C600" t="inlineStr"/>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>03.03.2023</t>
+        </is>
+      </c>
       <c r="D600" t="inlineStr">
         <is>
-          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E600" t="inlineStr"/>
@@ -20476,11 +20480,11 @@
     </row>
     <row r="601">
       <c r="A601" t="n">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C601" t="inlineStr">
@@ -20490,7 +20494,7 @@
       </c>
       <c r="D601" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
+          <t>Dosazení ŘJ kamer</t>
         </is>
       </c>
       <c r="E601" t="inlineStr"/>
@@ -20509,24 +20513,24 @@
     </row>
     <row r="602">
       <c r="A602" t="n">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>844 013</t>
-        </is>
-      </c>
-      <c r="C602" t="inlineStr">
-        <is>
-          <t>03.03.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr"/>
       <c r="D602" t="inlineStr">
         <is>
-          <t>Dosazení ŘJ kamer</t>
-        </is>
-      </c>
-      <c r="E602" t="inlineStr"/>
+          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>hlášeno p. Škodovi</t>
+        </is>
+      </c>
       <c r="F602" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20542,24 +20546,20 @@
     </row>
     <row r="603">
       <c r="A603" t="n">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="B603" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C603" t="inlineStr"/>
       <c r="D603" t="inlineStr">
         <is>
-          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
-        </is>
-      </c>
-      <c r="E603" t="inlineStr">
-        <is>
-          <t>hlášeno p. Škodovi</t>
-        </is>
-      </c>
+          <t>ŘJ kamer dosazena z 013</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr"/>
       <c r="F603" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20575,17 +20575,21 @@
     </row>
     <row r="604">
       <c r="A604" t="n">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B604" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C604" t="inlineStr"/>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>02.09.2023</t>
+        </is>
+      </c>
       <c r="D604" t="inlineStr">
         <is>
-          <t>ŘJ kamer dosazena z 013</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E604" t="inlineStr"/>
@@ -20604,24 +20608,24 @@
     </row>
     <row r="605">
       <c r="A605" t="n">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B605" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C605" t="inlineStr">
-        <is>
-          <t>02.09.2023</t>
-        </is>
-      </c>
+      <c r="C605" t="inlineStr"/>
       <c r="D605" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
-        </is>
-      </c>
-      <c r="E605" t="inlineStr"/>
+          <t>dosazen opraveny MIREL</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+        </is>
+      </c>
       <c r="F605" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20637,22 +20641,22 @@
     </row>
     <row r="606">
       <c r="A606" t="n">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B606" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C606" t="inlineStr"/>
       <c r="D606" t="inlineStr">
         <is>
-          <t>dosazen opraveny MIREL</t>
+          <t>Odpojen trojcestný ventil na A i B</t>
         </is>
       </c>
       <c r="E606" t="inlineStr">
         <is>
-          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+          <t>Zapojeny zpět 24.2.2023</t>
         </is>
       </c>
       <c r="F606" t="inlineStr">
@@ -20670,24 +20674,20 @@
     </row>
     <row r="607">
       <c r="A607" t="n">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B607" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C607" t="inlineStr"/>
       <c r="D607" t="inlineStr">
         <is>
-          <t>Odpojen trojcestný ventil na A i B</t>
-        </is>
-      </c>
-      <c r="E607" t="inlineStr">
-        <is>
-          <t>Zapojeny zpět 24.2.2023</t>
-        </is>
-      </c>
+          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr"/>
       <c r="F607" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20703,17 +20703,21 @@
     </row>
     <row r="608">
       <c r="A608" t="n">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B608" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C608" t="inlineStr"/>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>01.10.2023</t>
+        </is>
+      </c>
       <c r="D608" t="inlineStr">
         <is>
-          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E608" t="inlineStr"/>
@@ -20732,21 +20736,17 @@
     </row>
     <row r="609">
       <c r="A609" t="n">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C609" t="inlineStr">
-        <is>
-          <t>01.10.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr"/>
       <c r="D609" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
         </is>
       </c>
       <c r="E609" t="inlineStr"/>
@@ -20765,17 +20765,17 @@
     </row>
     <row r="610">
       <c r="A610" t="n">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B610" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C610" t="inlineStr"/>
       <c r="D610" t="inlineStr">
         <is>
-          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
+          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
         </is>
       </c>
       <c r="E610" t="inlineStr"/>
@@ -20794,7 +20794,7 @@
     </row>
     <row r="611">
       <c r="A611" t="n">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B611" t="inlineStr">
         <is>
@@ -20804,7 +20804,7 @@
       <c r="C611" t="inlineStr"/>
       <c r="D611" t="inlineStr">
         <is>
-          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
+          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
         </is>
       </c>
       <c r="E611" t="inlineStr"/>
@@ -20823,20 +20823,24 @@
     </row>
     <row r="612">
       <c r="A612" t="n">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B612" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C612" t="inlineStr"/>
       <c r="D612" t="inlineStr">
         <is>
-          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
-        </is>
-      </c>
-      <c r="E612" t="inlineStr"/>
+          <t>Přišel opravený Mirel ve skladu</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>dosazen na 29.12.2022</t>
+        </is>
+      </c>
       <c r="F612" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20852,22 +20856,26 @@
     </row>
     <row r="613">
       <c r="A613" t="n">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C613" t="inlineStr"/>
+          <t>844 014</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>12.06.2022</t>
+        </is>
+      </c>
       <c r="D613" t="inlineStr">
         <is>
-          <t>Přišel opravený Mirel ve skladu</t>
+          <t>rychloměr do opravy hazí !!</t>
         </is>
       </c>
       <c r="E613" t="inlineStr">
         <is>
-          <t>dosazen na 29.12.2022</t>
+          <t>zapujcen z 844 028 z veselí</t>
         </is>
       </c>
       <c r="F613" t="inlineStr">
@@ -20885,11 +20893,11 @@
     </row>
     <row r="614">
       <c r="A614" t="n">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B614" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C614" t="inlineStr">
@@ -20899,14 +20907,10 @@
       </c>
       <c r="D614" t="inlineStr">
         <is>
-          <t>rychloměr do opravy hazí !!</t>
-        </is>
-      </c>
-      <c r="E614" t="inlineStr">
-        <is>
-          <t>zapujcen z 844 028 z veselí</t>
-        </is>
-      </c>
+          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr"/>
       <c r="F614" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20922,24 +20926,28 @@
     </row>
     <row r="615">
       <c r="A615" t="n">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C615" t="inlineStr">
         <is>
-          <t>12.06.2022</t>
+          <t>12.03.2022</t>
         </is>
       </c>
       <c r="D615" t="inlineStr">
         <is>
-          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
-        </is>
-      </c>
-      <c r="E615" t="inlineStr"/>
+          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>bude řešit Škoda</t>
+        </is>
+      </c>
       <c r="F615" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20955,26 +20963,22 @@
     </row>
     <row r="616">
       <c r="A616" t="n">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B616" t="inlineStr">
         <is>
           <t>844 003</t>
         </is>
       </c>
-      <c r="C616" t="inlineStr">
-        <is>
-          <t>12.03.2022</t>
-        </is>
-      </c>
+      <c r="C616" t="inlineStr"/>
       <c r="D616" t="inlineStr">
         <is>
-          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+          <t>na A strane asi vadna expanzní nadrz topení ?</t>
         </is>
       </c>
       <c r="E616" t="inlineStr">
         <is>
-          <t>bude řešit Škoda</t>
+          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
         </is>
       </c>
       <c r="F616" t="inlineStr">
@@ -20992,22 +20996,22 @@
     </row>
     <row r="617">
       <c r="A617" t="n">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C617" t="inlineStr"/>
       <c r="D617" t="inlineStr">
         <is>
-          <t>na A strane asi vadna expanzní nadrz topení ?</t>
+          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
         </is>
       </c>
       <c r="E617" t="inlineStr">
         <is>
-          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
+          <t>nová obrazovka hazela vykricnik porad</t>
         </is>
       </c>
       <c r="F617" t="inlineStr">
@@ -21025,24 +21029,24 @@
     </row>
     <row r="618">
       <c r="A618" t="n">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B618" t="inlineStr">
         <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C618" t="inlineStr"/>
+          <t>842 010</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>11.06.2022</t>
+        </is>
+      </c>
       <c r="D618" t="inlineStr">
         <is>
-          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
-        </is>
-      </c>
-      <c r="E618" t="inlineStr">
-        <is>
-          <t>nová obrazovka hazela vykricnik porad</t>
-        </is>
-      </c>
+          <t>Přehození karty TBA v DPV na 842 036</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr"/>
       <c r="F618" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21058,11 +21062,11 @@
     </row>
     <row r="619">
       <c r="A619" t="n">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>842 010</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C619" t="inlineStr">
@@ -21072,7 +21076,7 @@
       </c>
       <c r="D619" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 036</t>
+          <t>Přehození karty TBA v DPV na 842 010</t>
         </is>
       </c>
       <c r="E619" t="inlineStr"/>
@@ -21091,11 +21095,11 @@
     </row>
     <row r="620">
       <c r="A620" t="n">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C620" t="inlineStr">
@@ -21105,10 +21109,14 @@
       </c>
       <c r="D620" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 010</t>
-        </is>
-      </c>
-      <c r="E620" t="inlineStr"/>
+          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>mirel byl špatný po opravě</t>
+        </is>
+      </c>
       <c r="F620" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21124,26 +21132,26 @@
     </row>
     <row r="621">
       <c r="A621" t="n">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C621" t="inlineStr">
         <is>
-          <t>11.06.2022</t>
+          <t>11.05.2022</t>
         </is>
       </c>
       <c r="D621" t="inlineStr">
         <is>
-          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
         </is>
       </c>
       <c r="E621" t="inlineStr">
         <is>
-          <t>mirel byl špatný po opravě</t>
+          <t>25.11. opraveno</t>
         </is>
       </c>
       <c r="F621" t="inlineStr">
@@ -21161,11 +21169,11 @@
     </row>
     <row r="622">
       <c r="A622" t="n">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C622" t="inlineStr">
@@ -21175,14 +21183,10 @@
       </c>
       <c r="D622" t="inlineStr">
         <is>
-          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
-        </is>
-      </c>
-      <c r="E622" t="inlineStr">
-        <is>
-          <t>25.11. opraveno</t>
-        </is>
-      </c>
+          <t>VESELÍ R3 (odjela)</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr"/>
       <c r="F622" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21198,24 +21202,24 @@
     </row>
     <row r="623">
       <c r="A623" t="n">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B623" t="inlineStr">
         <is>
-          <t>844 020</t>
-        </is>
-      </c>
-      <c r="C623" t="inlineStr">
-        <is>
-          <t>11.05.2022</t>
-        </is>
-      </c>
+          <t>814 190</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr"/>
       <c r="D623" t="inlineStr">
         <is>
-          <t>VESELÍ R3 (odjela)</t>
-        </is>
-      </c>
-      <c r="E623" t="inlineStr"/>
+          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>hlášeno p.Škodovi</t>
+        </is>
+      </c>
       <c r="F623" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21231,22 +21235,22 @@
     </row>
     <row r="624">
       <c r="A624" t="n">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>814 190</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C624" t="inlineStr"/>
       <c r="D624" t="inlineStr">
         <is>
-          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
         </is>
       </c>
       <c r="E624" t="inlineStr">
         <is>
-          <t>hlášeno p.Škodovi</t>
+          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
         </is>
       </c>
       <c r="F624" t="inlineStr">
@@ -21264,24 +21268,20 @@
     </row>
     <row r="625">
       <c r="A625" t="n">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B625" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C625" t="inlineStr"/>
       <c r="D625" t="inlineStr">
         <is>
-          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
-        </is>
-      </c>
-      <c r="E625" t="inlineStr">
-        <is>
-          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
-        </is>
-      </c>
+          <t>dosazen předzesilovač linky</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr"/>
       <c r="F625" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21297,20 +21297,28 @@
     </row>
     <row r="626">
       <c r="A626" t="n">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B626" t="inlineStr">
         <is>
           <t>814 073</t>
         </is>
       </c>
-      <c r="C626" t="inlineStr"/>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>09.07.2022</t>
+        </is>
+      </c>
       <c r="D626" t="inlineStr">
         <is>
-          <t>dosazen předzesilovač linky</t>
-        </is>
-      </c>
-      <c r="E626" t="inlineStr"/>
+          <t>chybějící díl</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>předzasilovač linky - objednán nový</t>
+        </is>
+      </c>
       <c r="F626" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21326,26 +21334,26 @@
     </row>
     <row r="627">
       <c r="A627" t="n">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 003</t>
         </is>
       </c>
       <c r="C627" t="inlineStr">
         <is>
-          <t>09.07.2022</t>
+          <t>09.03.2022</t>
         </is>
       </c>
       <c r="D627" t="inlineStr">
         <is>
-          <t>chybějící díl</t>
+          <t>dosazen díl</t>
         </is>
       </c>
       <c r="E627" t="inlineStr">
         <is>
-          <t>předzasilovač linky - objednán nový</t>
+          <t>dosazen předzasilovač linky A23</t>
         </is>
       </c>
       <c r="F627" t="inlineStr">
@@ -21363,26 +21371,22 @@
     </row>
     <row r="628">
       <c r="A628" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C628" t="inlineStr">
-        <is>
-          <t>09.03.2022</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr"/>
       <c r="D628" t="inlineStr">
         <is>
-          <t>dosazen díl</t>
+          <t>oprava dveří na B pravé po směru jízdy</t>
         </is>
       </c>
       <c r="E628" t="inlineStr">
         <is>
-          <t>dosazen předzasilovač linky A23</t>
+          <t>vadný motorek</t>
         </is>
       </c>
       <c r="F628" t="inlineStr">
@@ -21400,22 +21404,22 @@
     </row>
     <row r="629">
       <c r="A629" t="n">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C629" t="inlineStr"/>
       <c r="D629" t="inlineStr">
         <is>
-          <t>oprava dveří na B pravé po směru jízdy</t>
+          <t>vadné čidlo množství písku M5</t>
         </is>
       </c>
       <c r="E629" t="inlineStr">
         <is>
-          <t>vadný motorek</t>
+          <t>2. osa pravo po smeru jizdy z B</t>
         </is>
       </c>
       <c r="F629" t="inlineStr">
@@ -21433,22 +21437,22 @@
     </row>
     <row r="630">
       <c r="A630" t="n">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C630" t="inlineStr"/>
       <c r="D630" t="inlineStr">
         <is>
-          <t>vadné čidlo množství písku M5</t>
+          <t>rychloměr dán do skladu na opravu</t>
         </is>
       </c>
       <c r="E630" t="inlineStr">
         <is>
-          <t>2. osa pravo po smeru jizdy z B</t>
+          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
         </is>
       </c>
       <c r="F630" t="inlineStr">
@@ -21466,22 +21470,22 @@
     </row>
     <row r="631">
       <c r="A631" t="n">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C631" t="inlineStr"/>
       <c r="D631" t="inlineStr">
         <is>
-          <t>rychloměr dán do skladu na opravu</t>
+          <t>rychloměr nekomunikuje</t>
         </is>
       </c>
       <c r="E631" t="inlineStr">
         <is>
-          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
+          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
         </is>
       </c>
       <c r="F631" t="inlineStr">
@@ -21499,22 +21503,26 @@
     </row>
     <row r="632">
       <c r="A632" t="n">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>844 022</t>
-        </is>
-      </c>
-      <c r="C632" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>10.08.2021</t>
+        </is>
+      </c>
       <c r="D632" t="inlineStr">
         <is>
-          <t>rychloměr nekomunikuje</t>
+          <t>dosazeny díly</t>
         </is>
       </c>
       <c r="E632" t="inlineStr">
         <is>
-          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
+          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
         </is>
       </c>
       <c r="F632" t="inlineStr">
@@ -21532,18 +21540,14 @@
     </row>
     <row r="633">
       <c r="A633" t="n">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B633" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C633" t="inlineStr">
-        <is>
-          <t>10.08.2021</t>
-        </is>
-      </c>
+      <c r="C633" t="inlineStr"/>
       <c r="D633" t="inlineStr">
         <is>
           <t>dosazeny díly</t>
@@ -21551,7 +21555,7 @@
       </c>
       <c r="E633" t="inlineStr">
         <is>
-          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
+          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
         </is>
       </c>
       <c r="F633" t="inlineStr">
@@ -21569,22 +21573,26 @@
     </row>
     <row r="634">
       <c r="A634" t="n">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B634" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C634" t="inlineStr"/>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>09.06.2021</t>
+        </is>
+      </c>
       <c r="D634" t="inlineStr">
         <is>
-          <t>dosazeny díly</t>
+          <t>Chybějící díly z důvodu použití na jinou lok.</t>
         </is>
       </c>
       <c r="E634" t="inlineStr">
         <is>
-          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
+          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
         </is>
       </c>
       <c r="F634" t="inlineStr">
@@ -21602,28 +21610,16 @@
     </row>
     <row r="635">
       <c r="A635" t="n">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C635" t="inlineStr">
-        <is>
-          <t>09.06.2021</t>
-        </is>
-      </c>
-      <c r="D635" t="inlineStr">
-        <is>
-          <t>Chybějící díly z důvodu použití na jinou lok.</t>
-        </is>
-      </c>
-      <c r="E635" t="inlineStr">
-        <is>
-          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
-        </is>
-      </c>
+          <t>842 015</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr"/>
+      <c r="D635" t="inlineStr"/>
+      <c r="E635" t="inlineStr"/>
       <c r="F635" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21639,15 +21635,19 @@
     </row>
     <row r="636">
       <c r="A636" t="n">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C636" t="inlineStr"/>
-      <c r="D636" t="inlineStr"/>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>výměna obrazovky Lokel na 914</t>
+        </is>
+      </c>
       <c r="E636" t="inlineStr"/>
       <c r="F636" t="inlineStr">
         <is>
@@ -21664,17 +21664,17 @@
     </row>
     <row r="637">
       <c r="A637" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C637" t="inlineStr"/>
       <c r="D637" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E637" t="inlineStr"/>
@@ -21693,17 +21693,17 @@
     </row>
     <row r="638">
       <c r="A638" t="n">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C638" t="inlineStr"/>
       <c r="D638" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E638" t="inlineStr"/>
@@ -21722,7 +21722,7 @@
     </row>
     <row r="639">
       <c r="A639" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B639" t="inlineStr">
         <is>
@@ -21732,10 +21732,14 @@
       <c r="C639" t="inlineStr"/>
       <c r="D639" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E639" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F639" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21751,24 +21755,20 @@
     </row>
     <row r="640">
       <c r="A640" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C640" t="inlineStr"/>
       <c r="D640" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E640" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr"/>
       <c r="F640" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21784,7 +21784,7 @@
     </row>
     <row r="641">
       <c r="A641" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B641" t="inlineStr">
         <is>
@@ -21794,7 +21794,7 @@
       <c r="C641" t="inlineStr"/>
       <c r="D641" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E641" t="inlineStr"/>
@@ -21813,17 +21813,17 @@
     </row>
     <row r="642">
       <c r="A642" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C642" t="inlineStr"/>
       <c r="D642" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E642" t="inlineStr"/>
@@ -21842,20 +21842,24 @@
     </row>
     <row r="643">
       <c r="A643" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C643" t="inlineStr"/>
       <c r="D643" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E643" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F643" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21871,7 +21875,7 @@
     </row>
     <row r="644">
       <c r="A644" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B644" t="inlineStr">
         <is>
@@ -21881,12 +21885,12 @@
       <c r="C644" t="inlineStr"/>
       <c r="D644" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F644" t="inlineStr">
@@ -21904,24 +21908,24 @@
     </row>
     <row r="645">
       <c r="A645" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C645" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D645" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E645" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr"/>
       <c r="F645" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21937,7 +21941,7 @@
     </row>
     <row r="646">
       <c r="A646" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B646" t="inlineStr">
         <is>
@@ -21946,12 +21950,12 @@
       </c>
       <c r="C646" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D646" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E646" t="inlineStr"/>
@@ -21970,7 +21974,7 @@
     </row>
     <row r="647">
       <c r="A647" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B647" t="inlineStr">
         <is>
@@ -21984,7 +21988,7 @@
       </c>
       <c r="D647" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E647" t="inlineStr"/>
@@ -22003,7 +22007,7 @@
     </row>
     <row r="648">
       <c r="A648" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B648" t="inlineStr">
         <is>
@@ -22017,10 +22021,14 @@
       </c>
       <c r="D648" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E648" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F648" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22036,7 +22044,7 @@
     </row>
     <row r="649">
       <c r="A649" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B649" t="inlineStr">
         <is>
@@ -22050,12 +22058,12 @@
       </c>
       <c r="D649" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E649" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F649" t="inlineStr">
@@ -22073,7 +22081,7 @@
     </row>
     <row r="650">
       <c r="A650" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B650" t="inlineStr">
         <is>
@@ -22087,14 +22095,10 @@
       </c>
       <c r="D650" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E650" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr"/>
       <c r="F650" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22110,24 +22114,24 @@
     </row>
     <row r="651">
       <c r="A651" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C651" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr"/>
       <c r="D651" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E651" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F651" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22143,24 +22147,20 @@
     </row>
     <row r="652">
       <c r="A652" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C652" t="inlineStr"/>
       <c r="D652" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E652" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr"/>
       <c r="F652" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22176,17 +22176,17 @@
     </row>
     <row r="653">
       <c r="A653" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C653" t="inlineStr"/>
       <c r="D653" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E653" t="inlineStr"/>
@@ -22205,7 +22205,7 @@
     </row>
     <row r="654">
       <c r="A654" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B654" t="inlineStr">
         <is>
@@ -22215,10 +22215,14 @@
       <c r="C654" t="inlineStr"/>
       <c r="D654" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E654" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F654" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22234,24 +22238,20 @@
     </row>
     <row r="655">
       <c r="A655" t="n">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C655" t="inlineStr"/>
       <c r="D655" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E655" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr"/>
       <c r="F655" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22267,7 +22267,7 @@
     </row>
     <row r="656">
       <c r="A656" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B656" t="inlineStr">
         <is>
@@ -22277,7 +22277,7 @@
       <c r="C656" t="inlineStr"/>
       <c r="D656" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E656" t="inlineStr"/>
@@ -22296,20 +22296,24 @@
     </row>
     <row r="657">
       <c r="A657" t="n">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C657" t="inlineStr"/>
       <c r="D657" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
-        </is>
-      </c>
-      <c r="E657" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F657" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22325,7 +22329,7 @@
     </row>
     <row r="658">
       <c r="A658" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B658" t="inlineStr">
         <is>
@@ -22335,14 +22339,10 @@
       <c r="C658" t="inlineStr"/>
       <c r="D658" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E658" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr"/>
       <c r="F658" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22358,7 +22358,7 @@
     </row>
     <row r="659">
       <c r="A659" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B659" t="inlineStr">
         <is>
@@ -22368,10 +22368,14 @@
       <c r="C659" t="inlineStr"/>
       <c r="D659" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E659" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F659" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22387,7 +22391,7 @@
     </row>
     <row r="660">
       <c r="A660" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B660" t="inlineStr">
         <is>
@@ -22397,14 +22401,10 @@
       <c r="C660" t="inlineStr"/>
       <c r="D660" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E660" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr"/>
       <c r="F660" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22420,7 +22420,7 @@
     </row>
     <row r="661">
       <c r="A661" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B661" t="inlineStr">
         <is>
@@ -22430,7 +22430,7 @@
       <c r="C661" t="inlineStr"/>
       <c r="D661" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E661" t="inlineStr"/>
@@ -22449,7 +22449,7 @@
     </row>
     <row r="662">
       <c r="A662" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B662" t="inlineStr">
         <is>
@@ -22459,10 +22459,14 @@
       <c r="C662" t="inlineStr"/>
       <c r="D662" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E662" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F662" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22478,7 +22482,7 @@
     </row>
     <row r="663">
       <c r="A663" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B663" t="inlineStr">
         <is>
@@ -22488,12 +22492,12 @@
       <c r="C663" t="inlineStr"/>
       <c r="D663" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E663" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F663" t="inlineStr">
@@ -22511,7 +22515,7 @@
     </row>
     <row r="664">
       <c r="A664" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B664" t="inlineStr">
         <is>
@@ -22521,12 +22525,12 @@
       <c r="C664" t="inlineStr"/>
       <c r="D664" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E664" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F664" t="inlineStr">
@@ -22544,24 +22548,20 @@
     </row>
     <row r="665">
       <c r="A665" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C665" t="inlineStr"/>
       <c r="D665" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E665" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr"/>
       <c r="F665" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22577,7 +22577,7 @@
     </row>
     <row r="666">
       <c r="A666" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B666" t="inlineStr">
         <is>
@@ -22587,10 +22587,14 @@
       <c r="C666" t="inlineStr"/>
       <c r="D666" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E666" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F666" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22606,7 +22610,7 @@
     </row>
     <row r="667">
       <c r="A667" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B667" t="inlineStr">
         <is>
@@ -22616,12 +22620,12 @@
       <c r="C667" t="inlineStr"/>
       <c r="D667" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E667" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F667" t="inlineStr">
@@ -22639,7 +22643,7 @@
     </row>
     <row r="668">
       <c r="A668" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B668" t="inlineStr">
         <is>
@@ -22649,14 +22653,10 @@
       <c r="C668" t="inlineStr"/>
       <c r="D668" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E668" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr"/>
       <c r="F668" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22672,17 +22672,17 @@
     </row>
     <row r="669">
       <c r="A669" t="n">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C669" t="inlineStr"/>
       <c r="D669" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E669" t="inlineStr"/>
@@ -22701,7 +22701,7 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
@@ -22711,10 +22711,14 @@
       <c r="C670" t="inlineStr"/>
       <c r="D670" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E670" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F670" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22730,22 +22734,22 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C671" t="inlineStr"/>
       <c r="D671" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E671" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F671" t="inlineStr">
@@ -22763,7 +22767,7 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
@@ -22773,12 +22777,12 @@
       <c r="C672" t="inlineStr"/>
       <c r="D672" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E672" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F672" t="inlineStr">
@@ -22796,24 +22800,20 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C673" t="inlineStr"/>
       <c r="D673" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E673" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr"/>
       <c r="F673" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22829,23 +22829,27 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C674" t="inlineStr"/>
       <c r="D674" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E674" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F674" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G674" t="inlineStr"/>
@@ -22858,27 +22862,23 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C675" t="inlineStr"/>
       <c r="D675" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E675" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr"/>
       <c r="F675" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G675" t="inlineStr"/>
@@ -22891,7 +22891,7 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
@@ -22901,7 +22901,7 @@
       <c r="C676" t="inlineStr"/>
       <c r="D676" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E676" t="inlineStr"/>
@@ -22920,7 +22920,7 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
@@ -22930,7 +22930,7 @@
       <c r="C677" t="inlineStr"/>
       <c r="D677" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E677" t="inlineStr"/>
@@ -22949,7 +22949,7 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
@@ -22959,7 +22959,7 @@
       <c r="C678" t="inlineStr"/>
       <c r="D678" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E678" t="inlineStr"/>
@@ -22978,7 +22978,7 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
@@ -22988,10 +22988,14 @@
       <c r="C679" t="inlineStr"/>
       <c r="D679" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E679" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F679" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23007,24 +23011,20 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C680" t="inlineStr"/>
       <c r="D680" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E680" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr"/>
       <c r="F680" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23040,7 +23040,7 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
@@ -23050,7 +23050,7 @@
       <c r="C681" t="inlineStr"/>
       <c r="D681" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E681" t="inlineStr"/>
@@ -23069,20 +23069,24 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C682" t="inlineStr"/>
       <c r="D682" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E682" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F682" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23098,27 +23102,23 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C683" t="inlineStr"/>
       <c r="D683" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E683" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr"/>
       <c r="F683" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G683" t="inlineStr"/>
@@ -23131,7 +23131,7 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
@@ -23141,7 +23141,7 @@
       <c r="C684" t="inlineStr"/>
       <c r="D684" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E684" t="inlineStr"/>
@@ -23160,23 +23160,27 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C685" t="inlineStr"/>
       <c r="D685" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E685" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F685" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G685" t="inlineStr"/>
@@ -23189,27 +23193,31 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C686" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D686" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E686" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F686" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G686" t="inlineStr"/>
@@ -23222,11 +23230,11 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C687" t="inlineStr">
@@ -23236,12 +23244,12 @@
       </c>
       <c r="D687" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E687" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F687" t="inlineStr">
@@ -23259,26 +23267,26 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C688" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D688" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E688" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F688" t="inlineStr">
@@ -23296,31 +23304,27 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C689" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D689" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E689" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr"/>
       <c r="F689" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G689" t="inlineStr"/>
@@ -23333,27 +23337,27 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C690" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D690" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E690" t="inlineStr"/>
       <c r="F690" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G690" t="inlineStr"/>
@@ -23366,27 +23370,27 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C691" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D691" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E691" t="inlineStr"/>
       <c r="F691" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G691" t="inlineStr"/>
@@ -23399,27 +23403,27 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C692" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D692" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E692" t="inlineStr"/>
       <c r="F692" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G692" t="inlineStr"/>
@@ -23432,24 +23436,28 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C693" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D693" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E693" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F693" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -23465,11 +23473,11 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C694" t="inlineStr">
@@ -23479,12 +23487,12 @@
       </c>
       <c r="D694" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E694" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F694" t="inlineStr">
@@ -23502,11 +23510,11 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C695" t="inlineStr">
@@ -23516,7 +23524,7 @@
       </c>
       <c r="D695" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E695" t="inlineStr">
@@ -23539,31 +23547,31 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C696" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D696" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E696" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F696" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G696" t="inlineStr"/>
@@ -23576,31 +23584,27 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C697" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D697" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E697" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr"/>
       <c r="F697" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G697" t="inlineStr"/>
@@ -23613,27 +23617,31 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C698" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D698" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E698" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F698" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G698" t="inlineStr"/>
@@ -23646,26 +23654,22 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C699" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr"/>
       <c r="D699" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E699" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F699" t="inlineStr">
@@ -23683,30 +23687,38 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C700" t="inlineStr"/>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D700" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E700" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F700" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G700" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G700" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H700" t="inlineStr"/>
       <c r="I700" t="inlineStr">
         <is>
@@ -23716,38 +23728,34 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C701" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D701" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E701" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F701" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G701" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G701" t="inlineStr"/>
       <c r="H701" t="inlineStr"/>
       <c r="I701" t="inlineStr">
         <is>
@@ -23757,26 +23765,26 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C702" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D702" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E702" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F702" t="inlineStr">
@@ -23784,7 +23792,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G702" t="inlineStr"/>
+      <c r="G702" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H702" t="inlineStr"/>
       <c r="I702" t="inlineStr">
         <is>
@@ -23794,11 +23806,11 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C703" t="inlineStr">
@@ -23808,67 +23820,26 @@
       </c>
       <c r="D703" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E703" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F703" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G703" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H703" t="inlineStr"/>
       <c r="I703" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="704">
-      <c r="A704" t="n">
-        <v>763</v>
-      </c>
-      <c r="B704" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C704" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D704" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E704" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F704" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G704" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H704" t="inlineStr"/>
-      <c r="I704" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 581 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I703"/>
+  <dimension ref="A1:I702"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18488,7 +18488,7 @@
     </row>
     <row r="541">
       <c r="A541" t="n">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B541" t="inlineStr">
         <is>
@@ -18498,10 +18498,14 @@
       <c r="C541" t="inlineStr"/>
       <c r="D541" t="inlineStr">
         <is>
-          <t>MM</t>
-        </is>
-      </c>
-      <c r="E541" t="inlineStr"/>
+          <t>levé dveře na 914 se nezavírají</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>vadná optozávora - výměna</t>
+        </is>
+      </c>
       <c r="F541" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -18517,22 +18521,18 @@
     </row>
     <row r="542">
       <c r="A542" t="n">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>814 076</t>
         </is>
       </c>
       <c r="C542" t="inlineStr"/>
-      <c r="D542" t="inlineStr">
-        <is>
-          <t>levé dveře na 914 se nezavírají</t>
-        </is>
-      </c>
+      <c r="D542" t="inlineStr"/>
       <c r="E542" t="inlineStr">
         <is>
-          <t>vadná optozávora - výměna</t>
+          <t>vyčtení rychloměru</t>
         </is>
       </c>
       <c r="F542" t="inlineStr">
@@ -18550,18 +18550,26 @@
     </row>
     <row r="543">
       <c r="A543" t="n">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>814 076</t>
-        </is>
-      </c>
-      <c r="C543" t="inlineStr"/>
-      <c r="D543" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>22.06.2023</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>nasvěcuje se poruha mazání nákolků !MOK (přední stanoviště)</t>
+        </is>
+      </c>
       <c r="E543" t="inlineStr">
         <is>
-          <t>vyčtení rychloměru</t>
+          <t>při navolení přepínače SA90 do polohy plnění se závada cca 3x projevila,bohužel jsem nestihl doběhnout k obrazovce dřív než se zablokovala. Ale pravděpodobně nespína signál MOP (spíná ventil co pouští vzduch). Udělal jsem ještě profuk. Pravděpodobně to bylo někde přicpané a nedošlo ke změně tlaku na tlakáčích v bloku A61. Pro jistotu jsem ještě přehodil v DPV IN karty (první s druhou) a OUT karty.</t>
         </is>
       </c>
       <c r="F543" t="inlineStr">
@@ -18579,26 +18587,22 @@
     </row>
     <row r="544">
       <c r="A544" t="n">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C544" t="inlineStr">
-        <is>
-          <t>22.06.2023</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr"/>
       <c r="D544" t="inlineStr">
         <is>
-          <t>nasvěcuje se poruha mazání nákolků !MOK (přední stanoviště)</t>
+          <t>často se navěcuje požár rozvaděče</t>
         </is>
       </c>
       <c r="E544" t="inlineStr">
         <is>
-          <t>při navolení přepínače SA90 do polohy plnění se závada cca 3x projevila,bohužel jsem nestihl doběhnout k obrazovce dřív než se zablokovala. Ale pravděpodobně nespína signál MOP (spíná ventil co pouští vzduch). Udělal jsem ještě profuk. Pravděpodobně to bylo někde přicpané a nedošlo ke změně tlaku na tlakáčích v bloku A61. Pro jistotu jsem ještě přehodil v DPV IN karty (první s druhou) a OUT karty.</t>
+          <t>neprojevilo se,výměna čidla požáru v RTO</t>
         </is>
       </c>
       <c r="F544" t="inlineStr">
@@ -18616,22 +18620,22 @@
     </row>
     <row r="545">
       <c r="A545" t="n">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C545" t="inlineStr"/>
       <c r="D545" t="inlineStr">
         <is>
-          <t>často se navěcuje požár rozvaděče</t>
+          <t>levé schody  na A nejdou</t>
         </is>
       </c>
       <c r="E545" t="inlineStr">
         <is>
-          <t>neprojevilo se,výměna čidla požáru v RTO</t>
+          <t>nečistoy kolem motoru+řemen</t>
         </is>
       </c>
       <c r="F545" t="inlineStr">
@@ -18649,22 +18653,22 @@
     </row>
     <row r="546">
       <c r="A546" t="n">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C546" t="inlineStr"/>
       <c r="D546" t="inlineStr">
         <is>
-          <t>levé schody  na A nejdou</t>
+          <t>údajne obrazovka IS v sekci B nad průchozími dveřmi ( směrem od WC) po tmě</t>
         </is>
       </c>
       <c r="E546" t="inlineStr">
         <is>
-          <t>nečistoy kolem motoru+řemen</t>
+          <t>neprojevilo se,kontrola konektorů,poklep obrazovka.Vše OK</t>
         </is>
       </c>
       <c r="F546" t="inlineStr">
@@ -18682,7 +18686,7 @@
     </row>
     <row r="547">
       <c r="A547" t="n">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B547" t="inlineStr">
         <is>
@@ -18692,12 +18696,12 @@
       <c r="C547" t="inlineStr"/>
       <c r="D547" t="inlineStr">
         <is>
-          <t>údajne obrazovka IS v sekci B nad průchozími dveřmi ( směrem od WC) po tmě</t>
+          <t>údajně problikává chyba čidla měření nafty</t>
         </is>
       </c>
       <c r="E547" t="inlineStr">
         <is>
-          <t>neprojevilo se,kontrola konektorů,poklep obrazovka.Vše OK</t>
+          <t>nenapsali jakého,neprojevilo se</t>
         </is>
       </c>
       <c r="F547" t="inlineStr">
@@ -18715,22 +18719,22 @@
     </row>
     <row r="548">
       <c r="A548" t="n">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B548" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C548" t="inlineStr"/>
       <c r="D548" t="inlineStr">
         <is>
-          <t>údajně problikává chyba čidla měření nafty</t>
+          <t>nechladí</t>
         </is>
       </c>
       <c r="E548" t="inlineStr">
         <is>
-          <t>nenapsali jakého,neprojevilo se</t>
+          <t>vydný proporcionální ventil,výměna</t>
         </is>
       </c>
       <c r="F548" t="inlineStr">
@@ -18748,22 +18752,22 @@
     </row>
     <row r="549">
       <c r="A549" t="n">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>842 015</t>
         </is>
       </c>
       <c r="C549" t="inlineStr"/>
       <c r="D549" t="inlineStr">
         <is>
-          <t>nechladí</t>
+          <t>někdy nejde brzda PB</t>
         </is>
       </c>
       <c r="E549" t="inlineStr">
         <is>
-          <t>vydný proporcionální ventil,výměna</t>
+          <t>výměna ventilu YV 61 včetně cívky</t>
         </is>
       </c>
       <c r="F549" t="inlineStr">
@@ -18781,22 +18785,22 @@
     </row>
     <row r="550">
       <c r="A550" t="n">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C550" t="inlineStr"/>
       <c r="D550" t="inlineStr">
         <is>
-          <t>někdy nejde brzda PB</t>
+          <t>v B salónu ukazuje prostřední čidlo 0°C</t>
         </is>
       </c>
       <c r="E550" t="inlineStr">
         <is>
-          <t>výměna ventilu YV 61 včetně cívky</t>
+          <t>po zahýbáním káblíku co vede ze stěny do svorkovnice čidla vše OK. Prodřený drát cca 5 cm od konce. Nasazení smršťovačky,přesvorkování dutinek</t>
         </is>
       </c>
       <c r="F550" t="inlineStr">
@@ -18814,22 +18818,22 @@
     </row>
     <row r="551">
       <c r="A551" t="n">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C551" t="inlineStr"/>
       <c r="D551" t="inlineStr">
         <is>
-          <t>v B salónu ukazuje prostřední čidlo 0°C</t>
+          <t>neukazuje vodoznak,pravá strana</t>
         </is>
       </c>
       <c r="E551" t="inlineStr">
         <is>
-          <t>po zahýbáním káblíku co vede ze stěny do svorkovnice čidla vše OK. Prodřený drát cca 5 cm od konce. Nasazení smršťovačky,přesvorkování dutinek</t>
+          <t>výměna</t>
         </is>
       </c>
       <c r="F551" t="inlineStr">
@@ -18847,22 +18851,22 @@
     </row>
     <row r="552">
       <c r="A552" t="n">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B552" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C552" t="inlineStr"/>
       <c r="D552" t="inlineStr">
         <is>
-          <t>neukazuje vodoznak,pravá strana</t>
+          <t>opět slabý výkon</t>
         </is>
       </c>
       <c r="E552" t="inlineStr">
         <is>
-          <t>výměna</t>
+          <t>byly "vyběhané" kloubky na táhlu AČ,výměna.Seřízení pákový,při 25% 930 otáček</t>
         </is>
       </c>
       <c r="F552" t="inlineStr">
@@ -18880,22 +18884,22 @@
     </row>
     <row r="553">
       <c r="A553" t="n">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>814 118</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C553" t="inlineStr"/>
       <c r="D553" t="inlineStr">
         <is>
-          <t>opět slabý výkon</t>
+          <t>údajně nejde ARR z B</t>
         </is>
       </c>
       <c r="E553" t="inlineStr">
         <is>
-          <t>byly "vyběhané" kloubky na táhlu AČ,výměna.Seřízení pákový,při 25% 930 otáček</t>
+          <t>neprojevilo se,neměněno</t>
         </is>
       </c>
       <c r="F553" t="inlineStr">
@@ -18913,7 +18917,7 @@
     </row>
     <row r="554">
       <c r="A554" t="n">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B554" t="inlineStr">
         <is>
@@ -18923,12 +18927,12 @@
       <c r="C554" t="inlineStr"/>
       <c r="D554" t="inlineStr">
         <is>
-          <t>údajně nejde ARR z B</t>
+          <t>v A salónu ukazuje prostřední čidlo -17°C</t>
         </is>
       </c>
       <c r="E554" t="inlineStr">
         <is>
-          <t>neprojevilo se,neměněno</t>
+          <t>ve skutečnosti se jedná o čidlo u měchů. 6.9.2021 se přehazovali vstupy do ŘJ mezi měchy a prostředkem. Chyba byla v prostředku. 2 roky pak byl klid. Proměření ohmicky cesty,vstupy dány zpět jak mají být. Pokud se vrátí zase v prostředku,chyba v ŘJ</t>
         </is>
       </c>
       <c r="F554" t="inlineStr">
@@ -18946,22 +18950,22 @@
     </row>
     <row r="555">
       <c r="A555" t="n">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="B555" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>029 227</t>
         </is>
       </c>
       <c r="C555" t="inlineStr"/>
       <c r="D555" t="inlineStr">
         <is>
-          <t>v A salónu ukazuje prostřední čidlo -17°C</t>
+          <t>porucha dveří elektr.</t>
         </is>
       </c>
       <c r="E555" t="inlineStr">
         <is>
-          <t>ve skutečnosti se jedná o čidlo u měchů. 6.9.2021 se přehazovali vstupy do ŘJ mezi měchy a prostředkem. Chyba byla v prostředku. 2 roky pak byl klid. Proměření ohmicky cesty,vstupy dány zpět jak mají být. Pokud se vrátí zase v prostředku,chyba v ŘJ</t>
+          <t>neprojevilo se , přezkoušení stran</t>
         </is>
       </c>
       <c r="F555" t="inlineStr">
@@ -18979,22 +18983,22 @@
     </row>
     <row r="556">
       <c r="A556" t="n">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B556" t="inlineStr">
         <is>
-          <t>029 227</t>
+          <t>742 263</t>
         </is>
       </c>
       <c r="C556" t="inlineStr"/>
       <c r="D556" t="inlineStr">
         <is>
-          <t>porucha dveří elektr.</t>
+          <t>při startu dlouho promázává, nejde zkrácený start</t>
         </is>
       </c>
       <c r="E556" t="inlineStr">
         <is>
-          <t>neprojevilo se , přezkoušení stran</t>
+          <t>vše bylo funkční , zkrácený start spíná při 49°C přesto výměna YCR7</t>
         </is>
       </c>
       <c r="F556" t="inlineStr">
@@ -19012,7 +19016,7 @@
     </row>
     <row r="557">
       <c r="A557" t="n">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B557" t="inlineStr">
         <is>
@@ -19022,12 +19026,12 @@
       <c r="C557" t="inlineStr"/>
       <c r="D557" t="inlineStr">
         <is>
-          <t>při startu dlouho promázává, nejde zkrácený start</t>
+          <t>porucha dveří elektr.</t>
         </is>
       </c>
       <c r="E557" t="inlineStr">
         <is>
-          <t>vše bylo funkční , zkrácený start spíná při 49°C přesto výměna YCR7</t>
+          <t>neprojevilo se , přezkoušení stran</t>
         </is>
       </c>
       <c r="F557" t="inlineStr">
@@ -19045,22 +19049,22 @@
     </row>
     <row r="558">
       <c r="A558" t="n">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B558" t="inlineStr">
         <is>
-          <t>742 263</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C558" t="inlineStr"/>
       <c r="D558" t="inlineStr">
         <is>
-          <t>porucha dveří elektr.</t>
+          <t>IS se rozpadá, ztráci komunikaci mezi stan.</t>
         </is>
       </c>
       <c r="E558" t="inlineStr">
         <is>
-          <t>neprojevilo se , přezkoušení stran</t>
+          <t>dotlační konektoru ale vše bylo funkční</t>
         </is>
       </c>
       <c r="F558" t="inlineStr">
@@ -19078,7 +19082,7 @@
     </row>
     <row r="559">
       <c r="A559" t="n">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B559" t="inlineStr">
         <is>
@@ -19088,12 +19092,12 @@
       <c r="C559" t="inlineStr"/>
       <c r="D559" t="inlineStr">
         <is>
-          <t>IS se rozpadá, ztráci komunikaci mezi stan.</t>
+          <t>parkovací brzda nevybaví KBS</t>
         </is>
       </c>
       <c r="E559" t="inlineStr">
         <is>
-          <t>dotlační konektoru ale vše bylo funkční</t>
+          <t>seřízení tlaku</t>
         </is>
       </c>
       <c r="F559" t="inlineStr">
@@ -19111,7 +19115,7 @@
     </row>
     <row r="560">
       <c r="A560" t="n">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="B560" t="inlineStr">
         <is>
@@ -19121,12 +19125,12 @@
       <c r="C560" t="inlineStr"/>
       <c r="D560" t="inlineStr">
         <is>
-          <t>parkovací brzda nevybaví KBS</t>
+          <t>únik oleje na 6. válci</t>
         </is>
       </c>
       <c r="E560" t="inlineStr">
         <is>
-          <t>seřízení tlaku</t>
+          <t>výměna</t>
         </is>
       </c>
       <c r="F560" t="inlineStr">
@@ -19144,7 +19148,7 @@
     </row>
     <row r="561">
       <c r="A561" t="n">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B561" t="inlineStr">
         <is>
@@ -19154,12 +19158,12 @@
       <c r="C561" t="inlineStr"/>
       <c r="D561" t="inlineStr">
         <is>
-          <t>únik oleje na 6. válci</t>
+          <t>nesvítí červené poziční světlo</t>
         </is>
       </c>
       <c r="E561" t="inlineStr">
         <is>
-          <t>výměna</t>
+          <t>zapojení vodiče 735 byl odpojený (výměna obou světel na stan 914)</t>
         </is>
       </c>
       <c r="F561" t="inlineStr">
@@ -19177,22 +19181,22 @@
     </row>
     <row r="562">
       <c r="A562" t="n">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C562" t="inlineStr"/>
       <c r="D562" t="inlineStr">
         <is>
-          <t>nesvítí červené poziční světlo</t>
+          <t>nelze odbrzdit, tlak ve válcích zůstáva 0,3 bar závada jen z 914</t>
         </is>
       </c>
       <c r="E562" t="inlineStr">
         <is>
-          <t>zapojení vodiče 735 byl odpojený (výměna obou světel na stan 914)</t>
+          <t>zk. Jízda OK</t>
         </is>
       </c>
       <c r="F562" t="inlineStr">
@@ -19210,22 +19214,22 @@
     </row>
     <row r="563">
       <c r="A563" t="n">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="B563" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C563" t="inlineStr"/>
       <c r="D563" t="inlineStr">
         <is>
-          <t>nelze odbrzdit, tlak ve válcích zůstáva 0,3 bar závada jen z 914</t>
+          <t>2.SM samovolně zvyšuje otáčky, seřízení GAC</t>
         </is>
       </c>
       <c r="E563" t="inlineStr">
         <is>
-          <t>zk. Jízda OK</t>
+          <t>přístě vyměnit GAC musela jet ven</t>
         </is>
       </c>
       <c r="F563" t="inlineStr">
@@ -19243,22 +19247,22 @@
     </row>
     <row r="564">
       <c r="A564" t="n">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="B564" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C564" t="inlineStr"/>
       <c r="D564" t="inlineStr">
         <is>
-          <t>2.SM samovolně zvyšuje otáčky, seřízení GAC</t>
+          <t>nehlási IS na stan. A</t>
         </is>
       </c>
       <c r="E564" t="inlineStr">
         <is>
-          <t>přístě vyměnit GAC musela jet ven</t>
+          <t>ztlumen potenciometr</t>
         </is>
       </c>
       <c r="F564" t="inlineStr">
@@ -19276,7 +19280,7 @@
     </row>
     <row r="565">
       <c r="A565" t="n">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B565" t="inlineStr">
         <is>
@@ -19286,12 +19290,12 @@
       <c r="C565" t="inlineStr"/>
       <c r="D565" t="inlineStr">
         <is>
-          <t>nehlási IS na stan. A</t>
+          <t>lednice nechladí</t>
         </is>
       </c>
       <c r="E565" t="inlineStr">
         <is>
-          <t>ztlumen potenciometr</t>
+          <t>odzkoušeno OK</t>
         </is>
       </c>
       <c r="F565" t="inlineStr">
@@ -19309,7 +19313,7 @@
     </row>
     <row r="566">
       <c r="A566" t="n">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B566" t="inlineStr">
         <is>
@@ -19319,12 +19323,12 @@
       <c r="C566" t="inlineStr"/>
       <c r="D566" t="inlineStr">
         <is>
-          <t>lednice nechladí</t>
+          <t>údajně rázy převodovky</t>
         </is>
       </c>
       <c r="E566" t="inlineStr">
         <is>
-          <t>odzkoušeno OK</t>
+          <t>řesí p. Šípek vyčítal jsi obě HMP</t>
         </is>
       </c>
       <c r="F566" t="inlineStr">
@@ -19342,22 +19346,22 @@
     </row>
     <row r="567">
       <c r="A567" t="n">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C567" t="inlineStr"/>
       <c r="D567" t="inlineStr">
         <is>
-          <t>údajně rázy převodovky</t>
+          <t>lok. Nejde nastartovat</t>
         </is>
       </c>
       <c r="E567" t="inlineStr">
         <is>
-          <t>řesí p. Šípek vyčítal jsi obě HMP</t>
+          <t>naftová netěsnost</t>
         </is>
       </c>
       <c r="F567" t="inlineStr">
@@ -19375,22 +19379,22 @@
     </row>
     <row r="568">
       <c r="A568" t="n">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C568" t="inlineStr"/>
       <c r="D568" t="inlineStr">
         <is>
-          <t>lok. Nejde nastartovat</t>
+          <t>izolačni stav odztraněny zkraty na vodiči 80 a 50</t>
         </is>
       </c>
       <c r="E568" t="inlineStr">
         <is>
-          <t>naftová netěsnost</t>
+          <t>startéry vyfoukany,ale nakonec výměna M2(volný pomocný vodič) seřízení GAC 2. SM , zkušební jízda se zdá v pořádku</t>
         </is>
       </c>
       <c r="F568" t="inlineStr">
@@ -19408,24 +19412,24 @@
     </row>
     <row r="569">
       <c r="A569" t="n">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B569" t="inlineStr">
         <is>
-          <t>842 035</t>
-        </is>
-      </c>
-      <c r="C569" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>06.12.2023</t>
+        </is>
+      </c>
       <c r="D569" t="inlineStr">
         <is>
-          <t>izolačni stav odztraněny zkraty na vodiči 80 a 50</t>
-        </is>
-      </c>
-      <c r="E569" t="inlineStr">
-        <is>
-          <t>startéry vyfoukany,ale nakonec výměna M2(volný pomocný vodič) seřízení GAC 2. SM , zkušební jízda se zdá v pořádku</t>
-        </is>
-      </c>
+          <t>Výměna obrazovky na 914 (občas zamrzá)</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr"/>
       <c r="F569" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19441,11 +19445,11 @@
     </row>
     <row r="570">
       <c r="A570" t="n">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>814 003</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C570" t="inlineStr">
@@ -19455,7 +19459,7 @@
       </c>
       <c r="D570" t="inlineStr">
         <is>
-          <t>Výměna obrazovky na 914 (občas zamrzá)</t>
+          <t>údajně se rozpadá IS přezkoušeno (kontrola konektoru)</t>
         </is>
       </c>
       <c r="E570" t="inlineStr"/>
@@ -19474,11 +19478,11 @@
     </row>
     <row r="571">
       <c r="A571" t="n">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B571" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 072</t>
         </is>
       </c>
       <c r="C571" t="inlineStr">
@@ -19488,7 +19492,7 @@
       </c>
       <c r="D571" t="inlineStr">
         <is>
-          <t>údajně se rozpadá IS přezkoušeno (kontrola konektoru)</t>
+          <t>tozpadáva se IS, oprava dispeleje na 914 byl volný</t>
         </is>
       </c>
       <c r="E571" t="inlineStr"/>
@@ -19507,24 +19511,28 @@
     </row>
     <row r="572">
       <c r="A572" t="n">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>814 072</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C572" t="inlineStr">
         <is>
-          <t>06.12.2023</t>
+          <t>06.11.2023</t>
         </is>
       </c>
       <c r="D572" t="inlineStr">
         <is>
-          <t>tozpadáva se IS, oprava dispeleje na 914 byl volný</t>
-        </is>
-      </c>
-      <c r="E572" t="inlineStr"/>
+          <t>tabule vnitřní , venkovní nekomunikují</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>výměna konektoru C na 914</t>
+        </is>
+      </c>
       <c r="F572" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19540,11 +19548,11 @@
     </row>
     <row r="573">
       <c r="A573" t="n">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>814 118</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C573" t="inlineStr">
@@ -19554,12 +19562,12 @@
       </c>
       <c r="D573" t="inlineStr">
         <is>
-          <t>tabule vnitřní , venkovní nekomunikují</t>
+          <t>korekce vody 2</t>
         </is>
       </c>
       <c r="E573" t="inlineStr">
         <is>
-          <t>výměna konektoru C na 914</t>
+          <t>izolačni stav špatný  stáhlé zemni relé</t>
         </is>
       </c>
       <c r="F573" t="inlineStr">
@@ -19577,11 +19585,11 @@
     </row>
     <row r="574">
       <c r="A574" t="n">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C574" t="inlineStr">
@@ -19591,14 +19599,10 @@
       </c>
       <c r="D574" t="inlineStr">
         <is>
-          <t>korekce vody 2</t>
-        </is>
-      </c>
-      <c r="E574" t="inlineStr">
-        <is>
-          <t>izolačni stav špatný  stáhlé zemni relé</t>
-        </is>
-      </c>
+          <t>výměna ARR na B stan. Nefunkční</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr"/>
       <c r="F574" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19614,21 +19618,21 @@
     </row>
     <row r="575">
       <c r="A575" t="n">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="B575" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>842 011</t>
         </is>
       </c>
       <c r="C575" t="inlineStr">
         <is>
-          <t>06.11.2023</t>
+          <t>06.10.2023</t>
         </is>
       </c>
       <c r="D575" t="inlineStr">
         <is>
-          <t>výměna ARR na B stan. Nefunkční</t>
+          <t>udajně zateklo do pultu na 2st.(kontrola)</t>
         </is>
       </c>
       <c r="E575" t="inlineStr"/>
@@ -19647,11 +19651,11 @@
     </row>
     <row r="576">
       <c r="A576" t="n">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B576" t="inlineStr">
         <is>
-          <t>842 011</t>
+          <t>842 021</t>
         </is>
       </c>
       <c r="C576" t="inlineStr">
@@ -19661,10 +19665,14 @@
       </c>
       <c r="D576" t="inlineStr">
         <is>
-          <t>udajně zateklo do pultu na 2st.(kontrola)</t>
-        </is>
-      </c>
-      <c r="E576" t="inlineStr"/>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>vadné čidlo vody v míse</t>
+        </is>
+      </c>
       <c r="F576" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19680,26 +19688,26 @@
     </row>
     <row r="577">
       <c r="A577" t="n">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>842 021</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C577" t="inlineStr">
         <is>
-          <t>06.10.2023</t>
+          <t>06.09.2023</t>
         </is>
       </c>
       <c r="D577" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>Nejdou dvěře WC</t>
         </is>
       </c>
       <c r="E577" t="inlineStr">
         <is>
-          <t>vadné čidlo vody v míse</t>
+          <t>upadlý drát na přepínači funkce WC (zapnuto,bez dveří, vypnuto). Seřízení zámykání dveří. Frýdek</t>
         </is>
       </c>
       <c r="F577" t="inlineStr">
@@ -19717,11 +19725,11 @@
     </row>
     <row r="578">
       <c r="A578" t="n">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C578" t="inlineStr">
@@ -19731,12 +19739,12 @@
       </c>
       <c r="D578" t="inlineStr">
         <is>
-          <t>Nejdou dvěře WC</t>
+          <t>údajně nejdou někdy schody u levých dveří strany A</t>
         </is>
       </c>
       <c r="E578" t="inlineStr">
         <is>
-          <t>upadlý drát na přepínači funkce WC (zapnuto,bez dveří, vypnuto). Seřízení zámykání dveří. Frýdek</t>
+          <t>vyčištění od kamínků,odzkoušení-OK</t>
         </is>
       </c>
       <c r="F578" t="inlineStr">
@@ -19754,26 +19762,26 @@
     </row>
     <row r="579">
       <c r="A579" t="n">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="B579" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C579" t="inlineStr">
         <is>
-          <t>06.09.2023</t>
+          <t>06.08.2023</t>
         </is>
       </c>
       <c r="D579" t="inlineStr">
         <is>
-          <t>údajně nejdou někdy schody u levých dveří strany A</t>
+          <t>zapůjčena z HB</t>
         </is>
       </c>
       <c r="E579" t="inlineStr">
         <is>
-          <t>vyčištění od kamínků,odzkoušení-OK</t>
+          <t>nahrány data IS ( funguje preš radiostanici)</t>
         </is>
       </c>
       <c r="F579" t="inlineStr">
@@ -19791,11 +19799,11 @@
     </row>
     <row r="580">
       <c r="A580" t="n">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B580" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C580" t="inlineStr">
@@ -19805,12 +19813,12 @@
       </c>
       <c r="D580" t="inlineStr">
         <is>
-          <t>zapůjčena z HB</t>
+          <t>Opět problémy se startováním</t>
         </is>
       </c>
       <c r="E580" t="inlineStr">
         <is>
-          <t>nahrány data IS ( funguje preš radiostanici)</t>
+          <t>(asi už vadný capos kondy)říkali veselani jak tu byli</t>
         </is>
       </c>
       <c r="F580" t="inlineStr">
@@ -19828,7 +19836,7 @@
     </row>
     <row r="581">
       <c r="A581" t="n">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="B581" t="inlineStr">
         <is>
@@ -19842,12 +19850,12 @@
       </c>
       <c r="D581" t="inlineStr">
         <is>
-          <t>Opět problémy se startováním</t>
+          <t>oprava hlasitosti na stanovišti A</t>
         </is>
       </c>
       <c r="E581" t="inlineStr">
         <is>
-          <t>(asi už vadný capos kondy)říkali veselani jak tu byli</t>
+          <t>přechod na kontaktech u reproduktoru v pultě</t>
         </is>
       </c>
       <c r="F581" t="inlineStr">
@@ -19865,11 +19873,11 @@
     </row>
     <row r="582">
       <c r="A582" t="n">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="B582" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C582" t="inlineStr">
@@ -19879,12 +19887,12 @@
       </c>
       <c r="D582" t="inlineStr">
         <is>
-          <t>oprava hlasitosti na stanovišti A</t>
+          <t>výměna ARR na B</t>
         </is>
       </c>
       <c r="E582" t="inlineStr">
         <is>
-          <t>přechod na kontaktech u reproduktoru v pultě</t>
+          <t>vadná linka CAN</t>
         </is>
       </c>
       <c r="F582" t="inlineStr">
@@ -19902,26 +19910,26 @@
     </row>
     <row r="583">
       <c r="A583" t="n">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B583" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>842 015</t>
         </is>
       </c>
       <c r="C583" t="inlineStr">
         <is>
-          <t>06.08.2023</t>
+          <t>06.07.2023</t>
         </is>
       </c>
       <c r="D583" t="inlineStr">
         <is>
-          <t>výměna ARR na B</t>
+          <t>někdy nejde brzda PB</t>
         </is>
       </c>
       <c r="E583" t="inlineStr">
         <is>
-          <t>vadná linka CAN</t>
+          <t>výměna karty DS a OUT z 842 025</t>
         </is>
       </c>
       <c r="F583" t="inlineStr">
@@ -19939,11 +19947,11 @@
     </row>
     <row r="584">
       <c r="A584" t="n">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B584" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C584" t="inlineStr">
@@ -19953,14 +19961,10 @@
       </c>
       <c r="D584" t="inlineStr">
         <is>
-          <t>někdy nejde brzda PB</t>
-        </is>
-      </c>
-      <c r="E584" t="inlineStr">
-        <is>
-          <t>výměna karty DS a OUT z 842 025</t>
-        </is>
-      </c>
+          <t>dosazeny karty z 842 015 (DS a OUT)</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr"/>
       <c r="F584" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -19976,11 +19980,11 @@
     </row>
     <row r="585">
       <c r="A585" t="n">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B585" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C585" t="inlineStr">
@@ -19990,10 +19994,14 @@
       </c>
       <c r="D585" t="inlineStr">
         <is>
-          <t>dosazeny karty z 842 015 (DS a OUT)</t>
-        </is>
-      </c>
-      <c r="E585" t="inlineStr"/>
+          <t>dosazen asi 5 dobíječ na B funkční</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>ve skladu nefunkční jenom (má řešit asi Mlíčko)</t>
+        </is>
+      </c>
       <c r="F585" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20009,28 +20017,24 @@
     </row>
     <row r="586">
       <c r="A586" t="n">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="B586" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 076</t>
         </is>
       </c>
       <c r="C586" t="inlineStr">
         <is>
-          <t>06.07.2023</t>
+          <t>06.06.2023</t>
         </is>
       </c>
       <c r="D586" t="inlineStr">
         <is>
-          <t>dosazen asi 5 dobíječ na B funkční</t>
-        </is>
-      </c>
-      <c r="E586" t="inlineStr">
-        <is>
-          <t>ve skladu nefunkční jenom (má řešit asi Mlíčko)</t>
-        </is>
-      </c>
+          <t>NEHODA V HOLEŠOVĚ</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr"/>
       <c r="F586" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20046,21 +20050,17 @@
     </row>
     <row r="587">
       <c r="A587" t="n">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="B587" t="inlineStr">
         <is>
-          <t>814 076</t>
-        </is>
-      </c>
-      <c r="C587" t="inlineStr">
-        <is>
-          <t>06.06.2023</t>
-        </is>
-      </c>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr"/>
       <c r="D587" t="inlineStr">
         <is>
-          <t>NEHODA V HOLEŠOVĚ</t>
+          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
         </is>
       </c>
       <c r="E587" t="inlineStr"/>
@@ -20079,7 +20079,7 @@
     </row>
     <row r="588">
       <c r="A588" t="n">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="B588" t="inlineStr">
         <is>
@@ -20089,7 +20089,7 @@
       <c r="C588" t="inlineStr"/>
       <c r="D588" t="inlineStr">
         <is>
-          <t>Přehpození rámových modulu AD-blue mezi A a B</t>
+          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
         </is>
       </c>
       <c r="E588" t="inlineStr"/>
@@ -20108,7 +20108,7 @@
     </row>
     <row r="589">
       <c r="A589" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B589" t="inlineStr">
         <is>
@@ -20118,7 +20118,7 @@
       <c r="C589" t="inlineStr"/>
       <c r="D589" t="inlineStr">
         <is>
-          <t>vypadáva jistič dobíječe na A straně objednán nový</t>
+          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
         </is>
       </c>
       <c r="E589" t="inlineStr"/>
@@ -20137,20 +20137,24 @@
     </row>
     <row r="590">
       <c r="A590" t="n">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B590" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C590" t="inlineStr"/>
       <c r="D590" t="inlineStr">
         <is>
-          <t>neztrácí se AD blue výměna difuzoru  na motoru A</t>
-        </is>
-      </c>
-      <c r="E590" t="inlineStr"/>
+          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>vyměnili dobíječ stacionární (Veselí)</t>
+        </is>
+      </c>
       <c r="F590" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20166,22 +20170,22 @@
     </row>
     <row r="591">
       <c r="A591" t="n">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B591" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C591" t="inlineStr"/>
       <c r="D591" t="inlineStr">
         <is>
-          <t>Generátor záruka do 23.5.2023 Veselí hlášeno i stacionární dobíječ + přetápění oddílů</t>
+          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
         </is>
       </c>
       <c r="E591" t="inlineStr">
         <is>
-          <t>vyměnili dobíječ stacionární (Veselí)</t>
+          <t>jela ven</t>
         </is>
       </c>
       <c r="F591" t="inlineStr">
@@ -20199,24 +20203,20 @@
     </row>
     <row r="592">
       <c r="A592" t="n">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C592" t="inlineStr"/>
       <c r="D592" t="inlineStr">
         <is>
-          <t>Nedobíjí B stan. Na obrazovce chyba přehřátí vinutí generátoru po resetu vše jelo. Pak už se závada nenasvítila</t>
-        </is>
-      </c>
-      <c r="E592" t="inlineStr">
-        <is>
-          <t>jela ven</t>
-        </is>
-      </c>
+          <t>seřízení kamer přes program v notasu(obraz)</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr"/>
       <c r="F592" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20232,20 +20232,24 @@
     </row>
     <row r="593">
       <c r="A593" t="n">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C593" t="inlineStr"/>
       <c r="D593" t="inlineStr">
         <is>
-          <t>seřízení kamer přes program v notasu(obraz)</t>
-        </is>
-      </c>
-      <c r="E593" t="inlineStr"/>
+          <t>po startu někdy nenabíjí "B"</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+        </is>
+      </c>
       <c r="F593" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20261,22 +20265,22 @@
     </row>
     <row r="594">
       <c r="A594" t="n">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B594" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C594" t="inlineStr"/>
       <c r="D594" t="inlineStr">
         <is>
-          <t>po startu někdy nenabíjí "B"</t>
+          <t>2. motor korekce vody  vystup</t>
         </is>
       </c>
       <c r="E594" t="inlineStr">
         <is>
-          <t>Přehození reg. RD100.7 mezi" A" a "B"</t>
+          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
         </is>
       </c>
       <c r="F594" t="inlineStr">
@@ -20294,24 +20298,24 @@
     </row>
     <row r="595">
       <c r="A595" t="n">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>842 035</t>
-        </is>
-      </c>
-      <c r="C595" t="inlineStr"/>
+          <t>844 021</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>04.12.2023</t>
+        </is>
+      </c>
       <c r="D595" t="inlineStr">
         <is>
-          <t>2. motor korekce vody  vystup</t>
-        </is>
-      </c>
-      <c r="E595" t="inlineStr">
-        <is>
-          <t>jsou vyměněny obě čidla i převodníky, karta ADA s 1. motorem</t>
-        </is>
-      </c>
+          <t>Výměna motoru A</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr"/>
       <c r="F595" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20327,21 +20331,17 @@
     </row>
     <row r="596">
       <c r="A596" t="n">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="B596" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C596" t="inlineStr">
-        <is>
-          <t>04.12.2023</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr"/>
       <c r="D596" t="inlineStr">
         <is>
-          <t>Výměna motoru A</t>
+          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
         </is>
       </c>
       <c r="E596" t="inlineStr"/>
@@ -20360,17 +20360,17 @@
     </row>
     <row r="597">
       <c r="A597" t="n">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B597" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C597" t="inlineStr"/>
       <c r="D597" t="inlineStr">
         <is>
-          <t>opravení spřáhla vadny tlakový spínač SP18 na B</t>
+          <t>dosazena nahadni Mirelka + NO z 844 013</t>
         </is>
       </c>
       <c r="E597" t="inlineStr"/>
@@ -20389,17 +20389,17 @@
     </row>
     <row r="598">
       <c r="A598" t="n">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B598" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 062</t>
         </is>
       </c>
       <c r="C598" t="inlineStr"/>
       <c r="D598" t="inlineStr">
         <is>
-          <t>dosazena nahadni Mirelka + NO z 844 013</t>
+          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
         </is>
       </c>
       <c r="E598" t="inlineStr"/>
@@ -20418,17 +20418,21 @@
     </row>
     <row r="599">
       <c r="A599" t="n">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>814 062</t>
-        </is>
-      </c>
-      <c r="C599" t="inlineStr"/>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>03.03.2023</t>
+        </is>
+      </c>
       <c r="D599" t="inlineStr">
         <is>
-          <t>Vadná komunikace s obrazovkou Lokel (vadná černá karta)</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E599" t="inlineStr"/>
@@ -20447,11 +20451,11 @@
     </row>
     <row r="600">
       <c r="A600" t="n">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B600" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C600" t="inlineStr">
@@ -20461,7 +20465,7 @@
       </c>
       <c r="D600" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
+          <t>Dosazení ŘJ kamer</t>
         </is>
       </c>
       <c r="E600" t="inlineStr"/>
@@ -20480,24 +20484,24 @@
     </row>
     <row r="601">
       <c r="A601" t="n">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>844 013</t>
-        </is>
-      </c>
-      <c r="C601" t="inlineStr">
-        <is>
-          <t>03.03.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr"/>
       <c r="D601" t="inlineStr">
         <is>
-          <t>Dosazení ŘJ kamer</t>
-        </is>
-      </c>
-      <c r="E601" t="inlineStr"/>
+          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>hlášeno p. Škodovi</t>
+        </is>
+      </c>
       <c r="F601" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20513,24 +20517,20 @@
     </row>
     <row r="602">
       <c r="A602" t="n">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C602" t="inlineStr"/>
       <c r="D602" t="inlineStr">
         <is>
-          <t>zjistěna vypálena svorkovnice na A za rozvaděčem, 100 a 98</t>
-        </is>
-      </c>
-      <c r="E602" t="inlineStr">
-        <is>
-          <t>hlášeno p. Škodovi</t>
-        </is>
-      </c>
+          <t>ŘJ kamer dosazena z 013</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr"/>
       <c r="F602" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20546,17 +20546,21 @@
     </row>
     <row r="603">
       <c r="A603" t="n">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B603" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C603" t="inlineStr"/>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>02.09.2023</t>
+        </is>
+      </c>
       <c r="D603" t="inlineStr">
         <is>
-          <t>ŘJ kamer dosazena z 013</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E603" t="inlineStr"/>
@@ -20575,24 +20579,24 @@
     </row>
     <row r="604">
       <c r="A604" t="n">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B604" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C604" t="inlineStr">
-        <is>
-          <t>02.09.2023</t>
-        </is>
-      </c>
+      <c r="C604" t="inlineStr"/>
       <c r="D604" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
-        </is>
-      </c>
-      <c r="E604" t="inlineStr"/>
+          <t>dosazen opraveny MIREL</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+        </is>
+      </c>
       <c r="F604" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20608,22 +20612,22 @@
     </row>
     <row r="605">
       <c r="A605" t="n">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C605" t="inlineStr"/>
       <c r="D605" t="inlineStr">
         <is>
-          <t>dosazen opraveny MIREL</t>
+          <t>Odpojen trojcestný ventil na A i B</t>
         </is>
       </c>
       <c r="E605" t="inlineStr">
         <is>
-          <t>opět špatné 2.3. odebrány i návěstní opakovače</t>
+          <t>Zapojeny zpět 24.2.2023</t>
         </is>
       </c>
       <c r="F605" t="inlineStr">
@@ -20641,24 +20645,20 @@
     </row>
     <row r="606">
       <c r="A606" t="n">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B606" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C606" t="inlineStr"/>
       <c r="D606" t="inlineStr">
         <is>
-          <t>Odpojen trojcestný ventil na A i B</t>
-        </is>
-      </c>
-      <c r="E606" t="inlineStr">
-        <is>
-          <t>Zapojeny zpět 24.2.2023</t>
-        </is>
-      </c>
+          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr"/>
       <c r="F606" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20674,17 +20674,21 @@
     </row>
     <row r="607">
       <c r="A607" t="n">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B607" t="inlineStr">
         <is>
           <t>844 021</t>
         </is>
       </c>
-      <c r="C607" t="inlineStr"/>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>01.10.2023</t>
+        </is>
+      </c>
       <c r="D607" t="inlineStr">
         <is>
-          <t>Na B nenabíjelo (klíňák na hraně ,natáhnutý) v depu bylo vše OK</t>
+          <t>odebran kamerovy systém zapůjčen na 013</t>
         </is>
       </c>
       <c r="E607" t="inlineStr"/>
@@ -20703,21 +20707,17 @@
     </row>
     <row r="608">
       <c r="A608" t="n">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="B608" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C608" t="inlineStr">
-        <is>
-          <t>01.10.2023</t>
-        </is>
-      </c>
+          <t>844 003</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr"/>
       <c r="D608" t="inlineStr">
         <is>
-          <t>odebran kamerovy systém zapůjčen na 013</t>
+          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
         </is>
       </c>
       <c r="E608" t="inlineStr"/>
@@ -20736,17 +20736,17 @@
     </row>
     <row r="609">
       <c r="A609" t="n">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C609" t="inlineStr"/>
       <c r="D609" t="inlineStr">
         <is>
-          <t>dosazen dobíječ původní z 014 s jinou ŘJ komunikační</t>
+          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
         </is>
       </c>
       <c r="E609" t="inlineStr"/>
@@ -20765,7 +20765,7 @@
     </row>
     <row r="610">
       <c r="A610" t="n">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B610" t="inlineStr">
         <is>
@@ -20775,7 +20775,7 @@
       <c r="C610" t="inlineStr"/>
       <c r="D610" t="inlineStr">
         <is>
-          <t>dosazen dobíječ z 003 z B strany stála na topení</t>
+          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
         </is>
       </c>
       <c r="E610" t="inlineStr"/>
@@ -20794,20 +20794,24 @@
     </row>
     <row r="611">
       <c r="A611" t="n">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B611" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C611" t="inlineStr"/>
       <c r="D611" t="inlineStr">
         <is>
-          <t>Na A výměna dobíječe ze skladu (původní neukazoval napětí,proud a teplotu)</t>
-        </is>
-      </c>
-      <c r="E611" t="inlineStr"/>
+          <t>Přišel opravený Mirel ve skladu</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>dosazen na 29.12.2022</t>
+        </is>
+      </c>
       <c r="F611" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20823,22 +20827,26 @@
     </row>
     <row r="612">
       <c r="A612" t="n">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B612" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C612" t="inlineStr"/>
+          <t>844 014</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>12.06.2022</t>
+        </is>
+      </c>
       <c r="D612" t="inlineStr">
         <is>
-          <t>Přišel opravený Mirel ve skladu</t>
+          <t>rychloměr do opravy hazí !!</t>
         </is>
       </c>
       <c r="E612" t="inlineStr">
         <is>
-          <t>dosazen na 29.12.2022</t>
+          <t>zapujcen z 844 028 z veselí</t>
         </is>
       </c>
       <c r="F612" t="inlineStr">
@@ -20856,11 +20864,11 @@
     </row>
     <row r="613">
       <c r="A613" t="n">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C613" t="inlineStr">
@@ -20870,14 +20878,10 @@
       </c>
       <c r="D613" t="inlineStr">
         <is>
-          <t>rychloměr do opravy hazí !!</t>
-        </is>
-      </c>
-      <c r="E613" t="inlineStr">
-        <is>
-          <t>zapujcen z 844 028 z veselí</t>
-        </is>
-      </c>
+          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr"/>
       <c r="F613" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20893,24 +20897,28 @@
     </row>
     <row r="614">
       <c r="A614" t="n">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B614" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C614" t="inlineStr">
         <is>
-          <t>12.06.2022</t>
+          <t>12.03.2022</t>
         </is>
       </c>
       <c r="D614" t="inlineStr">
         <is>
-          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
-        </is>
-      </c>
-      <c r="E614" t="inlineStr"/>
+          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>bude řešit Škoda</t>
+        </is>
+      </c>
       <c r="F614" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20926,26 +20934,22 @@
     </row>
     <row r="615">
       <c r="A615" t="n">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B615" t="inlineStr">
         <is>
           <t>844 003</t>
         </is>
       </c>
-      <c r="C615" t="inlineStr">
-        <is>
-          <t>12.03.2022</t>
-        </is>
-      </c>
+      <c r="C615" t="inlineStr"/>
       <c r="D615" t="inlineStr">
         <is>
-          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+          <t>na A strane asi vadna expanzní nadrz topení ?</t>
         </is>
       </c>
       <c r="E615" t="inlineStr">
         <is>
-          <t>bude řešit Škoda</t>
+          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
         </is>
       </c>
       <c r="F615" t="inlineStr">
@@ -20963,22 +20967,22 @@
     </row>
     <row r="616">
       <c r="A616" t="n">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B616" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C616" t="inlineStr"/>
       <c r="D616" t="inlineStr">
         <is>
-          <t>na A strane asi vadna expanzní nadrz topení ?</t>
+          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
         </is>
       </c>
       <c r="E616" t="inlineStr">
         <is>
-          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
+          <t>nová obrazovka hazela vykricnik porad</t>
         </is>
       </c>
       <c r="F616" t="inlineStr">
@@ -20996,24 +21000,24 @@
     </row>
     <row r="617">
       <c r="A617" t="n">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C617" t="inlineStr"/>
+          <t>842 010</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>11.06.2022</t>
+        </is>
+      </c>
       <c r="D617" t="inlineStr">
         <is>
-          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
-        </is>
-      </c>
-      <c r="E617" t="inlineStr">
-        <is>
-          <t>nová obrazovka hazela vykricnik porad</t>
-        </is>
-      </c>
+          <t>Přehození karty TBA v DPV na 842 036</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr"/>
       <c r="F617" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21029,11 +21033,11 @@
     </row>
     <row r="618">
       <c r="A618" t="n">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B618" t="inlineStr">
         <is>
-          <t>842 010</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C618" t="inlineStr">
@@ -21043,7 +21047,7 @@
       </c>
       <c r="D618" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 036</t>
+          <t>Přehození karty TBA v DPV na 842 010</t>
         </is>
       </c>
       <c r="E618" t="inlineStr"/>
@@ -21062,11 +21066,11 @@
     </row>
     <row r="619">
       <c r="A619" t="n">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C619" t="inlineStr">
@@ -21076,10 +21080,14 @@
       </c>
       <c r="D619" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 010</t>
-        </is>
-      </c>
-      <c r="E619" t="inlineStr"/>
+          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>mirel byl špatný po opravě</t>
+        </is>
+      </c>
       <c r="F619" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21095,26 +21103,26 @@
     </row>
     <row r="620">
       <c r="A620" t="n">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>11.06.2022</t>
+          <t>11.05.2022</t>
         </is>
       </c>
       <c r="D620" t="inlineStr">
         <is>
-          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
         </is>
       </c>
       <c r="E620" t="inlineStr">
         <is>
-          <t>mirel byl špatný po opravě</t>
+          <t>25.11. opraveno</t>
         </is>
       </c>
       <c r="F620" t="inlineStr">
@@ -21132,11 +21140,11 @@
     </row>
     <row r="621">
       <c r="A621" t="n">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C621" t="inlineStr">
@@ -21146,14 +21154,10 @@
       </c>
       <c r="D621" t="inlineStr">
         <is>
-          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
-        </is>
-      </c>
-      <c r="E621" t="inlineStr">
-        <is>
-          <t>25.11. opraveno</t>
-        </is>
-      </c>
+          <t>VESELÍ R3 (odjela)</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr"/>
       <c r="F621" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21169,24 +21173,24 @@
     </row>
     <row r="622">
       <c r="A622" t="n">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>844 020</t>
-        </is>
-      </c>
-      <c r="C622" t="inlineStr">
-        <is>
-          <t>11.05.2022</t>
-        </is>
-      </c>
+          <t>814 190</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr"/>
       <c r="D622" t="inlineStr">
         <is>
-          <t>VESELÍ R3 (odjela)</t>
-        </is>
-      </c>
-      <c r="E622" t="inlineStr"/>
+          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>hlášeno p.Škodovi</t>
+        </is>
+      </c>
       <c r="F622" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21202,22 +21206,22 @@
     </row>
     <row r="623">
       <c r="A623" t="n">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B623" t="inlineStr">
         <is>
-          <t>814 190</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C623" t="inlineStr"/>
       <c r="D623" t="inlineStr">
         <is>
-          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
         </is>
       </c>
       <c r="E623" t="inlineStr">
         <is>
-          <t>hlášeno p.Škodovi</t>
+          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
         </is>
       </c>
       <c r="F623" t="inlineStr">
@@ -21235,24 +21239,20 @@
     </row>
     <row r="624">
       <c r="A624" t="n">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C624" t="inlineStr"/>
       <c r="D624" t="inlineStr">
         <is>
-          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
-        </is>
-      </c>
-      <c r="E624" t="inlineStr">
-        <is>
-          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
-        </is>
-      </c>
+          <t>dosazen předzesilovač linky</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr"/>
       <c r="F624" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21268,20 +21268,28 @@
     </row>
     <row r="625">
       <c r="A625" t="n">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B625" t="inlineStr">
         <is>
           <t>814 073</t>
         </is>
       </c>
-      <c r="C625" t="inlineStr"/>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>09.07.2022</t>
+        </is>
+      </c>
       <c r="D625" t="inlineStr">
         <is>
-          <t>dosazen předzesilovač linky</t>
-        </is>
-      </c>
-      <c r="E625" t="inlineStr"/>
+          <t>chybějící díl</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>předzasilovač linky - objednán nový</t>
+        </is>
+      </c>
       <c r="F625" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21297,26 +21305,26 @@
     </row>
     <row r="626">
       <c r="A626" t="n">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 003</t>
         </is>
       </c>
       <c r="C626" t="inlineStr">
         <is>
-          <t>09.07.2022</t>
+          <t>09.03.2022</t>
         </is>
       </c>
       <c r="D626" t="inlineStr">
         <is>
-          <t>chybějící díl</t>
+          <t>dosazen díl</t>
         </is>
       </c>
       <c r="E626" t="inlineStr">
         <is>
-          <t>předzasilovač linky - objednán nový</t>
+          <t>dosazen předzasilovač linky A23</t>
         </is>
       </c>
       <c r="F626" t="inlineStr">
@@ -21334,26 +21342,22 @@
     </row>
     <row r="627">
       <c r="A627" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C627" t="inlineStr">
-        <is>
-          <t>09.03.2022</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr"/>
       <c r="D627" t="inlineStr">
         <is>
-          <t>dosazen díl</t>
+          <t>oprava dveří na B pravé po směru jízdy</t>
         </is>
       </c>
       <c r="E627" t="inlineStr">
         <is>
-          <t>dosazen předzasilovač linky A23</t>
+          <t>vadný motorek</t>
         </is>
       </c>
       <c r="F627" t="inlineStr">
@@ -21371,22 +21375,22 @@
     </row>
     <row r="628">
       <c r="A628" t="n">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C628" t="inlineStr"/>
       <c r="D628" t="inlineStr">
         <is>
-          <t>oprava dveří na B pravé po směru jízdy</t>
+          <t>vadné čidlo množství písku M5</t>
         </is>
       </c>
       <c r="E628" t="inlineStr">
         <is>
-          <t>vadný motorek</t>
+          <t>2. osa pravo po smeru jizdy z B</t>
         </is>
       </c>
       <c r="F628" t="inlineStr">
@@ -21404,22 +21408,22 @@
     </row>
     <row r="629">
       <c r="A629" t="n">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C629" t="inlineStr"/>
       <c r="D629" t="inlineStr">
         <is>
-          <t>vadné čidlo množství písku M5</t>
+          <t>rychloměr dán do skladu na opravu</t>
         </is>
       </c>
       <c r="E629" t="inlineStr">
         <is>
-          <t>2. osa pravo po smeru jizdy z B</t>
+          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
         </is>
       </c>
       <c r="F629" t="inlineStr">
@@ -21437,22 +21441,22 @@
     </row>
     <row r="630">
       <c r="A630" t="n">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C630" t="inlineStr"/>
       <c r="D630" t="inlineStr">
         <is>
-          <t>rychloměr dán do skladu na opravu</t>
+          <t>rychloměr nekomunikuje</t>
         </is>
       </c>
       <c r="E630" t="inlineStr">
         <is>
-          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
+          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
         </is>
       </c>
       <c r="F630" t="inlineStr">
@@ -21470,22 +21474,26 @@
     </row>
     <row r="631">
       <c r="A631" t="n">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>844 022</t>
-        </is>
-      </c>
-      <c r="C631" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>10.08.2021</t>
+        </is>
+      </c>
       <c r="D631" t="inlineStr">
         <is>
-          <t>rychloměr nekomunikuje</t>
+          <t>dosazeny díly</t>
         </is>
       </c>
       <c r="E631" t="inlineStr">
         <is>
-          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
+          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
         </is>
       </c>
       <c r="F631" t="inlineStr">
@@ -21503,18 +21511,14 @@
     </row>
     <row r="632">
       <c r="A632" t="n">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B632" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C632" t="inlineStr">
-        <is>
-          <t>10.08.2021</t>
-        </is>
-      </c>
+      <c r="C632" t="inlineStr"/>
       <c r="D632" t="inlineStr">
         <is>
           <t>dosazeny díly</t>
@@ -21522,7 +21526,7 @@
       </c>
       <c r="E632" t="inlineStr">
         <is>
-          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
+          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
         </is>
       </c>
       <c r="F632" t="inlineStr">
@@ -21540,22 +21544,26 @@
     </row>
     <row r="633">
       <c r="A633" t="n">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B633" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C633" t="inlineStr"/>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>09.06.2021</t>
+        </is>
+      </c>
       <c r="D633" t="inlineStr">
         <is>
-          <t>dosazeny díly</t>
+          <t>Chybějící díly z důvodu použití na jinou lok.</t>
         </is>
       </c>
       <c r="E633" t="inlineStr">
         <is>
-          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
+          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
         </is>
       </c>
       <c r="F633" t="inlineStr">
@@ -21573,28 +21581,16 @@
     </row>
     <row r="634">
       <c r="A634" t="n">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C634" t="inlineStr">
-        <is>
-          <t>09.06.2021</t>
-        </is>
-      </c>
-      <c r="D634" t="inlineStr">
-        <is>
-          <t>Chybějící díly z důvodu použití na jinou lok.</t>
-        </is>
-      </c>
-      <c r="E634" t="inlineStr">
-        <is>
-          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
-        </is>
-      </c>
+          <t>842 015</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr"/>
+      <c r="D634" t="inlineStr"/>
+      <c r="E634" t="inlineStr"/>
       <c r="F634" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21610,15 +21606,19 @@
     </row>
     <row r="635">
       <c r="A635" t="n">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C635" t="inlineStr"/>
-      <c r="D635" t="inlineStr"/>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>výměna obrazovky Lokel na 914</t>
+        </is>
+      </c>
       <c r="E635" t="inlineStr"/>
       <c r="F635" t="inlineStr">
         <is>
@@ -21635,17 +21635,17 @@
     </row>
     <row r="636">
       <c r="A636" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C636" t="inlineStr"/>
       <c r="D636" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E636" t="inlineStr"/>
@@ -21664,17 +21664,17 @@
     </row>
     <row r="637">
       <c r="A637" t="n">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C637" t="inlineStr"/>
       <c r="D637" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E637" t="inlineStr"/>
@@ -21693,7 +21693,7 @@
     </row>
     <row r="638">
       <c r="A638" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B638" t="inlineStr">
         <is>
@@ -21703,10 +21703,14 @@
       <c r="C638" t="inlineStr"/>
       <c r="D638" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E638" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F638" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21722,24 +21726,20 @@
     </row>
     <row r="639">
       <c r="A639" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C639" t="inlineStr"/>
       <c r="D639" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E639" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr"/>
       <c r="F639" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21755,7 +21755,7 @@
     </row>
     <row r="640">
       <c r="A640" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B640" t="inlineStr">
         <is>
@@ -21765,7 +21765,7 @@
       <c r="C640" t="inlineStr"/>
       <c r="D640" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E640" t="inlineStr"/>
@@ -21784,17 +21784,17 @@
     </row>
     <row r="641">
       <c r="A641" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C641" t="inlineStr"/>
       <c r="D641" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E641" t="inlineStr"/>
@@ -21813,20 +21813,24 @@
     </row>
     <row r="642">
       <c r="A642" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C642" t="inlineStr"/>
       <c r="D642" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E642" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F642" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21842,7 +21846,7 @@
     </row>
     <row r="643">
       <c r="A643" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B643" t="inlineStr">
         <is>
@@ -21852,12 +21856,12 @@
       <c r="C643" t="inlineStr"/>
       <c r="D643" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E643" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F643" t="inlineStr">
@@ -21875,24 +21879,24 @@
     </row>
     <row r="644">
       <c r="A644" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C644" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D644" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E644" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr"/>
       <c r="F644" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21908,7 +21912,7 @@
     </row>
     <row r="645">
       <c r="A645" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B645" t="inlineStr">
         <is>
@@ -21917,12 +21921,12 @@
       </c>
       <c r="C645" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D645" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E645" t="inlineStr"/>
@@ -21941,7 +21945,7 @@
     </row>
     <row r="646">
       <c r="A646" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B646" t="inlineStr">
         <is>
@@ -21955,7 +21959,7 @@
       </c>
       <c r="D646" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E646" t="inlineStr"/>
@@ -21974,7 +21978,7 @@
     </row>
     <row r="647">
       <c r="A647" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B647" t="inlineStr">
         <is>
@@ -21988,10 +21992,14 @@
       </c>
       <c r="D647" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E647" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F647" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22007,7 +22015,7 @@
     </row>
     <row r="648">
       <c r="A648" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B648" t="inlineStr">
         <is>
@@ -22021,12 +22029,12 @@
       </c>
       <c r="D648" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E648" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F648" t="inlineStr">
@@ -22044,7 +22052,7 @@
     </row>
     <row r="649">
       <c r="A649" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B649" t="inlineStr">
         <is>
@@ -22058,14 +22066,10 @@
       </c>
       <c r="D649" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E649" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr"/>
       <c r="F649" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22081,24 +22085,24 @@
     </row>
     <row r="650">
       <c r="A650" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C650" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr"/>
       <c r="D650" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E650" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F650" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22114,24 +22118,20 @@
     </row>
     <row r="651">
       <c r="A651" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C651" t="inlineStr"/>
       <c r="D651" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E651" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr"/>
       <c r="F651" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22147,17 +22147,17 @@
     </row>
     <row r="652">
       <c r="A652" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C652" t="inlineStr"/>
       <c r="D652" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E652" t="inlineStr"/>
@@ -22176,7 +22176,7 @@
     </row>
     <row r="653">
       <c r="A653" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B653" t="inlineStr">
         <is>
@@ -22186,10 +22186,14 @@
       <c r="C653" t="inlineStr"/>
       <c r="D653" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E653" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F653" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22205,24 +22209,20 @@
     </row>
     <row r="654">
       <c r="A654" t="n">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C654" t="inlineStr"/>
       <c r="D654" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E654" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr"/>
       <c r="F654" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22238,7 +22238,7 @@
     </row>
     <row r="655">
       <c r="A655" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B655" t="inlineStr">
         <is>
@@ -22248,7 +22248,7 @@
       <c r="C655" t="inlineStr"/>
       <c r="D655" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E655" t="inlineStr"/>
@@ -22267,20 +22267,24 @@
     </row>
     <row r="656">
       <c r="A656" t="n">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C656" t="inlineStr"/>
       <c r="D656" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
-        </is>
-      </c>
-      <c r="E656" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F656" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22296,7 +22300,7 @@
     </row>
     <row r="657">
       <c r="A657" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B657" t="inlineStr">
         <is>
@@ -22306,14 +22310,10 @@
       <c r="C657" t="inlineStr"/>
       <c r="D657" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E657" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr"/>
       <c r="F657" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22329,7 +22329,7 @@
     </row>
     <row r="658">
       <c r="A658" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B658" t="inlineStr">
         <is>
@@ -22339,10 +22339,14 @@
       <c r="C658" t="inlineStr"/>
       <c r="D658" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E658" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F658" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22358,7 +22362,7 @@
     </row>
     <row r="659">
       <c r="A659" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B659" t="inlineStr">
         <is>
@@ -22368,14 +22372,10 @@
       <c r="C659" t="inlineStr"/>
       <c r="D659" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E659" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr"/>
       <c r="F659" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22391,7 +22391,7 @@
     </row>
     <row r="660">
       <c r="A660" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B660" t="inlineStr">
         <is>
@@ -22401,7 +22401,7 @@
       <c r="C660" t="inlineStr"/>
       <c r="D660" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E660" t="inlineStr"/>
@@ -22420,7 +22420,7 @@
     </row>
     <row r="661">
       <c r="A661" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B661" t="inlineStr">
         <is>
@@ -22430,10 +22430,14 @@
       <c r="C661" t="inlineStr"/>
       <c r="D661" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E661" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F661" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22449,7 +22453,7 @@
     </row>
     <row r="662">
       <c r="A662" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B662" t="inlineStr">
         <is>
@@ -22459,12 +22463,12 @@
       <c r="C662" t="inlineStr"/>
       <c r="D662" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E662" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F662" t="inlineStr">
@@ -22482,7 +22486,7 @@
     </row>
     <row r="663">
       <c r="A663" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B663" t="inlineStr">
         <is>
@@ -22492,12 +22496,12 @@
       <c r="C663" t="inlineStr"/>
       <c r="D663" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E663" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F663" t="inlineStr">
@@ -22515,24 +22519,20 @@
     </row>
     <row r="664">
       <c r="A664" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C664" t="inlineStr"/>
       <c r="D664" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E664" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr"/>
       <c r="F664" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22548,7 +22548,7 @@
     </row>
     <row r="665">
       <c r="A665" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B665" t="inlineStr">
         <is>
@@ -22558,10 +22558,14 @@
       <c r="C665" t="inlineStr"/>
       <c r="D665" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E665" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F665" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22577,7 +22581,7 @@
     </row>
     <row r="666">
       <c r="A666" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B666" t="inlineStr">
         <is>
@@ -22587,12 +22591,12 @@
       <c r="C666" t="inlineStr"/>
       <c r="D666" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E666" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F666" t="inlineStr">
@@ -22610,7 +22614,7 @@
     </row>
     <row r="667">
       <c r="A667" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B667" t="inlineStr">
         <is>
@@ -22620,14 +22624,10 @@
       <c r="C667" t="inlineStr"/>
       <c r="D667" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E667" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr"/>
       <c r="F667" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22643,17 +22643,17 @@
     </row>
     <row r="668">
       <c r="A668" t="n">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="B668" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C668" t="inlineStr"/>
       <c r="D668" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E668" t="inlineStr"/>
@@ -22672,7 +22672,7 @@
     </row>
     <row r="669">
       <c r="A669" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B669" t="inlineStr">
         <is>
@@ -22682,10 +22682,14 @@
       <c r="C669" t="inlineStr"/>
       <c r="D669" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E669" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F669" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22701,22 +22705,22 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C670" t="inlineStr"/>
       <c r="D670" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E670" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F670" t="inlineStr">
@@ -22734,7 +22738,7 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
@@ -22744,12 +22748,12 @@
       <c r="C671" t="inlineStr"/>
       <c r="D671" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E671" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F671" t="inlineStr">
@@ -22767,24 +22771,20 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C672" t="inlineStr"/>
       <c r="D672" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E672" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr"/>
       <c r="F672" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22800,23 +22800,27 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C673" t="inlineStr"/>
       <c r="D673" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E673" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F673" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G673" t="inlineStr"/>
@@ -22829,27 +22833,23 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C674" t="inlineStr"/>
       <c r="D674" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E674" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr"/>
       <c r="F674" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G674" t="inlineStr"/>
@@ -22862,7 +22862,7 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
@@ -22872,7 +22872,7 @@
       <c r="C675" t="inlineStr"/>
       <c r="D675" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E675" t="inlineStr"/>
@@ -22891,7 +22891,7 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
@@ -22901,7 +22901,7 @@
       <c r="C676" t="inlineStr"/>
       <c r="D676" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E676" t="inlineStr"/>
@@ -22920,7 +22920,7 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
@@ -22930,7 +22930,7 @@
       <c r="C677" t="inlineStr"/>
       <c r="D677" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E677" t="inlineStr"/>
@@ -22949,7 +22949,7 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
@@ -22959,10 +22959,14 @@
       <c r="C678" t="inlineStr"/>
       <c r="D678" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E678" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F678" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22978,24 +22982,20 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C679" t="inlineStr"/>
       <c r="D679" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E679" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr"/>
       <c r="F679" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23011,7 +23011,7 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
@@ -23021,7 +23021,7 @@
       <c r="C680" t="inlineStr"/>
       <c r="D680" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E680" t="inlineStr"/>
@@ -23040,20 +23040,24 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C681" t="inlineStr"/>
       <c r="D681" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E681" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F681" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23069,27 +23073,23 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C682" t="inlineStr"/>
       <c r="D682" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E682" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr"/>
       <c r="F682" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G682" t="inlineStr"/>
@@ -23102,7 +23102,7 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
@@ -23112,7 +23112,7 @@
       <c r="C683" t="inlineStr"/>
       <c r="D683" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E683" t="inlineStr"/>
@@ -23131,23 +23131,27 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C684" t="inlineStr"/>
       <c r="D684" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E684" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F684" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G684" t="inlineStr"/>
@@ -23160,27 +23164,31 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C685" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D685" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E685" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F685" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G685" t="inlineStr"/>
@@ -23193,11 +23201,11 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C686" t="inlineStr">
@@ -23207,12 +23215,12 @@
       </c>
       <c r="D686" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E686" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F686" t="inlineStr">
@@ -23230,26 +23238,26 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C687" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D687" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E687" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F687" t="inlineStr">
@@ -23267,31 +23275,27 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C688" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D688" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E688" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr"/>
       <c r="F688" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G688" t="inlineStr"/>
@@ -23304,27 +23308,27 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C689" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D689" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E689" t="inlineStr"/>
       <c r="F689" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G689" t="inlineStr"/>
@@ -23337,27 +23341,27 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C690" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D690" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E690" t="inlineStr"/>
       <c r="F690" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G690" t="inlineStr"/>
@@ -23370,27 +23374,27 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C691" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D691" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E691" t="inlineStr"/>
       <c r="F691" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G691" t="inlineStr"/>
@@ -23403,24 +23407,28 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C692" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D692" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E692" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F692" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -23436,11 +23444,11 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C693" t="inlineStr">
@@ -23450,12 +23458,12 @@
       </c>
       <c r="D693" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E693" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F693" t="inlineStr">
@@ -23473,11 +23481,11 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C694" t="inlineStr">
@@ -23487,7 +23495,7 @@
       </c>
       <c r="D694" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E694" t="inlineStr">
@@ -23510,31 +23518,31 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C695" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D695" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E695" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F695" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G695" t="inlineStr"/>
@@ -23547,31 +23555,27 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C696" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D696" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E696" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr"/>
       <c r="F696" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G696" t="inlineStr"/>
@@ -23584,27 +23588,31 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C697" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D697" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E697" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F697" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G697" t="inlineStr"/>
@@ -23617,26 +23625,22 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C698" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr"/>
       <c r="D698" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E698" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F698" t="inlineStr">
@@ -23654,30 +23658,38 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C699" t="inlineStr"/>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D699" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E699" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F699" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G699" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G699" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H699" t="inlineStr"/>
       <c r="I699" t="inlineStr">
         <is>
@@ -23687,38 +23699,34 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C700" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D700" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E700" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F700" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G700" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G700" t="inlineStr"/>
       <c r="H700" t="inlineStr"/>
       <c r="I700" t="inlineStr">
         <is>
@@ -23728,26 +23736,26 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C701" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D701" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E701" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F701" t="inlineStr">
@@ -23755,7 +23763,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G701" t="inlineStr"/>
+      <c r="G701" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H701" t="inlineStr"/>
       <c r="I701" t="inlineStr">
         <is>
@@ -23765,11 +23777,11 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C702" t="inlineStr">
@@ -23779,67 +23791,26 @@
       </c>
       <c r="D702" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E702" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F702" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G702" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H702" t="inlineStr"/>
       <c r="I702" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="703">
-      <c r="A703" t="n">
-        <v>763</v>
-      </c>
-      <c r="B703" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C703" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D703" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E703" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F703" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G703" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H703" t="inlineStr"/>
-      <c r="I703" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Smazána závada ID 658 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I702"/>
+  <dimension ref="A1:I701"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20794,22 +20794,26 @@
     </row>
     <row r="611">
       <c r="A611" t="n">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="B611" t="inlineStr">
         <is>
-          <t>844 021</t>
-        </is>
-      </c>
-      <c r="C611" t="inlineStr"/>
+          <t>844 014</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>12.06.2022</t>
+        </is>
+      </c>
       <c r="D611" t="inlineStr">
         <is>
-          <t>Přišel opravený Mirel ve skladu</t>
+          <t>rychloměr do opravy hazí !!</t>
         </is>
       </c>
       <c r="E611" t="inlineStr">
         <is>
-          <t>dosazen na 29.12.2022</t>
+          <t>zapujcen z 844 028 z veselí</t>
         </is>
       </c>
       <c r="F611" t="inlineStr">
@@ -20827,11 +20831,11 @@
     </row>
     <row r="612">
       <c r="A612" t="n">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B612" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C612" t="inlineStr">
@@ -20841,14 +20845,10 @@
       </c>
       <c r="D612" t="inlineStr">
         <is>
-          <t>rychloměr do opravy hazí !!</t>
-        </is>
-      </c>
-      <c r="E612" t="inlineStr">
-        <is>
-          <t>zapujcen z 844 028 z veselí</t>
-        </is>
-      </c>
+          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr"/>
       <c r="F612" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20864,24 +20864,28 @@
     </row>
     <row r="613">
       <c r="A613" t="n">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C613" t="inlineStr">
         <is>
-          <t>12.06.2022</t>
+          <t>12.03.2022</t>
         </is>
       </c>
       <c r="D613" t="inlineStr">
         <is>
-          <t>odebrán rychloměr a poslán do opravy,10.1.2023 zapůjčen rychloměr z Veselí 844 028</t>
-        </is>
-      </c>
-      <c r="E613" t="inlineStr"/>
+          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>bude řešit Škoda</t>
+        </is>
+      </c>
       <c r="F613" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -20897,26 +20901,22 @@
     </row>
     <row r="614">
       <c r="A614" t="n">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B614" t="inlineStr">
         <is>
           <t>844 003</t>
         </is>
       </c>
-      <c r="C614" t="inlineStr">
-        <is>
-          <t>12.03.2022</t>
-        </is>
-      </c>
+      <c r="C614" t="inlineStr"/>
       <c r="D614" t="inlineStr">
         <is>
-          <t>Na B v klimatizaci (na hoře)odpojen trojcestny ventil ovladání a ručne otevřený</t>
+          <t>na A strane asi vadna expanzní nadrz topení ?</t>
         </is>
       </c>
       <c r="E614" t="inlineStr">
         <is>
-          <t>bude řešit Škoda</t>
+          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
         </is>
       </c>
       <c r="F614" t="inlineStr">
@@ -20934,22 +20934,22 @@
     </row>
     <row r="615">
       <c r="A615" t="n">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C615" t="inlineStr"/>
       <c r="D615" t="inlineStr">
         <is>
-          <t>na A strane asi vadna expanzní nadrz topení ?</t>
+          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
         </is>
       </c>
       <c r="E615" t="inlineStr">
         <is>
-          <t>bylo tam moc natlaceneho vzduchu !!!!!</t>
+          <t>nová obrazovka hazela vykricnik porad</t>
         </is>
       </c>
       <c r="F615" t="inlineStr">
@@ -20967,24 +20967,24 @@
     </row>
     <row r="616">
       <c r="A616" t="n">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B616" t="inlineStr">
         <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C616" t="inlineStr"/>
+          <t>842 010</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>11.06.2022</t>
+        </is>
+      </c>
       <c r="D616" t="inlineStr">
         <is>
-          <t>Výměna IO boxu na straně A dosazena puvodni obrazovka</t>
-        </is>
-      </c>
-      <c r="E616" t="inlineStr">
-        <is>
-          <t>nová obrazovka hazela vykricnik porad</t>
-        </is>
-      </c>
+          <t>Přehození karty TBA v DPV na 842 036</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr"/>
       <c r="F616" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21000,11 +21000,11 @@
     </row>
     <row r="617">
       <c r="A617" t="n">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>842 010</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C617" t="inlineStr">
@@ -21014,7 +21014,7 @@
       </c>
       <c r="D617" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 036</t>
+          <t>Přehození karty TBA v DPV na 842 010</t>
         </is>
       </c>
       <c r="E617" t="inlineStr"/>
@@ -21033,11 +21033,11 @@
     </row>
     <row r="618">
       <c r="A618" t="n">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B618" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C618" t="inlineStr">
@@ -21047,10 +21047,14 @@
       </c>
       <c r="D618" t="inlineStr">
         <is>
-          <t>Přehození karty TBA v DPV na 842 010</t>
-        </is>
-      </c>
-      <c r="E618" t="inlineStr"/>
+          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>mirel byl špatný po opravě</t>
+        </is>
+      </c>
       <c r="F618" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21066,26 +21070,26 @@
     </row>
     <row r="619">
       <c r="A619" t="n">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>814 029</t>
         </is>
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>11.06.2022</t>
+          <t>11.05.2022</t>
         </is>
       </c>
       <c r="D619" t="inlineStr">
         <is>
-          <t>Dosazena MIREL po opravě nahradní zpet do Brna</t>
+          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
         </is>
       </c>
       <c r="E619" t="inlineStr">
         <is>
-          <t>mirel byl špatný po opravě</t>
+          <t>25.11. opraveno</t>
         </is>
       </c>
       <c r="F619" t="inlineStr">
@@ -21103,11 +21107,11 @@
     </row>
     <row r="620">
       <c r="A620" t="n">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>814 029</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C620" t="inlineStr">
@@ -21117,14 +21121,10 @@
       </c>
       <c r="D620" t="inlineStr">
         <is>
-          <t>Vadný konektor na 914 mikrofonu musí se koupit</t>
-        </is>
-      </c>
-      <c r="E620" t="inlineStr">
-        <is>
-          <t>25.11. opraveno</t>
-        </is>
-      </c>
+          <t>VESELÍ R3 (odjela)</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr"/>
       <c r="F620" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21140,24 +21140,24 @@
     </row>
     <row r="621">
       <c r="A621" t="n">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>844 020</t>
-        </is>
-      </c>
-      <c r="C621" t="inlineStr">
-        <is>
-          <t>11.05.2022</t>
-        </is>
-      </c>
+          <t>814 190</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr"/>
       <c r="D621" t="inlineStr">
         <is>
-          <t>VESELÍ R3 (odjela)</t>
-        </is>
-      </c>
-      <c r="E621" t="inlineStr"/>
+          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>hlášeno p.Škodovi</t>
+        </is>
+      </c>
       <c r="F621" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21173,22 +21173,22 @@
     </row>
     <row r="622">
       <c r="A622" t="n">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>814 190</t>
+          <t>842 035</t>
         </is>
       </c>
       <c r="C622" t="inlineStr"/>
       <c r="D622" t="inlineStr">
         <is>
-          <t>WC zajimavá kabeláž výměna BVH01 zamykaji se dveře</t>
+          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
         </is>
       </c>
       <c r="E622" t="inlineStr">
         <is>
-          <t>hlášeno p.Škodovi</t>
+          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
         </is>
       </c>
       <c r="F622" t="inlineStr">
@@ -21206,24 +21206,20 @@
     </row>
     <row r="623">
       <c r="A623" t="n">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B623" t="inlineStr">
         <is>
-          <t>842 035</t>
+          <t>814 073</t>
         </is>
       </c>
       <c r="C623" t="inlineStr"/>
       <c r="D623" t="inlineStr">
         <is>
-          <t>1.motor se hřeje na 95 C a 2.na 80C</t>
-        </is>
-      </c>
-      <c r="E623" t="inlineStr">
-        <is>
-          <t>asi vadné (žádné) termostaty. Voda do chladiče šla moc brzy. Motoráři po konzultaci s mistry neřešili</t>
-        </is>
-      </c>
+          <t>dosazen předzesilovač linky</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr"/>
       <c r="F623" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21239,20 +21235,28 @@
     </row>
     <row r="624">
       <c r="A624" t="n">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B624" t="inlineStr">
         <is>
           <t>814 073</t>
         </is>
       </c>
-      <c r="C624" t="inlineStr"/>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>09.07.2022</t>
+        </is>
+      </c>
       <c r="D624" t="inlineStr">
         <is>
-          <t>dosazen předzesilovač linky</t>
-        </is>
-      </c>
-      <c r="E624" t="inlineStr"/>
+          <t>chybějící díl</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>předzasilovač linky - objednán nový</t>
+        </is>
+      </c>
       <c r="F624" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21268,26 +21272,26 @@
     </row>
     <row r="625">
       <c r="A625" t="n">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B625" t="inlineStr">
         <is>
-          <t>814 073</t>
+          <t>814 003</t>
         </is>
       </c>
       <c r="C625" t="inlineStr">
         <is>
-          <t>09.07.2022</t>
+          <t>09.03.2022</t>
         </is>
       </c>
       <c r="D625" t="inlineStr">
         <is>
-          <t>chybějící díl</t>
+          <t>dosazen díl</t>
         </is>
       </c>
       <c r="E625" t="inlineStr">
         <is>
-          <t>předzasilovač linky - objednán nový</t>
+          <t>dosazen předzasilovač linky A23</t>
         </is>
       </c>
       <c r="F625" t="inlineStr">
@@ -21305,26 +21309,22 @@
     </row>
     <row r="626">
       <c r="A626" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C626" t="inlineStr">
-        <is>
-          <t>09.03.2022</t>
-        </is>
-      </c>
+          <t>844 020</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr"/>
       <c r="D626" t="inlineStr">
         <is>
-          <t>dosazen díl</t>
+          <t>oprava dveří na B pravé po směru jízdy</t>
         </is>
       </c>
       <c r="E626" t="inlineStr">
         <is>
-          <t>dosazen předzasilovač linky A23</t>
+          <t>vadný motorek</t>
         </is>
       </c>
       <c r="F626" t="inlineStr">
@@ -21342,22 +21342,22 @@
     </row>
     <row r="627">
       <c r="A627" t="n">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C627" t="inlineStr"/>
       <c r="D627" t="inlineStr">
         <is>
-          <t>oprava dveří na B pravé po směru jízdy</t>
+          <t>vadné čidlo množství písku M5</t>
         </is>
       </c>
       <c r="E627" t="inlineStr">
         <is>
-          <t>vadný motorek</t>
+          <t>2. osa pravo po smeru jizdy z B</t>
         </is>
       </c>
       <c r="F627" t="inlineStr">
@@ -21375,22 +21375,22 @@
     </row>
     <row r="628">
       <c r="A628" t="n">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C628" t="inlineStr"/>
       <c r="D628" t="inlineStr">
         <is>
-          <t>vadné čidlo množství písku M5</t>
+          <t>rychloměr dán do skladu na opravu</t>
         </is>
       </c>
       <c r="E628" t="inlineStr">
         <is>
-          <t>2. osa pravo po smeru jizdy z B</t>
+          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
         </is>
       </c>
       <c r="F628" t="inlineStr">
@@ -21408,22 +21408,22 @@
     </row>
     <row r="629">
       <c r="A629" t="n">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C629" t="inlineStr"/>
       <c r="D629" t="inlineStr">
         <is>
-          <t>rychloměr dán do skladu na opravu</t>
+          <t>rychloměr nekomunikuje</t>
         </is>
       </c>
       <c r="E629" t="inlineStr">
         <is>
-          <t>chyby 60,22,445 a 462, červený vykříčník a špatný čas při smazání poruch vše v pořádku</t>
+          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
         </is>
       </c>
       <c r="F629" t="inlineStr">
@@ -21441,22 +21441,26 @@
     </row>
     <row r="630">
       <c r="A630" t="n">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>844 022</t>
-        </is>
-      </c>
-      <c r="C630" t="inlineStr"/>
+          <t>814 003</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>10.08.2021</t>
+        </is>
+      </c>
       <c r="D630" t="inlineStr">
         <is>
-          <t>rychloměr nekomunikuje</t>
+          <t>dosazeny díly</t>
         </is>
       </c>
       <c r="E630" t="inlineStr">
         <is>
-          <t>výměna rychloněru,dosazen zapůjčený z Veselí (844 028)</t>
+          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
         </is>
       </c>
       <c r="F630" t="inlineStr">
@@ -21474,18 +21478,14 @@
     </row>
     <row r="631">
       <c r="A631" t="n">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B631" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C631" t="inlineStr">
-        <is>
-          <t>10.08.2021</t>
-        </is>
-      </c>
+      <c r="C631" t="inlineStr"/>
       <c r="D631" t="inlineStr">
         <is>
           <t>dosazeny díly</t>
@@ -21493,7 +21493,7 @@
       </c>
       <c r="E631" t="inlineStr">
         <is>
-          <t>tempo,předzesilovač A23 vezl to p.škoda</t>
+          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
         </is>
       </c>
       <c r="F631" t="inlineStr">
@@ -21511,22 +21511,26 @@
     </row>
     <row r="632">
       <c r="A632" t="n">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B632" t="inlineStr">
         <is>
           <t>814 003</t>
         </is>
       </c>
-      <c r="C632" t="inlineStr"/>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>09.06.2021</t>
+        </is>
+      </c>
       <c r="D632" t="inlineStr">
         <is>
-          <t>dosazeny díly</t>
+          <t>Chybějící díly z důvodu použití na jinou lok.</t>
         </is>
       </c>
       <c r="E632" t="inlineStr">
         <is>
-          <t>tempo na 814,mikrotelefon, zemní relé(chybí tempo 914, A23), jela do VESELÍ</t>
+          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
         </is>
       </c>
       <c r="F632" t="inlineStr">
@@ -21544,28 +21548,16 @@
     </row>
     <row r="633">
       <c r="A633" t="n">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>814 003</t>
-        </is>
-      </c>
-      <c r="C633" t="inlineStr">
-        <is>
-          <t>09.06.2021</t>
-        </is>
-      </c>
-      <c r="D633" t="inlineStr">
-        <is>
-          <t>Chybějící díly z důvodu použití na jinou lok.</t>
-        </is>
-      </c>
-      <c r="E633" t="inlineStr">
-        <is>
-          <t>Tempo,zemní relé,mikrotelefon,předzesilovač A23</t>
-        </is>
-      </c>
+          <t>842 015</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr"/>
+      <c r="D633" t="inlineStr"/>
+      <c r="E633" t="inlineStr"/>
       <c r="F633" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21581,15 +21573,19 @@
     </row>
     <row r="634">
       <c r="A634" t="n">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>842 015</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C634" t="inlineStr"/>
-      <c r="D634" t="inlineStr"/>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>výměna obrazovky Lokel na 914</t>
+        </is>
+      </c>
       <c r="E634" t="inlineStr"/>
       <c r="F634" t="inlineStr">
         <is>
@@ -21606,17 +21602,17 @@
     </row>
     <row r="635">
       <c r="A635" t="n">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>814 052</t>
         </is>
       </c>
       <c r="C635" t="inlineStr"/>
       <c r="D635" t="inlineStr">
         <is>
-          <t>výměna obrazovky Lokel na 914</t>
+          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
         </is>
       </c>
       <c r="E635" t="inlineStr"/>
@@ -21635,17 +21631,17 @@
     </row>
     <row r="636">
       <c r="A636" t="n">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>814 052</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C636" t="inlineStr"/>
       <c r="D636" t="inlineStr">
         <is>
-          <t>třepe se motor při 1200 ot/min výměna čerpadla</t>
+          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
         </is>
       </c>
       <c r="E636" t="inlineStr"/>
@@ -21664,7 +21660,7 @@
     </row>
     <row r="637">
       <c r="A637" t="n">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B637" t="inlineStr">
         <is>
@@ -21674,10 +21670,14 @@
       <c r="C637" t="inlineStr"/>
       <c r="D637" t="inlineStr">
         <is>
-          <t>byly špatně zapojeny ventily ovladáni oddílu u měchu byl ovládán z oddílu za stanovištěm opraveno 22.3.2024</t>
-        </is>
-      </c>
-      <c r="E637" t="inlineStr"/>
+          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>výměna proporciálního ventilu</t>
+        </is>
+      </c>
       <c r="F637" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21693,24 +21693,20 @@
     </row>
     <row r="638">
       <c r="A638" t="n">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>814 187</t>
         </is>
       </c>
       <c r="C638" t="inlineStr"/>
       <c r="D638" t="inlineStr">
         <is>
-          <t>špatně chladí motor závada se na brzdě neprojevila ,</t>
-        </is>
-      </c>
-      <c r="E638" t="inlineStr">
-        <is>
-          <t>výměna proporciálního ventilu</t>
-        </is>
-      </c>
+          <t>odebrany 2x obrazovka tempo</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr"/>
       <c r="F638" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21726,7 +21722,7 @@
     </row>
     <row r="639">
       <c r="A639" t="n">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B639" t="inlineStr">
         <is>
@@ -21736,7 +21732,7 @@
       <c r="C639" t="inlineStr"/>
       <c r="D639" t="inlineStr">
         <is>
-          <t>odebrany 2x obrazovka tempo</t>
+          <t>odebrana obrazovka lokel</t>
         </is>
       </c>
       <c r="E639" t="inlineStr"/>
@@ -21755,17 +21751,17 @@
     </row>
     <row r="640">
       <c r="A640" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>814 187</t>
+          <t>814 189</t>
         </is>
       </c>
       <c r="C640" t="inlineStr"/>
       <c r="D640" t="inlineStr">
         <is>
-          <t>odebrana obrazovka lokel</t>
+          <t>nefunční IS neprojevilo se</t>
         </is>
       </c>
       <c r="E640" t="inlineStr"/>
@@ -21784,20 +21780,24 @@
     </row>
     <row r="641">
       <c r="A641" t="n">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>814 189</t>
+          <t>814 118</t>
         </is>
       </c>
       <c r="C641" t="inlineStr"/>
       <c r="D641" t="inlineStr">
         <is>
-          <t>nefunční IS neprojevilo se</t>
-        </is>
-      </c>
-      <c r="E641" t="inlineStr"/>
+          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>výkon je stejný jak po poslední opravě OK</t>
+        </is>
+      </c>
       <c r="F641" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21813,7 +21813,7 @@
     </row>
     <row r="642">
       <c r="A642" t="n">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B642" t="inlineStr">
         <is>
@@ -21823,12 +21823,12 @@
       <c r="C642" t="inlineStr"/>
       <c r="D642" t="inlineStr">
         <is>
-          <t>údajně slabý výkon (nedá se sní rozjet)</t>
+          <t>vyčtení převodovky</t>
         </is>
       </c>
       <c r="E642" t="inlineStr">
         <is>
-          <t>výkon je stejný jak po poslední opravě OK</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F642" t="inlineStr">
@@ -21846,24 +21846,24 @@
     </row>
     <row r="643">
       <c r="A643" t="n">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>814 118</t>
-        </is>
-      </c>
-      <c r="C643" t="inlineStr"/>
+          <t>842 011</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>08.10.2025</t>
+        </is>
+      </c>
       <c r="D643" t="inlineStr">
         <is>
-          <t>vyčtení převodovky</t>
-        </is>
-      </c>
-      <c r="E643" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
+          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr"/>
       <c r="F643" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21879,7 +21879,7 @@
     </row>
     <row r="644">
       <c r="A644" t="n">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B644" t="inlineStr">
         <is>
@@ -21888,12 +21888,12 @@
       </c>
       <c r="C644" t="inlineStr">
         <is>
-          <t>08.10.2025</t>
+          <t>21.11.2025</t>
         </is>
       </c>
       <c r="D644" t="inlineStr">
         <is>
-          <t>start SM1 OK, SM2 asi se nevrací startér divné kvičení</t>
+          <t>dosazení ventilátoru v rozv.</t>
         </is>
       </c>
       <c r="E644" t="inlineStr"/>
@@ -21912,7 +21912,7 @@
     </row>
     <row r="645">
       <c r="A645" t="n">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B645" t="inlineStr">
         <is>
@@ -21926,7 +21926,7 @@
       </c>
       <c r="D645" t="inlineStr">
         <is>
-          <t>dosazení ventilátoru v rozv.</t>
+          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
         </is>
       </c>
       <c r="E645" t="inlineStr"/>
@@ -21945,7 +21945,7 @@
     </row>
     <row r="646">
       <c r="A646" t="n">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B646" t="inlineStr">
         <is>
@@ -21959,10 +21959,14 @@
       </c>
       <c r="D646" t="inlineStr">
         <is>
-          <t>výměna vadného stropního ventilátoru v malém oddíle</t>
-        </is>
-      </c>
-      <c r="E646" t="inlineStr"/>
+          <t>oprava ZnZ na stan. 2 nesvítila</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>vadný blok BRN02</t>
+        </is>
+      </c>
       <c r="F646" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -21978,7 +21982,7 @@
     </row>
     <row r="647">
       <c r="A647" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B647" t="inlineStr">
         <is>
@@ -21992,12 +21996,12 @@
       </c>
       <c r="D647" t="inlineStr">
         <is>
-          <t>oprava ZnZ na stan. 2 nesvítila</t>
+          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
         </is>
       </c>
       <c r="E647" t="inlineStr">
         <is>
-          <t>vadný blok BRN02</t>
+          <t>neco v hydrostatu</t>
         </is>
       </c>
       <c r="F647" t="inlineStr">
@@ -22015,7 +22019,7 @@
     </row>
     <row r="648">
       <c r="A648" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="B648" t="inlineStr">
         <is>
@@ -22029,14 +22033,10 @@
       </c>
       <c r="D648" t="inlineStr">
         <is>
-          <t>na 2. motoru nebyla závada ve startéru ale mechanicka</t>
-        </is>
-      </c>
-      <c r="E648" t="inlineStr">
-        <is>
-          <t>neco v hydrostatu</t>
-        </is>
-      </c>
+          <t>na 1. motoru jede chlazení naplno pořád</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr"/>
       <c r="F648" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22052,24 +22052,24 @@
     </row>
     <row r="649">
       <c r="A649" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>842 011</t>
-        </is>
-      </c>
-      <c r="C649" t="inlineStr">
-        <is>
-          <t>21.11.2025</t>
-        </is>
-      </c>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr"/>
       <c r="D649" t="inlineStr">
         <is>
-          <t>na 1. motoru jede chlazení naplno pořád</t>
-        </is>
-      </c>
-      <c r="E649" t="inlineStr"/>
+          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>výměna baterie v CPU DPV(vádna baterie)</t>
+        </is>
+      </c>
       <c r="F649" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22085,24 +22085,20 @@
     </row>
     <row r="650">
       <c r="A650" t="n">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 003</t>
         </is>
       </c>
       <c r="C650" t="inlineStr"/>
       <c r="D650" t="inlineStr">
         <is>
-          <t>v poruchách hlášení nesmyslné hlášky, čas i datum</t>
-        </is>
-      </c>
-      <c r="E650" t="inlineStr">
-        <is>
-          <t>výměna baterie v CPU DPV(vádna baterie)</t>
-        </is>
-      </c>
+          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr"/>
       <c r="F650" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22118,17 +22114,17 @@
     </row>
     <row r="651">
       <c r="A651" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>844 003</t>
+          <t>844 013</t>
         </is>
       </c>
       <c r="C651" t="inlineStr"/>
       <c r="D651" t="inlineStr">
         <is>
-          <t>na A zjištěny 2 čidla s nefunkčnímy ventilátory. Funkční pouze to za fírou</t>
+          <t>přehrání WiFi router firmware</t>
         </is>
       </c>
       <c r="E651" t="inlineStr"/>
@@ -22147,7 +22143,7 @@
     </row>
     <row r="652">
       <c r="A652" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B652" t="inlineStr">
         <is>
@@ -22157,10 +22153,14 @@
       <c r="C652" t="inlineStr"/>
       <c r="D652" t="inlineStr">
         <is>
-          <t>přehrání WiFi router firmware</t>
-        </is>
-      </c>
-      <c r="E652" t="inlineStr"/>
+          <t>v CAN údajně porucha požáru a klimatizace</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>neprojevillo se</t>
+        </is>
+      </c>
       <c r="F652" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22176,24 +22176,20 @@
     </row>
     <row r="653">
       <c r="A653" t="n">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>844 013</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C653" t="inlineStr"/>
       <c r="D653" t="inlineStr">
         <is>
-          <t>v CAN údajně porucha požáru a klimatizace</t>
-        </is>
-      </c>
-      <c r="E653" t="inlineStr">
-        <is>
-          <t>neprojevillo se</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr"/>
       <c r="F653" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22209,7 +22205,7 @@
     </row>
     <row r="654">
       <c r="A654" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B654" t="inlineStr">
         <is>
@@ -22219,7 +22215,7 @@
       <c r="C654" t="inlineStr"/>
       <c r="D654" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
+          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
         </is>
       </c>
       <c r="E654" t="inlineStr"/>
@@ -22238,20 +22234,24 @@
     </row>
     <row r="655">
       <c r="A655" t="n">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>844 014</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C655" t="inlineStr"/>
       <c r="D655" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 014, závada  byla na 844 025</t>
-        </is>
-      </c>
-      <c r="E655" t="inlineStr"/>
+          <t>nefunkční spřáhla</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>garance Veselí</t>
+        </is>
+      </c>
       <c r="F655" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22267,7 +22267,7 @@
     </row>
     <row r="656">
       <c r="A656" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B656" t="inlineStr">
         <is>
@@ -22277,14 +22277,10 @@
       <c r="C656" t="inlineStr"/>
       <c r="D656" t="inlineStr">
         <is>
-          <t>nefunkční spřáhla</t>
-        </is>
-      </c>
-      <c r="E656" t="inlineStr">
-        <is>
-          <t>garance Veselí</t>
-        </is>
-      </c>
+          <t>přehráni WIFI routeru firmware</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr"/>
       <c r="F656" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22300,7 +22296,7 @@
     </row>
     <row r="657">
       <c r="A657" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B657" t="inlineStr">
         <is>
@@ -22310,10 +22306,14 @@
       <c r="C657" t="inlineStr"/>
       <c r="D657" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E657" t="inlineStr"/>
+          <t>T-Webasto ukazuje 13 stupňů</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
+        </is>
+      </c>
       <c r="F657" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22329,7 +22329,7 @@
     </row>
     <row r="658">
       <c r="A658" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B658" t="inlineStr">
         <is>
@@ -22339,14 +22339,10 @@
       <c r="C658" t="inlineStr"/>
       <c r="D658" t="inlineStr">
         <is>
-          <t>T-Webasto ukazuje 13 stupňů</t>
-        </is>
-      </c>
-      <c r="E658" t="inlineStr">
-        <is>
-          <t>výměna na B čidla teploty sání, teploty byly dobré</t>
-        </is>
-      </c>
+          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr"/>
       <c r="F658" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22362,7 +22358,7 @@
     </row>
     <row r="659">
       <c r="A659" t="n">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="B659" t="inlineStr">
         <is>
@@ -22372,7 +22368,7 @@
       <c r="C659" t="inlineStr"/>
       <c r="D659" t="inlineStr">
         <is>
-          <t>v nástupním oddíle A nesvítí půlka světel výměna měniče OK</t>
+          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
         </is>
       </c>
       <c r="E659" t="inlineStr"/>
@@ -22391,7 +22387,7 @@
     </row>
     <row r="660">
       <c r="A660" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B660" t="inlineStr">
         <is>
@@ -22401,10 +22397,14 @@
       <c r="C660" t="inlineStr"/>
       <c r="D660" t="inlineStr">
         <is>
-          <t>nastaveni průměru kol ukazoval špatnou rychlost</t>
-        </is>
-      </c>
-      <c r="E660" t="inlineStr"/>
+          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>CD telematika</t>
+        </is>
+      </c>
       <c r="F660" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22420,7 +22420,7 @@
     </row>
     <row r="661">
       <c r="A661" t="n">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B661" t="inlineStr">
         <is>
@@ -22430,12 +22430,12 @@
       <c r="C661" t="inlineStr"/>
       <c r="D661" t="inlineStr">
         <is>
-          <t>výměna obrazovky radiostan a IS na A kmitala</t>
+          <t>nejdou přeředit směry na žádné straně</t>
         </is>
       </c>
       <c r="E661" t="inlineStr">
         <is>
-          <t>CD telematika</t>
+          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
         </is>
       </c>
       <c r="F661" t="inlineStr">
@@ -22453,7 +22453,7 @@
     </row>
     <row r="662">
       <c r="A662" t="n">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B662" t="inlineStr">
         <is>
@@ -22463,12 +22463,12 @@
       <c r="C662" t="inlineStr"/>
       <c r="D662" t="inlineStr">
         <is>
-          <t>nejdou přeředit směry na žádné straně</t>
+          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
         </is>
       </c>
       <c r="E662" t="inlineStr">
         <is>
-          <t>nebylo seplé rele KR10, blokovaly to vadné protismyky (lze vyčíst v programu který je aktivní</t>
+          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
         </is>
       </c>
       <c r="F662" t="inlineStr">
@@ -22486,24 +22486,20 @@
     </row>
     <row r="663">
       <c r="A663" t="n">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C663" t="inlineStr"/>
       <c r="D663" t="inlineStr">
         <is>
-          <t>zkušební jízda AŽD  na ETCS, a příjezdu do depa už nenastartovala</t>
-        </is>
-      </c>
-      <c r="E663" t="inlineStr">
-        <is>
-          <t>chyba Capos , podle chyb na měniči špatný odpor na X3 upadlý</t>
-        </is>
-      </c>
+          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr"/>
       <c r="F663" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22519,7 +22515,7 @@
     </row>
     <row r="664">
       <c r="A664" t="n">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B664" t="inlineStr">
         <is>
@@ -22529,10 +22525,14 @@
       <c r="C664" t="inlineStr"/>
       <c r="D664" t="inlineStr">
         <is>
-          <t>klimatizace na B salón často vypíná nízký tlak, výměna snímače tlaku</t>
-        </is>
-      </c>
-      <c r="E664" t="inlineStr"/>
+          <t>stále chyba AD blue</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+        </is>
+      </c>
       <c r="F664" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22548,7 +22548,7 @@
     </row>
     <row r="665">
       <c r="A665" t="n">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B665" t="inlineStr">
         <is>
@@ -22558,12 +22558,12 @@
       <c r="C665" t="inlineStr"/>
       <c r="D665" t="inlineStr">
         <is>
-          <t>stále chyba AD blue</t>
+          <t>klima A opět vysoký tlak</t>
         </is>
       </c>
       <c r="E665" t="inlineStr">
         <is>
-          <t>stále chyba ventilu močoviny a ohřívače na difuzoru (difuzorem to není), podařilo se smaazt chybu diagnostiky, černá krabička se nestihla přehodit co je nad převodovkou (žlutý konektor)</t>
+          <t>neprojevilo se</t>
         </is>
       </c>
       <c r="F665" t="inlineStr">
@@ -22581,7 +22581,7 @@
     </row>
     <row r="666">
       <c r="A666" t="n">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B666" t="inlineStr">
         <is>
@@ -22591,14 +22591,10 @@
       <c r="C666" t="inlineStr"/>
       <c r="D666" t="inlineStr">
         <is>
-          <t>klima A opět vysoký tlak</t>
-        </is>
-      </c>
-      <c r="E666" t="inlineStr">
-        <is>
-          <t>neprojevilo se</t>
-        </is>
-      </c>
+          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr"/>
       <c r="F666" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22614,17 +22610,17 @@
     </row>
     <row r="667">
       <c r="A667" t="n">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 022</t>
         </is>
       </c>
       <c r="C667" t="inlineStr"/>
       <c r="D667" t="inlineStr">
         <is>
-          <t>nejde nastartocat motor B (těžjý start, ale motor nastartoval,vyčtena chyba NOX A</t>
+          <t>přehráni WIFI routeru firmware</t>
         </is>
       </c>
       <c r="E667" t="inlineStr"/>
@@ -22643,7 +22639,7 @@
     </row>
     <row r="668">
       <c r="A668" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B668" t="inlineStr">
         <is>
@@ -22653,10 +22649,14 @@
       <c r="C668" t="inlineStr"/>
       <c r="D668" t="inlineStr">
         <is>
-          <t>přehráni WIFI routeru firmware</t>
-        </is>
-      </c>
-      <c r="E668" t="inlineStr"/>
+          <t>přehození switche z A s 844 027</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>podezřelé byly na 844 027</t>
+        </is>
+      </c>
       <c r="F668" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22672,22 +22672,22 @@
     </row>
     <row r="669">
       <c r="A669" t="n">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>844 022</t>
+          <t>844 025</t>
         </is>
       </c>
       <c r="C669" t="inlineStr"/>
       <c r="D669" t="inlineStr">
         <is>
-          <t>přehození switche z A s 844 027</t>
+          <t>vadný pedál na A</t>
         </is>
       </c>
       <c r="E669" t="inlineStr">
         <is>
-          <t>podezřelé byly na 844 027</t>
+          <t>výměna pružiny</t>
         </is>
       </c>
       <c r="F669" t="inlineStr">
@@ -22705,7 +22705,7 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
@@ -22715,12 +22715,12 @@
       <c r="C670" t="inlineStr"/>
       <c r="D670" t="inlineStr">
         <is>
-          <t>vadný pedál na A</t>
+          <t>dobíjení B za jízdy silně kmitá</t>
         </is>
       </c>
       <c r="E670" t="inlineStr">
         <is>
-          <t>výměna pružiny</t>
+          <t>klíno. Řemeny</t>
         </is>
       </c>
       <c r="F670" t="inlineStr">
@@ -22738,24 +22738,20 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>844 025</t>
+          <t>844 026</t>
         </is>
       </c>
       <c r="C671" t="inlineStr"/>
       <c r="D671" t="inlineStr">
         <is>
-          <t>dobíjení B za jízdy silně kmitá</t>
-        </is>
-      </c>
-      <c r="E671" t="inlineStr">
-        <is>
-          <t>klíno. Řemeny</t>
-        </is>
-      </c>
+          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr"/>
       <c r="F671" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22771,23 +22767,27 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>844 026</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C672" t="inlineStr"/>
       <c r="D672" t="inlineStr">
         <is>
-          <t>levé dveře na B se samy otevírají po zavření výměna kabelu motoru byl vadný</t>
-        </is>
-      </c>
-      <c r="E672" t="inlineStr"/>
+          <t>na A rozbit malý konektor ŘJ motoru</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>opraven a vyrobena provizorní krytka</t>
+        </is>
+      </c>
       <c r="F672" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G672" t="inlineStr"/>
@@ -22800,27 +22800,23 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C673" t="inlineStr"/>
       <c r="D673" t="inlineStr">
         <is>
-          <t>na A rozbit malý konektor ŘJ motoru</t>
-        </is>
-      </c>
-      <c r="E673" t="inlineStr">
-        <is>
-          <t>opraven a vyrobena provizorní krytka</t>
-        </is>
-      </c>
+          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr"/>
       <c r="F673" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G673" t="inlineStr"/>
@@ -22833,7 +22829,7 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
@@ -22843,7 +22839,7 @@
       <c r="C674" t="inlineStr"/>
       <c r="D674" t="inlineStr">
         <is>
-          <t>přehození A3.1 z 844 026 - chyba byla na 844 026</t>
+          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
         </is>
       </c>
       <c r="E674" t="inlineStr"/>
@@ -22862,7 +22858,7 @@
     </row>
     <row r="675">
       <c r="A675" t="n">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B675" t="inlineStr">
         <is>
@@ -22872,7 +22868,7 @@
       <c r="C675" t="inlineStr"/>
       <c r="D675" t="inlineStr">
         <is>
-          <t>na B dveře levé uvoněný motorek a vadné čidlo výměna</t>
+          <t>na A vadné tlačítko bdělosti výměna pravé</t>
         </is>
       </c>
       <c r="E675" t="inlineStr"/>
@@ -22891,7 +22887,7 @@
     </row>
     <row r="676">
       <c r="A676" t="n">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B676" t="inlineStr">
         <is>
@@ -22901,7 +22897,7 @@
       <c r="C676" t="inlineStr"/>
       <c r="D676" t="inlineStr">
         <is>
-          <t>na A vadné tlačítko bdělosti výměna pravé</t>
+          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
         </is>
       </c>
       <c r="E676" t="inlineStr"/>
@@ -22920,7 +22916,7 @@
     </row>
     <row r="677">
       <c r="A677" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B677" t="inlineStr">
         <is>
@@ -22930,10 +22926,14 @@
       <c r="C677" t="inlineStr"/>
       <c r="D677" t="inlineStr">
         <is>
-          <t>dveře na B pravé neotvírají ,sjetý ozubený řemen, a unašeč motoru výměna</t>
-        </is>
-      </c>
-      <c r="E677" t="inlineStr"/>
+          <t>vadné vstupní čidlo teploty výfukových plynů</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
+        </is>
+      </c>
       <c r="F677" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22949,24 +22949,20 @@
     </row>
     <row r="678">
       <c r="A678" t="n">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>954 212</t>
         </is>
       </c>
       <c r="C678" t="inlineStr"/>
       <c r="D678" t="inlineStr">
         <is>
-          <t>vadné vstupní čidlo teploty výfukových plynů</t>
-        </is>
-      </c>
-      <c r="E678" t="inlineStr">
-        <is>
-          <t>dosahovalo teploty 800 C, a kolísa skokově</t>
-        </is>
-      </c>
+          <t>nefunkční signalizace dobíjení externí</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr"/>
       <c r="F678" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -22982,7 +22978,7 @@
     </row>
     <row r="679">
       <c r="A679" t="n">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B679" t="inlineStr">
         <is>
@@ -22992,7 +22988,7 @@
       <c r="C679" t="inlineStr"/>
       <c r="D679" t="inlineStr">
         <is>
-          <t>nefunkční signalizace dobíjení externí</t>
+          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
         </is>
       </c>
       <c r="E679" t="inlineStr"/>
@@ -23011,20 +23007,24 @@
     </row>
     <row r="680">
       <c r="A680" t="n">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>954 212</t>
+          <t>954 214</t>
         </is>
       </c>
       <c r="C680" t="inlineStr"/>
       <c r="D680" t="inlineStr">
         <is>
-          <t>Oprava signazace dobíjení dosazený správný dobíječ s relé</t>
-        </is>
-      </c>
-      <c r="E680" t="inlineStr"/>
+          <t>přijea na poruchu protismyku</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>nebyla zkušebka</t>
+        </is>
+      </c>
       <c r="F680" t="inlineStr">
         <is>
           <t>Neuvedeno</t>
@@ -23040,27 +23040,23 @@
     </row>
     <row r="681">
       <c r="A681" t="n">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B681" t="inlineStr">
         <is>
-          <t>954 214</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C681" t="inlineStr"/>
       <c r="D681" t="inlineStr">
         <is>
-          <t>přijea na poruchu protismyku</t>
-        </is>
-      </c>
-      <c r="E681" t="inlineStr">
-        <is>
-          <t>nebyla zkušebka</t>
-        </is>
-      </c>
+          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr"/>
       <c r="F681" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G681" t="inlineStr"/>
@@ -23073,7 +23069,7 @@
     </row>
     <row r="682">
       <c r="A682" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B682" t="inlineStr">
         <is>
@@ -23083,7 +23079,7 @@
       <c r="C682" t="inlineStr"/>
       <c r="D682" t="inlineStr">
         <is>
-          <t>Stopnutí motoru na A 3.6.2026 výměna A2.6, nyní výměna A2.7</t>
+          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
         </is>
       </c>
       <c r="E682" t="inlineStr"/>
@@ -23102,23 +23098,27 @@
     </row>
     <row r="683">
       <c r="A683" t="n">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 190</t>
         </is>
       </c>
       <c r="C683" t="inlineStr"/>
       <c r="D683" t="inlineStr">
         <is>
-          <t>Chyba CAN a stopnutí motoru A dříve výměna A2.6 dnes A2.7</t>
-        </is>
-      </c>
-      <c r="E683" t="inlineStr"/>
+          <t>asdasda</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>asdasd</t>
+        </is>
+      </c>
       <c r="F683" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Neuvedeno</t>
         </is>
       </c>
       <c r="G683" t="inlineStr"/>
@@ -23131,27 +23131,31 @@
     </row>
     <row r="684">
       <c r="A684" t="n">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>814 190</t>
-        </is>
-      </c>
-      <c r="C684" t="inlineStr"/>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>19.08.2026</t>
+        </is>
+      </c>
       <c r="D684" t="inlineStr">
         <is>
-          <t>asdasda</t>
+          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
         </is>
       </c>
       <c r="E684" t="inlineStr">
         <is>
-          <t>asdasd</t>
+          <t>Výměna A2.7</t>
         </is>
       </c>
       <c r="F684" t="inlineStr">
         <is>
-          <t>Neuvedeno</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G684" t="inlineStr"/>
@@ -23164,11 +23168,11 @@
     </row>
     <row r="685">
       <c r="A685" t="n">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>814 143</t>
         </is>
       </c>
       <c r="C685" t="inlineStr">
@@ -23178,12 +23182,12 @@
       </c>
       <c r="D685" t="inlineStr">
         <is>
-          <t>Chyba na motoru CAN , dříve výměna A2.6</t>
+          <t>Nešly přeřadit směry</t>
         </is>
       </c>
       <c r="E685" t="inlineStr">
         <is>
-          <t>Výměna A2.7</t>
+          <t>Výměna čidla pro odblokování směru BC13</t>
         </is>
       </c>
       <c r="F685" t="inlineStr">
@@ -23201,26 +23205,26 @@
     </row>
     <row r="686">
       <c r="A686" t="n">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>814 143</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C686" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="D686" t="inlineStr">
         <is>
-          <t>Nešly přeřadit směry</t>
+          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
         </is>
       </c>
       <c r="E686" t="inlineStr">
         <is>
-          <t>Výměna čidla pro odblokování směru BC13</t>
+          <t>výměna A2.6</t>
         </is>
       </c>
       <c r="F686" t="inlineStr">
@@ -23238,31 +23242,27 @@
     </row>
     <row r="687">
       <c r="A687" t="n">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C687" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="D687" t="inlineStr">
         <is>
-          <t>červený alarm motoru A, v SE1 červeně svítí A2.6 a A2.7</t>
-        </is>
-      </c>
-      <c r="E687" t="inlineStr">
-        <is>
-          <t>výměna A2.6</t>
-        </is>
-      </c>
+          <t>Závaz motoru B</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr"/>
       <c r="F687" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G687" t="inlineStr"/>
@@ -23275,27 +23275,27 @@
     </row>
     <row r="688">
       <c r="A688" t="n">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>844 020</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C688" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>01.08.2026</t>
         </is>
       </c>
       <c r="D688" t="inlineStr">
         <is>
-          <t>Závaz motoru B</t>
+          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
         </is>
       </c>
       <c r="E688" t="inlineStr"/>
       <c r="F688" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G688" t="inlineStr"/>
@@ -23308,27 +23308,27 @@
     </row>
     <row r="689">
       <c r="A689" t="n">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C689" t="inlineStr">
         <is>
-          <t>01.08.2026</t>
+          <t>11.08.2026</t>
         </is>
       </c>
       <c r="D689" t="inlineStr">
         <is>
-          <t>Opět chybí číslo lokomotivy na provozní obrazovce</t>
+          <t>Zavaz motoru B</t>
         </is>
       </c>
       <c r="E689" t="inlineStr"/>
       <c r="F689" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G689" t="inlineStr"/>
@@ -23341,27 +23341,27 @@
     </row>
     <row r="690">
       <c r="A690" t="n">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 021</t>
         </is>
       </c>
       <c r="C690" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="D690" t="inlineStr">
         <is>
-          <t>Zavaz motoru B</t>
+          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
         </is>
       </c>
       <c r="E690" t="inlineStr"/>
       <c r="F690" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G690" t="inlineStr"/>
@@ -23374,24 +23374,28 @@
     </row>
     <row r="691">
       <c r="A691" t="n">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>844 021</t>
+          <t>954 218</t>
         </is>
       </c>
       <c r="C691" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="D691" t="inlineStr">
         <is>
-          <t>Porucha Aksel, neprovilo se pokud se bude opakovat vyměnit</t>
-        </is>
-      </c>
-      <c r="E691" t="inlineStr"/>
+          <t>Zhasínají světla v oddíle</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>výměna bíle karty XC13</t>
+        </is>
+      </c>
       <c r="F691" t="inlineStr">
         <is>
           <t>Elektrická výzbroj</t>
@@ -23407,11 +23411,11 @@
     </row>
     <row r="692">
       <c r="A692" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>954 218</t>
+          <t>842 036</t>
         </is>
       </c>
       <c r="C692" t="inlineStr">
@@ -23421,12 +23425,12 @@
       </c>
       <c r="D692" t="inlineStr">
         <is>
-          <t>Zhasínají světla v oddíle</t>
+          <t>MSV výměna BIS02</t>
         </is>
       </c>
       <c r="E692" t="inlineStr">
         <is>
-          <t>výměna bíle karty XC13</t>
+          <t>MSV</t>
         </is>
       </c>
       <c r="F692" t="inlineStr">
@@ -23444,11 +23448,11 @@
     </row>
     <row r="693">
       <c r="A693" t="n">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>842 036</t>
+          <t>842 025</t>
         </is>
       </c>
       <c r="C693" t="inlineStr">
@@ -23458,7 +23462,7 @@
       </c>
       <c r="D693" t="inlineStr">
         <is>
-          <t>MSV výměna BIS02</t>
+          <t>Výměna BIS02</t>
         </is>
       </c>
       <c r="E693" t="inlineStr">
@@ -23481,31 +23485,31 @@
     </row>
     <row r="694">
       <c r="A694" t="n">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>842 025</t>
+          <t>844 029</t>
         </is>
       </c>
       <c r="C694" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D694" t="inlineStr">
         <is>
-          <t>Výměna BIS02</t>
+          <t>Výměna spalovacího motoru na podvozku B.</t>
         </is>
       </c>
       <c r="E694" t="inlineStr">
         <is>
-          <t>MSV</t>
+          <t>závaz</t>
         </is>
       </c>
       <c r="F694" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G694" t="inlineStr"/>
@@ -23518,31 +23522,27 @@
     </row>
     <row r="695">
       <c r="A695" t="n">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
-          <t>844 029</t>
+          <t>814 188</t>
         </is>
       </c>
       <c r="C695" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>21.08.2026</t>
         </is>
       </c>
       <c r="D695" t="inlineStr">
         <is>
-          <t>Výměna spalovacího motoru na podvozku B.</t>
-        </is>
-      </c>
-      <c r="E695" t="inlineStr">
-        <is>
-          <t>závaz</t>
-        </is>
-      </c>
+          <t>Dosazení Validátorů po R1.</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr"/>
       <c r="F695" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
+          <t>IS - Infosystém</t>
         </is>
       </c>
       <c r="G695" t="inlineStr"/>
@@ -23555,27 +23555,31 @@
     </row>
     <row r="696">
       <c r="A696" t="n">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
-          <t>814 188</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C696" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D696" t="inlineStr">
         <is>
-          <t>Dosazení Validátorů po R1.</t>
-        </is>
-      </c>
-      <c r="E696" t="inlineStr"/>
+          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>Prohozní s 844 015 - A2.6</t>
+        </is>
+      </c>
       <c r="F696" t="inlineStr">
         <is>
-          <t>IS - Infosystém</t>
+          <t>Elektrická výzbroj</t>
         </is>
       </c>
       <c r="G696" t="inlineStr"/>
@@ -23588,26 +23592,22 @@
     </row>
     <row r="697">
       <c r="A697" t="n">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>844 028</t>
-        </is>
-      </c>
-      <c r="C697" t="inlineStr">
-        <is>
-          <t>22.08.2026</t>
-        </is>
-      </c>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr"/>
       <c r="D697" t="inlineStr">
         <is>
-          <t>Opět přijela na chybu can a stopnutí motoru v CANU chyba A2.6 už byla měněna</t>
+          <t>Prohození A2.6</t>
         </is>
       </c>
       <c r="E697" t="inlineStr">
         <is>
-          <t>Prohozní s 844 015 - A2.6</t>
+          <t>Prohozní s 844 028 - A2.6</t>
         </is>
       </c>
       <c r="F697" t="inlineStr">
@@ -23625,30 +23625,38 @@
     </row>
     <row r="698">
       <c r="A698" t="n">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="B698" t="inlineStr">
         <is>
           <t>844 015</t>
         </is>
       </c>
-      <c r="C698" t="inlineStr"/>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>23.08.2026</t>
+        </is>
+      </c>
       <c r="D698" t="inlineStr">
         <is>
-          <t>Prohození A2.6</t>
+          <t>Vývaz motoru "B"</t>
         </is>
       </c>
       <c r="E698" t="inlineStr">
         <is>
-          <t>Prohozní s 844 028 - A2.6</t>
+          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
         </is>
       </c>
       <c r="F698" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
-        </is>
-      </c>
-      <c r="G698" t="inlineStr"/>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
+        </is>
+      </c>
       <c r="H698" t="inlineStr"/>
       <c r="I698" t="inlineStr">
         <is>
@@ -23658,38 +23666,34 @@
     </row>
     <row r="699">
       <c r="A699" t="n">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B699" t="inlineStr">
         <is>
-          <t>844 015</t>
+          <t>814 120</t>
         </is>
       </c>
       <c r="C699" t="inlineStr">
         <is>
-          <t>23.08.2026</t>
+          <t>22.08.2026</t>
         </is>
       </c>
       <c r="D699" t="inlineStr">
         <is>
-          <t>Vývaz motoru "B"</t>
+          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
         </is>
       </c>
       <c r="E699" t="inlineStr">
         <is>
-          <t>Odpojené pojistky FU1 a FU2 na obou stranách</t>
+          <t>Vadná černá karta v bobku</t>
         </is>
       </c>
       <c r="F699" t="inlineStr">
         <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G699" t="inlineStr">
-        <is>
-          <t>https://i.ibb.co/YFxzYsgQ/9cefdcb48550.jpg</t>
-        </is>
-      </c>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G699" t="inlineStr"/>
       <c r="H699" t="inlineStr"/>
       <c r="I699" t="inlineStr">
         <is>
@@ -23699,26 +23703,26 @@
     </row>
     <row r="700">
       <c r="A700" t="n">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>814 120</t>
+          <t>844 028</t>
         </is>
       </c>
       <c r="C700" t="inlineStr">
         <is>
-          <t>22.08.2026</t>
+          <t>23.08.2026</t>
         </is>
       </c>
       <c r="D700" t="inlineStr">
         <is>
-          <t>ARR při navolení spadne zpět na 0 nebo nejde navolit</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
         </is>
       </c>
       <c r="E700" t="inlineStr">
         <is>
-          <t>Vadná černá karta v bobku</t>
+          <t>závada viz video</t>
         </is>
       </c>
       <c r="F700" t="inlineStr">
@@ -23726,7 +23730,11 @@
           <t>Elektrická výzbroj</t>
         </is>
       </c>
-      <c r="G700" t="inlineStr"/>
+      <c r="G700" t="inlineStr">
+        <is>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+        </is>
+      </c>
       <c r="H700" t="inlineStr"/>
       <c r="I700" t="inlineStr">
         <is>
@@ -23736,11 +23744,11 @@
     </row>
     <row r="701">
       <c r="A701" t="n">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>844 028</t>
+          <t>844 014</t>
         </is>
       </c>
       <c r="C701" t="inlineStr">
@@ -23750,67 +23758,26 @@
       </c>
       <c r="D701" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
         </is>
       </c>
       <c r="E701" t="inlineStr">
         <is>
-          <t>závada viz video</t>
+          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
         </is>
       </c>
       <c r="F701" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G701" t="inlineStr">
         <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_762_VID-20260823-WA0000.mp4</t>
+          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
         </is>
       </c>
       <c r="H701" t="inlineStr"/>
       <c r="I701" t="inlineStr">
-        <is>
-          <t>Radek</t>
-        </is>
-      </c>
-    </row>
-    <row r="702">
-      <c r="A702" t="n">
-        <v>763</v>
-      </c>
-      <c r="B702" t="inlineStr">
-        <is>
-          <t>844 014</t>
-        </is>
-      </c>
-      <c r="C702" t="inlineStr">
-        <is>
-          <t>23.08.2026</t>
-        </is>
-      </c>
-      <c r="D702" t="inlineStr">
-        <is>
-          <t>Ráno a odpoledne po MM červený alarm motoru B CAPOS</t>
-        </is>
-      </c>
-      <c r="E702" t="inlineStr">
-        <is>
-          <t>Po restartu jističem a reset tlačítky ok … na měniči blikala  chyba ultracap viz. video</t>
-        </is>
-      </c>
-      <c r="F702" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G702" t="inlineStr">
-        <is>
-          <t>https://cdn.jsdelivr.net/gh/truckcsgofan-p5/evidence-zavad@main/docs_zavady_videa/zavada_763_IMG_4062.mov</t>
-        </is>
-      </c>
-      <c r="H702" t="inlineStr"/>
-      <c r="I702" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Hromadná úprava z tabulky (Petr) (autor: Petr)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -23717,7 +23717,7 @@
       </c>
       <c r="D700" t="inlineStr">
         <is>
-          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna</t>
+          <t>Opět přijela na poruchu motoru A CAN , předtím výměna A2.6 a A2.7 nýní nasimulováno pomocí A2.5 vyměněna. Nepomohlo nic. Nakonec vymena a2.0</t>
         </is>
       </c>
       <c r="E700" t="inlineStr">
@@ -23738,7 +23738,7 @@
       <c r="H700" t="inlineStr"/>
       <c r="I700" t="inlineStr">
         <is>
-          <t>Radek</t>
+          <t>Petr</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Přidána nová závada ID 764 (autor: Petr)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I701"/>
+  <dimension ref="A1:I702"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23783,6 +23783,43 @@
         </is>
       </c>
     </row>
+    <row r="702">
+      <c r="A702" t="n">
+        <v>764</v>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>854 020</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>28.08.2026</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>Udajne hlasi alarm neutral a i b pri jizde z A. Vyjezd do Branek. Tam jsme popojizdeli, zavada se nepodarila nasimulovat. Fira i tak odmidl s tim jet. Zavadacse stala 28.8.cca v 13:30. V SAMech zadny cerveny alarm</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr"/>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G702" t="inlineStr"/>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>Petr</t>
+        </is>
+      </c>
+      <c r="I702" t="inlineStr">
+        <is>
+          <t>Petr</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 765 (autor: Petr)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I702"/>
+  <dimension ref="A1:I703"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23820,6 +23820,43 @@
         </is>
       </c>
     </row>
+    <row r="703">
+      <c r="A703" t="n">
+        <v>765</v>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>854 020</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>28.08.2026</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>Udajne hlasi alarm neutral a i b pri jizde z A. Vyjezd do Branek. Tam jsme popojizdeli, zavada se nepodarila nasimulovat. Fira i tak odmidl s tim jet. Zavadacse stala 28.8.cca v 13:30. V SAMech zadny cerveny alarm</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr"/>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G703" t="inlineStr"/>
+      <c r="H703" t="inlineStr">
+        <is>
+          <t>Petr</t>
+        </is>
+      </c>
+      <c r="I703" t="inlineStr">
+        <is>
+          <t>Petr</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 766 (autor: Petr)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I703"/>
+  <dimension ref="A1:I704"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23857,6 +23857,43 @@
         </is>
       </c>
     </row>
+    <row r="704">
+      <c r="A704" t="n">
+        <v>766</v>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>854 020</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>28.08.2026</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>Udajne hlasi alarm neutral a i b pri jizde z A. Vyjezd do Branek. Tam jsme popojizdeli, zavada se nepodarila nasimulovat. Fira i tak odmidl s tim jet. Zavadacse stala 28.8.cca v 13:30. V SAMech zadny cerveny alarm</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr"/>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G704" t="inlineStr"/>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>Petr</t>
+        </is>
+      </c>
+      <c r="I704" t="inlineStr">
+        <is>
+          <t>Petr</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 767 (autor: Petr)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I704"/>
+  <dimension ref="A1:I705"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23894,6 +23894,43 @@
         </is>
       </c>
     </row>
+    <row r="705">
+      <c r="A705" t="n">
+        <v>767</v>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>854 020</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>28.08.2026</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>nahlášena chybová indikace „neutrál Mtu A i B“. Při následném odzkoušení a posunu ve stanici Branky se závadu nepodařilo nasimulovat. Diagnostický systém SAM neeviduje žádný aktivní červený alarm. Strojvedoucí odmítl další jízdu s vozidlem. Rikal ze zavada se stal 28.8. cca v 13:30</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr"/>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G705" t="inlineStr"/>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>Petr</t>
+        </is>
+      </c>
+      <c r="I705" t="inlineStr">
+        <is>
+          <t>Petr</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Smazána závada ID 765 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I704"/>
+  <dimension ref="A1:I703"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23785,7 +23785,7 @@
     </row>
     <row r="702">
       <c r="A702" t="n">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
@@ -23822,11 +23822,11 @@
     </row>
     <row r="703">
       <c r="A703" t="n">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>854 020</t>
+          <t>844 020</t>
         </is>
       </c>
       <c r="C703" t="inlineStr">
@@ -23836,13 +23836,13 @@
       </c>
       <c r="D703" t="inlineStr">
         <is>
-          <t>Udajne hlasi alarm neutral a i b pri jizde z A. Vyjezd do Branek. Tam jsme popojizdeli, zavada se nepodarila nasimulovat. Fira i tak odmidl s tim jet. Zavadacse stala 28.8.cca v 13:30. V SAMech zadny cerveny alarm</t>
+          <t>nahlášena chybová indikace „neutrál Mtu A i B“. Při následném odzkoušení a posunu ve stanici Branky se závadu nepodařilo nasimulovat. Diagnostický systém SAM neeviduje žádný aktivní červený alarm. Strojvedoucí odmítl další jízdu s vozidlem. Rikal ze zavada se stal 28.8. cca v 13:30</t>
         </is>
       </c>
       <c r="E703" t="inlineStr"/>
       <c r="F703" t="inlineStr">
         <is>
-          <t>Elektrická výzbroj</t>
+          <t>Spalovací motor / Pohon</t>
         </is>
       </c>
       <c r="G703" t="inlineStr"/>
@@ -23852,43 +23852,6 @@
         </is>
       </c>
       <c r="I703" t="inlineStr">
-        <is>
-          <t>Petr</t>
-        </is>
-      </c>
-    </row>
-    <row r="704">
-      <c r="A704" t="n">
-        <v>767</v>
-      </c>
-      <c r="B704" t="inlineStr">
-        <is>
-          <t>844 020</t>
-        </is>
-      </c>
-      <c r="C704" t="inlineStr">
-        <is>
-          <t>28.08.2026</t>
-        </is>
-      </c>
-      <c r="D704" t="inlineStr">
-        <is>
-          <t>nahlášena chybová indikace „neutrál Mtu A i B“. Při následném odzkoušení a posunu ve stanici Branky se závadu nepodařilo nasimulovat. Diagnostický systém SAM neeviduje žádný aktivní červený alarm. Strojvedoucí odmítl další jízdu s vozidlem. Rikal ze zavada se stal 28.8. cca v 13:30</t>
-        </is>
-      </c>
-      <c r="E704" t="inlineStr"/>
-      <c r="F704" t="inlineStr">
-        <is>
-          <t>Spalovací motor / Pohon</t>
-        </is>
-      </c>
-      <c r="G704" t="inlineStr"/>
-      <c r="H704" t="inlineStr">
-        <is>
-          <t>Petr</t>
-        </is>
-      </c>
-      <c r="I704" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Přidána nová závada ID 768 (autor: Dan)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I703"/>
+  <dimension ref="A1:I704"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23857,6 +23857,47 @@
         </is>
       </c>
     </row>
+    <row r="704">
+      <c r="A704" t="n">
+        <v>768</v>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>814 062</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>03.09.2026</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>Nejde nastartovat z 914 -&gt; Dalibor v Kroměříži neděláno</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>Bylo to už kdysi Roman kolem toho chodil, ale neprojevilo se</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G704" t="inlineStr"/>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>Dan</t>
+        </is>
+      </c>
+      <c r="I704" t="inlineStr">
+        <is>
+          <t>Dan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 769 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I704"/>
+  <dimension ref="A1:I705"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23898,6 +23898,43 @@
         </is>
       </c>
     </row>
+    <row r="705">
+      <c r="A705" t="n">
+        <v>769</v>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>05.09.2026</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>Motor celý od AD-Blue nebyl zapojený přívod močoviny do katalyzatoru</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr"/>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G705" t="inlineStr"/>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I705" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 770 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I705"/>
+  <dimension ref="A1:I706"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23935,6 +23935,43 @@
         </is>
       </c>
     </row>
+    <row r="706">
+      <c r="A706" t="n">
+        <v>770</v>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>844 028</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>05.09.2026</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>Chlazení na A jede na plno, vypadlý konektor na proporcionálním ventilu</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr"/>
+      <c r="F706" t="inlineStr">
+        <is>
+          <t>Spalovací motor / Pohon</t>
+        </is>
+      </c>
+      <c r="G706" t="inlineStr"/>
+      <c r="H706" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I706" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Úprava závady ID 768 (autor: Dan)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -23876,17 +23876,17 @@
           <t>Nejde nastartovat z 914 -&gt; Dalibor v Kroměříži neděláno</t>
         </is>
       </c>
-      <c r="E704" t="inlineStr">
-        <is>
-          <t>Bylo to už kdysi Roman kolem toho chodil, ale neprojevilo se</t>
-        </is>
-      </c>
+      <c r="E704" t="inlineStr"/>
       <c r="F704" t="inlineStr">
         <is>
           <t>Spalovací motor / Pohon</t>
         </is>
       </c>
-      <c r="G704" t="inlineStr"/>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="H704" t="inlineStr">
         <is>
           <t>Dan</t>

</xml_diff>

<commit_message>
Úprava závady ID 769 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -23882,11 +23882,7 @@
           <t>Spalovací motor / Pohon</t>
         </is>
       </c>
-      <c r="G704" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G704" t="inlineStr"/>
       <c r="H704" t="inlineStr">
         <is>
           <t>Dan</t>
@@ -23917,13 +23913,21 @@
           <t>Motor celý od AD-Blue nebyl zapojený přívod močoviny do katalyzatoru</t>
         </is>
       </c>
-      <c r="E705" t="inlineStr"/>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="F705" t="inlineStr">
         <is>
           <t>Spalovací motor / Pohon</t>
         </is>
       </c>
-      <c r="G705" t="inlineStr"/>
+      <c r="G705" t="inlineStr">
+        <is>
+          <t>https://i.ibb.co/tTHN8bpf/d0ae6b589974.jpg</t>
+        </is>
+      </c>
       <c r="H705" t="inlineStr">
         <is>
           <t>Radek</t>

</xml_diff>

<commit_message>
Přidána nová závada ID 771 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I706"/>
+  <dimension ref="A1:I707"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23913,11 +23913,7 @@
           <t>Motor celý od AD-Blue nebyl zapojený přívod močoviny do katalyzatoru</t>
         </is>
       </c>
-      <c r="E705" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E705" t="inlineStr"/>
       <c r="F705" t="inlineStr">
         <is>
           <t>Spalovací motor / Pohon</t>
@@ -23971,6 +23967,47 @@
         </is>
       </c>
       <c r="I706" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="n">
+        <v>771</v>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>844 015</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>06.09.2026</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>Výměna ŘJ motoru B vadný konektor na ŘJ dosazená nová ze skladu (nový motor)</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>Nastavení prvního spuštění AD-Blue</t>
+        </is>
+      </c>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G707" t="inlineStr"/>
+      <c r="H707" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I707" t="inlineStr">
         <is>
           <t>Radek</t>
         </is>

</xml_diff>

<commit_message>
Přidána nová závada ID 772 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I707"/>
+  <dimension ref="A1:I708"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24013,6 +24013,43 @@
         </is>
       </c>
     </row>
+    <row r="708">
+      <c r="A708" t="n">
+        <v>772</v>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>06.09.2026</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>Hlásí korekci vody I. Motoru , nejde chlazení, vadná elektronika na cívce proporcionálního ventilu</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr"/>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G708" t="inlineStr"/>
+      <c r="H708" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I708" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 773 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I708"/>
+  <dimension ref="A1:I709"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24050,6 +24050,47 @@
         </is>
       </c>
     </row>
+    <row r="709">
+      <c r="A709" t="n">
+        <v>773</v>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>844 029</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>08.09.2026</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>Tryskami protéká voda a trysky vadné</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>výměna celého WC</t>
+        </is>
+      </c>
+      <c r="F709" t="inlineStr">
+        <is>
+          <t>WC - systém</t>
+        </is>
+      </c>
+      <c r="G709" t="inlineStr"/>
+      <c r="H709" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I709" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přidána nová závada ID 774 (autor: Radek)
</commit_message>
<xml_diff>
--- a/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
+++ b/PREDAVKA_ELEKTRONICI_PRO_APPSHEET.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I709"/>
+  <dimension ref="A1:I710"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24091,6 +24091,43 @@
         </is>
       </c>
     </row>
+    <row r="710">
+      <c r="A710" t="n">
+        <v>774</v>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>842 025</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>11.09.2026</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>Na stanovišti B nejde dát páka do souhlasu, vadný spínač pro souhlas v páce výměna</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr"/>
+      <c r="F710" t="inlineStr">
+        <is>
+          <t>Elektrická výzbroj</t>
+        </is>
+      </c>
+      <c r="G710" t="inlineStr"/>
+      <c r="H710" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+      <c r="I710" t="inlineStr">
+        <is>
+          <t>Radek</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>